<commit_message>
Wagenpark_beheer.xlsx: lease-koop gesplitst in raming en jaar activering
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013EaFTgzjMaNvZvWgFM9YZf
</commit_message>
<xml_diff>
--- a/Wagenpark_beheer.xlsx
+++ b/Wagenpark_beheer.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="153">
   <si>
     <t xml:space="preserve">Voertuigen in gebruik</t>
   </si>
@@ -41,6 +41,9 @@
     <t xml:space="preserve">Harde cijfers: betaalde prijzen of bestaande afspraken. Nieuw V-nummer: typ direct onder de tabel. Bij vervanging: regel eerst kopiëren naar 'Buiten gebruik', dan hier overschrijven.</t>
   </si>
   <si>
+    <t xml:space="preserve">Koop: kolom H (werkelijk betaald). Lease-koop: kolom I t/m L (raming op basis van contract), kolom H blijft leeg.</t>
+  </si>
+  <si>
     <t xml:space="preserve">V-nummer</t>
   </si>
   <si>
@@ -62,10 +65,19 @@
     <t xml:space="preserve">Levensduur (jaar)</t>
   </si>
   <si>
-    <t xml:space="preserve">Aanschafkosten</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lease-koop: aanbetaling / extra / slotsom</t>
+    <t xml:space="preserve">Aanschafkosten (werkelijk)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lease-koop: aanbetaling (raming)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lease-koop: bijkomende kosten (raming)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lease-koop: slotbetaling (raming)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Te activeren in jaar</t>
   </si>
   <si>
     <t xml:space="preserve">Activakaart</t>
@@ -137,9 +149,6 @@
     <t xml:space="preserve">Jilles Eikelenboom</t>
   </si>
   <si>
-    <t xml:space="preserve">11.000 / 3.420 / 30.000</t>
-  </si>
-  <si>
     <t xml:space="preserve">V07</t>
   </si>
   <si>
@@ -182,9 +191,6 @@
     <t xml:space="preserve">Antoon Kemps</t>
   </si>
   <si>
-    <t xml:space="preserve">11.000 / 0 / 35.500</t>
-  </si>
-  <si>
     <t xml:space="preserve">V12</t>
   </si>
   <si>
@@ -218,16 +224,10 @@
     <t xml:space="preserve">Pascal Jonkman</t>
   </si>
   <si>
-    <t xml:space="preserve">11.000 / 0 / 30.000</t>
-  </si>
-  <si>
     <t xml:space="preserve">V16</t>
   </si>
   <si>
     <t xml:space="preserve">Mark Oerlemans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13.310 / 0 / 36.300</t>
   </si>
   <si>
     <t xml:space="preserve">V17</t>
@@ -586,14 +586,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDDEBF7"/>
-        <bgColor rgb="FFCCFFFF"/>
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFDDEBF7"/>
+        <bgColor rgb="FFCCFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -664,11 +664,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -676,15 +680,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -692,7 +692,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -700,7 +700,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -748,7 +748,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
+          <fgColor rgb="FFFFFF00"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -756,7 +756,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
+          <fgColor rgb="FF000000"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -830,9 +830,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblBuitenGebruik" displayName="tblBuitenGebruik" ref="A4:M15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A4:M15"/>
-  <tableColumns count="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblBuitenGebruik" displayName="tblBuitenGebruik" ref="A4:P15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A4:P15"/>
+  <tableColumns count="16">
     <tableColumn id="1" name="V-nummer"/>
     <tableColumn id="2" name="Kredietnummer"/>
     <tableColumn id="3" name="Kenteken"/>
@@ -840,20 +840,23 @@
     <tableColumn id="5" name="Berijder"/>
     <tableColumn id="6" name="Aanschafjaar"/>
     <tableColumn id="7" name="Levensduur (jaar)"/>
-    <tableColumn id="8" name="Aanschafkosten"/>
-    <tableColumn id="9" name="Lease-koop: aanbetaling / extra / slotsom"/>
-    <tableColumn id="10" name="Activakaart"/>
-    <tableColumn id="11" name="Exploitatienummer"/>
-    <tableColumn id="12" name="Leasesom 1 jaar"/>
-    <tableColumn id="13" name="Jaar buiten gebruik"/>
+    <tableColumn id="8" name="Aanschafkosten (werkelijk)"/>
+    <tableColumn id="9" name="Lease-koop: aanbetaling (raming)"/>
+    <tableColumn id="10" name="Lease-koop: bijkomende kosten (raming)"/>
+    <tableColumn id="11" name="Lease-koop: slotbetaling (raming)"/>
+    <tableColumn id="12" name="Te activeren in jaar"/>
+    <tableColumn id="13" name="Activakaart"/>
+    <tableColumn id="14" name="Exploitatienummer"/>
+    <tableColumn id="15" name="Leasesom 1 jaar"/>
+    <tableColumn id="16" name="Jaar buiten gebruik"/>
   </tableColumns>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblInGebruik" displayName="tblInGebruik" ref="A4:L31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A4:L31"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblInGebruik" displayName="tblInGebruik" ref="A4:O31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A4:O31"/>
+  <tableColumns count="15">
     <tableColumn id="1" name="V-nummer"/>
     <tableColumn id="2" name="Kredietnummer"/>
     <tableColumn id="3" name="Kenteken"/>
@@ -861,11 +864,14 @@
     <tableColumn id="5" name="Berijder"/>
     <tableColumn id="6" name="Aanschafjaar"/>
     <tableColumn id="7" name="Levensduur (jaar)"/>
-    <tableColumn id="8" name="Aanschafkosten"/>
-    <tableColumn id="9" name="Lease-koop: aanbetaling / extra / slotsom"/>
-    <tableColumn id="10" name="Activakaart"/>
-    <tableColumn id="11" name="Exploitatienummer"/>
-    <tableColumn id="12" name="Leasesom 1 jaar"/>
+    <tableColumn id="8" name="Aanschafkosten (werkelijk)"/>
+    <tableColumn id="9" name="Lease-koop: aanbetaling (raming)"/>
+    <tableColumn id="10" name="Lease-koop: bijkomende kosten (raming)"/>
+    <tableColumn id="11" name="Lease-koop: slotbetaling (raming)"/>
+    <tableColumn id="12" name="Te activeren in jaar"/>
+    <tableColumn id="13" name="Activakaart"/>
+    <tableColumn id="14" name="Exploitatienummer"/>
+    <tableColumn id="15" name="Leasesom 1 jaar"/>
   </tableColumns>
 </table>
 </file>
@@ -1050,7 +1056,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:O33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -1060,10 +1066,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="8" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1076,59 +1081,73 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>7205037</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>2024</v>
@@ -1139,28 +1158,31 @@
       <c r="H5" s="7" t="n">
         <v>248960</v>
       </c>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4" t="n">
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="4" t="n">
         <v>119</v>
       </c>
-      <c r="K5" s="4"/>
-      <c r="L5" s="7"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="7"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>7205034</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>2023</v>
@@ -1171,52 +1193,58 @@
       <c r="H6" s="7" t="n">
         <v>358180</v>
       </c>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4" t="n">
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="4" t="n">
         <v>625</v>
       </c>
-      <c r="K6" s="4"/>
-      <c r="L6" s="7"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="7"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="4" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>2012</v>
       </c>
       <c r="G7" s="6"/>
       <c r="H7" s="7"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="7"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>7205035</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>2024</v>
@@ -1227,28 +1255,31 @@
       <c r="H8" s="7" t="n">
         <v>72896</v>
       </c>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4" t="n">
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="4" t="n">
         <v>632</v>
       </c>
-      <c r="K8" s="4"/>
-      <c r="L8" s="7"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="7"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>7205053</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>2021</v>
@@ -1259,26 +1290,29 @@
       <c r="H9" s="7" t="n">
         <v>65000</v>
       </c>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="L9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="7"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>7205045</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>2026</v>
@@ -1286,35 +1320,42 @@
       <c r="G10" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="H10" s="7" t="n">
-        <v>44420</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4" t="n">
+      <c r="H10" s="7"/>
+      <c r="I10" s="7" t="n">
+        <v>11000</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>3420</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L10" s="5" t="n">
+        <v>2028</v>
+      </c>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4" t="n">
         <v>635901</v>
       </c>
-      <c r="L10" s="7" t="n">
+      <c r="O10" s="7" t="n">
         <v>11786.52</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>7205051</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>2013</v>
@@ -1325,28 +1366,31 @@
       <c r="H11" s="7" t="n">
         <v>65000</v>
       </c>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4" t="n">
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="5"/>
+      <c r="M11" s="4" t="n">
         <v>803</v>
       </c>
-      <c r="K11" s="4"/>
-      <c r="L11" s="7"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="7"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B12" s="4" t="n">
         <v>7205048</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>2026</v>
@@ -1354,37 +1398,44 @@
       <c r="G12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="H12" s="7" t="n">
-        <v>44420</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="J12" s="4" t="n">
+      <c r="H12" s="7"/>
+      <c r="I12" s="7" t="n">
+        <v>11000</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>3420</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L12" s="5" t="n">
+        <v>2028</v>
+      </c>
+      <c r="M12" s="4" t="n">
         <v>648</v>
       </c>
-      <c r="K12" s="4" t="n">
+      <c r="N12" s="4" t="n">
         <v>617901</v>
       </c>
-      <c r="L12" s="7" t="n">
+      <c r="O12" s="7" t="n">
         <v>11786.52</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>7205039</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>2024</v>
@@ -1395,28 +1446,31 @@
       <c r="H13" s="7" t="n">
         <v>38664</v>
       </c>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4" t="n">
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="4" t="n">
         <v>472</v>
       </c>
-      <c r="K13" s="4"/>
-      <c r="L13" s="7"/>
+      <c r="N13" s="4"/>
+      <c r="O13" s="7"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B14" s="4" t="n">
         <v>7205043</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F14" s="5" t="n">
         <v>2025</v>
@@ -1427,26 +1481,29 @@
       <c r="H14" s="7" t="n">
         <v>30093</v>
       </c>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4" t="n">
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="4" t="n">
         <v>461</v>
       </c>
-      <c r="K14" s="4"/>
-      <c r="L14" s="7"/>
+      <c r="N14" s="4"/>
+      <c r="O14" s="7"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B15" s="4" t="n">
         <v>7205046</v>
       </c>
       <c r="C15" s="4"/>
       <c r="D15" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F15" s="5" t="n">
         <v>2026</v>
@@ -1454,35 +1511,42 @@
       <c r="G15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="H15" s="7" t="n">
-        <v>46500</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4" t="n">
+      <c r="H15" s="7"/>
+      <c r="I15" s="7" t="n">
+        <v>11000</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>35500</v>
+      </c>
+      <c r="L15" s="5" t="n">
+        <v>2028</v>
+      </c>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4" t="n">
         <v>635901</v>
       </c>
-      <c r="L15" s="7" t="n">
+      <c r="O15" s="7" t="n">
         <v>13448.5289256198</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B16" s="4" t="n">
         <v>7205044</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>2024</v>
@@ -1493,28 +1557,31 @@
       <c r="H16" s="7" t="n">
         <v>65770</v>
       </c>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4" t="n">
+      <c r="I16" s="7"/>
+      <c r="J16" s="7"/>
+      <c r="K16" s="7"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="4" t="n">
         <v>465</v>
       </c>
-      <c r="K16" s="4"/>
-      <c r="L16" s="7"/>
+      <c r="N16" s="4"/>
+      <c r="O16" s="7"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B17" s="4" t="n">
         <v>7205052</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F17" s="5" t="n">
         <v>2017</v>
@@ -1525,28 +1592,31 @@
       <c r="H17" s="7" t="n">
         <v>65000</v>
       </c>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4" t="n">
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="5"/>
+      <c r="M17" s="4" t="n">
         <v>520</v>
       </c>
-      <c r="K17" s="4"/>
-      <c r="L17" s="7"/>
+      <c r="N17" s="4"/>
+      <c r="O17" s="7"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B18" s="4" t="n">
         <v>7205058</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>2018</v>
@@ -1557,24 +1627,27 @@
       <c r="H18" s="7" t="n">
         <v>45000</v>
       </c>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
-      <c r="L18" s="7"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="7"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="4"/>
+      <c r="N18" s="4"/>
+      <c r="O18" s="7"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B19" s="4" t="n">
         <v>7205033</v>
       </c>
       <c r="C19" s="4"/>
       <c r="D19" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F19" s="5" t="n">
         <v>2026</v>
@@ -1582,35 +1655,42 @@
       <c r="G19" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="H19" s="7" t="n">
-        <v>41000</v>
-      </c>
-      <c r="I19" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="J19" s="4" t="n">
+      <c r="H19" s="7"/>
+      <c r="I19" s="7" t="n">
+        <v>11000</v>
+      </c>
+      <c r="J19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="7" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L19" s="5" t="n">
+        <v>2028</v>
+      </c>
+      <c r="M19" s="4" t="n">
         <v>463</v>
       </c>
-      <c r="K19" s="4" t="n">
+      <c r="N19" s="4" t="n">
         <v>604901</v>
       </c>
-      <c r="L19" s="7" t="n">
+      <c r="O19" s="7" t="n">
         <v>11641.6859504132</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B20" s="4" t="n">
         <v>7205032</v>
       </c>
       <c r="C20" s="4"/>
       <c r="D20" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>2026</v>
@@ -1618,19 +1698,26 @@
       <c r="G20" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="H20" s="7" t="n">
-        <v>49610</v>
-      </c>
-      <c r="I20" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="J20" s="4" t="n">
+      <c r="H20" s="7"/>
+      <c r="I20" s="7" t="n">
+        <v>13310</v>
+      </c>
+      <c r="J20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="7" t="n">
+        <v>36300</v>
+      </c>
+      <c r="L20" s="5" t="n">
+        <v>2028</v>
+      </c>
+      <c r="M20" s="4" t="n">
         <v>776</v>
       </c>
-      <c r="K20" s="4" t="n">
+      <c r="N20" s="4" t="n">
         <v>630901</v>
       </c>
-      <c r="L20" s="7" t="n">
+      <c r="O20" s="7" t="n">
         <v>14085.84</v>
       </c>
     </row>
@@ -1645,7 +1732,7 @@
         <v>66</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>67</v>
@@ -1656,19 +1743,26 @@
       <c r="G21" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="H21" s="7" t="n">
-        <v>44420</v>
-      </c>
-      <c r="I21" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="J21" s="4" t="n">
+      <c r="H21" s="7"/>
+      <c r="I21" s="7" t="n">
+        <v>11000</v>
+      </c>
+      <c r="J21" s="7" t="n">
+        <v>3420</v>
+      </c>
+      <c r="K21" s="7" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L21" s="5" t="n">
+        <v>2028</v>
+      </c>
+      <c r="M21" s="4" t="n">
         <v>647</v>
       </c>
-      <c r="K21" s="4" t="n">
+      <c r="N21" s="4" t="n">
         <v>604901</v>
       </c>
-      <c r="L21" s="7" t="n">
+      <c r="O21" s="7" t="n">
         <v>11786.52</v>
       </c>
     </row>
@@ -1683,7 +1777,7 @@
         <v>69</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E22" s="4"/>
       <c r="F22" s="5" t="n">
@@ -1695,12 +1789,15 @@
       <c r="H22" s="7" t="n">
         <v>121968</v>
       </c>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4" t="n">
+      <c r="I22" s="7"/>
+      <c r="J22" s="7"/>
+      <c r="K22" s="7"/>
+      <c r="L22" s="5"/>
+      <c r="M22" s="4" t="n">
         <v>458</v>
       </c>
-      <c r="K22" s="4"/>
-      <c r="L22" s="7"/>
+      <c r="N22" s="4"/>
+      <c r="O22" s="7"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
@@ -1713,7 +1810,7 @@
         <v>71</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>72</v>
@@ -1727,12 +1824,15 @@
       <c r="H23" s="7" t="n">
         <v>80000</v>
       </c>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4" t="n">
+      <c r="I23" s="7"/>
+      <c r="J23" s="7"/>
+      <c r="K23" s="7"/>
+      <c r="L23" s="5"/>
+      <c r="M23" s="4" t="n">
         <v>823</v>
       </c>
-      <c r="K23" s="4"/>
-      <c r="L23" s="7"/>
+      <c r="N23" s="4"/>
+      <c r="O23" s="7"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
@@ -1743,7 +1843,7 @@
         <v>74</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>72</v>
@@ -1757,10 +1857,13 @@
       <c r="H24" s="7" t="n">
         <v>100000</v>
       </c>
-      <c r="I24" s="4"/>
-      <c r="J24" s="4"/>
-      <c r="K24" s="4"/>
-      <c r="L24" s="7"/>
+      <c r="I24" s="7"/>
+      <c r="J24" s="7"/>
+      <c r="K24" s="7"/>
+      <c r="L24" s="5"/>
+      <c r="M24" s="4"/>
+      <c r="N24" s="4"/>
+      <c r="O24" s="7"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
@@ -1773,7 +1876,7 @@
         <v>76</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>72</v>
@@ -1787,12 +1890,15 @@
       <c r="H25" s="7" t="n">
         <v>51100</v>
       </c>
-      <c r="I25" s="4"/>
-      <c r="J25" s="4" t="n">
+      <c r="I25" s="7"/>
+      <c r="J25" s="7"/>
+      <c r="K25" s="7"/>
+      <c r="L25" s="5"/>
+      <c r="M25" s="4" t="n">
         <v>518</v>
       </c>
-      <c r="K25" s="4"/>
-      <c r="L25" s="7"/>
+      <c r="N25" s="4"/>
+      <c r="O25" s="7"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
@@ -1803,7 +1909,7 @@
         <v>78</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>72</v>
@@ -1817,10 +1923,13 @@
       <c r="H26" s="7" t="n">
         <v>19000</v>
       </c>
-      <c r="I26" s="4"/>
-      <c r="J26" s="4"/>
-      <c r="K26" s="4"/>
-      <c r="L26" s="7"/>
+      <c r="I26" s="7"/>
+      <c r="J26" s="7"/>
+      <c r="K26" s="7"/>
+      <c r="L26" s="5"/>
+      <c r="M26" s="4"/>
+      <c r="N26" s="4"/>
+      <c r="O26" s="7"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
@@ -1833,7 +1942,7 @@
         <v>78</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>72</v>
@@ -1847,10 +1956,13 @@
       <c r="H27" s="7" t="n">
         <v>50000</v>
       </c>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
-      <c r="L27" s="7"/>
+      <c r="I27" s="7"/>
+      <c r="J27" s="7"/>
+      <c r="K27" s="7"/>
+      <c r="L27" s="5"/>
+      <c r="M27" s="4"/>
+      <c r="N27" s="4"/>
+      <c r="O27" s="7"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
@@ -1863,7 +1975,7 @@
         <v>81</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>82</v>
@@ -1877,10 +1989,13 @@
       <c r="H28" s="7" t="n">
         <v>45000</v>
       </c>
-      <c r="I28" s="4"/>
-      <c r="J28" s="4"/>
-      <c r="K28" s="4"/>
-      <c r="L28" s="7"/>
+      <c r="I28" s="7"/>
+      <c r="J28" s="7"/>
+      <c r="K28" s="7"/>
+      <c r="L28" s="5"/>
+      <c r="M28" s="4"/>
+      <c r="N28" s="4"/>
+      <c r="O28" s="7"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
@@ -1893,7 +2008,7 @@
         <v>84</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E29" s="4" t="s">
         <v>82</v>
@@ -1907,10 +2022,13 @@
       <c r="H29" s="7" t="n">
         <v>45000</v>
       </c>
-      <c r="I29" s="4"/>
-      <c r="J29" s="4"/>
-      <c r="K29" s="4"/>
-      <c r="L29" s="7"/>
+      <c r="I29" s="7"/>
+      <c r="J29" s="7"/>
+      <c r="K29" s="7"/>
+      <c r="L29" s="5"/>
+      <c r="M29" s="4"/>
+      <c r="N29" s="4"/>
+      <c r="O29" s="7"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
@@ -1921,7 +2039,7 @@
         <v>86</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>87</v>
@@ -1932,13 +2050,16 @@
       <c r="G30" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="H30" s="7" t="n">
-        <v>30000</v>
-      </c>
-      <c r="I30" s="4"/>
-      <c r="J30" s="4"/>
-      <c r="K30" s="4"/>
-      <c r="L30" s="7"/>
+      <c r="H30" s="7"/>
+      <c r="I30" s="8"/>
+      <c r="J30" s="8"/>
+      <c r="K30" s="8"/>
+      <c r="L30" s="5" t="n">
+        <v>2028</v>
+      </c>
+      <c r="M30" s="4"/>
+      <c r="N30" s="4"/>
+      <c r="O30" s="7"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
@@ -1951,7 +2072,7 @@
         <v>89</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>82</v>
@@ -1965,20 +2086,35 @@
       <c r="H31" s="7" t="n">
         <v>41530</v>
       </c>
-      <c r="I31" s="4"/>
-      <c r="J31" s="4" t="n">
+      <c r="I31" s="7"/>
+      <c r="J31" s="7"/>
+      <c r="K31" s="7"/>
+      <c r="L31" s="5"/>
+      <c r="M31" s="4" t="n">
         <v>631</v>
       </c>
-      <c r="K31" s="4"/>
-      <c r="L31" s="7"/>
+      <c r="N31" s="4"/>
+      <c r="O31" s="7"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G33" s="8" t="s">
+      <c r="G33" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="H33" s="9" t="n">
+      <c r="H33" s="10" t="n">
         <f aca="false">SUBTOTAL(109,H5:H31)</f>
-        <v>1908531</v>
+        <v>1608161</v>
+      </c>
+      <c r="I33" s="10" t="n">
+        <f aca="false">SUBTOTAL(109,I5:I31)</f>
+        <v>68310</v>
+      </c>
+      <c r="J33" s="10" t="n">
+        <f aca="false">SUBTOTAL(109,J5:J31)</f>
+        <v>10260</v>
+      </c>
+      <c r="K33" s="10" t="n">
+        <f aca="false">SUBTOTAL(109,K5:K31)</f>
+        <v>191800</v>
       </c>
     </row>
   </sheetData>
@@ -2027,18 +2163,18 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="9" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="C4" s="11" t="n">
+      <c r="C4" s="8" t="n">
         <v>10000</v>
       </c>
       <c r="F4" s="12" t="n">
@@ -2074,13 +2210,13 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="8" t="n">
         <v>5000</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="11" t="s">
         <v>97</v>
       </c>
       <c r="F5" s="14" t="n">
@@ -2117,13 +2253,13 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="C6" s="11" t="n">
+      <c r="C6" s="8" t="n">
         <v>7000</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="11" t="s">
         <v>99</v>
       </c>
       <c r="F6" s="14" t="n">
@@ -2160,10 +2296,10 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="C7" s="11" t="n">
+      <c r="C7" s="8" t="n">
         <v>35000</v>
       </c>
       <c r="E7" s="2" t="s">
@@ -2171,7 +2307,7 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="11" t="s">
         <v>102</v>
       </c>
       <c r="C8" s="12" t="n">
@@ -2182,7 +2318,7 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="11" t="s">
         <v>104</v>
       </c>
       <c r="C9" s="12" t="n">
@@ -2190,7 +2326,7 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="11" t="s">
         <v>105</v>
       </c>
       <c r="C10" s="12" t="n">
@@ -2198,25 +2334,25 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="8" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J15" s="8" t="s">
+      <c r="J15" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="K15" s="9" t="n">
+      <c r="K15" s="10" t="n">
         <f aca="false">SUM($K$17:$K$96)</f>
         <v>2047208</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>107</v>
@@ -2225,7 +2361,7 @@
         <v>108</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>109</v>
@@ -2263,11 +2399,11 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B17" s="15"/>
       <c r="C17" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>2027</v>
@@ -2317,11 +2453,11 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B18" s="15"/>
       <c r="C18" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>2027</v>
@@ -2371,11 +2507,11 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B19" s="15"/>
       <c r="C19" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D19" s="5" t="n">
         <v>2027</v>
@@ -2425,7 +2561,7 @@
       </c>
       <c r="B20" s="15"/>
       <c r="C20" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>2027</v>
@@ -2477,7 +2613,7 @@
       </c>
       <c r="B21" s="15"/>
       <c r="C21" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D21" s="5" t="n">
         <v>2027</v>
@@ -2531,7 +2667,7 @@
       </c>
       <c r="B22" s="15"/>
       <c r="C22" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D22" s="5" t="n">
         <v>2027</v>
@@ -2585,7 +2721,7 @@
       </c>
       <c r="B23" s="15"/>
       <c r="C23" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D23" s="5" t="n">
         <v>2028</v>
@@ -2635,11 +2771,11 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B24" s="15"/>
       <c r="C24" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D24" s="5" t="n">
         <v>2029</v>
@@ -2689,7 +2825,7 @@
       </c>
       <c r="B25" s="15"/>
       <c r="C25" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D25" s="5" t="n">
         <v>2029</v>
@@ -2741,7 +2877,7 @@
       </c>
       <c r="B26" s="15"/>
       <c r="C26" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D26" s="5" t="n">
         <v>2031</v>
@@ -2787,11 +2923,11 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B27" s="15"/>
       <c r="C27" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D27" s="5" t="n">
         <v>2032</v>
@@ -2839,7 +2975,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>123</v>
@@ -2890,11 +3026,11 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B29" s="15"/>
       <c r="C29" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D29" s="5" t="n">
         <v>2032</v>
@@ -2940,11 +3076,11 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B30" s="15"/>
       <c r="C30" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D30" s="5" t="n">
         <v>2032</v>
@@ -2990,11 +3126,11 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B31" s="15"/>
       <c r="C31" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D31" s="5" t="n">
         <v>2032</v>
@@ -3040,11 +3176,11 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B32" s="15"/>
       <c r="C32" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D32" s="5" t="n">
         <v>2033</v>
@@ -3094,7 +3230,7 @@
       </c>
       <c r="B33" s="15"/>
       <c r="C33" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D33" s="5" t="n">
         <v>2033</v>
@@ -3142,11 +3278,11 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B34" s="15"/>
       <c r="C34" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D34" s="5" t="n">
         <v>2034</v>
@@ -3192,11 +3328,11 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B35" s="15"/>
       <c r="C35" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D35" s="5" t="n">
         <v>2034</v>
@@ -3242,11 +3378,11 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B36" s="15"/>
       <c r="C36" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D36" s="5" t="n">
         <v>2034</v>
@@ -3292,11 +3428,11 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B37" s="15"/>
       <c r="C37" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D37" s="5" t="n">
         <v>2034</v>
@@ -3342,11 +3478,11 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B38" s="15"/>
       <c r="C38" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D38" s="5" t="n">
         <v>2034</v>
@@ -3396,7 +3532,7 @@
       </c>
       <c r="B39" s="15"/>
       <c r="C39" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D39" s="5" t="n">
         <v>2034</v>
@@ -3446,7 +3582,7 @@
       </c>
       <c r="B40" s="15"/>
       <c r="C40" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D40" s="5" t="n">
         <v>2034</v>
@@ -3498,7 +3634,7 @@
       </c>
       <c r="B41" s="15"/>
       <c r="C41" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D41" s="5" t="n">
         <v>2034</v>
@@ -3544,11 +3680,11 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B42" s="15"/>
       <c r="C42" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D42" s="5" t="n">
         <v>2035</v>
@@ -3600,7 +3736,7 @@
       </c>
       <c r="B43" s="15"/>
       <c r="C43" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D43" s="5" t="n">
         <v>2038</v>
@@ -5790,7 +5926,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:P15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -5800,11 +5936,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="8" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5819,58 +5954,67 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="P4" s="3" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4" t="s">
         <v>128</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>2014</v>
@@ -5879,27 +6023,30 @@
         <v>8</v>
       </c>
       <c r="H5" s="7"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="7"/>
-      <c r="M5" s="5" t="n">
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="5" t="n">
         <v>2026</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4" t="s">
         <v>129</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>2018</v>
@@ -5908,27 +6055,30 @@
         <v>8</v>
       </c>
       <c r="H6" s="7"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="5" t="n">
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="7"/>
+      <c r="P6" s="5" t="n">
         <v>2026</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="4" t="s">
         <v>130</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>2013</v>
@@ -5937,11 +6087,14 @@
         <v>8</v>
       </c>
       <c r="H7" s="7"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="5" t="n">
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="7"/>
+      <c r="P7" s="5" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -5956,7 +6109,7 @@
         <v>131</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>87</v>
@@ -5970,11 +6123,14 @@
       <c r="H8" s="7" t="n">
         <v>80000</v>
       </c>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="5" t="n">
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="7"/>
+      <c r="P8" s="5" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -5988,7 +6144,7 @@
       </c>
       <c r="D9" s="4"/>
       <c r="E9" s="4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>2007</v>
@@ -5999,11 +6155,14 @@
       <c r="H9" s="7" t="n">
         <v>65000</v>
       </c>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="L9" s="7"/>
-      <c r="M9" s="5" t="n">
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="7"/>
+      <c r="P9" s="5" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -6028,13 +6187,16 @@
       <c r="H10" s="7" t="n">
         <v>43000</v>
       </c>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4" t="s">
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="K10" s="4"/>
-      <c r="L10" s="7"/>
-      <c r="M10" s="17"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="7"/>
+      <c r="P10" s="17"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
@@ -6057,13 +6219,16 @@
       <c r="H11" s="7" t="n">
         <v>240000</v>
       </c>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4" t="s">
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="5"/>
+      <c r="M11" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="K11" s="4"/>
-      <c r="L11" s="7"/>
-      <c r="M11" s="17"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="7"/>
+      <c r="P11" s="17"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
@@ -6086,11 +6251,14 @@
       <c r="H12" s="7" t="n">
         <v>65000</v>
       </c>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="7"/>
-      <c r="M12" s="5" t="n">
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="5"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4"/>
+      <c r="O12" s="7"/>
+      <c r="P12" s="5" t="n">
         <v>2027</v>
       </c>
     </row>
@@ -6115,11 +6283,14 @@
       <c r="H13" s="7" t="n">
         <v>65000</v>
       </c>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
-      <c r="L13" s="7"/>
-      <c r="M13" s="5" t="n">
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="4"/>
+      <c r="N13" s="4"/>
+      <c r="O13" s="7"/>
+      <c r="P13" s="5" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -6142,11 +6313,14 @@
       <c r="H14" s="7" t="n">
         <v>65000</v>
       </c>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="7"/>
-      <c r="M14" s="5" t="n">
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="4"/>
+      <c r="N14" s="4"/>
+      <c r="O14" s="7"/>
+      <c r="P14" s="5" t="n">
         <v>2027</v>
       </c>
     </row>
@@ -6171,13 +6345,16 @@
       <c r="H15" s="7" t="n">
         <v>72000</v>
       </c>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4" t="s">
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="7"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="K15" s="4"/>
-      <c r="L15" s="7"/>
-      <c r="M15" s="17"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="7"/>
+      <c r="P15" s="17"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Wagenpark_beheer.xlsx: slotbetalingen vanaf 2027 op gemiddelde
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013EaFTgzjMaNvZvWgFM9YZf
</commit_message>
<xml_diff>
--- a/Wagenpark_beheer.xlsx
+++ b/Wagenpark_beheer.xlsx
@@ -41,7 +41,7 @@
     <t xml:space="preserve">Harde cijfers: betaalde prijzen of bestaande afspraken. Nieuw V-nummer: typ direct onder de tabel. Bij vervanging: regel eerst kopiëren naar 'Buiten gebruik', dan hier overschrijven.</t>
   </si>
   <si>
-    <t xml:space="preserve">Koop: kolom H (werkelijk betaald). Lease-koop: kolom I t/m L (raming op basis van contract), kolom H blijft leeg.</t>
+    <t xml:space="preserve">Koop: kolom H (werkelijk betaald). Lease-koop: kolom I t/m L, kolom H blijft leeg. Uitgaven vanaf 2027 = gemiddelde (groen), overschrijven met werkelijke uitgave zodra bekend.</t>
   </si>
   <si>
     <t xml:space="preserve">V-nummer</t>
@@ -504,7 +504,7 @@
     <numFmt numFmtId="166" formatCode="0"/>
     <numFmt numFmtId="167" formatCode="&quot;€ &quot;#,##0;&quot;-€ &quot;#,##0;\-"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -553,6 +553,13 @@
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF008000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -631,7 +638,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -664,15 +671,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -680,15 +683,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -696,7 +707,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -713,7 +724,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -749,6 +760,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF008000"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1327,8 +1346,9 @@
       <c r="J10" s="7" t="n">
         <v>3420</v>
       </c>
-      <c r="K10" s="7" t="n">
-        <v>30000</v>
+      <c r="K10" s="8" t="n">
+        <f aca="false">p_Slot</f>
+        <v>35000</v>
       </c>
       <c r="L10" s="5" t="n">
         <v>2028</v>
@@ -1405,8 +1425,9 @@
       <c r="J12" s="7" t="n">
         <v>3420</v>
       </c>
-      <c r="K12" s="7" t="n">
-        <v>30000</v>
+      <c r="K12" s="8" t="n">
+        <f aca="false">p_Slot</f>
+        <v>35000</v>
       </c>
       <c r="L12" s="5" t="n">
         <v>2028</v>
@@ -1518,8 +1539,9 @@
       <c r="J15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="7" t="n">
-        <v>35500</v>
+      <c r="K15" s="8" t="n">
+        <f aca="false">p_Slot</f>
+        <v>35000</v>
       </c>
       <c r="L15" s="5" t="n">
         <v>2028</v>
@@ -1662,8 +1684,9 @@
       <c r="J19" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="7" t="n">
-        <v>30000</v>
+      <c r="K19" s="8" t="n">
+        <f aca="false">p_Slot</f>
+        <v>35000</v>
       </c>
       <c r="L19" s="5" t="n">
         <v>2028</v>
@@ -1705,8 +1728,9 @@
       <c r="J20" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="K20" s="7" t="n">
-        <v>36300</v>
+      <c r="K20" s="8" t="n">
+        <f aca="false">p_Slot</f>
+        <v>35000</v>
       </c>
       <c r="L20" s="5" t="n">
         <v>2028</v>
@@ -1750,8 +1774,9 @@
       <c r="J21" s="7" t="n">
         <v>3420</v>
       </c>
-      <c r="K21" s="7" t="n">
-        <v>30000</v>
+      <c r="K21" s="8" t="n">
+        <f aca="false">p_Slot</f>
+        <v>35000</v>
       </c>
       <c r="L21" s="5" t="n">
         <v>2028</v>
@@ -2051,9 +2076,12 @@
         <v>8</v>
       </c>
       <c r="H30" s="7"/>
-      <c r="I30" s="8"/>
-      <c r="J30" s="8"/>
-      <c r="K30" s="8"/>
+      <c r="I30" s="9"/>
+      <c r="J30" s="9"/>
+      <c r="K30" s="8" t="n">
+        <f aca="false">p_Slot</f>
+        <v>35000</v>
+      </c>
       <c r="L30" s="5" t="n">
         <v>2028</v>
       </c>
@@ -2097,24 +2125,24 @@
       <c r="O31" s="7"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G33" s="9" t="s">
+      <c r="G33" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="H33" s="10" t="n">
+      <c r="H33" s="11" t="n">
         <f aca="false">SUBTOTAL(109,H5:H31)</f>
         <v>1608161</v>
       </c>
-      <c r="I33" s="10" t="n">
+      <c r="I33" s="11" t="n">
         <f aca="false">SUBTOTAL(109,I5:I31)</f>
         <v>68310</v>
       </c>
-      <c r="J33" s="10" t="n">
+      <c r="J33" s="11" t="n">
         <f aca="false">SUBTOTAL(109,J5:J31)</f>
         <v>10260</v>
       </c>
-      <c r="K33" s="10" t="n">
+      <c r="K33" s="11" t="n">
         <f aca="false">SUBTOTAL(109,K5:K31)</f>
-        <v>191800</v>
+        <v>245000</v>
       </c>
     </row>
   </sheetData>
@@ -2163,143 +2191,143 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="10" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="C4" s="8" t="n">
+      <c r="C4" s="9" t="n">
         <v>10000</v>
       </c>
-      <c r="F4" s="12" t="n">
+      <c r="F4" s="13" t="n">
         <v>2027</v>
       </c>
-      <c r="G4" s="13" t="n">
+      <c r="G4" s="14" t="n">
         <f aca="false">F4+1</f>
         <v>2028</v>
       </c>
-      <c r="H4" s="13" t="n">
+      <c r="H4" s="14" t="n">
         <f aca="false">G4+1</f>
         <v>2029</v>
       </c>
-      <c r="I4" s="13" t="n">
+      <c r="I4" s="14" t="n">
         <f aca="false">H4+1</f>
         <v>2030</v>
       </c>
-      <c r="J4" s="13" t="n">
+      <c r="J4" s="14" t="n">
         <f aca="false">I4+1</f>
         <v>2031</v>
       </c>
-      <c r="K4" s="13" t="n">
+      <c r="K4" s="14" t="n">
         <f aca="false">J4+1</f>
         <v>2032</v>
       </c>
-      <c r="L4" s="13" t="n">
+      <c r="L4" s="14" t="n">
         <f aca="false">K4+1</f>
         <v>2033</v>
       </c>
-      <c r="M4" s="13" t="n">
+      <c r="M4" s="14" t="n">
         <f aca="false">L4+1</f>
         <v>2034</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="C5" s="8" t="n">
+      <c r="C5" s="9" t="n">
         <v>5000</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="F5" s="14" t="n">
+      <c r="F5" s="15" t="n">
         <f aca="false">SUMIF($D$17:$D$96,F$4,$E$17:$E$96)+SUMIF($D$17:$D$96,F$4,$F$17:$F$96)+SUMIF($D$17:$D$96,F$4,$G$17:$G$96)+SUMIF($D$17:$D$96,F$4,$H$17:$H$96)+SUMIF($J$17:$J$96,F$4,$I$17:$I$96)</f>
         <v>322000</v>
       </c>
-      <c r="G5" s="14" t="n">
+      <c r="G5" s="15" t="n">
         <f aca="false">SUMIF($D$17:$D$96,G$4,$E$17:$E$96)+SUMIF($D$17:$D$96,G$4,$F$17:$F$96)+SUMIF($D$17:$D$96,G$4,$G$17:$G$96)+SUMIF($D$17:$D$96,G$4,$H$17:$H$96)+SUMIF($J$17:$J$96,G$4,$I$17:$I$96)</f>
         <v>50000</v>
       </c>
-      <c r="H5" s="14" t="n">
+      <c r="H5" s="15" t="n">
         <f aca="false">SUMIF($D$17:$D$96,H$4,$E$17:$E$96)+SUMIF($D$17:$D$96,H$4,$F$17:$F$96)+SUMIF($D$17:$D$96,H$4,$G$17:$G$96)+SUMIF($D$17:$D$96,H$4,$H$17:$H$96)+SUMIF($J$17:$J$96,H$4,$I$17:$I$96)</f>
         <v>157000</v>
       </c>
-      <c r="I5" s="14" t="n">
+      <c r="I5" s="15" t="n">
         <f aca="false">SUMIF($D$17:$D$96,I$4,$E$17:$E$96)+SUMIF($D$17:$D$96,I$4,$F$17:$F$96)+SUMIF($D$17:$D$96,I$4,$G$17:$G$96)+SUMIF($D$17:$D$96,I$4,$H$17:$H$96)+SUMIF($J$17:$J$96,I$4,$I$17:$I$96)</f>
         <v>0</v>
       </c>
-      <c r="J5" s="14" t="n">
+      <c r="J5" s="15" t="n">
         <f aca="false">SUMIF($D$17:$D$96,J$4,$E$17:$E$96)+SUMIF($D$17:$D$96,J$4,$F$17:$F$96)+SUMIF($D$17:$D$96,J$4,$G$17:$G$96)+SUMIF($D$17:$D$96,J$4,$H$17:$H$96)+SUMIF($J$17:$J$96,J$4,$I$17:$I$96)</f>
         <v>57000</v>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="K5" s="15" t="n">
         <f aca="false">SUMIF($D$17:$D$96,K$4,$E$17:$E$96)+SUMIF($D$17:$D$96,K$4,$F$17:$F$96)+SUMIF($D$17:$D$96,K$4,$G$17:$G$96)+SUMIF($D$17:$D$96,K$4,$H$17:$H$96)+SUMIF($J$17:$J$96,K$4,$I$17:$I$96)</f>
         <v>314960</v>
       </c>
-      <c r="L5" s="14" t="n">
+      <c r="L5" s="15" t="n">
         <f aca="false">SUMIF($D$17:$D$96,L$4,$E$17:$E$96)+SUMIF($D$17:$D$96,L$4,$F$17:$F$96)+SUMIF($D$17:$D$96,L$4,$G$17:$G$96)+SUMIF($D$17:$D$96,L$4,$H$17:$H$96)+SUMIF($J$17:$J$96,L$4,$I$17:$I$96)</f>
         <v>76000</v>
       </c>
-      <c r="M5" s="14" t="n">
+      <c r="M5" s="15" t="n">
         <f aca="false">SUMIF($D$17:$D$96,M$4,$E$17:$E$96)+SUMIF($D$17:$D$96,M$4,$F$17:$F$96)+SUMIF($D$17:$D$96,M$4,$G$17:$G$96)+SUMIF($D$17:$D$96,M$4,$H$17:$H$96)+SUMIF($J$17:$J$96,M$4,$I$17:$I$96)</f>
         <v>310100</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="9" t="n">
         <v>7000</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="F6" s="14" t="n">
+      <c r="F6" s="15" t="n">
         <f aca="false">SUMPRODUCT(($C$17:$C$96="Lease-koop")*($D$17:$D$96&lt;=F$4)*($J$17:$J$96&gt;F$4)*$N$17:$N$96)</f>
         <v>12000</v>
       </c>
-      <c r="G6" s="14" t="n">
+      <c r="G6" s="15" t="n">
         <f aca="false">SUMPRODUCT(($C$17:$C$96="Lease-koop")*($D$17:$D$96&lt;=G$4)*($J$17:$J$96&gt;G$4)*$N$17:$N$96)</f>
         <v>12000</v>
       </c>
-      <c r="H6" s="14" t="n">
+      <c r="H6" s="15" t="n">
         <f aca="false">SUMPRODUCT(($C$17:$C$96="Lease-koop")*($D$17:$D$96&lt;=H$4)*($J$17:$J$96&gt;H$4)*$N$17:$N$96)</f>
         <v>12000</v>
       </c>
-      <c r="I6" s="14" t="n">
+      <c r="I6" s="15" t="n">
         <f aca="false">SUMPRODUCT(($C$17:$C$96="Lease-koop")*($D$17:$D$96&lt;=I$4)*($J$17:$J$96&gt;I$4)*$N$17:$N$96)</f>
         <v>12000</v>
       </c>
-      <c r="J6" s="14" t="n">
+      <c r="J6" s="15" t="n">
         <f aca="false">SUMPRODUCT(($C$17:$C$96="Lease-koop")*($D$17:$D$96&lt;=J$4)*($J$17:$J$96&gt;J$4)*$N$17:$N$96)</f>
         <v>12000</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="K6" s="15" t="n">
         <f aca="false">SUMPRODUCT(($C$17:$C$96="Lease-koop")*($D$17:$D$96&lt;=K$4)*($J$17:$J$96&gt;K$4)*$N$17:$N$96)</f>
         <v>48000</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="L6" s="15" t="n">
         <f aca="false">SUMPRODUCT(($C$17:$C$96="Lease-koop")*($D$17:$D$96&lt;=L$4)*($J$17:$J$96&gt;L$4)*$N$17:$N$96)</f>
         <v>48000</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="M6" s="15" t="n">
         <f aca="false">SUMPRODUCT(($C$17:$C$96="Lease-koop")*($D$17:$D$96&lt;=M$4)*($J$17:$J$96&gt;M$4)*$N$17:$N$96)</f>
         <v>96000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="C7" s="8" t="n">
+      <c r="C7" s="9" t="n">
         <v>35000</v>
       </c>
       <c r="E7" s="2" t="s">
@@ -2307,10 +2335,10 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="13" t="n">
         <v>2</v>
       </c>
       <c r="E8" s="2" t="s">
@@ -2318,34 +2346,34 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="13" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="13" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="C11" s="8" t="n">
+      <c r="C11" s="9" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J15" s="9" t="s">
+      <c r="J15" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="K15" s="10" t="n">
+      <c r="K15" s="11" t="n">
         <f aca="false">SUM($K$17:$K$96)</f>
         <v>2047208</v>
       </c>
@@ -2401,49 +2429,49 @@
       <c r="A17" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B17" s="15"/>
+      <c r="B17" s="16"/>
       <c r="C17" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>2027</v>
       </c>
-      <c r="E17" s="14" t="n">
+      <c r="E17" s="15" t="n">
         <f aca="false">IF($C17="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F17" s="14" t="n">
+      <c r="F17" s="15" t="n">
         <f aca="false">IF($C17="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G17" s="14" t="n">
+      <c r="G17" s="15" t="n">
         <f aca="false">IF($C17="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>65000</v>
       </c>
-      <c r="I17" s="14" t="n">
+      <c r="I17" s="15" t="n">
         <f aca="false">IF($C17="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J17" s="16" t="n">
+      <c r="J17" s="17" t="n">
         <f aca="false">IF($C17="Lease-koop",D17+p_SlotJr,IF($C17="Koop",D17,0))</f>
         <v>2027</v>
       </c>
-      <c r="K17" s="14" t="n">
+      <c r="K17" s="15" t="n">
         <f aca="false">E17+F17+G17+H17+I17</f>
         <v>65000</v>
       </c>
-      <c r="L17" s="16" t="n">
+      <c r="L17" s="17" t="n">
         <f aca="false">IF($C17="Lease-koop",p_Afschr,IF($C17="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A17,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>8</v>
       </c>
-      <c r="M17" s="16" t="n">
+      <c r="M17" s="17" t="n">
         <f aca="false">IF($C17="Lease-koop",D17+p_Lev,IF(AND($C17="Koop",D17&gt;0),D17+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A17,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2035</v>
       </c>
-      <c r="N17" s="14" t="n">
+      <c r="N17" s="15" t="n">
         <f aca="false">IF($C17="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -2455,49 +2483,49 @@
       <c r="A18" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="15"/>
+      <c r="B18" s="16"/>
       <c r="C18" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>2027</v>
       </c>
-      <c r="E18" s="14" t="n">
+      <c r="E18" s="15" t="n">
         <f aca="false">IF($C18="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F18" s="14" t="n">
+      <c r="F18" s="15" t="n">
         <f aca="false">IF($C18="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G18" s="14" t="n">
+      <c r="G18" s="15" t="n">
         <f aca="false">IF($C18="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>65000</v>
       </c>
-      <c r="I18" s="14" t="n">
+      <c r="I18" s="15" t="n">
         <f aca="false">IF($C18="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J18" s="16" t="n">
+      <c r="J18" s="17" t="n">
         <f aca="false">IF($C18="Lease-koop",D18+p_SlotJr,IF($C18="Koop",D18,0))</f>
         <v>2027</v>
       </c>
-      <c r="K18" s="14" t="n">
+      <c r="K18" s="15" t="n">
         <f aca="false">E18+F18+G18+H18+I18</f>
         <v>65000</v>
       </c>
-      <c r="L18" s="16" t="n">
+      <c r="L18" s="17" t="n">
         <f aca="false">IF($C18="Lease-koop",p_Afschr,IF($C18="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A18,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>8</v>
       </c>
-      <c r="M18" s="16" t="n">
+      <c r="M18" s="17" t="n">
         <f aca="false">IF($C18="Lease-koop",D18+p_Lev,IF(AND($C18="Koop",D18&gt;0),D18+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A18,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2035</v>
       </c>
-      <c r="N18" s="14" t="n">
+      <c r="N18" s="15" t="n">
         <f aca="false">IF($C18="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -2509,47 +2537,47 @@
       <c r="A19" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B19" s="15"/>
+      <c r="B19" s="16"/>
       <c r="C19" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D19" s="5" t="n">
         <v>2027</v>
       </c>
-      <c r="E19" s="14" t="n">
+      <c r="E19" s="15" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F19" s="14" t="n">
+      <c r="F19" s="15" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G19" s="14" t="n">
+      <c r="G19" s="15" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H19" s="7"/>
-      <c r="I19" s="14" t="n">
+      <c r="I19" s="15" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J19" s="16" t="n">
+      <c r="J19" s="17" t="n">
         <f aca="false">IF($C19="Lease-koop",D19+p_SlotJr,IF($C19="Koop",D19,0))</f>
         <v>2029</v>
       </c>
-      <c r="K19" s="14" t="n">
+      <c r="K19" s="15" t="n">
         <f aca="false">E19+F19+G19+H19+I19</f>
         <v>57000</v>
       </c>
-      <c r="L19" s="16" t="n">
+      <c r="L19" s="17" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Afschr,IF($C19="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A19,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M19" s="16" t="n">
+      <c r="M19" s="17" t="n">
         <f aca="false">IF($C19="Lease-koop",D19+p_Lev,IF(AND($C19="Koop",D19&gt;0),D19+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A19,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2035</v>
       </c>
-      <c r="N19" s="14" t="n">
+      <c r="N19" s="15" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -2559,49 +2587,49 @@
       <c r="A20" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B20" s="15"/>
+      <c r="B20" s="16"/>
       <c r="C20" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>2027</v>
       </c>
-      <c r="E20" s="14" t="n">
+      <c r="E20" s="15" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F20" s="14" t="n">
+      <c r="F20" s="15" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G20" s="14" t="n">
+      <c r="G20" s="15" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>80000</v>
       </c>
-      <c r="I20" s="14" t="n">
+      <c r="I20" s="15" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J20" s="16" t="n">
+      <c r="J20" s="17" t="n">
         <f aca="false">IF($C20="Lease-koop",D20+p_SlotJr,IF($C20="Koop",D20,0))</f>
         <v>2027</v>
       </c>
-      <c r="K20" s="14" t="n">
+      <c r="K20" s="15" t="n">
         <f aca="false">E20+F20+G20+H20+I20</f>
         <v>80000</v>
       </c>
-      <c r="L20" s="16" t="n">
+      <c r="L20" s="17" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Afschr,IF($C20="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A20,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>15</v>
       </c>
-      <c r="M20" s="16" t="n">
+      <c r="M20" s="17" t="n">
         <f aca="false">IF($C20="Lease-koop",D20+p_Lev,IF(AND($C20="Koop",D20&gt;0),D20+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A20,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2042</v>
       </c>
-      <c r="N20" s="14" t="n">
+      <c r="N20" s="15" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -2611,49 +2639,49 @@
       <c r="A21" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B21" s="15"/>
+      <c r="B21" s="16"/>
       <c r="C21" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D21" s="5" t="n">
         <v>2027</v>
       </c>
-      <c r="E21" s="14" t="n">
+      <c r="E21" s="15" t="n">
         <f aca="false">IF($C21="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F21" s="14" t="n">
+      <c r="F21" s="15" t="n">
         <f aca="false">IF($C21="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G21" s="14" t="n">
+      <c r="G21" s="15" t="n">
         <f aca="false">IF($C21="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H21" s="7" t="n">
         <v>45000</v>
       </c>
-      <c r="I21" s="14" t="n">
+      <c r="I21" s="15" t="n">
         <f aca="false">IF($C21="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J21" s="16" t="n">
+      <c r="J21" s="17" t="n">
         <f aca="false">IF($C21="Lease-koop",D21+p_SlotJr,IF($C21="Koop",D21,0))</f>
         <v>2027</v>
       </c>
-      <c r="K21" s="14" t="n">
+      <c r="K21" s="15" t="n">
         <f aca="false">E21+F21+G21+H21+I21</f>
         <v>45000</v>
       </c>
-      <c r="L21" s="16" t="n">
+      <c r="L21" s="17" t="n">
         <f aca="false">IF($C21="Lease-koop",p_Afschr,IF($C21="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A21,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>8</v>
       </c>
-      <c r="M21" s="16" t="n">
+      <c r="M21" s="17" t="n">
         <f aca="false">IF($C21="Lease-koop",D21+p_Lev,IF(AND($C21="Koop",D21&gt;0),D21+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A21,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2035</v>
       </c>
-      <c r="N21" s="14" t="n">
+      <c r="N21" s="15" t="n">
         <f aca="false">IF($C21="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -2665,49 +2693,49 @@
       <c r="A22" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="B22" s="15"/>
+      <c r="B22" s="16"/>
       <c r="C22" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D22" s="5" t="n">
         <v>2027</v>
       </c>
-      <c r="E22" s="14" t="n">
+      <c r="E22" s="15" t="n">
         <f aca="false">IF($C22="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F22" s="14" t="n">
+      <c r="F22" s="15" t="n">
         <f aca="false">IF($C22="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G22" s="14" t="n">
+      <c r="G22" s="15" t="n">
         <f aca="false">IF($C22="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H22" s="7" t="n">
         <v>45000</v>
       </c>
-      <c r="I22" s="14" t="n">
+      <c r="I22" s="15" t="n">
         <f aca="false">IF($C22="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J22" s="16" t="n">
+      <c r="J22" s="17" t="n">
         <f aca="false">IF($C22="Lease-koop",D22+p_SlotJr,IF($C22="Koop",D22,0))</f>
         <v>2027</v>
       </c>
-      <c r="K22" s="14" t="n">
+      <c r="K22" s="15" t="n">
         <f aca="false">E22+F22+G22+H22+I22</f>
         <v>45000</v>
       </c>
-      <c r="L22" s="16" t="n">
+      <c r="L22" s="17" t="n">
         <f aca="false">IF($C22="Lease-koop",p_Afschr,IF($C22="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A22,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>8</v>
       </c>
-      <c r="M22" s="16" t="n">
+      <c r="M22" s="17" t="n">
         <f aca="false">IF($C22="Lease-koop",D22+p_Lev,IF(AND($C22="Koop",D22&gt;0),D22+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A22,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2035</v>
       </c>
-      <c r="N22" s="14" t="n">
+      <c r="N22" s="15" t="n">
         <f aca="false">IF($C22="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -2719,49 +2747,49 @@
       <c r="A23" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B23" s="15"/>
+      <c r="B23" s="16"/>
       <c r="C23" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D23" s="5" t="n">
         <v>2028</v>
       </c>
-      <c r="E23" s="14" t="n">
+      <c r="E23" s="15" t="n">
         <f aca="false">IF($C23="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F23" s="14" t="n">
+      <c r="F23" s="15" t="n">
         <f aca="false">IF($C23="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G23" s="14" t="n">
+      <c r="G23" s="15" t="n">
         <f aca="false">IF($C23="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H23" s="7" t="n">
         <v>50000</v>
       </c>
-      <c r="I23" s="14" t="n">
+      <c r="I23" s="15" t="n">
         <f aca="false">IF($C23="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J23" s="16" t="n">
+      <c r="J23" s="17" t="n">
         <f aca="false">IF($C23="Lease-koop",D23+p_SlotJr,IF($C23="Koop",D23,0))</f>
         <v>2028</v>
       </c>
-      <c r="K23" s="14" t="n">
+      <c r="K23" s="15" t="n">
         <f aca="false">E23+F23+G23+H23+I23</f>
         <v>50000</v>
       </c>
-      <c r="L23" s="16" t="n">
+      <c r="L23" s="17" t="n">
         <f aca="false">IF($C23="Lease-koop",p_Afschr,IF($C23="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A23,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>8</v>
       </c>
-      <c r="M23" s="16" t="n">
+      <c r="M23" s="17" t="n">
         <f aca="false">IF($C23="Lease-koop",D23+p_Lev,IF(AND($C23="Koop",D23&gt;0),D23+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A23,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2036</v>
       </c>
-      <c r="N23" s="14" t="n">
+      <c r="N23" s="15" t="n">
         <f aca="false">IF($C23="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -2773,47 +2801,47 @@
       <c r="A24" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B24" s="15"/>
+      <c r="B24" s="16"/>
       <c r="C24" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D24" s="5" t="n">
         <v>2029</v>
       </c>
-      <c r="E24" s="14" t="n">
+      <c r="E24" s="15" t="n">
         <f aca="false">IF($C24="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F24" s="14" t="n">
+      <c r="F24" s="15" t="n">
         <f aca="false">IF($C24="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G24" s="14" t="n">
+      <c r="G24" s="15" t="n">
         <f aca="false">IF($C24="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H24" s="7"/>
-      <c r="I24" s="14" t="n">
+      <c r="I24" s="15" t="n">
         <f aca="false">IF($C24="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J24" s="16" t="n">
+      <c r="J24" s="17" t="n">
         <f aca="false">IF($C24="Lease-koop",D24+p_SlotJr,IF($C24="Koop",D24,0))</f>
         <v>2031</v>
       </c>
-      <c r="K24" s="14" t="n">
+      <c r="K24" s="15" t="n">
         <f aca="false">E24+F24+G24+H24+I24</f>
         <v>57000</v>
       </c>
-      <c r="L24" s="16" t="n">
+      <c r="L24" s="17" t="n">
         <f aca="false">IF($C24="Lease-koop",p_Afschr,IF($C24="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A24,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M24" s="16" t="n">
+      <c r="M24" s="17" t="n">
         <f aca="false">IF($C24="Lease-koop",D24+p_Lev,IF(AND($C24="Koop",D24&gt;0),D24+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A24,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2037</v>
       </c>
-      <c r="N24" s="14" t="n">
+      <c r="N24" s="15" t="n">
         <f aca="false">IF($C24="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -2823,49 +2851,49 @@
       <c r="A25" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B25" s="15"/>
+      <c r="B25" s="16"/>
       <c r="C25" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="5" t="n">
         <v>2029</v>
       </c>
-      <c r="E25" s="14" t="n">
+      <c r="E25" s="15" t="n">
         <f aca="false">IF($C25="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F25" s="14" t="n">
+      <c r="F25" s="15" t="n">
         <f aca="false">IF($C25="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G25" s="14" t="n">
+      <c r="G25" s="15" t="n">
         <f aca="false">IF($C25="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H25" s="7" t="n">
         <v>100000</v>
       </c>
-      <c r="I25" s="14" t="n">
+      <c r="I25" s="15" t="n">
         <f aca="false">IF($C25="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J25" s="16" t="n">
+      <c r="J25" s="17" t="n">
         <f aca="false">IF($C25="Lease-koop",D25+p_SlotJr,IF($C25="Koop",D25,0))</f>
         <v>2029</v>
       </c>
-      <c r="K25" s="14" t="n">
+      <c r="K25" s="15" t="n">
         <f aca="false">E25+F25+G25+H25+I25</f>
         <v>100000</v>
       </c>
-      <c r="L25" s="16" t="n">
+      <c r="L25" s="17" t="n">
         <f aca="false">IF($C25="Lease-koop",p_Afschr,IF($C25="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A25,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>20</v>
       </c>
-      <c r="M25" s="16" t="n">
+      <c r="M25" s="17" t="n">
         <f aca="false">IF($C25="Lease-koop",D25+p_Lev,IF(AND($C25="Koop",D25&gt;0),D25+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A25,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2049</v>
       </c>
-      <c r="N25" s="14" t="n">
+      <c r="N25" s="15" t="n">
         <f aca="false">IF($C25="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -2875,47 +2903,47 @@
       <c r="A26" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B26" s="15"/>
+      <c r="B26" s="16"/>
       <c r="C26" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D26" s="5" t="n">
         <v>2031</v>
       </c>
-      <c r="E26" s="14" t="n">
+      <c r="E26" s="15" t="n">
         <f aca="false">IF($C26="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F26" s="14" t="n">
+      <c r="F26" s="15" t="n">
         <f aca="false">IF($C26="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G26" s="14" t="n">
+      <c r="G26" s="15" t="n">
         <f aca="false">IF($C26="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H26" s="7"/>
-      <c r="I26" s="14" t="n">
+      <c r="I26" s="15" t="n">
         <f aca="false">IF($C26="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J26" s="16" t="n">
+      <c r="J26" s="17" t="n">
         <f aca="false">IF($C26="Lease-koop",D26+p_SlotJr,IF($C26="Koop",D26,0))</f>
         <v>2033</v>
       </c>
-      <c r="K26" s="14" t="n">
+      <c r="K26" s="15" t="n">
         <f aca="false">E26+F26+G26+H26+I26</f>
         <v>57000</v>
       </c>
-      <c r="L26" s="16" t="n">
+      <c r="L26" s="17" t="n">
         <f aca="false">IF($C26="Lease-koop",p_Afschr,IF($C26="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A26,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M26" s="16" t="n">
+      <c r="M26" s="17" t="n">
         <f aca="false">IF($C26="Lease-koop",D26+p_Lev,IF(AND($C26="Koop",D26&gt;0),D26+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A26,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2039</v>
       </c>
-      <c r="N26" s="14" t="n">
+      <c r="N26" s="15" t="n">
         <f aca="false">IF($C26="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -2925,49 +2953,49 @@
       <c r="A27" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B27" s="15"/>
+      <c r="B27" s="16"/>
       <c r="C27" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D27" s="5" t="n">
         <v>2032</v>
       </c>
-      <c r="E27" s="14" t="n">
+      <c r="E27" s="15" t="n">
         <f aca="false">IF($C27="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F27" s="14" t="n">
+      <c r="F27" s="15" t="n">
         <f aca="false">IF($C27="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G27" s="14" t="n">
+      <c r="G27" s="15" t="n">
         <f aca="false">IF($C27="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H27" s="7" t="n">
         <v>248960</v>
       </c>
-      <c r="I27" s="14" t="n">
+      <c r="I27" s="15" t="n">
         <f aca="false">IF($C27="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J27" s="16" t="n">
+      <c r="J27" s="17" t="n">
         <f aca="false">IF($C27="Lease-koop",D27+p_SlotJr,IF($C27="Koop",D27,0))</f>
         <v>2032</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="K27" s="15" t="n">
         <f aca="false">E27+F27+G27+H27+I27</f>
         <v>248960</v>
       </c>
-      <c r="L27" s="16" t="n">
+      <c r="L27" s="17" t="n">
         <f aca="false">IF($C27="Lease-koop",p_Afschr,IF($C27="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A27,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>8</v>
       </c>
-      <c r="M27" s="16" t="n">
+      <c r="M27" s="17" t="n">
         <f aca="false">IF($C27="Lease-koop",D27+p_Lev,IF(AND($C27="Koop",D27&gt;0),D27+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A27,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2040</v>
       </c>
-      <c r="N27" s="14" t="n">
+      <c r="N27" s="15" t="n">
         <f aca="false">IF($C27="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -2983,40 +3011,40 @@
       <c r="D28" s="5" t="n">
         <v>2032</v>
       </c>
-      <c r="E28" s="14" t="n">
+      <c r="E28" s="15" t="n">
         <f aca="false">IF($C28="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F28" s="14" t="n">
+      <c r="F28" s="15" t="n">
         <f aca="false">IF($C28="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G28" s="14" t="n">
+      <c r="G28" s="15" t="n">
         <f aca="false">IF($C28="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H28" s="7"/>
-      <c r="I28" s="14" t="n">
+      <c r="I28" s="15" t="n">
         <f aca="false">IF($C28="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J28" s="16" t="n">
+      <c r="J28" s="17" t="n">
         <f aca="false">IF($C28="Lease-koop",D28+p_SlotJr,IF($C28="Koop",D28,0))</f>
         <v>0</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="K28" s="15" t="n">
         <f aca="false">E28+F28+G28+H28+I28</f>
         <v>0</v>
       </c>
-      <c r="L28" s="16" t="n">
+      <c r="L28" s="17" t="n">
         <f aca="false">IF($C28="Lease-koop",p_Afschr,IF($C28="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A28,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M28" s="16" t="n">
+      <c r="M28" s="17" t="n">
         <f aca="false">IF($C28="Lease-koop",D28+p_Lev,IF(AND($C28="Koop",D28&gt;0),D28+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A28,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N28" s="14" t="n">
+      <c r="N28" s="15" t="n">
         <f aca="false">IF($C28="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -3028,47 +3056,47 @@
       <c r="A29" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B29" s="15"/>
+      <c r="B29" s="16"/>
       <c r="C29" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D29" s="5" t="n">
         <v>2032</v>
       </c>
-      <c r="E29" s="14" t="n">
+      <c r="E29" s="15" t="n">
         <f aca="false">IF($C29="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F29" s="14" t="n">
+      <c r="F29" s="15" t="n">
         <f aca="false">IF($C29="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G29" s="14" t="n">
+      <c r="G29" s="15" t="n">
         <f aca="false">IF($C29="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H29" s="7"/>
-      <c r="I29" s="14" t="n">
+      <c r="I29" s="15" t="n">
         <f aca="false">IF($C29="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J29" s="16" t="n">
+      <c r="J29" s="17" t="n">
         <f aca="false">IF($C29="Lease-koop",D29+p_SlotJr,IF($C29="Koop",D29,0))</f>
         <v>2034</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="K29" s="15" t="n">
         <f aca="false">E29+F29+G29+H29+I29</f>
         <v>57000</v>
       </c>
-      <c r="L29" s="16" t="n">
+      <c r="L29" s="17" t="n">
         <f aca="false">IF($C29="Lease-koop",p_Afschr,IF($C29="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A29,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M29" s="16" t="n">
+      <c r="M29" s="17" t="n">
         <f aca="false">IF($C29="Lease-koop",D29+p_Lev,IF(AND($C29="Koop",D29&gt;0),D29+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A29,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2040</v>
       </c>
-      <c r="N29" s="14" t="n">
+      <c r="N29" s="15" t="n">
         <f aca="false">IF($C29="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3078,47 +3106,47 @@
       <c r="A30" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B30" s="15"/>
+      <c r="B30" s="16"/>
       <c r="C30" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D30" s="5" t="n">
         <v>2032</v>
       </c>
-      <c r="E30" s="14" t="n">
+      <c r="E30" s="15" t="n">
         <f aca="false">IF($C30="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F30" s="14" t="n">
+      <c r="F30" s="15" t="n">
         <f aca="false">IF($C30="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G30" s="14" t="n">
+      <c r="G30" s="15" t="n">
         <f aca="false">IF($C30="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H30" s="7"/>
-      <c r="I30" s="14" t="n">
+      <c r="I30" s="15" t="n">
         <f aca="false">IF($C30="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J30" s="16" t="n">
+      <c r="J30" s="17" t="n">
         <f aca="false">IF($C30="Lease-koop",D30+p_SlotJr,IF($C30="Koop",D30,0))</f>
         <v>2034</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="K30" s="15" t="n">
         <f aca="false">E30+F30+G30+H30+I30</f>
         <v>57000</v>
       </c>
-      <c r="L30" s="16" t="n">
+      <c r="L30" s="17" t="n">
         <f aca="false">IF($C30="Lease-koop",p_Afschr,IF($C30="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A30,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M30" s="16" t="n">
+      <c r="M30" s="17" t="n">
         <f aca="false">IF($C30="Lease-koop",D30+p_Lev,IF(AND($C30="Koop",D30&gt;0),D30+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A30,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2040</v>
       </c>
-      <c r="N30" s="14" t="n">
+      <c r="N30" s="15" t="n">
         <f aca="false">IF($C30="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3128,47 +3156,47 @@
       <c r="A31" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B31" s="15"/>
+      <c r="B31" s="16"/>
       <c r="C31" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D31" s="5" t="n">
         <v>2032</v>
       </c>
-      <c r="E31" s="14" t="n">
+      <c r="E31" s="15" t="n">
         <f aca="false">IF($C31="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F31" s="14" t="n">
+      <c r="F31" s="15" t="n">
         <f aca="false">IF($C31="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G31" s="14" t="n">
+      <c r="G31" s="15" t="n">
         <f aca="false">IF($C31="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H31" s="7"/>
-      <c r="I31" s="14" t="n">
+      <c r="I31" s="15" t="n">
         <f aca="false">IF($C31="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J31" s="16" t="n">
+      <c r="J31" s="17" t="n">
         <f aca="false">IF($C31="Lease-koop",D31+p_SlotJr,IF($C31="Koop",D31,0))</f>
         <v>2034</v>
       </c>
-      <c r="K31" s="14" t="n">
+      <c r="K31" s="15" t="n">
         <f aca="false">E31+F31+G31+H31+I31</f>
         <v>57000</v>
       </c>
-      <c r="L31" s="16" t="n">
+      <c r="L31" s="17" t="n">
         <f aca="false">IF($C31="Lease-koop",p_Afschr,IF($C31="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A31,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M31" s="16" t="n">
+      <c r="M31" s="17" t="n">
         <f aca="false">IF($C31="Lease-koop",D31+p_Lev,IF(AND($C31="Koop",D31&gt;0),D31+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A31,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2040</v>
       </c>
-      <c r="N31" s="14" t="n">
+      <c r="N31" s="15" t="n">
         <f aca="false">IF($C31="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3178,47 +3206,47 @@
       <c r="A32" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B32" s="15"/>
+      <c r="B32" s="16"/>
       <c r="C32" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D32" s="5" t="n">
         <v>2033</v>
       </c>
-      <c r="E32" s="14" t="n">
+      <c r="E32" s="15" t="n">
         <f aca="false">IF($C32="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F32" s="14" t="n">
+      <c r="F32" s="15" t="n">
         <f aca="false">IF($C32="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G32" s="14" t="n">
+      <c r="G32" s="15" t="n">
         <f aca="false">IF($C32="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H32" s="7"/>
-      <c r="I32" s="14" t="n">
+      <c r="I32" s="15" t="n">
         <f aca="false">IF($C32="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J32" s="16" t="n">
+      <c r="J32" s="17" t="n">
         <f aca="false">IF($C32="Lease-koop",D32+p_SlotJr,IF($C32="Koop",D32,0))</f>
         <v>2035</v>
       </c>
-      <c r="K32" s="14" t="n">
+      <c r="K32" s="15" t="n">
         <f aca="false">E32+F32+G32+H32+I32</f>
         <v>57000</v>
       </c>
-      <c r="L32" s="16" t="n">
+      <c r="L32" s="17" t="n">
         <f aca="false">IF($C32="Lease-koop",p_Afschr,IF($C32="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A32,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M32" s="16" t="n">
+      <c r="M32" s="17" t="n">
         <f aca="false">IF($C32="Lease-koop",D32+p_Lev,IF(AND($C32="Koop",D32&gt;0),D32+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A32,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2041</v>
       </c>
-      <c r="N32" s="14" t="n">
+      <c r="N32" s="15" t="n">
         <f aca="false">IF($C32="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3228,49 +3256,49 @@
       <c r="A33" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B33" s="15"/>
+      <c r="B33" s="16"/>
       <c r="C33" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D33" s="5" t="n">
         <v>2033</v>
       </c>
-      <c r="E33" s="14" t="n">
+      <c r="E33" s="15" t="n">
         <f aca="false">IF($C33="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F33" s="14" t="n">
+      <c r="F33" s="15" t="n">
         <f aca="false">IF($C33="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G33" s="14" t="n">
+      <c r="G33" s="15" t="n">
         <f aca="false">IF($C33="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H33" s="7" t="n">
         <v>19000</v>
       </c>
-      <c r="I33" s="14" t="n">
+      <c r="I33" s="15" t="n">
         <f aca="false">IF($C33="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J33" s="16" t="n">
+      <c r="J33" s="17" t="n">
         <f aca="false">IF($C33="Lease-koop",D33+p_SlotJr,IF($C33="Koop",D33,0))</f>
         <v>2033</v>
       </c>
-      <c r="K33" s="14" t="n">
+      <c r="K33" s="15" t="n">
         <f aca="false">E33+F33+G33+H33+I33</f>
         <v>19000</v>
       </c>
-      <c r="L33" s="16" t="n">
+      <c r="L33" s="17" t="n">
         <f aca="false">IF($C33="Lease-koop",p_Afschr,IF($C33="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A33,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>10</v>
       </c>
-      <c r="M33" s="16" t="n">
+      <c r="M33" s="17" t="n">
         <f aca="false">IF($C33="Lease-koop",D33+p_Lev,IF(AND($C33="Koop",D33&gt;0),D33+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A33,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2043</v>
       </c>
-      <c r="N33" s="14" t="n">
+      <c r="N33" s="15" t="n">
         <f aca="false">IF($C33="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -3280,47 +3308,47 @@
       <c r="A34" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B34" s="15"/>
+      <c r="B34" s="16"/>
       <c r="C34" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D34" s="5" t="n">
         <v>2034</v>
       </c>
-      <c r="E34" s="14" t="n">
+      <c r="E34" s="15" t="n">
         <f aca="false">IF($C34="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F34" s="14" t="n">
+      <c r="F34" s="15" t="n">
         <f aca="false">IF($C34="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G34" s="14" t="n">
+      <c r="G34" s="15" t="n">
         <f aca="false">IF($C34="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H34" s="7"/>
-      <c r="I34" s="14" t="n">
+      <c r="I34" s="15" t="n">
         <f aca="false">IF($C34="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J34" s="16" t="n">
+      <c r="J34" s="17" t="n">
         <f aca="false">IF($C34="Lease-koop",D34+p_SlotJr,IF($C34="Koop",D34,0))</f>
         <v>2036</v>
       </c>
-      <c r="K34" s="14" t="n">
+      <c r="K34" s="15" t="n">
         <f aca="false">E34+F34+G34+H34+I34</f>
         <v>57000</v>
       </c>
-      <c r="L34" s="16" t="n">
+      <c r="L34" s="17" t="n">
         <f aca="false">IF($C34="Lease-koop",p_Afschr,IF($C34="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A34,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M34" s="16" t="n">
+      <c r="M34" s="17" t="n">
         <f aca="false">IF($C34="Lease-koop",D34+p_Lev,IF(AND($C34="Koop",D34&gt;0),D34+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A34,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2042</v>
       </c>
-      <c r="N34" s="14" t="n">
+      <c r="N34" s="15" t="n">
         <f aca="false">IF($C34="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3330,47 +3358,47 @@
       <c r="A35" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B35" s="15"/>
+      <c r="B35" s="16"/>
       <c r="C35" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D35" s="5" t="n">
         <v>2034</v>
       </c>
-      <c r="E35" s="14" t="n">
+      <c r="E35" s="15" t="n">
         <f aca="false">IF($C35="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F35" s="14" t="n">
+      <c r="F35" s="15" t="n">
         <f aca="false">IF($C35="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G35" s="14" t="n">
+      <c r="G35" s="15" t="n">
         <f aca="false">IF($C35="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H35" s="7"/>
-      <c r="I35" s="14" t="n">
+      <c r="I35" s="15" t="n">
         <f aca="false">IF($C35="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J35" s="16" t="n">
+      <c r="J35" s="17" t="n">
         <f aca="false">IF($C35="Lease-koop",D35+p_SlotJr,IF($C35="Koop",D35,0))</f>
         <v>2036</v>
       </c>
-      <c r="K35" s="14" t="n">
+      <c r="K35" s="15" t="n">
         <f aca="false">E35+F35+G35+H35+I35</f>
         <v>57000</v>
       </c>
-      <c r="L35" s="16" t="n">
+      <c r="L35" s="17" t="n">
         <f aca="false">IF($C35="Lease-koop",p_Afschr,IF($C35="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A35,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M35" s="16" t="n">
+      <c r="M35" s="17" t="n">
         <f aca="false">IF($C35="Lease-koop",D35+p_Lev,IF(AND($C35="Koop",D35&gt;0),D35+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A35,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2042</v>
       </c>
-      <c r="N35" s="14" t="n">
+      <c r="N35" s="15" t="n">
         <f aca="false">IF($C35="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3380,47 +3408,47 @@
       <c r="A36" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B36" s="15"/>
+      <c r="B36" s="16"/>
       <c r="C36" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D36" s="5" t="n">
         <v>2034</v>
       </c>
-      <c r="E36" s="14" t="n">
+      <c r="E36" s="15" t="n">
         <f aca="false">IF($C36="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F36" s="14" t="n">
+      <c r="F36" s="15" t="n">
         <f aca="false">IF($C36="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G36" s="14" t="n">
+      <c r="G36" s="15" t="n">
         <f aca="false">IF($C36="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H36" s="7"/>
-      <c r="I36" s="14" t="n">
+      <c r="I36" s="15" t="n">
         <f aca="false">IF($C36="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J36" s="16" t="n">
+      <c r="J36" s="17" t="n">
         <f aca="false">IF($C36="Lease-koop",D36+p_SlotJr,IF($C36="Koop",D36,0))</f>
         <v>2036</v>
       </c>
-      <c r="K36" s="14" t="n">
+      <c r="K36" s="15" t="n">
         <f aca="false">E36+F36+G36+H36+I36</f>
         <v>57000</v>
       </c>
-      <c r="L36" s="16" t="n">
+      <c r="L36" s="17" t="n">
         <f aca="false">IF($C36="Lease-koop",p_Afschr,IF($C36="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A36,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M36" s="16" t="n">
+      <c r="M36" s="17" t="n">
         <f aca="false">IF($C36="Lease-koop",D36+p_Lev,IF(AND($C36="Koop",D36&gt;0),D36+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A36,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2042</v>
       </c>
-      <c r="N36" s="14" t="n">
+      <c r="N36" s="15" t="n">
         <f aca="false">IF($C36="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3430,47 +3458,47 @@
       <c r="A37" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B37" s="15"/>
+      <c r="B37" s="16"/>
       <c r="C37" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D37" s="5" t="n">
         <v>2034</v>
       </c>
-      <c r="E37" s="14" t="n">
+      <c r="E37" s="15" t="n">
         <f aca="false">IF($C37="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F37" s="14" t="n">
+      <c r="F37" s="15" t="n">
         <f aca="false">IF($C37="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G37" s="14" t="n">
+      <c r="G37" s="15" t="n">
         <f aca="false">IF($C37="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H37" s="7"/>
-      <c r="I37" s="14" t="n">
+      <c r="I37" s="15" t="n">
         <f aca="false">IF($C37="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J37" s="16" t="n">
+      <c r="J37" s="17" t="n">
         <f aca="false">IF($C37="Lease-koop",D37+p_SlotJr,IF($C37="Koop",D37,0))</f>
         <v>2036</v>
       </c>
-      <c r="K37" s="14" t="n">
+      <c r="K37" s="15" t="n">
         <f aca="false">E37+F37+G37+H37+I37</f>
         <v>57000</v>
       </c>
-      <c r="L37" s="16" t="n">
+      <c r="L37" s="17" t="n">
         <f aca="false">IF($C37="Lease-koop",p_Afschr,IF($C37="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A37,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M37" s="16" t="n">
+      <c r="M37" s="17" t="n">
         <f aca="false">IF($C37="Lease-koop",D37+p_Lev,IF(AND($C37="Koop",D37&gt;0),D37+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A37,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2042</v>
       </c>
-      <c r="N37" s="14" t="n">
+      <c r="N37" s="15" t="n">
         <f aca="false">IF($C37="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3480,47 +3508,47 @@
       <c r="A38" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B38" s="15"/>
+      <c r="B38" s="16"/>
       <c r="C38" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D38" s="5" t="n">
         <v>2034</v>
       </c>
-      <c r="E38" s="14" t="n">
+      <c r="E38" s="15" t="n">
         <f aca="false">IF($C38="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F38" s="14" t="n">
+      <c r="F38" s="15" t="n">
         <f aca="false">IF($C38="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G38" s="14" t="n">
+      <c r="G38" s="15" t="n">
         <f aca="false">IF($C38="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H38" s="7"/>
-      <c r="I38" s="14" t="n">
+      <c r="I38" s="15" t="n">
         <f aca="false">IF($C38="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J38" s="16" t="n">
+      <c r="J38" s="17" t="n">
         <f aca="false">IF($C38="Lease-koop",D38+p_SlotJr,IF($C38="Koop",D38,0))</f>
         <v>2036</v>
       </c>
-      <c r="K38" s="14" t="n">
+      <c r="K38" s="15" t="n">
         <f aca="false">E38+F38+G38+H38+I38</f>
         <v>57000</v>
       </c>
-      <c r="L38" s="16" t="n">
+      <c r="L38" s="17" t="n">
         <f aca="false">IF($C38="Lease-koop",p_Afschr,IF($C38="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A38,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M38" s="16" t="n">
+      <c r="M38" s="17" t="n">
         <f aca="false">IF($C38="Lease-koop",D38+p_Lev,IF(AND($C38="Koop",D38&gt;0),D38+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A38,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2042</v>
       </c>
-      <c r="N38" s="14" t="n">
+      <c r="N38" s="15" t="n">
         <f aca="false">IF($C38="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3530,47 +3558,47 @@
       <c r="A39" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B39" s="15"/>
+      <c r="B39" s="16"/>
       <c r="C39" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D39" s="5" t="n">
         <v>2034</v>
       </c>
-      <c r="E39" s="14" t="n">
+      <c r="E39" s="15" t="n">
         <f aca="false">IF($C39="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F39" s="14" t="n">
+      <c r="F39" s="15" t="n">
         <f aca="false">IF($C39="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G39" s="14" t="n">
+      <c r="G39" s="15" t="n">
         <f aca="false">IF($C39="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H39" s="7"/>
-      <c r="I39" s="14" t="n">
+      <c r="I39" s="15" t="n">
         <f aca="false">IF($C39="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J39" s="16" t="n">
+      <c r="J39" s="17" t="n">
         <f aca="false">IF($C39="Lease-koop",D39+p_SlotJr,IF($C39="Koop",D39,0))</f>
         <v>2036</v>
       </c>
-      <c r="K39" s="14" t="n">
+      <c r="K39" s="15" t="n">
         <f aca="false">E39+F39+G39+H39+I39</f>
         <v>57000</v>
       </c>
-      <c r="L39" s="16" t="n">
+      <c r="L39" s="17" t="n">
         <f aca="false">IF($C39="Lease-koop",p_Afschr,IF($C39="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A39,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M39" s="16" t="n">
+      <c r="M39" s="17" t="n">
         <f aca="false">IF($C39="Lease-koop",D39+p_Lev,IF(AND($C39="Koop",D39&gt;0),D39+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A39,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2042</v>
       </c>
-      <c r="N39" s="14" t="n">
+      <c r="N39" s="15" t="n">
         <f aca="false">IF($C39="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3580,49 +3608,49 @@
       <c r="A40" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B40" s="15"/>
+      <c r="B40" s="16"/>
       <c r="C40" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D40" s="5" t="n">
         <v>2034</v>
       </c>
-      <c r="E40" s="14" t="n">
+      <c r="E40" s="15" t="n">
         <f aca="false">IF($C40="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F40" s="14" t="n">
+      <c r="F40" s="15" t="n">
         <f aca="false">IF($C40="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G40" s="14" t="n">
+      <c r="G40" s="15" t="n">
         <f aca="false">IF($C40="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H40" s="7" t="n">
         <v>51100</v>
       </c>
-      <c r="I40" s="14" t="n">
+      <c r="I40" s="15" t="n">
         <f aca="false">IF($C40="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J40" s="16" t="n">
+      <c r="J40" s="17" t="n">
         <f aca="false">IF($C40="Lease-koop",D40+p_SlotJr,IF($C40="Koop",D40,0))</f>
         <v>2034</v>
       </c>
-      <c r="K40" s="14" t="n">
+      <c r="K40" s="15" t="n">
         <f aca="false">E40+F40+G40+H40+I40</f>
         <v>51100</v>
       </c>
-      <c r="L40" s="16" t="n">
+      <c r="L40" s="17" t="n">
         <f aca="false">IF($C40="Lease-koop",p_Afschr,IF($C40="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A40,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>10</v>
       </c>
-      <c r="M40" s="16" t="n">
+      <c r="M40" s="17" t="n">
         <f aca="false">IF($C40="Lease-koop",D40+p_Lev,IF(AND($C40="Koop",D40&gt;0),D40+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A40,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2044</v>
       </c>
-      <c r="N40" s="14" t="n">
+      <c r="N40" s="15" t="n">
         <f aca="false">IF($C40="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -3632,47 +3660,47 @@
       <c r="A41" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B41" s="15"/>
+      <c r="B41" s="16"/>
       <c r="C41" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D41" s="5" t="n">
         <v>2034</v>
       </c>
-      <c r="E41" s="14" t="n">
+      <c r="E41" s="15" t="n">
         <f aca="false">IF($C41="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F41" s="14" t="n">
+      <c r="F41" s="15" t="n">
         <f aca="false">IF($C41="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G41" s="14" t="n">
+      <c r="G41" s="15" t="n">
         <f aca="false">IF($C41="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H41" s="7"/>
-      <c r="I41" s="14" t="n">
+      <c r="I41" s="15" t="n">
         <f aca="false">IF($C41="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J41" s="16" t="n">
+      <c r="J41" s="17" t="n">
         <f aca="false">IF($C41="Lease-koop",D41+p_SlotJr,IF($C41="Koop",D41,0))</f>
         <v>2036</v>
       </c>
-      <c r="K41" s="14" t="n">
+      <c r="K41" s="15" t="n">
         <f aca="false">E41+F41+G41+H41+I41</f>
         <v>57000</v>
       </c>
-      <c r="L41" s="16" t="n">
+      <c r="L41" s="17" t="n">
         <f aca="false">IF($C41="Lease-koop",p_Afschr,IF($C41="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A41,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M41" s="16" t="n">
+      <c r="M41" s="17" t="n">
         <f aca="false">IF($C41="Lease-koop",D41+p_Lev,IF(AND($C41="Koop",D41&gt;0),D41+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A41,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2042</v>
       </c>
-      <c r="N41" s="14" t="n">
+      <c r="N41" s="15" t="n">
         <f aca="false">IF($C41="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3682,49 +3710,49 @@
       <c r="A42" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B42" s="15"/>
+      <c r="B42" s="16"/>
       <c r="C42" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D42" s="5" t="n">
         <v>2035</v>
       </c>
-      <c r="E42" s="14" t="n">
+      <c r="E42" s="15" t="n">
         <f aca="false">IF($C42="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F42" s="14" t="n">
+      <c r="F42" s="15" t="n">
         <f aca="false">IF($C42="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G42" s="14" t="n">
+      <c r="G42" s="15" t="n">
         <f aca="false">IF($C42="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H42" s="7" t="n">
         <v>358180</v>
       </c>
-      <c r="I42" s="14" t="n">
+      <c r="I42" s="15" t="n">
         <f aca="false">IF($C42="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J42" s="16" t="n">
+      <c r="J42" s="17" t="n">
         <f aca="false">IF($C42="Lease-koop",D42+p_SlotJr,IF($C42="Koop",D42,0))</f>
         <v>2035</v>
       </c>
-      <c r="K42" s="14" t="n">
+      <c r="K42" s="15" t="n">
         <f aca="false">E42+F42+G42+H42+I42</f>
         <v>358180</v>
       </c>
-      <c r="L42" s="16" t="n">
+      <c r="L42" s="17" t="n">
         <f aca="false">IF($C42="Lease-koop",p_Afschr,IF($C42="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A42,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>12</v>
       </c>
-      <c r="M42" s="16" t="n">
+      <c r="M42" s="17" t="n">
         <f aca="false">IF($C42="Lease-koop",D42+p_Lev,IF(AND($C42="Koop",D42&gt;0),D42+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A42,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2047</v>
       </c>
-      <c r="N42" s="14" t="n">
+      <c r="N42" s="15" t="n">
         <f aca="false">IF($C42="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -3734,49 +3762,49 @@
       <c r="A43" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B43" s="15"/>
+      <c r="B43" s="16"/>
       <c r="C43" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D43" s="5" t="n">
         <v>2038</v>
       </c>
-      <c r="E43" s="14" t="n">
+      <c r="E43" s="15" t="n">
         <f aca="false">IF($C43="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F43" s="14" t="n">
+      <c r="F43" s="15" t="n">
         <f aca="false">IF($C43="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G43" s="14" t="n">
+      <c r="G43" s="15" t="n">
         <f aca="false">IF($C43="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H43" s="7" t="n">
         <v>121968</v>
       </c>
-      <c r="I43" s="14" t="n">
+      <c r="I43" s="15" t="n">
         <f aca="false">IF($C43="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J43" s="16" t="n">
+      <c r="J43" s="17" t="n">
         <f aca="false">IF($C43="Lease-koop",D43+p_SlotJr,IF($C43="Koop",D43,0))</f>
         <v>2038</v>
       </c>
-      <c r="K43" s="14" t="n">
+      <c r="K43" s="15" t="n">
         <f aca="false">E43+F43+G43+H43+I43</f>
         <v>121968</v>
       </c>
-      <c r="L43" s="16" t="n">
+      <c r="L43" s="17" t="n">
         <f aca="false">IF($C43="Lease-koop",p_Afschr,IF($C43="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A43,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>15</v>
       </c>
-      <c r="M43" s="16" t="n">
+      <c r="M43" s="17" t="n">
         <f aca="false">IF($C43="Lease-koop",D43+p_Lev,IF(AND($C43="Koop",D43&gt;0),D43+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A43,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2053</v>
       </c>
-      <c r="N43" s="14" t="n">
+      <c r="N43" s="15" t="n">
         <f aca="false">IF($C43="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -3784,2120 +3812,2120 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D44" s="5"/>
-      <c r="E44" s="14" t="n">
+      <c r="E44" s="15" t="n">
         <f aca="false">IF($C44="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F44" s="14" t="n">
+      <c r="F44" s="15" t="n">
         <f aca="false">IF($C44="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G44" s="14" t="n">
+      <c r="G44" s="15" t="n">
         <f aca="false">IF($C44="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H44" s="7"/>
-      <c r="I44" s="14" t="n">
+      <c r="I44" s="15" t="n">
         <f aca="false">IF($C44="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J44" s="16" t="n">
+      <c r="J44" s="17" t="n">
         <f aca="false">IF($C44="Lease-koop",D44+p_SlotJr,IF($C44="Koop",D44,0))</f>
         <v>0</v>
       </c>
-      <c r="K44" s="14" t="n">
+      <c r="K44" s="15" t="n">
         <f aca="false">E44+F44+G44+H44+I44</f>
         <v>0</v>
       </c>
-      <c r="L44" s="16" t="n">
+      <c r="L44" s="17" t="n">
         <f aca="false">IF($C44="Lease-koop",p_Afschr,IF($C44="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A44,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M44" s="16" t="n">
+      <c r="M44" s="17" t="n">
         <f aca="false">IF($C44="Lease-koop",D44+p_Lev,IF(AND($C44="Koop",D44&gt;0),D44+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A44,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N44" s="14" t="n">
+      <c r="N44" s="15" t="n">
         <f aca="false">IF($C44="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D45" s="5"/>
-      <c r="E45" s="14" t="n">
+      <c r="E45" s="15" t="n">
         <f aca="false">IF($C45="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F45" s="14" t="n">
+      <c r="F45" s="15" t="n">
         <f aca="false">IF($C45="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G45" s="14" t="n">
+      <c r="G45" s="15" t="n">
         <f aca="false">IF($C45="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H45" s="7"/>
-      <c r="I45" s="14" t="n">
+      <c r="I45" s="15" t="n">
         <f aca="false">IF($C45="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J45" s="16" t="n">
+      <c r="J45" s="17" t="n">
         <f aca="false">IF($C45="Lease-koop",D45+p_SlotJr,IF($C45="Koop",D45,0))</f>
         <v>0</v>
       </c>
-      <c r="K45" s="14" t="n">
+      <c r="K45" s="15" t="n">
         <f aca="false">E45+F45+G45+H45+I45</f>
         <v>0</v>
       </c>
-      <c r="L45" s="16" t="n">
+      <c r="L45" s="17" t="n">
         <f aca="false">IF($C45="Lease-koop",p_Afschr,IF($C45="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A45,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M45" s="16" t="n">
+      <c r="M45" s="17" t="n">
         <f aca="false">IF($C45="Lease-koop",D45+p_Lev,IF(AND($C45="Koop",D45&gt;0),D45+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A45,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N45" s="14" t="n">
+      <c r="N45" s="15" t="n">
         <f aca="false">IF($C45="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D46" s="5"/>
-      <c r="E46" s="14" t="n">
+      <c r="E46" s="15" t="n">
         <f aca="false">IF($C46="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F46" s="14" t="n">
+      <c r="F46" s="15" t="n">
         <f aca="false">IF($C46="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G46" s="14" t="n">
+      <c r="G46" s="15" t="n">
         <f aca="false">IF($C46="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H46" s="7"/>
-      <c r="I46" s="14" t="n">
+      <c r="I46" s="15" t="n">
         <f aca="false">IF($C46="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J46" s="16" t="n">
+      <c r="J46" s="17" t="n">
         <f aca="false">IF($C46="Lease-koop",D46+p_SlotJr,IF($C46="Koop",D46,0))</f>
         <v>0</v>
       </c>
-      <c r="K46" s="14" t="n">
+      <c r="K46" s="15" t="n">
         <f aca="false">E46+F46+G46+H46+I46</f>
         <v>0</v>
       </c>
-      <c r="L46" s="16" t="n">
+      <c r="L46" s="17" t="n">
         <f aca="false">IF($C46="Lease-koop",p_Afschr,IF($C46="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A46,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M46" s="16" t="n">
+      <c r="M46" s="17" t="n">
         <f aca="false">IF($C46="Lease-koop",D46+p_Lev,IF(AND($C46="Koop",D46&gt;0),D46+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A46,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N46" s="14" t="n">
+      <c r="N46" s="15" t="n">
         <f aca="false">IF($C46="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D47" s="5"/>
-      <c r="E47" s="14" t="n">
+      <c r="E47" s="15" t="n">
         <f aca="false">IF($C47="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F47" s="14" t="n">
+      <c r="F47" s="15" t="n">
         <f aca="false">IF($C47="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G47" s="14" t="n">
+      <c r="G47" s="15" t="n">
         <f aca="false">IF($C47="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H47" s="7"/>
-      <c r="I47" s="14" t="n">
+      <c r="I47" s="15" t="n">
         <f aca="false">IF($C47="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J47" s="16" t="n">
+      <c r="J47" s="17" t="n">
         <f aca="false">IF($C47="Lease-koop",D47+p_SlotJr,IF($C47="Koop",D47,0))</f>
         <v>0</v>
       </c>
-      <c r="K47" s="14" t="n">
+      <c r="K47" s="15" t="n">
         <f aca="false">E47+F47+G47+H47+I47</f>
         <v>0</v>
       </c>
-      <c r="L47" s="16" t="n">
+      <c r="L47" s="17" t="n">
         <f aca="false">IF($C47="Lease-koop",p_Afschr,IF($C47="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A47,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M47" s="16" t="n">
+      <c r="M47" s="17" t="n">
         <f aca="false">IF($C47="Lease-koop",D47+p_Lev,IF(AND($C47="Koop",D47&gt;0),D47+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A47,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N47" s="14" t="n">
+      <c r="N47" s="15" t="n">
         <f aca="false">IF($C47="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D48" s="5"/>
-      <c r="E48" s="14" t="n">
+      <c r="E48" s="15" t="n">
         <f aca="false">IF($C48="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F48" s="14" t="n">
+      <c r="F48" s="15" t="n">
         <f aca="false">IF($C48="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G48" s="14" t="n">
+      <c r="G48" s="15" t="n">
         <f aca="false">IF($C48="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H48" s="7"/>
-      <c r="I48" s="14" t="n">
+      <c r="I48" s="15" t="n">
         <f aca="false">IF($C48="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J48" s="16" t="n">
+      <c r="J48" s="17" t="n">
         <f aca="false">IF($C48="Lease-koop",D48+p_SlotJr,IF($C48="Koop",D48,0))</f>
         <v>0</v>
       </c>
-      <c r="K48" s="14" t="n">
+      <c r="K48" s="15" t="n">
         <f aca="false">E48+F48+G48+H48+I48</f>
         <v>0</v>
       </c>
-      <c r="L48" s="16" t="n">
+      <c r="L48" s="17" t="n">
         <f aca="false">IF($C48="Lease-koop",p_Afschr,IF($C48="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A48,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M48" s="16" t="n">
+      <c r="M48" s="17" t="n">
         <f aca="false">IF($C48="Lease-koop",D48+p_Lev,IF(AND($C48="Koop",D48&gt;0),D48+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A48,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N48" s="14" t="n">
+      <c r="N48" s="15" t="n">
         <f aca="false">IF($C48="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D49" s="5"/>
-      <c r="E49" s="14" t="n">
+      <c r="E49" s="15" t="n">
         <f aca="false">IF($C49="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F49" s="14" t="n">
+      <c r="F49" s="15" t="n">
         <f aca="false">IF($C49="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G49" s="14" t="n">
+      <c r="G49" s="15" t="n">
         <f aca="false">IF($C49="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H49" s="7"/>
-      <c r="I49" s="14" t="n">
+      <c r="I49" s="15" t="n">
         <f aca="false">IF($C49="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J49" s="16" t="n">
+      <c r="J49" s="17" t="n">
         <f aca="false">IF($C49="Lease-koop",D49+p_SlotJr,IF($C49="Koop",D49,0))</f>
         <v>0</v>
       </c>
-      <c r="K49" s="14" t="n">
+      <c r="K49" s="15" t="n">
         <f aca="false">E49+F49+G49+H49+I49</f>
         <v>0</v>
       </c>
-      <c r="L49" s="16" t="n">
+      <c r="L49" s="17" t="n">
         <f aca="false">IF($C49="Lease-koop",p_Afschr,IF($C49="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A49,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M49" s="16" t="n">
+      <c r="M49" s="17" t="n">
         <f aca="false">IF($C49="Lease-koop",D49+p_Lev,IF(AND($C49="Koop",D49&gt;0),D49+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A49,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N49" s="14" t="n">
+      <c r="N49" s="15" t="n">
         <f aca="false">IF($C49="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D50" s="5"/>
-      <c r="E50" s="14" t="n">
+      <c r="E50" s="15" t="n">
         <f aca="false">IF($C50="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F50" s="14" t="n">
+      <c r="F50" s="15" t="n">
         <f aca="false">IF($C50="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G50" s="14" t="n">
+      <c r="G50" s="15" t="n">
         <f aca="false">IF($C50="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H50" s="7"/>
-      <c r="I50" s="14" t="n">
+      <c r="I50" s="15" t="n">
         <f aca="false">IF($C50="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J50" s="16" t="n">
+      <c r="J50" s="17" t="n">
         <f aca="false">IF($C50="Lease-koop",D50+p_SlotJr,IF($C50="Koop",D50,0))</f>
         <v>0</v>
       </c>
-      <c r="K50" s="14" t="n">
+      <c r="K50" s="15" t="n">
         <f aca="false">E50+F50+G50+H50+I50</f>
         <v>0</v>
       </c>
-      <c r="L50" s="16" t="n">
+      <c r="L50" s="17" t="n">
         <f aca="false">IF($C50="Lease-koop",p_Afschr,IF($C50="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A50,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M50" s="16" t="n">
+      <c r="M50" s="17" t="n">
         <f aca="false">IF($C50="Lease-koop",D50+p_Lev,IF(AND($C50="Koop",D50&gt;0),D50+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A50,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N50" s="14" t="n">
+      <c r="N50" s="15" t="n">
         <f aca="false">IF($C50="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D51" s="5"/>
-      <c r="E51" s="14" t="n">
+      <c r="E51" s="15" t="n">
         <f aca="false">IF($C51="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F51" s="14" t="n">
+      <c r="F51" s="15" t="n">
         <f aca="false">IF($C51="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G51" s="14" t="n">
+      <c r="G51" s="15" t="n">
         <f aca="false">IF($C51="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H51" s="7"/>
-      <c r="I51" s="14" t="n">
+      <c r="I51" s="15" t="n">
         <f aca="false">IF($C51="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J51" s="16" t="n">
+      <c r="J51" s="17" t="n">
         <f aca="false">IF($C51="Lease-koop",D51+p_SlotJr,IF($C51="Koop",D51,0))</f>
         <v>0</v>
       </c>
-      <c r="K51" s="14" t="n">
+      <c r="K51" s="15" t="n">
         <f aca="false">E51+F51+G51+H51+I51</f>
         <v>0</v>
       </c>
-      <c r="L51" s="16" t="n">
+      <c r="L51" s="17" t="n">
         <f aca="false">IF($C51="Lease-koop",p_Afschr,IF($C51="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A51,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M51" s="16" t="n">
+      <c r="M51" s="17" t="n">
         <f aca="false">IF($C51="Lease-koop",D51+p_Lev,IF(AND($C51="Koop",D51&gt;0),D51+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A51,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N51" s="14" t="n">
+      <c r="N51" s="15" t="n">
         <f aca="false">IF($C51="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D52" s="5"/>
-      <c r="E52" s="14" t="n">
+      <c r="E52" s="15" t="n">
         <f aca="false">IF($C52="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F52" s="14" t="n">
+      <c r="F52" s="15" t="n">
         <f aca="false">IF($C52="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G52" s="14" t="n">
+      <c r="G52" s="15" t="n">
         <f aca="false">IF($C52="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H52" s="7"/>
-      <c r="I52" s="14" t="n">
+      <c r="I52" s="15" t="n">
         <f aca="false">IF($C52="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J52" s="16" t="n">
+      <c r="J52" s="17" t="n">
         <f aca="false">IF($C52="Lease-koop",D52+p_SlotJr,IF($C52="Koop",D52,0))</f>
         <v>0</v>
       </c>
-      <c r="K52" s="14" t="n">
+      <c r="K52" s="15" t="n">
         <f aca="false">E52+F52+G52+H52+I52</f>
         <v>0</v>
       </c>
-      <c r="L52" s="16" t="n">
+      <c r="L52" s="17" t="n">
         <f aca="false">IF($C52="Lease-koop",p_Afschr,IF($C52="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A52,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M52" s="16" t="n">
+      <c r="M52" s="17" t="n">
         <f aca="false">IF($C52="Lease-koop",D52+p_Lev,IF(AND($C52="Koop",D52&gt;0),D52+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A52,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N52" s="14" t="n">
+      <c r="N52" s="15" t="n">
         <f aca="false">IF($C52="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D53" s="5"/>
-      <c r="E53" s="14" t="n">
+      <c r="E53" s="15" t="n">
         <f aca="false">IF($C53="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F53" s="14" t="n">
+      <c r="F53" s="15" t="n">
         <f aca="false">IF($C53="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G53" s="14" t="n">
+      <c r="G53" s="15" t="n">
         <f aca="false">IF($C53="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H53" s="7"/>
-      <c r="I53" s="14" t="n">
+      <c r="I53" s="15" t="n">
         <f aca="false">IF($C53="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J53" s="16" t="n">
+      <c r="J53" s="17" t="n">
         <f aca="false">IF($C53="Lease-koop",D53+p_SlotJr,IF($C53="Koop",D53,0))</f>
         <v>0</v>
       </c>
-      <c r="K53" s="14" t="n">
+      <c r="K53" s="15" t="n">
         <f aca="false">E53+F53+G53+H53+I53</f>
         <v>0</v>
       </c>
-      <c r="L53" s="16" t="n">
+      <c r="L53" s="17" t="n">
         <f aca="false">IF($C53="Lease-koop",p_Afschr,IF($C53="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A53,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M53" s="16" t="n">
+      <c r="M53" s="17" t="n">
         <f aca="false">IF($C53="Lease-koop",D53+p_Lev,IF(AND($C53="Koop",D53&gt;0),D53+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A53,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N53" s="14" t="n">
+      <c r="N53" s="15" t="n">
         <f aca="false">IF($C53="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D54" s="5"/>
-      <c r="E54" s="14" t="n">
+      <c r="E54" s="15" t="n">
         <f aca="false">IF($C54="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F54" s="14" t="n">
+      <c r="F54" s="15" t="n">
         <f aca="false">IF($C54="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G54" s="14" t="n">
+      <c r="G54" s="15" t="n">
         <f aca="false">IF($C54="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H54" s="7"/>
-      <c r="I54" s="14" t="n">
+      <c r="I54" s="15" t="n">
         <f aca="false">IF($C54="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J54" s="16" t="n">
+      <c r="J54" s="17" t="n">
         <f aca="false">IF($C54="Lease-koop",D54+p_SlotJr,IF($C54="Koop",D54,0))</f>
         <v>0</v>
       </c>
-      <c r="K54" s="14" t="n">
+      <c r="K54" s="15" t="n">
         <f aca="false">E54+F54+G54+H54+I54</f>
         <v>0</v>
       </c>
-      <c r="L54" s="16" t="n">
+      <c r="L54" s="17" t="n">
         <f aca="false">IF($C54="Lease-koop",p_Afschr,IF($C54="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A54,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M54" s="16" t="n">
+      <c r="M54" s="17" t="n">
         <f aca="false">IF($C54="Lease-koop",D54+p_Lev,IF(AND($C54="Koop",D54&gt;0),D54+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A54,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N54" s="14" t="n">
+      <c r="N54" s="15" t="n">
         <f aca="false">IF($C54="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D55" s="5"/>
-      <c r="E55" s="14" t="n">
+      <c r="E55" s="15" t="n">
         <f aca="false">IF($C55="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F55" s="14" t="n">
+      <c r="F55" s="15" t="n">
         <f aca="false">IF($C55="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G55" s="14" t="n">
+      <c r="G55" s="15" t="n">
         <f aca="false">IF($C55="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H55" s="7"/>
-      <c r="I55" s="14" t="n">
+      <c r="I55" s="15" t="n">
         <f aca="false">IF($C55="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J55" s="16" t="n">
+      <c r="J55" s="17" t="n">
         <f aca="false">IF($C55="Lease-koop",D55+p_SlotJr,IF($C55="Koop",D55,0))</f>
         <v>0</v>
       </c>
-      <c r="K55" s="14" t="n">
+      <c r="K55" s="15" t="n">
         <f aca="false">E55+F55+G55+H55+I55</f>
         <v>0</v>
       </c>
-      <c r="L55" s="16" t="n">
+      <c r="L55" s="17" t="n">
         <f aca="false">IF($C55="Lease-koop",p_Afschr,IF($C55="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A55,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M55" s="16" t="n">
+      <c r="M55" s="17" t="n">
         <f aca="false">IF($C55="Lease-koop",D55+p_Lev,IF(AND($C55="Koop",D55&gt;0),D55+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A55,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N55" s="14" t="n">
+      <c r="N55" s="15" t="n">
         <f aca="false">IF($C55="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D56" s="5"/>
-      <c r="E56" s="14" t="n">
+      <c r="E56" s="15" t="n">
         <f aca="false">IF($C56="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F56" s="14" t="n">
+      <c r="F56" s="15" t="n">
         <f aca="false">IF($C56="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G56" s="14" t="n">
+      <c r="G56" s="15" t="n">
         <f aca="false">IF($C56="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H56" s="7"/>
-      <c r="I56" s="14" t="n">
+      <c r="I56" s="15" t="n">
         <f aca="false">IF($C56="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J56" s="16" t="n">
+      <c r="J56" s="17" t="n">
         <f aca="false">IF($C56="Lease-koop",D56+p_SlotJr,IF($C56="Koop",D56,0))</f>
         <v>0</v>
       </c>
-      <c r="K56" s="14" t="n">
+      <c r="K56" s="15" t="n">
         <f aca="false">E56+F56+G56+H56+I56</f>
         <v>0</v>
       </c>
-      <c r="L56" s="16" t="n">
+      <c r="L56" s="17" t="n">
         <f aca="false">IF($C56="Lease-koop",p_Afschr,IF($C56="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A56,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M56" s="16" t="n">
+      <c r="M56" s="17" t="n">
         <f aca="false">IF($C56="Lease-koop",D56+p_Lev,IF(AND($C56="Koop",D56&gt;0),D56+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A56,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N56" s="14" t="n">
+      <c r="N56" s="15" t="n">
         <f aca="false">IF($C56="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D57" s="5"/>
-      <c r="E57" s="14" t="n">
+      <c r="E57" s="15" t="n">
         <f aca="false">IF($C57="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F57" s="14" t="n">
+      <c r="F57" s="15" t="n">
         <f aca="false">IF($C57="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G57" s="14" t="n">
+      <c r="G57" s="15" t="n">
         <f aca="false">IF($C57="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H57" s="7"/>
-      <c r="I57" s="14" t="n">
+      <c r="I57" s="15" t="n">
         <f aca="false">IF($C57="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J57" s="16" t="n">
+      <c r="J57" s="17" t="n">
         <f aca="false">IF($C57="Lease-koop",D57+p_SlotJr,IF($C57="Koop",D57,0))</f>
         <v>0</v>
       </c>
-      <c r="K57" s="14" t="n">
+      <c r="K57" s="15" t="n">
         <f aca="false">E57+F57+G57+H57+I57</f>
         <v>0</v>
       </c>
-      <c r="L57" s="16" t="n">
+      <c r="L57" s="17" t="n">
         <f aca="false">IF($C57="Lease-koop",p_Afschr,IF($C57="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A57,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M57" s="16" t="n">
+      <c r="M57" s="17" t="n">
         <f aca="false">IF($C57="Lease-koop",D57+p_Lev,IF(AND($C57="Koop",D57&gt;0),D57+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A57,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N57" s="14" t="n">
+      <c r="N57" s="15" t="n">
         <f aca="false">IF($C57="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D58" s="5"/>
-      <c r="E58" s="14" t="n">
+      <c r="E58" s="15" t="n">
         <f aca="false">IF($C58="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F58" s="14" t="n">
+      <c r="F58" s="15" t="n">
         <f aca="false">IF($C58="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G58" s="14" t="n">
+      <c r="G58" s="15" t="n">
         <f aca="false">IF($C58="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H58" s="7"/>
-      <c r="I58" s="14" t="n">
+      <c r="I58" s="15" t="n">
         <f aca="false">IF($C58="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J58" s="16" t="n">
+      <c r="J58" s="17" t="n">
         <f aca="false">IF($C58="Lease-koop",D58+p_SlotJr,IF($C58="Koop",D58,0))</f>
         <v>0</v>
       </c>
-      <c r="K58" s="14" t="n">
+      <c r="K58" s="15" t="n">
         <f aca="false">E58+F58+G58+H58+I58</f>
         <v>0</v>
       </c>
-      <c r="L58" s="16" t="n">
+      <c r="L58" s="17" t="n">
         <f aca="false">IF($C58="Lease-koop",p_Afschr,IF($C58="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A58,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M58" s="16" t="n">
+      <c r="M58" s="17" t="n">
         <f aca="false">IF($C58="Lease-koop",D58+p_Lev,IF(AND($C58="Koop",D58&gt;0),D58+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A58,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N58" s="14" t="n">
+      <c r="N58" s="15" t="n">
         <f aca="false">IF($C58="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D59" s="5"/>
-      <c r="E59" s="14" t="n">
+      <c r="E59" s="15" t="n">
         <f aca="false">IF($C59="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F59" s="14" t="n">
+      <c r="F59" s="15" t="n">
         <f aca="false">IF($C59="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G59" s="14" t="n">
+      <c r="G59" s="15" t="n">
         <f aca="false">IF($C59="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H59" s="7"/>
-      <c r="I59" s="14" t="n">
+      <c r="I59" s="15" t="n">
         <f aca="false">IF($C59="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J59" s="16" t="n">
+      <c r="J59" s="17" t="n">
         <f aca="false">IF($C59="Lease-koop",D59+p_SlotJr,IF($C59="Koop",D59,0))</f>
         <v>0</v>
       </c>
-      <c r="K59" s="14" t="n">
+      <c r="K59" s="15" t="n">
         <f aca="false">E59+F59+G59+H59+I59</f>
         <v>0</v>
       </c>
-      <c r="L59" s="16" t="n">
+      <c r="L59" s="17" t="n">
         <f aca="false">IF($C59="Lease-koop",p_Afschr,IF($C59="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A59,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M59" s="16" t="n">
+      <c r="M59" s="17" t="n">
         <f aca="false">IF($C59="Lease-koop",D59+p_Lev,IF(AND($C59="Koop",D59&gt;0),D59+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A59,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N59" s="14" t="n">
+      <c r="N59" s="15" t="n">
         <f aca="false">IF($C59="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D60" s="5"/>
-      <c r="E60" s="14" t="n">
+      <c r="E60" s="15" t="n">
         <f aca="false">IF($C60="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F60" s="14" t="n">
+      <c r="F60" s="15" t="n">
         <f aca="false">IF($C60="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G60" s="14" t="n">
+      <c r="G60" s="15" t="n">
         <f aca="false">IF($C60="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H60" s="7"/>
-      <c r="I60" s="14" t="n">
+      <c r="I60" s="15" t="n">
         <f aca="false">IF($C60="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J60" s="16" t="n">
+      <c r="J60" s="17" t="n">
         <f aca="false">IF($C60="Lease-koop",D60+p_SlotJr,IF($C60="Koop",D60,0))</f>
         <v>0</v>
       </c>
-      <c r="K60" s="14" t="n">
+      <c r="K60" s="15" t="n">
         <f aca="false">E60+F60+G60+H60+I60</f>
         <v>0</v>
       </c>
-      <c r="L60" s="16" t="n">
+      <c r="L60" s="17" t="n">
         <f aca="false">IF($C60="Lease-koop",p_Afschr,IF($C60="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A60,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M60" s="16" t="n">
+      <c r="M60" s="17" t="n">
         <f aca="false">IF($C60="Lease-koop",D60+p_Lev,IF(AND($C60="Koop",D60&gt;0),D60+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A60,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N60" s="14" t="n">
+      <c r="N60" s="15" t="n">
         <f aca="false">IF($C60="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D61" s="5"/>
-      <c r="E61" s="14" t="n">
+      <c r="E61" s="15" t="n">
         <f aca="false">IF($C61="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F61" s="14" t="n">
+      <c r="F61" s="15" t="n">
         <f aca="false">IF($C61="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G61" s="14" t="n">
+      <c r="G61" s="15" t="n">
         <f aca="false">IF($C61="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H61" s="7"/>
-      <c r="I61" s="14" t="n">
+      <c r="I61" s="15" t="n">
         <f aca="false">IF($C61="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J61" s="16" t="n">
+      <c r="J61" s="17" t="n">
         <f aca="false">IF($C61="Lease-koop",D61+p_SlotJr,IF($C61="Koop",D61,0))</f>
         <v>0</v>
       </c>
-      <c r="K61" s="14" t="n">
+      <c r="K61" s="15" t="n">
         <f aca="false">E61+F61+G61+H61+I61</f>
         <v>0</v>
       </c>
-      <c r="L61" s="16" t="n">
+      <c r="L61" s="17" t="n">
         <f aca="false">IF($C61="Lease-koop",p_Afschr,IF($C61="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A61,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M61" s="16" t="n">
+      <c r="M61" s="17" t="n">
         <f aca="false">IF($C61="Lease-koop",D61+p_Lev,IF(AND($C61="Koop",D61&gt;0),D61+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A61,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N61" s="14" t="n">
+      <c r="N61" s="15" t="n">
         <f aca="false">IF($C61="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D62" s="5"/>
-      <c r="E62" s="14" t="n">
+      <c r="E62" s="15" t="n">
         <f aca="false">IF($C62="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F62" s="14" t="n">
+      <c r="F62" s="15" t="n">
         <f aca="false">IF($C62="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G62" s="14" t="n">
+      <c r="G62" s="15" t="n">
         <f aca="false">IF($C62="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H62" s="7"/>
-      <c r="I62" s="14" t="n">
+      <c r="I62" s="15" t="n">
         <f aca="false">IF($C62="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J62" s="16" t="n">
+      <c r="J62" s="17" t="n">
         <f aca="false">IF($C62="Lease-koop",D62+p_SlotJr,IF($C62="Koop",D62,0))</f>
         <v>0</v>
       </c>
-      <c r="K62" s="14" t="n">
+      <c r="K62" s="15" t="n">
         <f aca="false">E62+F62+G62+H62+I62</f>
         <v>0</v>
       </c>
-      <c r="L62" s="16" t="n">
+      <c r="L62" s="17" t="n">
         <f aca="false">IF($C62="Lease-koop",p_Afschr,IF($C62="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A62,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M62" s="16" t="n">
+      <c r="M62" s="17" t="n">
         <f aca="false">IF($C62="Lease-koop",D62+p_Lev,IF(AND($C62="Koop",D62&gt;0),D62+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A62,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N62" s="14" t="n">
+      <c r="N62" s="15" t="n">
         <f aca="false">IF($C62="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D63" s="5"/>
-      <c r="E63" s="14" t="n">
+      <c r="E63" s="15" t="n">
         <f aca="false">IF($C63="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F63" s="14" t="n">
+      <c r="F63" s="15" t="n">
         <f aca="false">IF($C63="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G63" s="14" t="n">
+      <c r="G63" s="15" t="n">
         <f aca="false">IF($C63="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H63" s="7"/>
-      <c r="I63" s="14" t="n">
+      <c r="I63" s="15" t="n">
         <f aca="false">IF($C63="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J63" s="16" t="n">
+      <c r="J63" s="17" t="n">
         <f aca="false">IF($C63="Lease-koop",D63+p_SlotJr,IF($C63="Koop",D63,0))</f>
         <v>0</v>
       </c>
-      <c r="K63" s="14" t="n">
+      <c r="K63" s="15" t="n">
         <f aca="false">E63+F63+G63+H63+I63</f>
         <v>0</v>
       </c>
-      <c r="L63" s="16" t="n">
+      <c r="L63" s="17" t="n">
         <f aca="false">IF($C63="Lease-koop",p_Afschr,IF($C63="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A63,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M63" s="16" t="n">
+      <c r="M63" s="17" t="n">
         <f aca="false">IF($C63="Lease-koop",D63+p_Lev,IF(AND($C63="Koop",D63&gt;0),D63+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A63,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N63" s="14" t="n">
+      <c r="N63" s="15" t="n">
         <f aca="false">IF($C63="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D64" s="5"/>
-      <c r="E64" s="14" t="n">
+      <c r="E64" s="15" t="n">
         <f aca="false">IF($C64="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F64" s="14" t="n">
+      <c r="F64" s="15" t="n">
         <f aca="false">IF($C64="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G64" s="14" t="n">
+      <c r="G64" s="15" t="n">
         <f aca="false">IF($C64="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H64" s="7"/>
-      <c r="I64" s="14" t="n">
+      <c r="I64" s="15" t="n">
         <f aca="false">IF($C64="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J64" s="16" t="n">
+      <c r="J64" s="17" t="n">
         <f aca="false">IF($C64="Lease-koop",D64+p_SlotJr,IF($C64="Koop",D64,0))</f>
         <v>0</v>
       </c>
-      <c r="K64" s="14" t="n">
+      <c r="K64" s="15" t="n">
         <f aca="false">E64+F64+G64+H64+I64</f>
         <v>0</v>
       </c>
-      <c r="L64" s="16" t="n">
+      <c r="L64" s="17" t="n">
         <f aca="false">IF($C64="Lease-koop",p_Afschr,IF($C64="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A64,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M64" s="16" t="n">
+      <c r="M64" s="17" t="n">
         <f aca="false">IF($C64="Lease-koop",D64+p_Lev,IF(AND($C64="Koop",D64&gt;0),D64+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A64,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N64" s="14" t="n">
+      <c r="N64" s="15" t="n">
         <f aca="false">IF($C64="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D65" s="5"/>
-      <c r="E65" s="14" t="n">
+      <c r="E65" s="15" t="n">
         <f aca="false">IF($C65="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F65" s="14" t="n">
+      <c r="F65" s="15" t="n">
         <f aca="false">IF($C65="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G65" s="14" t="n">
+      <c r="G65" s="15" t="n">
         <f aca="false">IF($C65="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H65" s="7"/>
-      <c r="I65" s="14" t="n">
+      <c r="I65" s="15" t="n">
         <f aca="false">IF($C65="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J65" s="16" t="n">
+      <c r="J65" s="17" t="n">
         <f aca="false">IF($C65="Lease-koop",D65+p_SlotJr,IF($C65="Koop",D65,0))</f>
         <v>0</v>
       </c>
-      <c r="K65" s="14" t="n">
+      <c r="K65" s="15" t="n">
         <f aca="false">E65+F65+G65+H65+I65</f>
         <v>0</v>
       </c>
-      <c r="L65" s="16" t="n">
+      <c r="L65" s="17" t="n">
         <f aca="false">IF($C65="Lease-koop",p_Afschr,IF($C65="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A65,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M65" s="16" t="n">
+      <c r="M65" s="17" t="n">
         <f aca="false">IF($C65="Lease-koop",D65+p_Lev,IF(AND($C65="Koop",D65&gt;0),D65+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A65,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N65" s="14" t="n">
+      <c r="N65" s="15" t="n">
         <f aca="false">IF($C65="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D66" s="5"/>
-      <c r="E66" s="14" t="n">
+      <c r="E66" s="15" t="n">
         <f aca="false">IF($C66="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F66" s="14" t="n">
+      <c r="F66" s="15" t="n">
         <f aca="false">IF($C66="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G66" s="14" t="n">
+      <c r="G66" s="15" t="n">
         <f aca="false">IF($C66="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H66" s="7"/>
-      <c r="I66" s="14" t="n">
+      <c r="I66" s="15" t="n">
         <f aca="false">IF($C66="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J66" s="16" t="n">
+      <c r="J66" s="17" t="n">
         <f aca="false">IF($C66="Lease-koop",D66+p_SlotJr,IF($C66="Koop",D66,0))</f>
         <v>0</v>
       </c>
-      <c r="K66" s="14" t="n">
+      <c r="K66" s="15" t="n">
         <f aca="false">E66+F66+G66+H66+I66</f>
         <v>0</v>
       </c>
-      <c r="L66" s="16" t="n">
+      <c r="L66" s="17" t="n">
         <f aca="false">IF($C66="Lease-koop",p_Afschr,IF($C66="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A66,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M66" s="16" t="n">
+      <c r="M66" s="17" t="n">
         <f aca="false">IF($C66="Lease-koop",D66+p_Lev,IF(AND($C66="Koop",D66&gt;0),D66+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A66,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N66" s="14" t="n">
+      <c r="N66" s="15" t="n">
         <f aca="false">IF($C66="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D67" s="5"/>
-      <c r="E67" s="14" t="n">
+      <c r="E67" s="15" t="n">
         <f aca="false">IF($C67="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F67" s="14" t="n">
+      <c r="F67" s="15" t="n">
         <f aca="false">IF($C67="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G67" s="14" t="n">
+      <c r="G67" s="15" t="n">
         <f aca="false">IF($C67="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H67" s="7"/>
-      <c r="I67" s="14" t="n">
+      <c r="I67" s="15" t="n">
         <f aca="false">IF($C67="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J67" s="16" t="n">
+      <c r="J67" s="17" t="n">
         <f aca="false">IF($C67="Lease-koop",D67+p_SlotJr,IF($C67="Koop",D67,0))</f>
         <v>0</v>
       </c>
-      <c r="K67" s="14" t="n">
+      <c r="K67" s="15" t="n">
         <f aca="false">E67+F67+G67+H67+I67</f>
         <v>0</v>
       </c>
-      <c r="L67" s="16" t="n">
+      <c r="L67" s="17" t="n">
         <f aca="false">IF($C67="Lease-koop",p_Afschr,IF($C67="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A67,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M67" s="16" t="n">
+      <c r="M67" s="17" t="n">
         <f aca="false">IF($C67="Lease-koop",D67+p_Lev,IF(AND($C67="Koop",D67&gt;0),D67+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A67,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N67" s="14" t="n">
+      <c r="N67" s="15" t="n">
         <f aca="false">IF($C67="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D68" s="5"/>
-      <c r="E68" s="14" t="n">
+      <c r="E68" s="15" t="n">
         <f aca="false">IF($C68="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F68" s="14" t="n">
+      <c r="F68" s="15" t="n">
         <f aca="false">IF($C68="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G68" s="14" t="n">
+      <c r="G68" s="15" t="n">
         <f aca="false">IF($C68="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H68" s="7"/>
-      <c r="I68" s="14" t="n">
+      <c r="I68" s="15" t="n">
         <f aca="false">IF($C68="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J68" s="16" t="n">
+      <c r="J68" s="17" t="n">
         <f aca="false">IF($C68="Lease-koop",D68+p_SlotJr,IF($C68="Koop",D68,0))</f>
         <v>0</v>
       </c>
-      <c r="K68" s="14" t="n">
+      <c r="K68" s="15" t="n">
         <f aca="false">E68+F68+G68+H68+I68</f>
         <v>0</v>
       </c>
-      <c r="L68" s="16" t="n">
+      <c r="L68" s="17" t="n">
         <f aca="false">IF($C68="Lease-koop",p_Afschr,IF($C68="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A68,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M68" s="16" t="n">
+      <c r="M68" s="17" t="n">
         <f aca="false">IF($C68="Lease-koop",D68+p_Lev,IF(AND($C68="Koop",D68&gt;0),D68+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A68,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N68" s="14" t="n">
+      <c r="N68" s="15" t="n">
         <f aca="false">IF($C68="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D69" s="5"/>
-      <c r="E69" s="14" t="n">
+      <c r="E69" s="15" t="n">
         <f aca="false">IF($C69="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F69" s="14" t="n">
+      <c r="F69" s="15" t="n">
         <f aca="false">IF($C69="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G69" s="14" t="n">
+      <c r="G69" s="15" t="n">
         <f aca="false">IF($C69="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H69" s="7"/>
-      <c r="I69" s="14" t="n">
+      <c r="I69" s="15" t="n">
         <f aca="false">IF($C69="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J69" s="16" t="n">
+      <c r="J69" s="17" t="n">
         <f aca="false">IF($C69="Lease-koop",D69+p_SlotJr,IF($C69="Koop",D69,0))</f>
         <v>0</v>
       </c>
-      <c r="K69" s="14" t="n">
+      <c r="K69" s="15" t="n">
         <f aca="false">E69+F69+G69+H69+I69</f>
         <v>0</v>
       </c>
-      <c r="L69" s="16" t="n">
+      <c r="L69" s="17" t="n">
         <f aca="false">IF($C69="Lease-koop",p_Afschr,IF($C69="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A69,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M69" s="16" t="n">
+      <c r="M69" s="17" t="n">
         <f aca="false">IF($C69="Lease-koop",D69+p_Lev,IF(AND($C69="Koop",D69&gt;0),D69+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A69,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N69" s="14" t="n">
+      <c r="N69" s="15" t="n">
         <f aca="false">IF($C69="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D70" s="5"/>
-      <c r="E70" s="14" t="n">
+      <c r="E70" s="15" t="n">
         <f aca="false">IF($C70="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F70" s="14" t="n">
+      <c r="F70" s="15" t="n">
         <f aca="false">IF($C70="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G70" s="14" t="n">
+      <c r="G70" s="15" t="n">
         <f aca="false">IF($C70="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H70" s="7"/>
-      <c r="I70" s="14" t="n">
+      <c r="I70" s="15" t="n">
         <f aca="false">IF($C70="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J70" s="16" t="n">
+      <c r="J70" s="17" t="n">
         <f aca="false">IF($C70="Lease-koop",D70+p_SlotJr,IF($C70="Koop",D70,0))</f>
         <v>0</v>
       </c>
-      <c r="K70" s="14" t="n">
+      <c r="K70" s="15" t="n">
         <f aca="false">E70+F70+G70+H70+I70</f>
         <v>0</v>
       </c>
-      <c r="L70" s="16" t="n">
+      <c r="L70" s="17" t="n">
         <f aca="false">IF($C70="Lease-koop",p_Afschr,IF($C70="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A70,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M70" s="16" t="n">
+      <c r="M70" s="17" t="n">
         <f aca="false">IF($C70="Lease-koop",D70+p_Lev,IF(AND($C70="Koop",D70&gt;0),D70+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A70,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N70" s="14" t="n">
+      <c r="N70" s="15" t="n">
         <f aca="false">IF($C70="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D71" s="5"/>
-      <c r="E71" s="14" t="n">
+      <c r="E71" s="15" t="n">
         <f aca="false">IF($C71="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F71" s="14" t="n">
+      <c r="F71" s="15" t="n">
         <f aca="false">IF($C71="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G71" s="14" t="n">
+      <c r="G71" s="15" t="n">
         <f aca="false">IF($C71="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H71" s="7"/>
-      <c r="I71" s="14" t="n">
+      <c r="I71" s="15" t="n">
         <f aca="false">IF($C71="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J71" s="16" t="n">
+      <c r="J71" s="17" t="n">
         <f aca="false">IF($C71="Lease-koop",D71+p_SlotJr,IF($C71="Koop",D71,0))</f>
         <v>0</v>
       </c>
-      <c r="K71" s="14" t="n">
+      <c r="K71" s="15" t="n">
         <f aca="false">E71+F71+G71+H71+I71</f>
         <v>0</v>
       </c>
-      <c r="L71" s="16" t="n">
+      <c r="L71" s="17" t="n">
         <f aca="false">IF($C71="Lease-koop",p_Afschr,IF($C71="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A71,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M71" s="16" t="n">
+      <c r="M71" s="17" t="n">
         <f aca="false">IF($C71="Lease-koop",D71+p_Lev,IF(AND($C71="Koop",D71&gt;0),D71+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A71,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N71" s="14" t="n">
+      <c r="N71" s="15" t="n">
         <f aca="false">IF($C71="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D72" s="5"/>
-      <c r="E72" s="14" t="n">
+      <c r="E72" s="15" t="n">
         <f aca="false">IF($C72="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F72" s="14" t="n">
+      <c r="F72" s="15" t="n">
         <f aca="false">IF($C72="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G72" s="14" t="n">
+      <c r="G72" s="15" t="n">
         <f aca="false">IF($C72="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H72" s="7"/>
-      <c r="I72" s="14" t="n">
+      <c r="I72" s="15" t="n">
         <f aca="false">IF($C72="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J72" s="16" t="n">
+      <c r="J72" s="17" t="n">
         <f aca="false">IF($C72="Lease-koop",D72+p_SlotJr,IF($C72="Koop",D72,0))</f>
         <v>0</v>
       </c>
-      <c r="K72" s="14" t="n">
+      <c r="K72" s="15" t="n">
         <f aca="false">E72+F72+G72+H72+I72</f>
         <v>0</v>
       </c>
-      <c r="L72" s="16" t="n">
+      <c r="L72" s="17" t="n">
         <f aca="false">IF($C72="Lease-koop",p_Afschr,IF($C72="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A72,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M72" s="16" t="n">
+      <c r="M72" s="17" t="n">
         <f aca="false">IF($C72="Lease-koop",D72+p_Lev,IF(AND($C72="Koop",D72&gt;0),D72+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A72,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N72" s="14" t="n">
+      <c r="N72" s="15" t="n">
         <f aca="false">IF($C72="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D73" s="5"/>
-      <c r="E73" s="14" t="n">
+      <c r="E73" s="15" t="n">
         <f aca="false">IF($C73="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F73" s="14" t="n">
+      <c r="F73" s="15" t="n">
         <f aca="false">IF($C73="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G73" s="14" t="n">
+      <c r="G73" s="15" t="n">
         <f aca="false">IF($C73="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H73" s="7"/>
-      <c r="I73" s="14" t="n">
+      <c r="I73" s="15" t="n">
         <f aca="false">IF($C73="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J73" s="16" t="n">
+      <c r="J73" s="17" t="n">
         <f aca="false">IF($C73="Lease-koop",D73+p_SlotJr,IF($C73="Koop",D73,0))</f>
         <v>0</v>
       </c>
-      <c r="K73" s="14" t="n">
+      <c r="K73" s="15" t="n">
         <f aca="false">E73+F73+G73+H73+I73</f>
         <v>0</v>
       </c>
-      <c r="L73" s="16" t="n">
+      <c r="L73" s="17" t="n">
         <f aca="false">IF($C73="Lease-koop",p_Afschr,IF($C73="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A73,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M73" s="16" t="n">
+      <c r="M73" s="17" t="n">
         <f aca="false">IF($C73="Lease-koop",D73+p_Lev,IF(AND($C73="Koop",D73&gt;0),D73+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A73,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N73" s="14" t="n">
+      <c r="N73" s="15" t="n">
         <f aca="false">IF($C73="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D74" s="5"/>
-      <c r="E74" s="14" t="n">
+      <c r="E74" s="15" t="n">
         <f aca="false">IF($C74="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F74" s="14" t="n">
+      <c r="F74" s="15" t="n">
         <f aca="false">IF($C74="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G74" s="14" t="n">
+      <c r="G74" s="15" t="n">
         <f aca="false">IF($C74="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H74" s="7"/>
-      <c r="I74" s="14" t="n">
+      <c r="I74" s="15" t="n">
         <f aca="false">IF($C74="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J74" s="16" t="n">
+      <c r="J74" s="17" t="n">
         <f aca="false">IF($C74="Lease-koop",D74+p_SlotJr,IF($C74="Koop",D74,0))</f>
         <v>0</v>
       </c>
-      <c r="K74" s="14" t="n">
+      <c r="K74" s="15" t="n">
         <f aca="false">E74+F74+G74+H74+I74</f>
         <v>0</v>
       </c>
-      <c r="L74" s="16" t="n">
+      <c r="L74" s="17" t="n">
         <f aca="false">IF($C74="Lease-koop",p_Afschr,IF($C74="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A74,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M74" s="16" t="n">
+      <c r="M74" s="17" t="n">
         <f aca="false">IF($C74="Lease-koop",D74+p_Lev,IF(AND($C74="Koop",D74&gt;0),D74+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A74,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N74" s="14" t="n">
+      <c r="N74" s="15" t="n">
         <f aca="false">IF($C74="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D75" s="5"/>
-      <c r="E75" s="14" t="n">
+      <c r="E75" s="15" t="n">
         <f aca="false">IF($C75="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F75" s="14" t="n">
+      <c r="F75" s="15" t="n">
         <f aca="false">IF($C75="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G75" s="14" t="n">
+      <c r="G75" s="15" t="n">
         <f aca="false">IF($C75="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H75" s="7"/>
-      <c r="I75" s="14" t="n">
+      <c r="I75" s="15" t="n">
         <f aca="false">IF($C75="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J75" s="16" t="n">
+      <c r="J75" s="17" t="n">
         <f aca="false">IF($C75="Lease-koop",D75+p_SlotJr,IF($C75="Koop",D75,0))</f>
         <v>0</v>
       </c>
-      <c r="K75" s="14" t="n">
+      <c r="K75" s="15" t="n">
         <f aca="false">E75+F75+G75+H75+I75</f>
         <v>0</v>
       </c>
-      <c r="L75" s="16" t="n">
+      <c r="L75" s="17" t="n">
         <f aca="false">IF($C75="Lease-koop",p_Afschr,IF($C75="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A75,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M75" s="16" t="n">
+      <c r="M75" s="17" t="n">
         <f aca="false">IF($C75="Lease-koop",D75+p_Lev,IF(AND($C75="Koop",D75&gt;0),D75+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A75,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N75" s="14" t="n">
+      <c r="N75" s="15" t="n">
         <f aca="false">IF($C75="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D76" s="5"/>
-      <c r="E76" s="14" t="n">
+      <c r="E76" s="15" t="n">
         <f aca="false">IF($C76="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F76" s="14" t="n">
+      <c r="F76" s="15" t="n">
         <f aca="false">IF($C76="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G76" s="14" t="n">
+      <c r="G76" s="15" t="n">
         <f aca="false">IF($C76="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H76" s="7"/>
-      <c r="I76" s="14" t="n">
+      <c r="I76" s="15" t="n">
         <f aca="false">IF($C76="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J76" s="16" t="n">
+      <c r="J76" s="17" t="n">
         <f aca="false">IF($C76="Lease-koop",D76+p_SlotJr,IF($C76="Koop",D76,0))</f>
         <v>0</v>
       </c>
-      <c r="K76" s="14" t="n">
+      <c r="K76" s="15" t="n">
         <f aca="false">E76+F76+G76+H76+I76</f>
         <v>0</v>
       </c>
-      <c r="L76" s="16" t="n">
+      <c r="L76" s="17" t="n">
         <f aca="false">IF($C76="Lease-koop",p_Afschr,IF($C76="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A76,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M76" s="16" t="n">
+      <c r="M76" s="17" t="n">
         <f aca="false">IF($C76="Lease-koop",D76+p_Lev,IF(AND($C76="Koop",D76&gt;0),D76+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A76,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N76" s="14" t="n">
+      <c r="N76" s="15" t="n">
         <f aca="false">IF($C76="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D77" s="5"/>
-      <c r="E77" s="14" t="n">
+      <c r="E77" s="15" t="n">
         <f aca="false">IF($C77="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F77" s="14" t="n">
+      <c r="F77" s="15" t="n">
         <f aca="false">IF($C77="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G77" s="14" t="n">
+      <c r="G77" s="15" t="n">
         <f aca="false">IF($C77="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H77" s="7"/>
-      <c r="I77" s="14" t="n">
+      <c r="I77" s="15" t="n">
         <f aca="false">IF($C77="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J77" s="16" t="n">
+      <c r="J77" s="17" t="n">
         <f aca="false">IF($C77="Lease-koop",D77+p_SlotJr,IF($C77="Koop",D77,0))</f>
         <v>0</v>
       </c>
-      <c r="K77" s="14" t="n">
+      <c r="K77" s="15" t="n">
         <f aca="false">E77+F77+G77+H77+I77</f>
         <v>0</v>
       </c>
-      <c r="L77" s="16" t="n">
+      <c r="L77" s="17" t="n">
         <f aca="false">IF($C77="Lease-koop",p_Afschr,IF($C77="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A77,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M77" s="16" t="n">
+      <c r="M77" s="17" t="n">
         <f aca="false">IF($C77="Lease-koop",D77+p_Lev,IF(AND($C77="Koop",D77&gt;0),D77+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A77,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N77" s="14" t="n">
+      <c r="N77" s="15" t="n">
         <f aca="false">IF($C77="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D78" s="5"/>
-      <c r="E78" s="14" t="n">
+      <c r="E78" s="15" t="n">
         <f aca="false">IF($C78="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F78" s="14" t="n">
+      <c r="F78" s="15" t="n">
         <f aca="false">IF($C78="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G78" s="14" t="n">
+      <c r="G78" s="15" t="n">
         <f aca="false">IF($C78="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H78" s="7"/>
-      <c r="I78" s="14" t="n">
+      <c r="I78" s="15" t="n">
         <f aca="false">IF($C78="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J78" s="16" t="n">
+      <c r="J78" s="17" t="n">
         <f aca="false">IF($C78="Lease-koop",D78+p_SlotJr,IF($C78="Koop",D78,0))</f>
         <v>0</v>
       </c>
-      <c r="K78" s="14" t="n">
+      <c r="K78" s="15" t="n">
         <f aca="false">E78+F78+G78+H78+I78</f>
         <v>0</v>
       </c>
-      <c r="L78" s="16" t="n">
+      <c r="L78" s="17" t="n">
         <f aca="false">IF($C78="Lease-koop",p_Afschr,IF($C78="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A78,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M78" s="16" t="n">
+      <c r="M78" s="17" t="n">
         <f aca="false">IF($C78="Lease-koop",D78+p_Lev,IF(AND($C78="Koop",D78&gt;0),D78+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A78,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N78" s="14" t="n">
+      <c r="N78" s="15" t="n">
         <f aca="false">IF($C78="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D79" s="5"/>
-      <c r="E79" s="14" t="n">
+      <c r="E79" s="15" t="n">
         <f aca="false">IF($C79="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F79" s="14" t="n">
+      <c r="F79" s="15" t="n">
         <f aca="false">IF($C79="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G79" s="14" t="n">
+      <c r="G79" s="15" t="n">
         <f aca="false">IF($C79="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H79" s="7"/>
-      <c r="I79" s="14" t="n">
+      <c r="I79" s="15" t="n">
         <f aca="false">IF($C79="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J79" s="16" t="n">
+      <c r="J79" s="17" t="n">
         <f aca="false">IF($C79="Lease-koop",D79+p_SlotJr,IF($C79="Koop",D79,0))</f>
         <v>0</v>
       </c>
-      <c r="K79" s="14" t="n">
+      <c r="K79" s="15" t="n">
         <f aca="false">E79+F79+G79+H79+I79</f>
         <v>0</v>
       </c>
-      <c r="L79" s="16" t="n">
+      <c r="L79" s="17" t="n">
         <f aca="false">IF($C79="Lease-koop",p_Afschr,IF($C79="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A79,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M79" s="16" t="n">
+      <c r="M79" s="17" t="n">
         <f aca="false">IF($C79="Lease-koop",D79+p_Lev,IF(AND($C79="Koop",D79&gt;0),D79+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A79,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N79" s="14" t="n">
+      <c r="N79" s="15" t="n">
         <f aca="false">IF($C79="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D80" s="5"/>
-      <c r="E80" s="14" t="n">
+      <c r="E80" s="15" t="n">
         <f aca="false">IF($C80="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F80" s="14" t="n">
+      <c r="F80" s="15" t="n">
         <f aca="false">IF($C80="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G80" s="14" t="n">
+      <c r="G80" s="15" t="n">
         <f aca="false">IF($C80="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H80" s="7"/>
-      <c r="I80" s="14" t="n">
+      <c r="I80" s="15" t="n">
         <f aca="false">IF($C80="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J80" s="16" t="n">
+      <c r="J80" s="17" t="n">
         <f aca="false">IF($C80="Lease-koop",D80+p_SlotJr,IF($C80="Koop",D80,0))</f>
         <v>0</v>
       </c>
-      <c r="K80" s="14" t="n">
+      <c r="K80" s="15" t="n">
         <f aca="false">E80+F80+G80+H80+I80</f>
         <v>0</v>
       </c>
-      <c r="L80" s="16" t="n">
+      <c r="L80" s="17" t="n">
         <f aca="false">IF($C80="Lease-koop",p_Afschr,IF($C80="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A80,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M80" s="16" t="n">
+      <c r="M80" s="17" t="n">
         <f aca="false">IF($C80="Lease-koop",D80+p_Lev,IF(AND($C80="Koop",D80&gt;0),D80+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A80,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N80" s="14" t="n">
+      <c r="N80" s="15" t="n">
         <f aca="false">IF($C80="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D81" s="5"/>
-      <c r="E81" s="14" t="n">
+      <c r="E81" s="15" t="n">
         <f aca="false">IF($C81="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F81" s="14" t="n">
+      <c r="F81" s="15" t="n">
         <f aca="false">IF($C81="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G81" s="14" t="n">
+      <c r="G81" s="15" t="n">
         <f aca="false">IF($C81="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H81" s="7"/>
-      <c r="I81" s="14" t="n">
+      <c r="I81" s="15" t="n">
         <f aca="false">IF($C81="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J81" s="16" t="n">
+      <c r="J81" s="17" t="n">
         <f aca="false">IF($C81="Lease-koop",D81+p_SlotJr,IF($C81="Koop",D81,0))</f>
         <v>0</v>
       </c>
-      <c r="K81" s="14" t="n">
+      <c r="K81" s="15" t="n">
         <f aca="false">E81+F81+G81+H81+I81</f>
         <v>0</v>
       </c>
-      <c r="L81" s="16" t="n">
+      <c r="L81" s="17" t="n">
         <f aca="false">IF($C81="Lease-koop",p_Afschr,IF($C81="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A81,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M81" s="16" t="n">
+      <c r="M81" s="17" t="n">
         <f aca="false">IF($C81="Lease-koop",D81+p_Lev,IF(AND($C81="Koop",D81&gt;0),D81+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A81,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N81" s="14" t="n">
+      <c r="N81" s="15" t="n">
         <f aca="false">IF($C81="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D82" s="5"/>
-      <c r="E82" s="14" t="n">
+      <c r="E82" s="15" t="n">
         <f aca="false">IF($C82="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F82" s="14" t="n">
+      <c r="F82" s="15" t="n">
         <f aca="false">IF($C82="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G82" s="14" t="n">
+      <c r="G82" s="15" t="n">
         <f aca="false">IF($C82="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H82" s="7"/>
-      <c r="I82" s="14" t="n">
+      <c r="I82" s="15" t="n">
         <f aca="false">IF($C82="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J82" s="16" t="n">
+      <c r="J82" s="17" t="n">
         <f aca="false">IF($C82="Lease-koop",D82+p_SlotJr,IF($C82="Koop",D82,0))</f>
         <v>0</v>
       </c>
-      <c r="K82" s="14" t="n">
+      <c r="K82" s="15" t="n">
         <f aca="false">E82+F82+G82+H82+I82</f>
         <v>0</v>
       </c>
-      <c r="L82" s="16" t="n">
+      <c r="L82" s="17" t="n">
         <f aca="false">IF($C82="Lease-koop",p_Afschr,IF($C82="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A82,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M82" s="16" t="n">
+      <c r="M82" s="17" t="n">
         <f aca="false">IF($C82="Lease-koop",D82+p_Lev,IF(AND($C82="Koop",D82&gt;0),D82+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A82,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N82" s="14" t="n">
+      <c r="N82" s="15" t="n">
         <f aca="false">IF($C82="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D83" s="5"/>
-      <c r="E83" s="14" t="n">
+      <c r="E83" s="15" t="n">
         <f aca="false">IF($C83="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F83" s="14" t="n">
+      <c r="F83" s="15" t="n">
         <f aca="false">IF($C83="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G83" s="14" t="n">
+      <c r="G83" s="15" t="n">
         <f aca="false">IF($C83="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H83" s="7"/>
-      <c r="I83" s="14" t="n">
+      <c r="I83" s="15" t="n">
         <f aca="false">IF($C83="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J83" s="16" t="n">
+      <c r="J83" s="17" t="n">
         <f aca="false">IF($C83="Lease-koop",D83+p_SlotJr,IF($C83="Koop",D83,0))</f>
         <v>0</v>
       </c>
-      <c r="K83" s="14" t="n">
+      <c r="K83" s="15" t="n">
         <f aca="false">E83+F83+G83+H83+I83</f>
         <v>0</v>
       </c>
-      <c r="L83" s="16" t="n">
+      <c r="L83" s="17" t="n">
         <f aca="false">IF($C83="Lease-koop",p_Afschr,IF($C83="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A83,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M83" s="16" t="n">
+      <c r="M83" s="17" t="n">
         <f aca="false">IF($C83="Lease-koop",D83+p_Lev,IF(AND($C83="Koop",D83&gt;0),D83+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A83,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N83" s="14" t="n">
+      <c r="N83" s="15" t="n">
         <f aca="false">IF($C83="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D84" s="5"/>
-      <c r="E84" s="14" t="n">
+      <c r="E84" s="15" t="n">
         <f aca="false">IF($C84="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F84" s="14" t="n">
+      <c r="F84" s="15" t="n">
         <f aca="false">IF($C84="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G84" s="14" t="n">
+      <c r="G84" s="15" t="n">
         <f aca="false">IF($C84="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H84" s="7"/>
-      <c r="I84" s="14" t="n">
+      <c r="I84" s="15" t="n">
         <f aca="false">IF($C84="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J84" s="16" t="n">
+      <c r="J84" s="17" t="n">
         <f aca="false">IF($C84="Lease-koop",D84+p_SlotJr,IF($C84="Koop",D84,0))</f>
         <v>0</v>
       </c>
-      <c r="K84" s="14" t="n">
+      <c r="K84" s="15" t="n">
         <f aca="false">E84+F84+G84+H84+I84</f>
         <v>0</v>
       </c>
-      <c r="L84" s="16" t="n">
+      <c r="L84" s="17" t="n">
         <f aca="false">IF($C84="Lease-koop",p_Afschr,IF($C84="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A84,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M84" s="16" t="n">
+      <c r="M84" s="17" t="n">
         <f aca="false">IF($C84="Lease-koop",D84+p_Lev,IF(AND($C84="Koop",D84&gt;0),D84+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A84,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N84" s="14" t="n">
+      <c r="N84" s="15" t="n">
         <f aca="false">IF($C84="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D85" s="5"/>
-      <c r="E85" s="14" t="n">
+      <c r="E85" s="15" t="n">
         <f aca="false">IF($C85="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F85" s="14" t="n">
+      <c r="F85" s="15" t="n">
         <f aca="false">IF($C85="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G85" s="14" t="n">
+      <c r="G85" s="15" t="n">
         <f aca="false">IF($C85="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H85" s="7"/>
-      <c r="I85" s="14" t="n">
+      <c r="I85" s="15" t="n">
         <f aca="false">IF($C85="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J85" s="16" t="n">
+      <c r="J85" s="17" t="n">
         <f aca="false">IF($C85="Lease-koop",D85+p_SlotJr,IF($C85="Koop",D85,0))</f>
         <v>0</v>
       </c>
-      <c r="K85" s="14" t="n">
+      <c r="K85" s="15" t="n">
         <f aca="false">E85+F85+G85+H85+I85</f>
         <v>0</v>
       </c>
-      <c r="L85" s="16" t="n">
+      <c r="L85" s="17" t="n">
         <f aca="false">IF($C85="Lease-koop",p_Afschr,IF($C85="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A85,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M85" s="16" t="n">
+      <c r="M85" s="17" t="n">
         <f aca="false">IF($C85="Lease-koop",D85+p_Lev,IF(AND($C85="Koop",D85&gt;0),D85+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A85,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N85" s="14" t="n">
+      <c r="N85" s="15" t="n">
         <f aca="false">IF($C85="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D86" s="5"/>
-      <c r="E86" s="14" t="n">
+      <c r="E86" s="15" t="n">
         <f aca="false">IF($C86="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F86" s="14" t="n">
+      <c r="F86" s="15" t="n">
         <f aca="false">IF($C86="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G86" s="14" t="n">
+      <c r="G86" s="15" t="n">
         <f aca="false">IF($C86="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H86" s="7"/>
-      <c r="I86" s="14" t="n">
+      <c r="I86" s="15" t="n">
         <f aca="false">IF($C86="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J86" s="16" t="n">
+      <c r="J86" s="17" t="n">
         <f aca="false">IF($C86="Lease-koop",D86+p_SlotJr,IF($C86="Koop",D86,0))</f>
         <v>0</v>
       </c>
-      <c r="K86" s="14" t="n">
+      <c r="K86" s="15" t="n">
         <f aca="false">E86+F86+G86+H86+I86</f>
         <v>0</v>
       </c>
-      <c r="L86" s="16" t="n">
+      <c r="L86" s="17" t="n">
         <f aca="false">IF($C86="Lease-koop",p_Afschr,IF($C86="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A86,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M86" s="16" t="n">
+      <c r="M86" s="17" t="n">
         <f aca="false">IF($C86="Lease-koop",D86+p_Lev,IF(AND($C86="Koop",D86&gt;0),D86+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A86,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N86" s="14" t="n">
+      <c r="N86" s="15" t="n">
         <f aca="false">IF($C86="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D87" s="5"/>
-      <c r="E87" s="14" t="n">
+      <c r="E87" s="15" t="n">
         <f aca="false">IF($C87="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F87" s="14" t="n">
+      <c r="F87" s="15" t="n">
         <f aca="false">IF($C87="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G87" s="14" t="n">
+      <c r="G87" s="15" t="n">
         <f aca="false">IF($C87="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H87" s="7"/>
-      <c r="I87" s="14" t="n">
+      <c r="I87" s="15" t="n">
         <f aca="false">IF($C87="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J87" s="16" t="n">
+      <c r="J87" s="17" t="n">
         <f aca="false">IF($C87="Lease-koop",D87+p_SlotJr,IF($C87="Koop",D87,0))</f>
         <v>0</v>
       </c>
-      <c r="K87" s="14" t="n">
+      <c r="K87" s="15" t="n">
         <f aca="false">E87+F87+G87+H87+I87</f>
         <v>0</v>
       </c>
-      <c r="L87" s="16" t="n">
+      <c r="L87" s="17" t="n">
         <f aca="false">IF($C87="Lease-koop",p_Afschr,IF($C87="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A87,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M87" s="16" t="n">
+      <c r="M87" s="17" t="n">
         <f aca="false">IF($C87="Lease-koop",D87+p_Lev,IF(AND($C87="Koop",D87&gt;0),D87+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A87,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N87" s="14" t="n">
+      <c r="N87" s="15" t="n">
         <f aca="false">IF($C87="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D88" s="5"/>
-      <c r="E88" s="14" t="n">
+      <c r="E88" s="15" t="n">
         <f aca="false">IF($C88="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F88" s="14" t="n">
+      <c r="F88" s="15" t="n">
         <f aca="false">IF($C88="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G88" s="14" t="n">
+      <c r="G88" s="15" t="n">
         <f aca="false">IF($C88="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H88" s="7"/>
-      <c r="I88" s="14" t="n">
+      <c r="I88" s="15" t="n">
         <f aca="false">IF($C88="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J88" s="16" t="n">
+      <c r="J88" s="17" t="n">
         <f aca="false">IF($C88="Lease-koop",D88+p_SlotJr,IF($C88="Koop",D88,0))</f>
         <v>0</v>
       </c>
-      <c r="K88" s="14" t="n">
+      <c r="K88" s="15" t="n">
         <f aca="false">E88+F88+G88+H88+I88</f>
         <v>0</v>
       </c>
-      <c r="L88" s="16" t="n">
+      <c r="L88" s="17" t="n">
         <f aca="false">IF($C88="Lease-koop",p_Afschr,IF($C88="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A88,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M88" s="16" t="n">
+      <c r="M88" s="17" t="n">
         <f aca="false">IF($C88="Lease-koop",D88+p_Lev,IF(AND($C88="Koop",D88&gt;0),D88+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A88,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N88" s="14" t="n">
+      <c r="N88" s="15" t="n">
         <f aca="false">IF($C88="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D89" s="5"/>
-      <c r="E89" s="14" t="n">
+      <c r="E89" s="15" t="n">
         <f aca="false">IF($C89="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F89" s="14" t="n">
+      <c r="F89" s="15" t="n">
         <f aca="false">IF($C89="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G89" s="14" t="n">
+      <c r="G89" s="15" t="n">
         <f aca="false">IF($C89="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H89" s="7"/>
-      <c r="I89" s="14" t="n">
+      <c r="I89" s="15" t="n">
         <f aca="false">IF($C89="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J89" s="16" t="n">
+      <c r="J89" s="17" t="n">
         <f aca="false">IF($C89="Lease-koop",D89+p_SlotJr,IF($C89="Koop",D89,0))</f>
         <v>0</v>
       </c>
-      <c r="K89" s="14" t="n">
+      <c r="K89" s="15" t="n">
         <f aca="false">E89+F89+G89+H89+I89</f>
         <v>0</v>
       </c>
-      <c r="L89" s="16" t="n">
+      <c r="L89" s="17" t="n">
         <f aca="false">IF($C89="Lease-koop",p_Afschr,IF($C89="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A89,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M89" s="16" t="n">
+      <c r="M89" s="17" t="n">
         <f aca="false">IF($C89="Lease-koop",D89+p_Lev,IF(AND($C89="Koop",D89&gt;0),D89+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A89,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N89" s="14" t="n">
+      <c r="N89" s="15" t="n">
         <f aca="false">IF($C89="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D90" s="5"/>
-      <c r="E90" s="14" t="n">
+      <c r="E90" s="15" t="n">
         <f aca="false">IF($C90="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F90" s="14" t="n">
+      <c r="F90" s="15" t="n">
         <f aca="false">IF($C90="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G90" s="14" t="n">
+      <c r="G90" s="15" t="n">
         <f aca="false">IF($C90="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H90" s="7"/>
-      <c r="I90" s="14" t="n">
+      <c r="I90" s="15" t="n">
         <f aca="false">IF($C90="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J90" s="16" t="n">
+      <c r="J90" s="17" t="n">
         <f aca="false">IF($C90="Lease-koop",D90+p_SlotJr,IF($C90="Koop",D90,0))</f>
         <v>0</v>
       </c>
-      <c r="K90" s="14" t="n">
+      <c r="K90" s="15" t="n">
         <f aca="false">E90+F90+G90+H90+I90</f>
         <v>0</v>
       </c>
-      <c r="L90" s="16" t="n">
+      <c r="L90" s="17" t="n">
         <f aca="false">IF($C90="Lease-koop",p_Afschr,IF($C90="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A90,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M90" s="16" t="n">
+      <c r="M90" s="17" t="n">
         <f aca="false">IF($C90="Lease-koop",D90+p_Lev,IF(AND($C90="Koop",D90&gt;0),D90+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A90,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N90" s="14" t="n">
+      <c r="N90" s="15" t="n">
         <f aca="false">IF($C90="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D91" s="5"/>
-      <c r="E91" s="14" t="n">
+      <c r="E91" s="15" t="n">
         <f aca="false">IF($C91="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F91" s="14" t="n">
+      <c r="F91" s="15" t="n">
         <f aca="false">IF($C91="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G91" s="14" t="n">
+      <c r="G91" s="15" t="n">
         <f aca="false">IF($C91="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H91" s="7"/>
-      <c r="I91" s="14" t="n">
+      <c r="I91" s="15" t="n">
         <f aca="false">IF($C91="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J91" s="16" t="n">
+      <c r="J91" s="17" t="n">
         <f aca="false">IF($C91="Lease-koop",D91+p_SlotJr,IF($C91="Koop",D91,0))</f>
         <v>0</v>
       </c>
-      <c r="K91" s="14" t="n">
+      <c r="K91" s="15" t="n">
         <f aca="false">E91+F91+G91+H91+I91</f>
         <v>0</v>
       </c>
-      <c r="L91" s="16" t="n">
+      <c r="L91" s="17" t="n">
         <f aca="false">IF($C91="Lease-koop",p_Afschr,IF($C91="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A91,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M91" s="16" t="n">
+      <c r="M91" s="17" t="n">
         <f aca="false">IF($C91="Lease-koop",D91+p_Lev,IF(AND($C91="Koop",D91&gt;0),D91+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A91,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N91" s="14" t="n">
+      <c r="N91" s="15" t="n">
         <f aca="false">IF($C91="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D92" s="5"/>
-      <c r="E92" s="14" t="n">
+      <c r="E92" s="15" t="n">
         <f aca="false">IF($C92="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F92" s="14" t="n">
+      <c r="F92" s="15" t="n">
         <f aca="false">IF($C92="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G92" s="14" t="n">
+      <c r="G92" s="15" t="n">
         <f aca="false">IF($C92="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H92" s="7"/>
-      <c r="I92" s="14" t="n">
+      <c r="I92" s="15" t="n">
         <f aca="false">IF($C92="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J92" s="16" t="n">
+      <c r="J92" s="17" t="n">
         <f aca="false">IF($C92="Lease-koop",D92+p_SlotJr,IF($C92="Koop",D92,0))</f>
         <v>0</v>
       </c>
-      <c r="K92" s="14" t="n">
+      <c r="K92" s="15" t="n">
         <f aca="false">E92+F92+G92+H92+I92</f>
         <v>0</v>
       </c>
-      <c r="L92" s="16" t="n">
+      <c r="L92" s="17" t="n">
         <f aca="false">IF($C92="Lease-koop",p_Afschr,IF($C92="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A92,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M92" s="16" t="n">
+      <c r="M92" s="17" t="n">
         <f aca="false">IF($C92="Lease-koop",D92+p_Lev,IF(AND($C92="Koop",D92&gt;0),D92+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A92,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N92" s="14" t="n">
+      <c r="N92" s="15" t="n">
         <f aca="false">IF($C92="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D93" s="5"/>
-      <c r="E93" s="14" t="n">
+      <c r="E93" s="15" t="n">
         <f aca="false">IF($C93="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F93" s="14" t="n">
+      <c r="F93" s="15" t="n">
         <f aca="false">IF($C93="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G93" s="14" t="n">
+      <c r="G93" s="15" t="n">
         <f aca="false">IF($C93="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H93" s="7"/>
-      <c r="I93" s="14" t="n">
+      <c r="I93" s="15" t="n">
         <f aca="false">IF($C93="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J93" s="16" t="n">
+      <c r="J93" s="17" t="n">
         <f aca="false">IF($C93="Lease-koop",D93+p_SlotJr,IF($C93="Koop",D93,0))</f>
         <v>0</v>
       </c>
-      <c r="K93" s="14" t="n">
+      <c r="K93" s="15" t="n">
         <f aca="false">E93+F93+G93+H93+I93</f>
         <v>0</v>
       </c>
-      <c r="L93" s="16" t="n">
+      <c r="L93" s="17" t="n">
         <f aca="false">IF($C93="Lease-koop",p_Afschr,IF($C93="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A93,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M93" s="16" t="n">
+      <c r="M93" s="17" t="n">
         <f aca="false">IF($C93="Lease-koop",D93+p_Lev,IF(AND($C93="Koop",D93&gt;0),D93+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A93,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N93" s="14" t="n">
+      <c r="N93" s="15" t="n">
         <f aca="false">IF($C93="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D94" s="5"/>
-      <c r="E94" s="14" t="n">
+      <c r="E94" s="15" t="n">
         <f aca="false">IF($C94="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F94" s="14" t="n">
+      <c r="F94" s="15" t="n">
         <f aca="false">IF($C94="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G94" s="14" t="n">
+      <c r="G94" s="15" t="n">
         <f aca="false">IF($C94="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H94" s="7"/>
-      <c r="I94" s="14" t="n">
+      <c r="I94" s="15" t="n">
         <f aca="false">IF($C94="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J94" s="16" t="n">
+      <c r="J94" s="17" t="n">
         <f aca="false">IF($C94="Lease-koop",D94+p_SlotJr,IF($C94="Koop",D94,0))</f>
         <v>0</v>
       </c>
-      <c r="K94" s="14" t="n">
+      <c r="K94" s="15" t="n">
         <f aca="false">E94+F94+G94+H94+I94</f>
         <v>0</v>
       </c>
-      <c r="L94" s="16" t="n">
+      <c r="L94" s="17" t="n">
         <f aca="false">IF($C94="Lease-koop",p_Afschr,IF($C94="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A94,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M94" s="16" t="n">
+      <c r="M94" s="17" t="n">
         <f aca="false">IF($C94="Lease-koop",D94+p_Lev,IF(AND($C94="Koop",D94&gt;0),D94+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A94,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N94" s="14" t="n">
+      <c r="N94" s="15" t="n">
         <f aca="false">IF($C94="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D95" s="5"/>
-      <c r="E95" s="14" t="n">
+      <c r="E95" s="15" t="n">
         <f aca="false">IF($C95="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F95" s="14" t="n">
+      <c r="F95" s="15" t="n">
         <f aca="false">IF($C95="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G95" s="14" t="n">
+      <c r="G95" s="15" t="n">
         <f aca="false">IF($C95="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H95" s="7"/>
-      <c r="I95" s="14" t="n">
+      <c r="I95" s="15" t="n">
         <f aca="false">IF($C95="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J95" s="16" t="n">
+      <c r="J95" s="17" t="n">
         <f aca="false">IF($C95="Lease-koop",D95+p_SlotJr,IF($C95="Koop",D95,0))</f>
         <v>0</v>
       </c>
-      <c r="K95" s="14" t="n">
+      <c r="K95" s="15" t="n">
         <f aca="false">E95+F95+G95+H95+I95</f>
         <v>0</v>
       </c>
-      <c r="L95" s="16" t="n">
+      <c r="L95" s="17" t="n">
         <f aca="false">IF($C95="Lease-koop",p_Afschr,IF($C95="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A95,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M95" s="16" t="n">
+      <c r="M95" s="17" t="n">
         <f aca="false">IF($C95="Lease-koop",D95+p_Lev,IF(AND($C95="Koop",D95&gt;0),D95+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A95,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N95" s="14" t="n">
+      <c r="N95" s="15" t="n">
         <f aca="false">IF($C95="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D96" s="5"/>
-      <c r="E96" s="14" t="n">
+      <c r="E96" s="15" t="n">
         <f aca="false">IF($C96="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F96" s="14" t="n">
+      <c r="F96" s="15" t="n">
         <f aca="false">IF($C96="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G96" s="14" t="n">
+      <c r="G96" s="15" t="n">
         <f aca="false">IF($C96="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H96" s="7"/>
-      <c r="I96" s="14" t="n">
+      <c r="I96" s="15" t="n">
         <f aca="false">IF($C96="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J96" s="16" t="n">
+      <c r="J96" s="17" t="n">
         <f aca="false">IF($C96="Lease-koop",D96+p_SlotJr,IF($C96="Koop",D96,0))</f>
         <v>0</v>
       </c>
-      <c r="K96" s="14" t="n">
+      <c r="K96" s="15" t="n">
         <f aca="false">E96+F96+G96+H96+I96</f>
         <v>0</v>
       </c>
-      <c r="L96" s="16" t="n">
+      <c r="L96" s="17" t="n">
         <f aca="false">IF($C96="Lease-koop",p_Afschr,IF($C96="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A96,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M96" s="16" t="n">
+      <c r="M96" s="17" t="n">
         <f aca="false">IF($C96="Lease-koop",D96+p_Lev,IF(AND($C96="Koop",D96&gt;0),D96+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A96,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N96" s="14" t="n">
+      <c r="N96" s="15" t="n">
         <f aca="false">IF($C96="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -6196,7 +6224,7 @@
       </c>
       <c r="N10" s="4"/>
       <c r="O10" s="7"/>
-      <c r="P10" s="17"/>
+      <c r="P10" s="18"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
@@ -6228,7 +6256,7 @@
       </c>
       <c r="N11" s="4"/>
       <c r="O11" s="7"/>
-      <c r="P11" s="17"/>
+      <c r="P11" s="18"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
@@ -6354,7 +6382,7 @@
       </c>
       <c r="N15" s="4"/>
       <c r="O15" s="7"/>
-      <c r="P15" s="17"/>
+      <c r="P15" s="18"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Wagenpark_beheer.xlsx: alle tekst zwart
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013EaFTgzjMaNvZvWgFM9YZf
</commit_message>
<xml_diff>
--- a/Wagenpark_beheer.xlsx
+++ b/Wagenpark_beheer.xlsx
@@ -41,7 +41,7 @@
     <t xml:space="preserve">Harde cijfers: betaalde prijzen of bestaande afspraken. Nieuw V-nummer: typ direct onder de tabel. Bij vervanging: regel eerst kopiëren naar 'Buiten gebruik', dan hier overschrijven.</t>
   </si>
   <si>
-    <t xml:space="preserve">Koop: kolom H (werkelijk betaald). Lease-koop: kolom I t/m L, kolom H blijft leeg. Uitgaven vanaf 2027 = gemiddelde (groen), overschrijven met werkelijke uitgave zodra bekend.</t>
+    <t xml:space="preserve">Koop: kolom H (werkelijk betaald). Lease-koop: kolom I t/m L, kolom H blijft leeg. Uitgaven vanaf 2027 = gemiddelde, overschrijven met werkelijke uitgave zodra bekend.</t>
   </si>
   <si>
     <t xml:space="preserve">V-nummer</t>
@@ -311,7 +311,7 @@
     <t xml:space="preserve">Vervangingsinvesteringen</t>
   </si>
   <si>
-    <t xml:space="preserve">Per V-nummer de eerstvolgende aanschaf, op volgorde van aanschafjaar. Blauw/geel = invullen, zwart = berekend.</t>
+    <t xml:space="preserve">Per V-nummer de eerstvolgende aanschaf, op volgorde van aanschafjaar. Geel = nog invullen.</t>
   </si>
   <si>
     <t xml:space="preserve">Standaardbedragen</t>
@@ -504,7 +504,7 @@
     <numFmt numFmtId="166" formatCode="0"/>
     <numFmt numFmtId="167" formatCode="&quot;€ &quot;#,##0;&quot;-€ &quot;#,##0;\-"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -552,26 +552,12 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF008000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -638,7 +624,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -671,23 +657,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="167" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -695,19 +673,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -724,7 +694,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="5">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -743,14 +713,6 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF0000FF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor rgb="FFFFFFFF"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
@@ -760,14 +722,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF008000"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1346,7 +1300,7 @@
       <c r="J10" s="7" t="n">
         <v>3420</v>
       </c>
-      <c r="K10" s="8" t="n">
+      <c r="K10" s="7" t="n">
         <f aca="false">p_Slot</f>
         <v>35000</v>
       </c>
@@ -1425,7 +1379,7 @@
       <c r="J12" s="7" t="n">
         <v>3420</v>
       </c>
-      <c r="K12" s="8" t="n">
+      <c r="K12" s="7" t="n">
         <f aca="false">p_Slot</f>
         <v>35000</v>
       </c>
@@ -1539,7 +1493,7 @@
       <c r="J15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="8" t="n">
+      <c r="K15" s="7" t="n">
         <f aca="false">p_Slot</f>
         <v>35000</v>
       </c>
@@ -1684,7 +1638,7 @@
       <c r="J19" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="8" t="n">
+      <c r="K19" s="7" t="n">
         <f aca="false">p_Slot</f>
         <v>35000</v>
       </c>
@@ -1728,7 +1682,7 @@
       <c r="J20" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="K20" s="8" t="n">
+      <c r="K20" s="7" t="n">
         <f aca="false">p_Slot</f>
         <v>35000</v>
       </c>
@@ -1774,7 +1728,7 @@
       <c r="J21" s="7" t="n">
         <v>3420</v>
       </c>
-      <c r="K21" s="8" t="n">
+      <c r="K21" s="7" t="n">
         <f aca="false">p_Slot</f>
         <v>35000</v>
       </c>
@@ -2076,9 +2030,9 @@
         <v>8</v>
       </c>
       <c r="H30" s="7"/>
-      <c r="I30" s="9"/>
-      <c r="J30" s="9"/>
-      <c r="K30" s="8" t="n">
+      <c r="I30" s="8"/>
+      <c r="J30" s="8"/>
+      <c r="K30" s="7" t="n">
         <f aca="false">p_Slot</f>
         <v>35000</v>
       </c>
@@ -2125,22 +2079,22 @@
       <c r="O31" s="7"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G33" s="10" t="s">
+      <c r="G33" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="H33" s="11" t="n">
+      <c r="H33" s="10" t="n">
         <f aca="false">SUBTOTAL(109,H5:H31)</f>
         <v>1608161</v>
       </c>
-      <c r="I33" s="11" t="n">
+      <c r="I33" s="10" t="n">
         <f aca="false">SUBTOTAL(109,I5:I31)</f>
         <v>68310</v>
       </c>
-      <c r="J33" s="11" t="n">
+      <c r="J33" s="10" t="n">
         <f aca="false">SUBTOTAL(109,J5:J31)</f>
         <v>10260</v>
       </c>
-      <c r="K33" s="11" t="n">
+      <c r="K33" s="10" t="n">
         <f aca="false">SUBTOTAL(109,K5:K31)</f>
         <v>245000</v>
       </c>
@@ -2191,143 +2145,143 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="9" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="C4" s="9" t="n">
+      <c r="C4" s="8" t="n">
         <v>10000</v>
       </c>
-      <c r="F4" s="13" t="n">
+      <c r="F4" s="11" t="n">
         <v>2027</v>
       </c>
-      <c r="G4" s="14" t="n">
+      <c r="G4" s="12" t="n">
         <f aca="false">F4+1</f>
         <v>2028</v>
       </c>
-      <c r="H4" s="14" t="n">
+      <c r="H4" s="12" t="n">
         <f aca="false">G4+1</f>
         <v>2029</v>
       </c>
-      <c r="I4" s="14" t="n">
+      <c r="I4" s="12" t="n">
         <f aca="false">H4+1</f>
         <v>2030</v>
       </c>
-      <c r="J4" s="14" t="n">
+      <c r="J4" s="12" t="n">
         <f aca="false">I4+1</f>
         <v>2031</v>
       </c>
-      <c r="K4" s="14" t="n">
+      <c r="K4" s="12" t="n">
         <f aca="false">J4+1</f>
         <v>2032</v>
       </c>
-      <c r="L4" s="14" t="n">
+      <c r="L4" s="12" t="n">
         <f aca="false">K4+1</f>
         <v>2033</v>
       </c>
-      <c r="M4" s="14" t="n">
+      <c r="M4" s="12" t="n">
         <f aca="false">L4+1</f>
         <v>2034</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="8" t="n">
         <v>5000</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="F5" s="15" t="n">
+      <c r="F5" s="7" t="n">
         <f aca="false">SUMIF($D$17:$D$96,F$4,$E$17:$E$96)+SUMIF($D$17:$D$96,F$4,$F$17:$F$96)+SUMIF($D$17:$D$96,F$4,$G$17:$G$96)+SUMIF($D$17:$D$96,F$4,$H$17:$H$96)+SUMIF($J$17:$J$96,F$4,$I$17:$I$96)</f>
         <v>322000</v>
       </c>
-      <c r="G5" s="15" t="n">
+      <c r="G5" s="7" t="n">
         <f aca="false">SUMIF($D$17:$D$96,G$4,$E$17:$E$96)+SUMIF($D$17:$D$96,G$4,$F$17:$F$96)+SUMIF($D$17:$D$96,G$4,$G$17:$G$96)+SUMIF($D$17:$D$96,G$4,$H$17:$H$96)+SUMIF($J$17:$J$96,G$4,$I$17:$I$96)</f>
         <v>50000</v>
       </c>
-      <c r="H5" s="15" t="n">
+      <c r="H5" s="7" t="n">
         <f aca="false">SUMIF($D$17:$D$96,H$4,$E$17:$E$96)+SUMIF($D$17:$D$96,H$4,$F$17:$F$96)+SUMIF($D$17:$D$96,H$4,$G$17:$G$96)+SUMIF($D$17:$D$96,H$4,$H$17:$H$96)+SUMIF($J$17:$J$96,H$4,$I$17:$I$96)</f>
         <v>157000</v>
       </c>
-      <c r="I5" s="15" t="n">
+      <c r="I5" s="7" t="n">
         <f aca="false">SUMIF($D$17:$D$96,I$4,$E$17:$E$96)+SUMIF($D$17:$D$96,I$4,$F$17:$F$96)+SUMIF($D$17:$D$96,I$4,$G$17:$G$96)+SUMIF($D$17:$D$96,I$4,$H$17:$H$96)+SUMIF($J$17:$J$96,I$4,$I$17:$I$96)</f>
         <v>0</v>
       </c>
-      <c r="J5" s="15" t="n">
+      <c r="J5" s="7" t="n">
         <f aca="false">SUMIF($D$17:$D$96,J$4,$E$17:$E$96)+SUMIF($D$17:$D$96,J$4,$F$17:$F$96)+SUMIF($D$17:$D$96,J$4,$G$17:$G$96)+SUMIF($D$17:$D$96,J$4,$H$17:$H$96)+SUMIF($J$17:$J$96,J$4,$I$17:$I$96)</f>
         <v>57000</v>
       </c>
-      <c r="K5" s="15" t="n">
+      <c r="K5" s="7" t="n">
         <f aca="false">SUMIF($D$17:$D$96,K$4,$E$17:$E$96)+SUMIF($D$17:$D$96,K$4,$F$17:$F$96)+SUMIF($D$17:$D$96,K$4,$G$17:$G$96)+SUMIF($D$17:$D$96,K$4,$H$17:$H$96)+SUMIF($J$17:$J$96,K$4,$I$17:$I$96)</f>
         <v>314960</v>
       </c>
-      <c r="L5" s="15" t="n">
+      <c r="L5" s="7" t="n">
         <f aca="false">SUMIF($D$17:$D$96,L$4,$E$17:$E$96)+SUMIF($D$17:$D$96,L$4,$F$17:$F$96)+SUMIF($D$17:$D$96,L$4,$G$17:$G$96)+SUMIF($D$17:$D$96,L$4,$H$17:$H$96)+SUMIF($J$17:$J$96,L$4,$I$17:$I$96)</f>
         <v>76000</v>
       </c>
-      <c r="M5" s="15" t="n">
+      <c r="M5" s="7" t="n">
         <f aca="false">SUMIF($D$17:$D$96,M$4,$E$17:$E$96)+SUMIF($D$17:$D$96,M$4,$F$17:$F$96)+SUMIF($D$17:$D$96,M$4,$G$17:$G$96)+SUMIF($D$17:$D$96,M$4,$H$17:$H$96)+SUMIF($J$17:$J$96,M$4,$I$17:$I$96)</f>
         <v>310100</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="C6" s="9" t="n">
+      <c r="C6" s="8" t="n">
         <v>7000</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="F6" s="15" t="n">
+      <c r="F6" s="7" t="n">
         <f aca="false">SUMPRODUCT(($C$17:$C$96="Lease-koop")*($D$17:$D$96&lt;=F$4)*($J$17:$J$96&gt;F$4)*$N$17:$N$96)</f>
         <v>12000</v>
       </c>
-      <c r="G6" s="15" t="n">
+      <c r="G6" s="7" t="n">
         <f aca="false">SUMPRODUCT(($C$17:$C$96="Lease-koop")*($D$17:$D$96&lt;=G$4)*($J$17:$J$96&gt;G$4)*$N$17:$N$96)</f>
         <v>12000</v>
       </c>
-      <c r="H6" s="15" t="n">
+      <c r="H6" s="7" t="n">
         <f aca="false">SUMPRODUCT(($C$17:$C$96="Lease-koop")*($D$17:$D$96&lt;=H$4)*($J$17:$J$96&gt;H$4)*$N$17:$N$96)</f>
         <v>12000</v>
       </c>
-      <c r="I6" s="15" t="n">
+      <c r="I6" s="7" t="n">
         <f aca="false">SUMPRODUCT(($C$17:$C$96="Lease-koop")*($D$17:$D$96&lt;=I$4)*($J$17:$J$96&gt;I$4)*$N$17:$N$96)</f>
         <v>12000</v>
       </c>
-      <c r="J6" s="15" t="n">
+      <c r="J6" s="7" t="n">
         <f aca="false">SUMPRODUCT(($C$17:$C$96="Lease-koop")*($D$17:$D$96&lt;=J$4)*($J$17:$J$96&gt;J$4)*$N$17:$N$96)</f>
         <v>12000</v>
       </c>
-      <c r="K6" s="15" t="n">
+      <c r="K6" s="7" t="n">
         <f aca="false">SUMPRODUCT(($C$17:$C$96="Lease-koop")*($D$17:$D$96&lt;=K$4)*($J$17:$J$96&gt;K$4)*$N$17:$N$96)</f>
         <v>48000</v>
       </c>
-      <c r="L6" s="15" t="n">
+      <c r="L6" s="7" t="n">
         <f aca="false">SUMPRODUCT(($C$17:$C$96="Lease-koop")*($D$17:$D$96&lt;=L$4)*($J$17:$J$96&gt;L$4)*$N$17:$N$96)</f>
         <v>48000</v>
       </c>
-      <c r="M6" s="15" t="n">
+      <c r="M6" s="7" t="n">
         <f aca="false">SUMPRODUCT(($C$17:$C$96="Lease-koop")*($D$17:$D$96&lt;=M$4)*($J$17:$J$96&gt;M$4)*$N$17:$N$96)</f>
         <v>96000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="8" t="n">
         <v>35000</v>
       </c>
       <c r="E7" s="2" t="s">
@@ -2335,10 +2289,10 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="11" t="n">
         <v>2</v>
       </c>
       <c r="E8" s="2" t="s">
@@ -2346,34 +2300,34 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="11" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="11" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="C11" s="9" t="n">
+      <c r="C11" s="8" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J15" s="10" t="s">
+      <c r="J15" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="K15" s="11" t="n">
+      <c r="K15" s="10" t="n">
         <f aca="false">SUM($K$17:$K$96)</f>
         <v>2047208</v>
       </c>
@@ -2429,49 +2383,49 @@
       <c r="A17" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B17" s="16"/>
+      <c r="B17" s="13"/>
       <c r="C17" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>2027</v>
       </c>
-      <c r="E17" s="15" t="n">
+      <c r="E17" s="7" t="n">
         <f aca="false">IF($C17="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F17" s="15" t="n">
+      <c r="F17" s="7" t="n">
         <f aca="false">IF($C17="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G17" s="15" t="n">
+      <c r="G17" s="7" t="n">
         <f aca="false">IF($C17="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>65000</v>
       </c>
-      <c r="I17" s="15" t="n">
+      <c r="I17" s="7" t="n">
         <f aca="false">IF($C17="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J17" s="17" t="n">
+      <c r="J17" s="5" t="n">
         <f aca="false">IF($C17="Lease-koop",D17+p_SlotJr,IF($C17="Koop",D17,0))</f>
         <v>2027</v>
       </c>
-      <c r="K17" s="15" t="n">
+      <c r="K17" s="7" t="n">
         <f aca="false">E17+F17+G17+H17+I17</f>
         <v>65000</v>
       </c>
-      <c r="L17" s="17" t="n">
+      <c r="L17" s="5" t="n">
         <f aca="false">IF($C17="Lease-koop",p_Afschr,IF($C17="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A17,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>8</v>
       </c>
-      <c r="M17" s="17" t="n">
+      <c r="M17" s="5" t="n">
         <f aca="false">IF($C17="Lease-koop",D17+p_Lev,IF(AND($C17="Koop",D17&gt;0),D17+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A17,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2035</v>
       </c>
-      <c r="N17" s="15" t="n">
+      <c r="N17" s="7" t="n">
         <f aca="false">IF($C17="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -2483,49 +2437,49 @@
       <c r="A18" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="16"/>
+      <c r="B18" s="13"/>
       <c r="C18" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>2027</v>
       </c>
-      <c r="E18" s="15" t="n">
+      <c r="E18" s="7" t="n">
         <f aca="false">IF($C18="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F18" s="15" t="n">
+      <c r="F18" s="7" t="n">
         <f aca="false">IF($C18="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G18" s="15" t="n">
+      <c r="G18" s="7" t="n">
         <f aca="false">IF($C18="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>65000</v>
       </c>
-      <c r="I18" s="15" t="n">
+      <c r="I18" s="7" t="n">
         <f aca="false">IF($C18="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J18" s="17" t="n">
+      <c r="J18" s="5" t="n">
         <f aca="false">IF($C18="Lease-koop",D18+p_SlotJr,IF($C18="Koop",D18,0))</f>
         <v>2027</v>
       </c>
-      <c r="K18" s="15" t="n">
+      <c r="K18" s="7" t="n">
         <f aca="false">E18+F18+G18+H18+I18</f>
         <v>65000</v>
       </c>
-      <c r="L18" s="17" t="n">
+      <c r="L18" s="5" t="n">
         <f aca="false">IF($C18="Lease-koop",p_Afschr,IF($C18="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A18,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>8</v>
       </c>
-      <c r="M18" s="17" t="n">
+      <c r="M18" s="5" t="n">
         <f aca="false">IF($C18="Lease-koop",D18+p_Lev,IF(AND($C18="Koop",D18&gt;0),D18+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A18,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2035</v>
       </c>
-      <c r="N18" s="15" t="n">
+      <c r="N18" s="7" t="n">
         <f aca="false">IF($C18="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -2537,47 +2491,47 @@
       <c r="A19" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B19" s="16"/>
+      <c r="B19" s="13"/>
       <c r="C19" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D19" s="5" t="n">
         <v>2027</v>
       </c>
-      <c r="E19" s="15" t="n">
+      <c r="E19" s="7" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F19" s="15" t="n">
+      <c r="F19" s="7" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G19" s="15" t="n">
+      <c r="G19" s="7" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H19" s="7"/>
-      <c r="I19" s="15" t="n">
+      <c r="I19" s="7" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J19" s="17" t="n">
+      <c r="J19" s="5" t="n">
         <f aca="false">IF($C19="Lease-koop",D19+p_SlotJr,IF($C19="Koop",D19,0))</f>
         <v>2029</v>
       </c>
-      <c r="K19" s="15" t="n">
+      <c r="K19" s="7" t="n">
         <f aca="false">E19+F19+G19+H19+I19</f>
         <v>57000</v>
       </c>
-      <c r="L19" s="17" t="n">
+      <c r="L19" s="5" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Afschr,IF($C19="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A19,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M19" s="17" t="n">
+      <c r="M19" s="5" t="n">
         <f aca="false">IF($C19="Lease-koop",D19+p_Lev,IF(AND($C19="Koop",D19&gt;0),D19+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A19,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2035</v>
       </c>
-      <c r="N19" s="15" t="n">
+      <c r="N19" s="7" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -2587,49 +2541,49 @@
       <c r="A20" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B20" s="16"/>
+      <c r="B20" s="13"/>
       <c r="C20" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>2027</v>
       </c>
-      <c r="E20" s="15" t="n">
+      <c r="E20" s="7" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F20" s="15" t="n">
+      <c r="F20" s="7" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G20" s="15" t="n">
+      <c r="G20" s="7" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>80000</v>
       </c>
-      <c r="I20" s="15" t="n">
+      <c r="I20" s="7" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J20" s="17" t="n">
+      <c r="J20" s="5" t="n">
         <f aca="false">IF($C20="Lease-koop",D20+p_SlotJr,IF($C20="Koop",D20,0))</f>
         <v>2027</v>
       </c>
-      <c r="K20" s="15" t="n">
+      <c r="K20" s="7" t="n">
         <f aca="false">E20+F20+G20+H20+I20</f>
         <v>80000</v>
       </c>
-      <c r="L20" s="17" t="n">
+      <c r="L20" s="5" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Afschr,IF($C20="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A20,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>15</v>
       </c>
-      <c r="M20" s="17" t="n">
+      <c r="M20" s="5" t="n">
         <f aca="false">IF($C20="Lease-koop",D20+p_Lev,IF(AND($C20="Koop",D20&gt;0),D20+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A20,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2042</v>
       </c>
-      <c r="N20" s="15" t="n">
+      <c r="N20" s="7" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -2639,49 +2593,49 @@
       <c r="A21" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B21" s="16"/>
+      <c r="B21" s="13"/>
       <c r="C21" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D21" s="5" t="n">
         <v>2027</v>
       </c>
-      <c r="E21" s="15" t="n">
+      <c r="E21" s="7" t="n">
         <f aca="false">IF($C21="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F21" s="15" t="n">
+      <c r="F21" s="7" t="n">
         <f aca="false">IF($C21="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G21" s="15" t="n">
+      <c r="G21" s="7" t="n">
         <f aca="false">IF($C21="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H21" s="7" t="n">
         <v>45000</v>
       </c>
-      <c r="I21" s="15" t="n">
+      <c r="I21" s="7" t="n">
         <f aca="false">IF($C21="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J21" s="17" t="n">
+      <c r="J21" s="5" t="n">
         <f aca="false">IF($C21="Lease-koop",D21+p_SlotJr,IF($C21="Koop",D21,0))</f>
         <v>2027</v>
       </c>
-      <c r="K21" s="15" t="n">
+      <c r="K21" s="7" t="n">
         <f aca="false">E21+F21+G21+H21+I21</f>
         <v>45000</v>
       </c>
-      <c r="L21" s="17" t="n">
+      <c r="L21" s="5" t="n">
         <f aca="false">IF($C21="Lease-koop",p_Afschr,IF($C21="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A21,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>8</v>
       </c>
-      <c r="M21" s="17" t="n">
+      <c r="M21" s="5" t="n">
         <f aca="false">IF($C21="Lease-koop",D21+p_Lev,IF(AND($C21="Koop",D21&gt;0),D21+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A21,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2035</v>
       </c>
-      <c r="N21" s="15" t="n">
+      <c r="N21" s="7" t="n">
         <f aca="false">IF($C21="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -2693,49 +2647,49 @@
       <c r="A22" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="B22" s="16"/>
+      <c r="B22" s="13"/>
       <c r="C22" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D22" s="5" t="n">
         <v>2027</v>
       </c>
-      <c r="E22" s="15" t="n">
+      <c r="E22" s="7" t="n">
         <f aca="false">IF($C22="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F22" s="15" t="n">
+      <c r="F22" s="7" t="n">
         <f aca="false">IF($C22="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G22" s="15" t="n">
+      <c r="G22" s="7" t="n">
         <f aca="false">IF($C22="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H22" s="7" t="n">
         <v>45000</v>
       </c>
-      <c r="I22" s="15" t="n">
+      <c r="I22" s="7" t="n">
         <f aca="false">IF($C22="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J22" s="17" t="n">
+      <c r="J22" s="5" t="n">
         <f aca="false">IF($C22="Lease-koop",D22+p_SlotJr,IF($C22="Koop",D22,0))</f>
         <v>2027</v>
       </c>
-      <c r="K22" s="15" t="n">
+      <c r="K22" s="7" t="n">
         <f aca="false">E22+F22+G22+H22+I22</f>
         <v>45000</v>
       </c>
-      <c r="L22" s="17" t="n">
+      <c r="L22" s="5" t="n">
         <f aca="false">IF($C22="Lease-koop",p_Afschr,IF($C22="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A22,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>8</v>
       </c>
-      <c r="M22" s="17" t="n">
+      <c r="M22" s="5" t="n">
         <f aca="false">IF($C22="Lease-koop",D22+p_Lev,IF(AND($C22="Koop",D22&gt;0),D22+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A22,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2035</v>
       </c>
-      <c r="N22" s="15" t="n">
+      <c r="N22" s="7" t="n">
         <f aca="false">IF($C22="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -2747,49 +2701,49 @@
       <c r="A23" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B23" s="16"/>
+      <c r="B23" s="13"/>
       <c r="C23" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D23" s="5" t="n">
         <v>2028</v>
       </c>
-      <c r="E23" s="15" t="n">
+      <c r="E23" s="7" t="n">
         <f aca="false">IF($C23="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F23" s="15" t="n">
+      <c r="F23" s="7" t="n">
         <f aca="false">IF($C23="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G23" s="15" t="n">
+      <c r="G23" s="7" t="n">
         <f aca="false">IF($C23="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H23" s="7" t="n">
         <v>50000</v>
       </c>
-      <c r="I23" s="15" t="n">
+      <c r="I23" s="7" t="n">
         <f aca="false">IF($C23="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J23" s="17" t="n">
+      <c r="J23" s="5" t="n">
         <f aca="false">IF($C23="Lease-koop",D23+p_SlotJr,IF($C23="Koop",D23,0))</f>
         <v>2028</v>
       </c>
-      <c r="K23" s="15" t="n">
+      <c r="K23" s="7" t="n">
         <f aca="false">E23+F23+G23+H23+I23</f>
         <v>50000</v>
       </c>
-      <c r="L23" s="17" t="n">
+      <c r="L23" s="5" t="n">
         <f aca="false">IF($C23="Lease-koop",p_Afschr,IF($C23="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A23,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>8</v>
       </c>
-      <c r="M23" s="17" t="n">
+      <c r="M23" s="5" t="n">
         <f aca="false">IF($C23="Lease-koop",D23+p_Lev,IF(AND($C23="Koop",D23&gt;0),D23+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A23,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2036</v>
       </c>
-      <c r="N23" s="15" t="n">
+      <c r="N23" s="7" t="n">
         <f aca="false">IF($C23="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -2801,47 +2755,47 @@
       <c r="A24" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B24" s="16"/>
+      <c r="B24" s="13"/>
       <c r="C24" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D24" s="5" t="n">
         <v>2029</v>
       </c>
-      <c r="E24" s="15" t="n">
+      <c r="E24" s="7" t="n">
         <f aca="false">IF($C24="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F24" s="15" t="n">
+      <c r="F24" s="7" t="n">
         <f aca="false">IF($C24="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G24" s="15" t="n">
+      <c r="G24" s="7" t="n">
         <f aca="false">IF($C24="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H24" s="7"/>
-      <c r="I24" s="15" t="n">
+      <c r="I24" s="7" t="n">
         <f aca="false">IF($C24="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J24" s="17" t="n">
+      <c r="J24" s="5" t="n">
         <f aca="false">IF($C24="Lease-koop",D24+p_SlotJr,IF($C24="Koop",D24,0))</f>
         <v>2031</v>
       </c>
-      <c r="K24" s="15" t="n">
+      <c r="K24" s="7" t="n">
         <f aca="false">E24+F24+G24+H24+I24</f>
         <v>57000</v>
       </c>
-      <c r="L24" s="17" t="n">
+      <c r="L24" s="5" t="n">
         <f aca="false">IF($C24="Lease-koop",p_Afschr,IF($C24="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A24,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M24" s="17" t="n">
+      <c r="M24" s="5" t="n">
         <f aca="false">IF($C24="Lease-koop",D24+p_Lev,IF(AND($C24="Koop",D24&gt;0),D24+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A24,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2037</v>
       </c>
-      <c r="N24" s="15" t="n">
+      <c r="N24" s="7" t="n">
         <f aca="false">IF($C24="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -2851,49 +2805,49 @@
       <c r="A25" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B25" s="16"/>
+      <c r="B25" s="13"/>
       <c r="C25" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="5" t="n">
         <v>2029</v>
       </c>
-      <c r="E25" s="15" t="n">
+      <c r="E25" s="7" t="n">
         <f aca="false">IF($C25="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F25" s="15" t="n">
+      <c r="F25" s="7" t="n">
         <f aca="false">IF($C25="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G25" s="15" t="n">
+      <c r="G25" s="7" t="n">
         <f aca="false">IF($C25="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H25" s="7" t="n">
         <v>100000</v>
       </c>
-      <c r="I25" s="15" t="n">
+      <c r="I25" s="7" t="n">
         <f aca="false">IF($C25="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J25" s="17" t="n">
+      <c r="J25" s="5" t="n">
         <f aca="false">IF($C25="Lease-koop",D25+p_SlotJr,IF($C25="Koop",D25,0))</f>
         <v>2029</v>
       </c>
-      <c r="K25" s="15" t="n">
+      <c r="K25" s="7" t="n">
         <f aca="false">E25+F25+G25+H25+I25</f>
         <v>100000</v>
       </c>
-      <c r="L25" s="17" t="n">
+      <c r="L25" s="5" t="n">
         <f aca="false">IF($C25="Lease-koop",p_Afschr,IF($C25="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A25,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>20</v>
       </c>
-      <c r="M25" s="17" t="n">
+      <c r="M25" s="5" t="n">
         <f aca="false">IF($C25="Lease-koop",D25+p_Lev,IF(AND($C25="Koop",D25&gt;0),D25+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A25,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2049</v>
       </c>
-      <c r="N25" s="15" t="n">
+      <c r="N25" s="7" t="n">
         <f aca="false">IF($C25="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -2903,47 +2857,47 @@
       <c r="A26" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B26" s="16"/>
+      <c r="B26" s="13"/>
       <c r="C26" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D26" s="5" t="n">
         <v>2031</v>
       </c>
-      <c r="E26" s="15" t="n">
+      <c r="E26" s="7" t="n">
         <f aca="false">IF($C26="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F26" s="15" t="n">
+      <c r="F26" s="7" t="n">
         <f aca="false">IF($C26="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G26" s="15" t="n">
+      <c r="G26" s="7" t="n">
         <f aca="false">IF($C26="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H26" s="7"/>
-      <c r="I26" s="15" t="n">
+      <c r="I26" s="7" t="n">
         <f aca="false">IF($C26="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J26" s="17" t="n">
+      <c r="J26" s="5" t="n">
         <f aca="false">IF($C26="Lease-koop",D26+p_SlotJr,IF($C26="Koop",D26,0))</f>
         <v>2033</v>
       </c>
-      <c r="K26" s="15" t="n">
+      <c r="K26" s="7" t="n">
         <f aca="false">E26+F26+G26+H26+I26</f>
         <v>57000</v>
       </c>
-      <c r="L26" s="17" t="n">
+      <c r="L26" s="5" t="n">
         <f aca="false">IF($C26="Lease-koop",p_Afschr,IF($C26="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A26,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M26" s="17" t="n">
+      <c r="M26" s="5" t="n">
         <f aca="false">IF($C26="Lease-koop",D26+p_Lev,IF(AND($C26="Koop",D26&gt;0),D26+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A26,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2039</v>
       </c>
-      <c r="N26" s="15" t="n">
+      <c r="N26" s="7" t="n">
         <f aca="false">IF($C26="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -2953,49 +2907,49 @@
       <c r="A27" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B27" s="16"/>
+      <c r="B27" s="13"/>
       <c r="C27" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D27" s="5" t="n">
         <v>2032</v>
       </c>
-      <c r="E27" s="15" t="n">
+      <c r="E27" s="7" t="n">
         <f aca="false">IF($C27="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F27" s="15" t="n">
+      <c r="F27" s="7" t="n">
         <f aca="false">IF($C27="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G27" s="15" t="n">
+      <c r="G27" s="7" t="n">
         <f aca="false">IF($C27="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H27" s="7" t="n">
         <v>248960</v>
       </c>
-      <c r="I27" s="15" t="n">
+      <c r="I27" s="7" t="n">
         <f aca="false">IF($C27="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J27" s="17" t="n">
+      <c r="J27" s="5" t="n">
         <f aca="false">IF($C27="Lease-koop",D27+p_SlotJr,IF($C27="Koop",D27,0))</f>
         <v>2032</v>
       </c>
-      <c r="K27" s="15" t="n">
+      <c r="K27" s="7" t="n">
         <f aca="false">E27+F27+G27+H27+I27</f>
         <v>248960</v>
       </c>
-      <c r="L27" s="17" t="n">
+      <c r="L27" s="5" t="n">
         <f aca="false">IF($C27="Lease-koop",p_Afschr,IF($C27="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A27,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>8</v>
       </c>
-      <c r="M27" s="17" t="n">
+      <c r="M27" s="5" t="n">
         <f aca="false">IF($C27="Lease-koop",D27+p_Lev,IF(AND($C27="Koop",D27&gt;0),D27+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A27,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2040</v>
       </c>
-      <c r="N27" s="15" t="n">
+      <c r="N27" s="7" t="n">
         <f aca="false">IF($C27="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -3011,40 +2965,40 @@
       <c r="D28" s="5" t="n">
         <v>2032</v>
       </c>
-      <c r="E28" s="15" t="n">
+      <c r="E28" s="7" t="n">
         <f aca="false">IF($C28="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F28" s="15" t="n">
+      <c r="F28" s="7" t="n">
         <f aca="false">IF($C28="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G28" s="15" t="n">
+      <c r="G28" s="7" t="n">
         <f aca="false">IF($C28="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H28" s="7"/>
-      <c r="I28" s="15" t="n">
+      <c r="I28" s="7" t="n">
         <f aca="false">IF($C28="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J28" s="17" t="n">
+      <c r="J28" s="5" t="n">
         <f aca="false">IF($C28="Lease-koop",D28+p_SlotJr,IF($C28="Koop",D28,0))</f>
         <v>0</v>
       </c>
-      <c r="K28" s="15" t="n">
+      <c r="K28" s="7" t="n">
         <f aca="false">E28+F28+G28+H28+I28</f>
         <v>0</v>
       </c>
-      <c r="L28" s="17" t="n">
+      <c r="L28" s="5" t="n">
         <f aca="false">IF($C28="Lease-koop",p_Afschr,IF($C28="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A28,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M28" s="17" t="n">
+      <c r="M28" s="5" t="n">
         <f aca="false">IF($C28="Lease-koop",D28+p_Lev,IF(AND($C28="Koop",D28&gt;0),D28+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A28,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N28" s="15" t="n">
+      <c r="N28" s="7" t="n">
         <f aca="false">IF($C28="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -3056,47 +3010,47 @@
       <c r="A29" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B29" s="16"/>
+      <c r="B29" s="13"/>
       <c r="C29" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D29" s="5" t="n">
         <v>2032</v>
       </c>
-      <c r="E29" s="15" t="n">
+      <c r="E29" s="7" t="n">
         <f aca="false">IF($C29="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F29" s="15" t="n">
+      <c r="F29" s="7" t="n">
         <f aca="false">IF($C29="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G29" s="15" t="n">
+      <c r="G29" s="7" t="n">
         <f aca="false">IF($C29="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H29" s="7"/>
-      <c r="I29" s="15" t="n">
+      <c r="I29" s="7" t="n">
         <f aca="false">IF($C29="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J29" s="17" t="n">
+      <c r="J29" s="5" t="n">
         <f aca="false">IF($C29="Lease-koop",D29+p_SlotJr,IF($C29="Koop",D29,0))</f>
         <v>2034</v>
       </c>
-      <c r="K29" s="15" t="n">
+      <c r="K29" s="7" t="n">
         <f aca="false">E29+F29+G29+H29+I29</f>
         <v>57000</v>
       </c>
-      <c r="L29" s="17" t="n">
+      <c r="L29" s="5" t="n">
         <f aca="false">IF($C29="Lease-koop",p_Afschr,IF($C29="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A29,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M29" s="17" t="n">
+      <c r="M29" s="5" t="n">
         <f aca="false">IF($C29="Lease-koop",D29+p_Lev,IF(AND($C29="Koop",D29&gt;0),D29+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A29,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2040</v>
       </c>
-      <c r="N29" s="15" t="n">
+      <c r="N29" s="7" t="n">
         <f aca="false">IF($C29="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3106,47 +3060,47 @@
       <c r="A30" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B30" s="16"/>
+      <c r="B30" s="13"/>
       <c r="C30" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D30" s="5" t="n">
         <v>2032</v>
       </c>
-      <c r="E30" s="15" t="n">
+      <c r="E30" s="7" t="n">
         <f aca="false">IF($C30="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F30" s="15" t="n">
+      <c r="F30" s="7" t="n">
         <f aca="false">IF($C30="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G30" s="15" t="n">
+      <c r="G30" s="7" t="n">
         <f aca="false">IF($C30="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H30" s="7"/>
-      <c r="I30" s="15" t="n">
+      <c r="I30" s="7" t="n">
         <f aca="false">IF($C30="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J30" s="17" t="n">
+      <c r="J30" s="5" t="n">
         <f aca="false">IF($C30="Lease-koop",D30+p_SlotJr,IF($C30="Koop",D30,0))</f>
         <v>2034</v>
       </c>
-      <c r="K30" s="15" t="n">
+      <c r="K30" s="7" t="n">
         <f aca="false">E30+F30+G30+H30+I30</f>
         <v>57000</v>
       </c>
-      <c r="L30" s="17" t="n">
+      <c r="L30" s="5" t="n">
         <f aca="false">IF($C30="Lease-koop",p_Afschr,IF($C30="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A30,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M30" s="17" t="n">
+      <c r="M30" s="5" t="n">
         <f aca="false">IF($C30="Lease-koop",D30+p_Lev,IF(AND($C30="Koop",D30&gt;0),D30+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A30,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2040</v>
       </c>
-      <c r="N30" s="15" t="n">
+      <c r="N30" s="7" t="n">
         <f aca="false">IF($C30="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3156,47 +3110,47 @@
       <c r="A31" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B31" s="16"/>
+      <c r="B31" s="13"/>
       <c r="C31" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D31" s="5" t="n">
         <v>2032</v>
       </c>
-      <c r="E31" s="15" t="n">
+      <c r="E31" s="7" t="n">
         <f aca="false">IF($C31="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F31" s="15" t="n">
+      <c r="F31" s="7" t="n">
         <f aca="false">IF($C31="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G31" s="15" t="n">
+      <c r="G31" s="7" t="n">
         <f aca="false">IF($C31="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H31" s="7"/>
-      <c r="I31" s="15" t="n">
+      <c r="I31" s="7" t="n">
         <f aca="false">IF($C31="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J31" s="17" t="n">
+      <c r="J31" s="5" t="n">
         <f aca="false">IF($C31="Lease-koop",D31+p_SlotJr,IF($C31="Koop",D31,0))</f>
         <v>2034</v>
       </c>
-      <c r="K31" s="15" t="n">
+      <c r="K31" s="7" t="n">
         <f aca="false">E31+F31+G31+H31+I31</f>
         <v>57000</v>
       </c>
-      <c r="L31" s="17" t="n">
+      <c r="L31" s="5" t="n">
         <f aca="false">IF($C31="Lease-koop",p_Afschr,IF($C31="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A31,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M31" s="17" t="n">
+      <c r="M31" s="5" t="n">
         <f aca="false">IF($C31="Lease-koop",D31+p_Lev,IF(AND($C31="Koop",D31&gt;0),D31+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A31,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2040</v>
       </c>
-      <c r="N31" s="15" t="n">
+      <c r="N31" s="7" t="n">
         <f aca="false">IF($C31="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3206,47 +3160,47 @@
       <c r="A32" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B32" s="16"/>
+      <c r="B32" s="13"/>
       <c r="C32" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D32" s="5" t="n">
         <v>2033</v>
       </c>
-      <c r="E32" s="15" t="n">
+      <c r="E32" s="7" t="n">
         <f aca="false">IF($C32="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F32" s="15" t="n">
+      <c r="F32" s="7" t="n">
         <f aca="false">IF($C32="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G32" s="15" t="n">
+      <c r="G32" s="7" t="n">
         <f aca="false">IF($C32="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H32" s="7"/>
-      <c r="I32" s="15" t="n">
+      <c r="I32" s="7" t="n">
         <f aca="false">IF($C32="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J32" s="17" t="n">
+      <c r="J32" s="5" t="n">
         <f aca="false">IF($C32="Lease-koop",D32+p_SlotJr,IF($C32="Koop",D32,0))</f>
         <v>2035</v>
       </c>
-      <c r="K32" s="15" t="n">
+      <c r="K32" s="7" t="n">
         <f aca="false">E32+F32+G32+H32+I32</f>
         <v>57000</v>
       </c>
-      <c r="L32" s="17" t="n">
+      <c r="L32" s="5" t="n">
         <f aca="false">IF($C32="Lease-koop",p_Afschr,IF($C32="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A32,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M32" s="17" t="n">
+      <c r="M32" s="5" t="n">
         <f aca="false">IF($C32="Lease-koop",D32+p_Lev,IF(AND($C32="Koop",D32&gt;0),D32+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A32,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2041</v>
       </c>
-      <c r="N32" s="15" t="n">
+      <c r="N32" s="7" t="n">
         <f aca="false">IF($C32="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3256,49 +3210,49 @@
       <c r="A33" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B33" s="16"/>
+      <c r="B33" s="13"/>
       <c r="C33" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D33" s="5" t="n">
         <v>2033</v>
       </c>
-      <c r="E33" s="15" t="n">
+      <c r="E33" s="7" t="n">
         <f aca="false">IF($C33="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F33" s="15" t="n">
+      <c r="F33" s="7" t="n">
         <f aca="false">IF($C33="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G33" s="15" t="n">
+      <c r="G33" s="7" t="n">
         <f aca="false">IF($C33="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H33" s="7" t="n">
         <v>19000</v>
       </c>
-      <c r="I33" s="15" t="n">
+      <c r="I33" s="7" t="n">
         <f aca="false">IF($C33="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J33" s="17" t="n">
+      <c r="J33" s="5" t="n">
         <f aca="false">IF($C33="Lease-koop",D33+p_SlotJr,IF($C33="Koop",D33,0))</f>
         <v>2033</v>
       </c>
-      <c r="K33" s="15" t="n">
+      <c r="K33" s="7" t="n">
         <f aca="false">E33+F33+G33+H33+I33</f>
         <v>19000</v>
       </c>
-      <c r="L33" s="17" t="n">
+      <c r="L33" s="5" t="n">
         <f aca="false">IF($C33="Lease-koop",p_Afschr,IF($C33="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A33,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>10</v>
       </c>
-      <c r="M33" s="17" t="n">
+      <c r="M33" s="5" t="n">
         <f aca="false">IF($C33="Lease-koop",D33+p_Lev,IF(AND($C33="Koop",D33&gt;0),D33+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A33,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2043</v>
       </c>
-      <c r="N33" s="15" t="n">
+      <c r="N33" s="7" t="n">
         <f aca="false">IF($C33="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -3308,47 +3262,47 @@
       <c r="A34" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B34" s="16"/>
+      <c r="B34" s="13"/>
       <c r="C34" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D34" s="5" t="n">
         <v>2034</v>
       </c>
-      <c r="E34" s="15" t="n">
+      <c r="E34" s="7" t="n">
         <f aca="false">IF($C34="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F34" s="15" t="n">
+      <c r="F34" s="7" t="n">
         <f aca="false">IF($C34="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G34" s="15" t="n">
+      <c r="G34" s="7" t="n">
         <f aca="false">IF($C34="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H34" s="7"/>
-      <c r="I34" s="15" t="n">
+      <c r="I34" s="7" t="n">
         <f aca="false">IF($C34="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J34" s="17" t="n">
+      <c r="J34" s="5" t="n">
         <f aca="false">IF($C34="Lease-koop",D34+p_SlotJr,IF($C34="Koop",D34,0))</f>
         <v>2036</v>
       </c>
-      <c r="K34" s="15" t="n">
+      <c r="K34" s="7" t="n">
         <f aca="false">E34+F34+G34+H34+I34</f>
         <v>57000</v>
       </c>
-      <c r="L34" s="17" t="n">
+      <c r="L34" s="5" t="n">
         <f aca="false">IF($C34="Lease-koop",p_Afschr,IF($C34="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A34,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M34" s="17" t="n">
+      <c r="M34" s="5" t="n">
         <f aca="false">IF($C34="Lease-koop",D34+p_Lev,IF(AND($C34="Koop",D34&gt;0),D34+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A34,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2042</v>
       </c>
-      <c r="N34" s="15" t="n">
+      <c r="N34" s="7" t="n">
         <f aca="false">IF($C34="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3358,47 +3312,47 @@
       <c r="A35" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B35" s="16"/>
+      <c r="B35" s="13"/>
       <c r="C35" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D35" s="5" t="n">
         <v>2034</v>
       </c>
-      <c r="E35" s="15" t="n">
+      <c r="E35" s="7" t="n">
         <f aca="false">IF($C35="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F35" s="15" t="n">
+      <c r="F35" s="7" t="n">
         <f aca="false">IF($C35="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G35" s="15" t="n">
+      <c r="G35" s="7" t="n">
         <f aca="false">IF($C35="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H35" s="7"/>
-      <c r="I35" s="15" t="n">
+      <c r="I35" s="7" t="n">
         <f aca="false">IF($C35="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J35" s="17" t="n">
+      <c r="J35" s="5" t="n">
         <f aca="false">IF($C35="Lease-koop",D35+p_SlotJr,IF($C35="Koop",D35,0))</f>
         <v>2036</v>
       </c>
-      <c r="K35" s="15" t="n">
+      <c r="K35" s="7" t="n">
         <f aca="false">E35+F35+G35+H35+I35</f>
         <v>57000</v>
       </c>
-      <c r="L35" s="17" t="n">
+      <c r="L35" s="5" t="n">
         <f aca="false">IF($C35="Lease-koop",p_Afschr,IF($C35="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A35,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M35" s="17" t="n">
+      <c r="M35" s="5" t="n">
         <f aca="false">IF($C35="Lease-koop",D35+p_Lev,IF(AND($C35="Koop",D35&gt;0),D35+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A35,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2042</v>
       </c>
-      <c r="N35" s="15" t="n">
+      <c r="N35" s="7" t="n">
         <f aca="false">IF($C35="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3408,47 +3362,47 @@
       <c r="A36" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B36" s="16"/>
+      <c r="B36" s="13"/>
       <c r="C36" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D36" s="5" t="n">
         <v>2034</v>
       </c>
-      <c r="E36" s="15" t="n">
+      <c r="E36" s="7" t="n">
         <f aca="false">IF($C36="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F36" s="15" t="n">
+      <c r="F36" s="7" t="n">
         <f aca="false">IF($C36="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G36" s="15" t="n">
+      <c r="G36" s="7" t="n">
         <f aca="false">IF($C36="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H36" s="7"/>
-      <c r="I36" s="15" t="n">
+      <c r="I36" s="7" t="n">
         <f aca="false">IF($C36="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J36" s="17" t="n">
+      <c r="J36" s="5" t="n">
         <f aca="false">IF($C36="Lease-koop",D36+p_SlotJr,IF($C36="Koop",D36,0))</f>
         <v>2036</v>
       </c>
-      <c r="K36" s="15" t="n">
+      <c r="K36" s="7" t="n">
         <f aca="false">E36+F36+G36+H36+I36</f>
         <v>57000</v>
       </c>
-      <c r="L36" s="17" t="n">
+      <c r="L36" s="5" t="n">
         <f aca="false">IF($C36="Lease-koop",p_Afschr,IF($C36="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A36,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M36" s="17" t="n">
+      <c r="M36" s="5" t="n">
         <f aca="false">IF($C36="Lease-koop",D36+p_Lev,IF(AND($C36="Koop",D36&gt;0),D36+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A36,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2042</v>
       </c>
-      <c r="N36" s="15" t="n">
+      <c r="N36" s="7" t="n">
         <f aca="false">IF($C36="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3458,47 +3412,47 @@
       <c r="A37" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B37" s="16"/>
+      <c r="B37" s="13"/>
       <c r="C37" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D37" s="5" t="n">
         <v>2034</v>
       </c>
-      <c r="E37" s="15" t="n">
+      <c r="E37" s="7" t="n">
         <f aca="false">IF($C37="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F37" s="15" t="n">
+      <c r="F37" s="7" t="n">
         <f aca="false">IF($C37="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G37" s="15" t="n">
+      <c r="G37" s="7" t="n">
         <f aca="false">IF($C37="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H37" s="7"/>
-      <c r="I37" s="15" t="n">
+      <c r="I37" s="7" t="n">
         <f aca="false">IF($C37="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J37" s="17" t="n">
+      <c r="J37" s="5" t="n">
         <f aca="false">IF($C37="Lease-koop",D37+p_SlotJr,IF($C37="Koop",D37,0))</f>
         <v>2036</v>
       </c>
-      <c r="K37" s="15" t="n">
+      <c r="K37" s="7" t="n">
         <f aca="false">E37+F37+G37+H37+I37</f>
         <v>57000</v>
       </c>
-      <c r="L37" s="17" t="n">
+      <c r="L37" s="5" t="n">
         <f aca="false">IF($C37="Lease-koop",p_Afschr,IF($C37="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A37,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M37" s="17" t="n">
+      <c r="M37" s="5" t="n">
         <f aca="false">IF($C37="Lease-koop",D37+p_Lev,IF(AND($C37="Koop",D37&gt;0),D37+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A37,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2042</v>
       </c>
-      <c r="N37" s="15" t="n">
+      <c r="N37" s="7" t="n">
         <f aca="false">IF($C37="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3508,47 +3462,47 @@
       <c r="A38" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B38" s="16"/>
+      <c r="B38" s="13"/>
       <c r="C38" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D38" s="5" t="n">
         <v>2034</v>
       </c>
-      <c r="E38" s="15" t="n">
+      <c r="E38" s="7" t="n">
         <f aca="false">IF($C38="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F38" s="15" t="n">
+      <c r="F38" s="7" t="n">
         <f aca="false">IF($C38="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G38" s="15" t="n">
+      <c r="G38" s="7" t="n">
         <f aca="false">IF($C38="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H38" s="7"/>
-      <c r="I38" s="15" t="n">
+      <c r="I38" s="7" t="n">
         <f aca="false">IF($C38="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J38" s="17" t="n">
+      <c r="J38" s="5" t="n">
         <f aca="false">IF($C38="Lease-koop",D38+p_SlotJr,IF($C38="Koop",D38,0))</f>
         <v>2036</v>
       </c>
-      <c r="K38" s="15" t="n">
+      <c r="K38" s="7" t="n">
         <f aca="false">E38+F38+G38+H38+I38</f>
         <v>57000</v>
       </c>
-      <c r="L38" s="17" t="n">
+      <c r="L38" s="5" t="n">
         <f aca="false">IF($C38="Lease-koop",p_Afschr,IF($C38="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A38,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M38" s="17" t="n">
+      <c r="M38" s="5" t="n">
         <f aca="false">IF($C38="Lease-koop",D38+p_Lev,IF(AND($C38="Koop",D38&gt;0),D38+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A38,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2042</v>
       </c>
-      <c r="N38" s="15" t="n">
+      <c r="N38" s="7" t="n">
         <f aca="false">IF($C38="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3558,47 +3512,47 @@
       <c r="A39" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B39" s="16"/>
+      <c r="B39" s="13"/>
       <c r="C39" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D39" s="5" t="n">
         <v>2034</v>
       </c>
-      <c r="E39" s="15" t="n">
+      <c r="E39" s="7" t="n">
         <f aca="false">IF($C39="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F39" s="15" t="n">
+      <c r="F39" s="7" t="n">
         <f aca="false">IF($C39="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G39" s="15" t="n">
+      <c r="G39" s="7" t="n">
         <f aca="false">IF($C39="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H39" s="7"/>
-      <c r="I39" s="15" t="n">
+      <c r="I39" s="7" t="n">
         <f aca="false">IF($C39="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J39" s="17" t="n">
+      <c r="J39" s="5" t="n">
         <f aca="false">IF($C39="Lease-koop",D39+p_SlotJr,IF($C39="Koop",D39,0))</f>
         <v>2036</v>
       </c>
-      <c r="K39" s="15" t="n">
+      <c r="K39" s="7" t="n">
         <f aca="false">E39+F39+G39+H39+I39</f>
         <v>57000</v>
       </c>
-      <c r="L39" s="17" t="n">
+      <c r="L39" s="5" t="n">
         <f aca="false">IF($C39="Lease-koop",p_Afschr,IF($C39="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A39,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M39" s="17" t="n">
+      <c r="M39" s="5" t="n">
         <f aca="false">IF($C39="Lease-koop",D39+p_Lev,IF(AND($C39="Koop",D39&gt;0),D39+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A39,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2042</v>
       </c>
-      <c r="N39" s="15" t="n">
+      <c r="N39" s="7" t="n">
         <f aca="false">IF($C39="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3608,49 +3562,49 @@
       <c r="A40" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B40" s="16"/>
+      <c r="B40" s="13"/>
       <c r="C40" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D40" s="5" t="n">
         <v>2034</v>
       </c>
-      <c r="E40" s="15" t="n">
+      <c r="E40" s="7" t="n">
         <f aca="false">IF($C40="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F40" s="15" t="n">
+      <c r="F40" s="7" t="n">
         <f aca="false">IF($C40="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G40" s="15" t="n">
+      <c r="G40" s="7" t="n">
         <f aca="false">IF($C40="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H40" s="7" t="n">
         <v>51100</v>
       </c>
-      <c r="I40" s="15" t="n">
+      <c r="I40" s="7" t="n">
         <f aca="false">IF($C40="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J40" s="17" t="n">
+      <c r="J40" s="5" t="n">
         <f aca="false">IF($C40="Lease-koop",D40+p_SlotJr,IF($C40="Koop",D40,0))</f>
         <v>2034</v>
       </c>
-      <c r="K40" s="15" t="n">
+      <c r="K40" s="7" t="n">
         <f aca="false">E40+F40+G40+H40+I40</f>
         <v>51100</v>
       </c>
-      <c r="L40" s="17" t="n">
+      <c r="L40" s="5" t="n">
         <f aca="false">IF($C40="Lease-koop",p_Afschr,IF($C40="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A40,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>10</v>
       </c>
-      <c r="M40" s="17" t="n">
+      <c r="M40" s="5" t="n">
         <f aca="false">IF($C40="Lease-koop",D40+p_Lev,IF(AND($C40="Koop",D40&gt;0),D40+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A40,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2044</v>
       </c>
-      <c r="N40" s="15" t="n">
+      <c r="N40" s="7" t="n">
         <f aca="false">IF($C40="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -3660,47 +3614,47 @@
       <c r="A41" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B41" s="16"/>
+      <c r="B41" s="13"/>
       <c r="C41" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D41" s="5" t="n">
         <v>2034</v>
       </c>
-      <c r="E41" s="15" t="n">
+      <c r="E41" s="7" t="n">
         <f aca="false">IF($C41="Lease-koop",p_Aanbet,0)</f>
         <v>10000</v>
       </c>
-      <c r="F41" s="15" t="n">
+      <c r="F41" s="7" t="n">
         <f aca="false">IF($C41="Lease-koop",p_Belet,0)</f>
         <v>5000</v>
       </c>
-      <c r="G41" s="15" t="n">
+      <c r="G41" s="7" t="n">
         <f aca="false">IF($C41="Lease-koop",p_Opbouw,0)</f>
         <v>7000</v>
       </c>
       <c r="H41" s="7"/>
-      <c r="I41" s="15" t="n">
+      <c r="I41" s="7" t="n">
         <f aca="false">IF($C41="Lease-koop",p_Slot,0)</f>
         <v>35000</v>
       </c>
-      <c r="J41" s="17" t="n">
+      <c r="J41" s="5" t="n">
         <f aca="false">IF($C41="Lease-koop",D41+p_SlotJr,IF($C41="Koop",D41,0))</f>
         <v>2036</v>
       </c>
-      <c r="K41" s="15" t="n">
+      <c r="K41" s="7" t="n">
         <f aca="false">E41+F41+G41+H41+I41</f>
         <v>57000</v>
       </c>
-      <c r="L41" s="17" t="n">
+      <c r="L41" s="5" t="n">
         <f aca="false">IF($C41="Lease-koop",p_Afschr,IF($C41="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A41,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>6</v>
       </c>
-      <c r="M41" s="17" t="n">
+      <c r="M41" s="5" t="n">
         <f aca="false">IF($C41="Lease-koop",D41+p_Lev,IF(AND($C41="Koop",D41&gt;0),D41+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A41,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2042</v>
       </c>
-      <c r="N41" s="15" t="n">
+      <c r="N41" s="7" t="n">
         <f aca="false">IF($C41="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
@@ -3710,49 +3664,49 @@
       <c r="A42" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B42" s="16"/>
+      <c r="B42" s="13"/>
       <c r="C42" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D42" s="5" t="n">
         <v>2035</v>
       </c>
-      <c r="E42" s="15" t="n">
+      <c r="E42" s="7" t="n">
         <f aca="false">IF($C42="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F42" s="15" t="n">
+      <c r="F42" s="7" t="n">
         <f aca="false">IF($C42="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G42" s="15" t="n">
+      <c r="G42" s="7" t="n">
         <f aca="false">IF($C42="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H42" s="7" t="n">
         <v>358180</v>
       </c>
-      <c r="I42" s="15" t="n">
+      <c r="I42" s="7" t="n">
         <f aca="false">IF($C42="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J42" s="17" t="n">
+      <c r="J42" s="5" t="n">
         <f aca="false">IF($C42="Lease-koop",D42+p_SlotJr,IF($C42="Koop",D42,0))</f>
         <v>2035</v>
       </c>
-      <c r="K42" s="15" t="n">
+      <c r="K42" s="7" t="n">
         <f aca="false">E42+F42+G42+H42+I42</f>
         <v>358180</v>
       </c>
-      <c r="L42" s="17" t="n">
+      <c r="L42" s="5" t="n">
         <f aca="false">IF($C42="Lease-koop",p_Afschr,IF($C42="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A42,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>12</v>
       </c>
-      <c r="M42" s="17" t="n">
+      <c r="M42" s="5" t="n">
         <f aca="false">IF($C42="Lease-koop",D42+p_Lev,IF(AND($C42="Koop",D42&gt;0),D42+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A42,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2047</v>
       </c>
-      <c r="N42" s="15" t="n">
+      <c r="N42" s="7" t="n">
         <f aca="false">IF($C42="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -3762,49 +3716,49 @@
       <c r="A43" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B43" s="16"/>
+      <c r="B43" s="13"/>
       <c r="C43" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D43" s="5" t="n">
         <v>2038</v>
       </c>
-      <c r="E43" s="15" t="n">
+      <c r="E43" s="7" t="n">
         <f aca="false">IF($C43="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F43" s="15" t="n">
+      <c r="F43" s="7" t="n">
         <f aca="false">IF($C43="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G43" s="15" t="n">
+      <c r="G43" s="7" t="n">
         <f aca="false">IF($C43="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H43" s="7" t="n">
         <v>121968</v>
       </c>
-      <c r="I43" s="15" t="n">
+      <c r="I43" s="7" t="n">
         <f aca="false">IF($C43="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J43" s="17" t="n">
+      <c r="J43" s="5" t="n">
         <f aca="false">IF($C43="Lease-koop",D43+p_SlotJr,IF($C43="Koop",D43,0))</f>
         <v>2038</v>
       </c>
-      <c r="K43" s="15" t="n">
+      <c r="K43" s="7" t="n">
         <f aca="false">E43+F43+G43+H43+I43</f>
         <v>121968</v>
       </c>
-      <c r="L43" s="17" t="n">
+      <c r="L43" s="5" t="n">
         <f aca="false">IF($C43="Lease-koop",p_Afschr,IF($C43="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A43,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>15</v>
       </c>
-      <c r="M43" s="17" t="n">
+      <c r="M43" s="5" t="n">
         <f aca="false">IF($C43="Lease-koop",D43+p_Lev,IF(AND($C43="Koop",D43&gt;0),D43+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A43,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>2053</v>
       </c>
-      <c r="N43" s="15" t="n">
+      <c r="N43" s="7" t="n">
         <f aca="false">IF($C43="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -3812,2120 +3766,2120 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D44" s="5"/>
-      <c r="E44" s="15" t="n">
+      <c r="E44" s="7" t="n">
         <f aca="false">IF($C44="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F44" s="15" t="n">
+      <c r="F44" s="7" t="n">
         <f aca="false">IF($C44="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G44" s="15" t="n">
+      <c r="G44" s="7" t="n">
         <f aca="false">IF($C44="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H44" s="7"/>
-      <c r="I44" s="15" t="n">
+      <c r="I44" s="7" t="n">
         <f aca="false">IF($C44="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J44" s="17" t="n">
+      <c r="J44" s="5" t="n">
         <f aca="false">IF($C44="Lease-koop",D44+p_SlotJr,IF($C44="Koop",D44,0))</f>
         <v>0</v>
       </c>
-      <c r="K44" s="15" t="n">
+      <c r="K44" s="7" t="n">
         <f aca="false">E44+F44+G44+H44+I44</f>
         <v>0</v>
       </c>
-      <c r="L44" s="17" t="n">
+      <c r="L44" s="5" t="n">
         <f aca="false">IF($C44="Lease-koop",p_Afschr,IF($C44="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A44,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M44" s="17" t="n">
+      <c r="M44" s="5" t="n">
         <f aca="false">IF($C44="Lease-koop",D44+p_Lev,IF(AND($C44="Koop",D44&gt;0),D44+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A44,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N44" s="15" t="n">
+      <c r="N44" s="7" t="n">
         <f aca="false">IF($C44="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D45" s="5"/>
-      <c r="E45" s="15" t="n">
+      <c r="E45" s="7" t="n">
         <f aca="false">IF($C45="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F45" s="15" t="n">
+      <c r="F45" s="7" t="n">
         <f aca="false">IF($C45="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G45" s="15" t="n">
+      <c r="G45" s="7" t="n">
         <f aca="false">IF($C45="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H45" s="7"/>
-      <c r="I45" s="15" t="n">
+      <c r="I45" s="7" t="n">
         <f aca="false">IF($C45="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J45" s="17" t="n">
+      <c r="J45" s="5" t="n">
         <f aca="false">IF($C45="Lease-koop",D45+p_SlotJr,IF($C45="Koop",D45,0))</f>
         <v>0</v>
       </c>
-      <c r="K45" s="15" t="n">
+      <c r="K45" s="7" t="n">
         <f aca="false">E45+F45+G45+H45+I45</f>
         <v>0</v>
       </c>
-      <c r="L45" s="17" t="n">
+      <c r="L45" s="5" t="n">
         <f aca="false">IF($C45="Lease-koop",p_Afschr,IF($C45="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A45,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M45" s="17" t="n">
+      <c r="M45" s="5" t="n">
         <f aca="false">IF($C45="Lease-koop",D45+p_Lev,IF(AND($C45="Koop",D45&gt;0),D45+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A45,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N45" s="15" t="n">
+      <c r="N45" s="7" t="n">
         <f aca="false">IF($C45="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D46" s="5"/>
-      <c r="E46" s="15" t="n">
+      <c r="E46" s="7" t="n">
         <f aca="false">IF($C46="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F46" s="15" t="n">
+      <c r="F46" s="7" t="n">
         <f aca="false">IF($C46="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G46" s="15" t="n">
+      <c r="G46" s="7" t="n">
         <f aca="false">IF($C46="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H46" s="7"/>
-      <c r="I46" s="15" t="n">
+      <c r="I46" s="7" t="n">
         <f aca="false">IF($C46="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J46" s="17" t="n">
+      <c r="J46" s="5" t="n">
         <f aca="false">IF($C46="Lease-koop",D46+p_SlotJr,IF($C46="Koop",D46,0))</f>
         <v>0</v>
       </c>
-      <c r="K46" s="15" t="n">
+      <c r="K46" s="7" t="n">
         <f aca="false">E46+F46+G46+H46+I46</f>
         <v>0</v>
       </c>
-      <c r="L46" s="17" t="n">
+      <c r="L46" s="5" t="n">
         <f aca="false">IF($C46="Lease-koop",p_Afschr,IF($C46="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A46,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M46" s="17" t="n">
+      <c r="M46" s="5" t="n">
         <f aca="false">IF($C46="Lease-koop",D46+p_Lev,IF(AND($C46="Koop",D46&gt;0),D46+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A46,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N46" s="15" t="n">
+      <c r="N46" s="7" t="n">
         <f aca="false">IF($C46="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D47" s="5"/>
-      <c r="E47" s="15" t="n">
+      <c r="E47" s="7" t="n">
         <f aca="false">IF($C47="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F47" s="15" t="n">
+      <c r="F47" s="7" t="n">
         <f aca="false">IF($C47="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G47" s="15" t="n">
+      <c r="G47" s="7" t="n">
         <f aca="false">IF($C47="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H47" s="7"/>
-      <c r="I47" s="15" t="n">
+      <c r="I47" s="7" t="n">
         <f aca="false">IF($C47="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J47" s="17" t="n">
+      <c r="J47" s="5" t="n">
         <f aca="false">IF($C47="Lease-koop",D47+p_SlotJr,IF($C47="Koop",D47,0))</f>
         <v>0</v>
       </c>
-      <c r="K47" s="15" t="n">
+      <c r="K47" s="7" t="n">
         <f aca="false">E47+F47+G47+H47+I47</f>
         <v>0</v>
       </c>
-      <c r="L47" s="17" t="n">
+      <c r="L47" s="5" t="n">
         <f aca="false">IF($C47="Lease-koop",p_Afschr,IF($C47="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A47,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M47" s="17" t="n">
+      <c r="M47" s="5" t="n">
         <f aca="false">IF($C47="Lease-koop",D47+p_Lev,IF(AND($C47="Koop",D47&gt;0),D47+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A47,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N47" s="15" t="n">
+      <c r="N47" s="7" t="n">
         <f aca="false">IF($C47="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D48" s="5"/>
-      <c r="E48" s="15" t="n">
+      <c r="E48" s="7" t="n">
         <f aca="false">IF($C48="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F48" s="15" t="n">
+      <c r="F48" s="7" t="n">
         <f aca="false">IF($C48="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G48" s="15" t="n">
+      <c r="G48" s="7" t="n">
         <f aca="false">IF($C48="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H48" s="7"/>
-      <c r="I48" s="15" t="n">
+      <c r="I48" s="7" t="n">
         <f aca="false">IF($C48="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J48" s="17" t="n">
+      <c r="J48" s="5" t="n">
         <f aca="false">IF($C48="Lease-koop",D48+p_SlotJr,IF($C48="Koop",D48,0))</f>
         <v>0</v>
       </c>
-      <c r="K48" s="15" t="n">
+      <c r="K48" s="7" t="n">
         <f aca="false">E48+F48+G48+H48+I48</f>
         <v>0</v>
       </c>
-      <c r="L48" s="17" t="n">
+      <c r="L48" s="5" t="n">
         <f aca="false">IF($C48="Lease-koop",p_Afschr,IF($C48="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A48,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M48" s="17" t="n">
+      <c r="M48" s="5" t="n">
         <f aca="false">IF($C48="Lease-koop",D48+p_Lev,IF(AND($C48="Koop",D48&gt;0),D48+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A48,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N48" s="15" t="n">
+      <c r="N48" s="7" t="n">
         <f aca="false">IF($C48="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D49" s="5"/>
-      <c r="E49" s="15" t="n">
+      <c r="E49" s="7" t="n">
         <f aca="false">IF($C49="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F49" s="15" t="n">
+      <c r="F49" s="7" t="n">
         <f aca="false">IF($C49="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G49" s="15" t="n">
+      <c r="G49" s="7" t="n">
         <f aca="false">IF($C49="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H49" s="7"/>
-      <c r="I49" s="15" t="n">
+      <c r="I49" s="7" t="n">
         <f aca="false">IF($C49="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J49" s="17" t="n">
+      <c r="J49" s="5" t="n">
         <f aca="false">IF($C49="Lease-koop",D49+p_SlotJr,IF($C49="Koop",D49,0))</f>
         <v>0</v>
       </c>
-      <c r="K49" s="15" t="n">
+      <c r="K49" s="7" t="n">
         <f aca="false">E49+F49+G49+H49+I49</f>
         <v>0</v>
       </c>
-      <c r="L49" s="17" t="n">
+      <c r="L49" s="5" t="n">
         <f aca="false">IF($C49="Lease-koop",p_Afschr,IF($C49="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A49,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M49" s="17" t="n">
+      <c r="M49" s="5" t="n">
         <f aca="false">IF($C49="Lease-koop",D49+p_Lev,IF(AND($C49="Koop",D49&gt;0),D49+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A49,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N49" s="15" t="n">
+      <c r="N49" s="7" t="n">
         <f aca="false">IF($C49="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D50" s="5"/>
-      <c r="E50" s="15" t="n">
+      <c r="E50" s="7" t="n">
         <f aca="false">IF($C50="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F50" s="15" t="n">
+      <c r="F50" s="7" t="n">
         <f aca="false">IF($C50="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G50" s="15" t="n">
+      <c r="G50" s="7" t="n">
         <f aca="false">IF($C50="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H50" s="7"/>
-      <c r="I50" s="15" t="n">
+      <c r="I50" s="7" t="n">
         <f aca="false">IF($C50="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J50" s="17" t="n">
+      <c r="J50" s="5" t="n">
         <f aca="false">IF($C50="Lease-koop",D50+p_SlotJr,IF($C50="Koop",D50,0))</f>
         <v>0</v>
       </c>
-      <c r="K50" s="15" t="n">
+      <c r="K50" s="7" t="n">
         <f aca="false">E50+F50+G50+H50+I50</f>
         <v>0</v>
       </c>
-      <c r="L50" s="17" t="n">
+      <c r="L50" s="5" t="n">
         <f aca="false">IF($C50="Lease-koop",p_Afschr,IF($C50="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A50,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M50" s="17" t="n">
+      <c r="M50" s="5" t="n">
         <f aca="false">IF($C50="Lease-koop",D50+p_Lev,IF(AND($C50="Koop",D50&gt;0),D50+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A50,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N50" s="15" t="n">
+      <c r="N50" s="7" t="n">
         <f aca="false">IF($C50="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D51" s="5"/>
-      <c r="E51" s="15" t="n">
+      <c r="E51" s="7" t="n">
         <f aca="false">IF($C51="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F51" s="15" t="n">
+      <c r="F51" s="7" t="n">
         <f aca="false">IF($C51="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G51" s="15" t="n">
+      <c r="G51" s="7" t="n">
         <f aca="false">IF($C51="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H51" s="7"/>
-      <c r="I51" s="15" t="n">
+      <c r="I51" s="7" t="n">
         <f aca="false">IF($C51="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J51" s="17" t="n">
+      <c r="J51" s="5" t="n">
         <f aca="false">IF($C51="Lease-koop",D51+p_SlotJr,IF($C51="Koop",D51,0))</f>
         <v>0</v>
       </c>
-      <c r="K51" s="15" t="n">
+      <c r="K51" s="7" t="n">
         <f aca="false">E51+F51+G51+H51+I51</f>
         <v>0</v>
       </c>
-      <c r="L51" s="17" t="n">
+      <c r="L51" s="5" t="n">
         <f aca="false">IF($C51="Lease-koop",p_Afschr,IF($C51="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A51,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M51" s="17" t="n">
+      <c r="M51" s="5" t="n">
         <f aca="false">IF($C51="Lease-koop",D51+p_Lev,IF(AND($C51="Koop",D51&gt;0),D51+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A51,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N51" s="15" t="n">
+      <c r="N51" s="7" t="n">
         <f aca="false">IF($C51="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D52" s="5"/>
-      <c r="E52" s="15" t="n">
+      <c r="E52" s="7" t="n">
         <f aca="false">IF($C52="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F52" s="15" t="n">
+      <c r="F52" s="7" t="n">
         <f aca="false">IF($C52="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G52" s="15" t="n">
+      <c r="G52" s="7" t="n">
         <f aca="false">IF($C52="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H52" s="7"/>
-      <c r="I52" s="15" t="n">
+      <c r="I52" s="7" t="n">
         <f aca="false">IF($C52="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J52" s="17" t="n">
+      <c r="J52" s="5" t="n">
         <f aca="false">IF($C52="Lease-koop",D52+p_SlotJr,IF($C52="Koop",D52,0))</f>
         <v>0</v>
       </c>
-      <c r="K52" s="15" t="n">
+      <c r="K52" s="7" t="n">
         <f aca="false">E52+F52+G52+H52+I52</f>
         <v>0</v>
       </c>
-      <c r="L52" s="17" t="n">
+      <c r="L52" s="5" t="n">
         <f aca="false">IF($C52="Lease-koop",p_Afschr,IF($C52="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A52,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M52" s="17" t="n">
+      <c r="M52" s="5" t="n">
         <f aca="false">IF($C52="Lease-koop",D52+p_Lev,IF(AND($C52="Koop",D52&gt;0),D52+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A52,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N52" s="15" t="n">
+      <c r="N52" s="7" t="n">
         <f aca="false">IF($C52="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D53" s="5"/>
-      <c r="E53" s="15" t="n">
+      <c r="E53" s="7" t="n">
         <f aca="false">IF($C53="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F53" s="15" t="n">
+      <c r="F53" s="7" t="n">
         <f aca="false">IF($C53="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G53" s="15" t="n">
+      <c r="G53" s="7" t="n">
         <f aca="false">IF($C53="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H53" s="7"/>
-      <c r="I53" s="15" t="n">
+      <c r="I53" s="7" t="n">
         <f aca="false">IF($C53="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J53" s="17" t="n">
+      <c r="J53" s="5" t="n">
         <f aca="false">IF($C53="Lease-koop",D53+p_SlotJr,IF($C53="Koop",D53,0))</f>
         <v>0</v>
       </c>
-      <c r="K53" s="15" t="n">
+      <c r="K53" s="7" t="n">
         <f aca="false">E53+F53+G53+H53+I53</f>
         <v>0</v>
       </c>
-      <c r="L53" s="17" t="n">
+      <c r="L53" s="5" t="n">
         <f aca="false">IF($C53="Lease-koop",p_Afschr,IF($C53="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A53,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M53" s="17" t="n">
+      <c r="M53" s="5" t="n">
         <f aca="false">IF($C53="Lease-koop",D53+p_Lev,IF(AND($C53="Koop",D53&gt;0),D53+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A53,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N53" s="15" t="n">
+      <c r="N53" s="7" t="n">
         <f aca="false">IF($C53="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D54" s="5"/>
-      <c r="E54" s="15" t="n">
+      <c r="E54" s="7" t="n">
         <f aca="false">IF($C54="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F54" s="15" t="n">
+      <c r="F54" s="7" t="n">
         <f aca="false">IF($C54="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G54" s="15" t="n">
+      <c r="G54" s="7" t="n">
         <f aca="false">IF($C54="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H54" s="7"/>
-      <c r="I54" s="15" t="n">
+      <c r="I54" s="7" t="n">
         <f aca="false">IF($C54="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J54" s="17" t="n">
+      <c r="J54" s="5" t="n">
         <f aca="false">IF($C54="Lease-koop",D54+p_SlotJr,IF($C54="Koop",D54,0))</f>
         <v>0</v>
       </c>
-      <c r="K54" s="15" t="n">
+      <c r="K54" s="7" t="n">
         <f aca="false">E54+F54+G54+H54+I54</f>
         <v>0</v>
       </c>
-      <c r="L54" s="17" t="n">
+      <c r="L54" s="5" t="n">
         <f aca="false">IF($C54="Lease-koop",p_Afschr,IF($C54="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A54,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M54" s="17" t="n">
+      <c r="M54" s="5" t="n">
         <f aca="false">IF($C54="Lease-koop",D54+p_Lev,IF(AND($C54="Koop",D54&gt;0),D54+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A54,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N54" s="15" t="n">
+      <c r="N54" s="7" t="n">
         <f aca="false">IF($C54="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D55" s="5"/>
-      <c r="E55" s="15" t="n">
+      <c r="E55" s="7" t="n">
         <f aca="false">IF($C55="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F55" s="15" t="n">
+      <c r="F55" s="7" t="n">
         <f aca="false">IF($C55="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G55" s="15" t="n">
+      <c r="G55" s="7" t="n">
         <f aca="false">IF($C55="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H55" s="7"/>
-      <c r="I55" s="15" t="n">
+      <c r="I55" s="7" t="n">
         <f aca="false">IF($C55="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J55" s="17" t="n">
+      <c r="J55" s="5" t="n">
         <f aca="false">IF($C55="Lease-koop",D55+p_SlotJr,IF($C55="Koop",D55,0))</f>
         <v>0</v>
       </c>
-      <c r="K55" s="15" t="n">
+      <c r="K55" s="7" t="n">
         <f aca="false">E55+F55+G55+H55+I55</f>
         <v>0</v>
       </c>
-      <c r="L55" s="17" t="n">
+      <c r="L55" s="5" t="n">
         <f aca="false">IF($C55="Lease-koop",p_Afschr,IF($C55="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A55,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M55" s="17" t="n">
+      <c r="M55" s="5" t="n">
         <f aca="false">IF($C55="Lease-koop",D55+p_Lev,IF(AND($C55="Koop",D55&gt;0),D55+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A55,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N55" s="15" t="n">
+      <c r="N55" s="7" t="n">
         <f aca="false">IF($C55="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D56" s="5"/>
-      <c r="E56" s="15" t="n">
+      <c r="E56" s="7" t="n">
         <f aca="false">IF($C56="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F56" s="15" t="n">
+      <c r="F56" s="7" t="n">
         <f aca="false">IF($C56="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G56" s="15" t="n">
+      <c r="G56" s="7" t="n">
         <f aca="false">IF($C56="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H56" s="7"/>
-      <c r="I56" s="15" t="n">
+      <c r="I56" s="7" t="n">
         <f aca="false">IF($C56="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J56" s="17" t="n">
+      <c r="J56" s="5" t="n">
         <f aca="false">IF($C56="Lease-koop",D56+p_SlotJr,IF($C56="Koop",D56,0))</f>
         <v>0</v>
       </c>
-      <c r="K56" s="15" t="n">
+      <c r="K56" s="7" t="n">
         <f aca="false">E56+F56+G56+H56+I56</f>
         <v>0</v>
       </c>
-      <c r="L56" s="17" t="n">
+      <c r="L56" s="5" t="n">
         <f aca="false">IF($C56="Lease-koop",p_Afschr,IF($C56="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A56,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M56" s="17" t="n">
+      <c r="M56" s="5" t="n">
         <f aca="false">IF($C56="Lease-koop",D56+p_Lev,IF(AND($C56="Koop",D56&gt;0),D56+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A56,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N56" s="15" t="n">
+      <c r="N56" s="7" t="n">
         <f aca="false">IF($C56="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D57" s="5"/>
-      <c r="E57" s="15" t="n">
+      <c r="E57" s="7" t="n">
         <f aca="false">IF($C57="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F57" s="15" t="n">
+      <c r="F57" s="7" t="n">
         <f aca="false">IF($C57="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G57" s="15" t="n">
+      <c r="G57" s="7" t="n">
         <f aca="false">IF($C57="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H57" s="7"/>
-      <c r="I57" s="15" t="n">
+      <c r="I57" s="7" t="n">
         <f aca="false">IF($C57="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J57" s="17" t="n">
+      <c r="J57" s="5" t="n">
         <f aca="false">IF($C57="Lease-koop",D57+p_SlotJr,IF($C57="Koop",D57,0))</f>
         <v>0</v>
       </c>
-      <c r="K57" s="15" t="n">
+      <c r="K57" s="7" t="n">
         <f aca="false">E57+F57+G57+H57+I57</f>
         <v>0</v>
       </c>
-      <c r="L57" s="17" t="n">
+      <c r="L57" s="5" t="n">
         <f aca="false">IF($C57="Lease-koop",p_Afschr,IF($C57="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A57,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M57" s="17" t="n">
+      <c r="M57" s="5" t="n">
         <f aca="false">IF($C57="Lease-koop",D57+p_Lev,IF(AND($C57="Koop",D57&gt;0),D57+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A57,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N57" s="15" t="n">
+      <c r="N57" s="7" t="n">
         <f aca="false">IF($C57="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D58" s="5"/>
-      <c r="E58" s="15" t="n">
+      <c r="E58" s="7" t="n">
         <f aca="false">IF($C58="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F58" s="15" t="n">
+      <c r="F58" s="7" t="n">
         <f aca="false">IF($C58="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G58" s="15" t="n">
+      <c r="G58" s="7" t="n">
         <f aca="false">IF($C58="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H58" s="7"/>
-      <c r="I58" s="15" t="n">
+      <c r="I58" s="7" t="n">
         <f aca="false">IF($C58="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J58" s="17" t="n">
+      <c r="J58" s="5" t="n">
         <f aca="false">IF($C58="Lease-koop",D58+p_SlotJr,IF($C58="Koop",D58,0))</f>
         <v>0</v>
       </c>
-      <c r="K58" s="15" t="n">
+      <c r="K58" s="7" t="n">
         <f aca="false">E58+F58+G58+H58+I58</f>
         <v>0</v>
       </c>
-      <c r="L58" s="17" t="n">
+      <c r="L58" s="5" t="n">
         <f aca="false">IF($C58="Lease-koop",p_Afschr,IF($C58="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A58,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M58" s="17" t="n">
+      <c r="M58" s="5" t="n">
         <f aca="false">IF($C58="Lease-koop",D58+p_Lev,IF(AND($C58="Koop",D58&gt;0),D58+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A58,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N58" s="15" t="n">
+      <c r="N58" s="7" t="n">
         <f aca="false">IF($C58="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D59" s="5"/>
-      <c r="E59" s="15" t="n">
+      <c r="E59" s="7" t="n">
         <f aca="false">IF($C59="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F59" s="15" t="n">
+      <c r="F59" s="7" t="n">
         <f aca="false">IF($C59="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G59" s="15" t="n">
+      <c r="G59" s="7" t="n">
         <f aca="false">IF($C59="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H59" s="7"/>
-      <c r="I59" s="15" t="n">
+      <c r="I59" s="7" t="n">
         <f aca="false">IF($C59="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J59" s="17" t="n">
+      <c r="J59" s="5" t="n">
         <f aca="false">IF($C59="Lease-koop",D59+p_SlotJr,IF($C59="Koop",D59,0))</f>
         <v>0</v>
       </c>
-      <c r="K59" s="15" t="n">
+      <c r="K59" s="7" t="n">
         <f aca="false">E59+F59+G59+H59+I59</f>
         <v>0</v>
       </c>
-      <c r="L59" s="17" t="n">
+      <c r="L59" s="5" t="n">
         <f aca="false">IF($C59="Lease-koop",p_Afschr,IF($C59="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A59,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M59" s="17" t="n">
+      <c r="M59" s="5" t="n">
         <f aca="false">IF($C59="Lease-koop",D59+p_Lev,IF(AND($C59="Koop",D59&gt;0),D59+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A59,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N59" s="15" t="n">
+      <c r="N59" s="7" t="n">
         <f aca="false">IF($C59="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D60" s="5"/>
-      <c r="E60" s="15" t="n">
+      <c r="E60" s="7" t="n">
         <f aca="false">IF($C60="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F60" s="15" t="n">
+      <c r="F60" s="7" t="n">
         <f aca="false">IF($C60="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G60" s="15" t="n">
+      <c r="G60" s="7" t="n">
         <f aca="false">IF($C60="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H60" s="7"/>
-      <c r="I60" s="15" t="n">
+      <c r="I60" s="7" t="n">
         <f aca="false">IF($C60="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J60" s="17" t="n">
+      <c r="J60" s="5" t="n">
         <f aca="false">IF($C60="Lease-koop",D60+p_SlotJr,IF($C60="Koop",D60,0))</f>
         <v>0</v>
       </c>
-      <c r="K60" s="15" t="n">
+      <c r="K60" s="7" t="n">
         <f aca="false">E60+F60+G60+H60+I60</f>
         <v>0</v>
       </c>
-      <c r="L60" s="17" t="n">
+      <c r="L60" s="5" t="n">
         <f aca="false">IF($C60="Lease-koop",p_Afschr,IF($C60="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A60,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M60" s="17" t="n">
+      <c r="M60" s="5" t="n">
         <f aca="false">IF($C60="Lease-koop",D60+p_Lev,IF(AND($C60="Koop",D60&gt;0),D60+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A60,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N60" s="15" t="n">
+      <c r="N60" s="7" t="n">
         <f aca="false">IF($C60="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D61" s="5"/>
-      <c r="E61" s="15" t="n">
+      <c r="E61" s="7" t="n">
         <f aca="false">IF($C61="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F61" s="15" t="n">
+      <c r="F61" s="7" t="n">
         <f aca="false">IF($C61="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G61" s="15" t="n">
+      <c r="G61" s="7" t="n">
         <f aca="false">IF($C61="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H61" s="7"/>
-      <c r="I61" s="15" t="n">
+      <c r="I61" s="7" t="n">
         <f aca="false">IF($C61="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J61" s="17" t="n">
+      <c r="J61" s="5" t="n">
         <f aca="false">IF($C61="Lease-koop",D61+p_SlotJr,IF($C61="Koop",D61,0))</f>
         <v>0</v>
       </c>
-      <c r="K61" s="15" t="n">
+      <c r="K61" s="7" t="n">
         <f aca="false">E61+F61+G61+H61+I61</f>
         <v>0</v>
       </c>
-      <c r="L61" s="17" t="n">
+      <c r="L61" s="5" t="n">
         <f aca="false">IF($C61="Lease-koop",p_Afschr,IF($C61="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A61,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M61" s="17" t="n">
+      <c r="M61" s="5" t="n">
         <f aca="false">IF($C61="Lease-koop",D61+p_Lev,IF(AND($C61="Koop",D61&gt;0),D61+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A61,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N61" s="15" t="n">
+      <c r="N61" s="7" t="n">
         <f aca="false">IF($C61="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D62" s="5"/>
-      <c r="E62" s="15" t="n">
+      <c r="E62" s="7" t="n">
         <f aca="false">IF($C62="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F62" s="15" t="n">
+      <c r="F62" s="7" t="n">
         <f aca="false">IF($C62="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G62" s="15" t="n">
+      <c r="G62" s="7" t="n">
         <f aca="false">IF($C62="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H62" s="7"/>
-      <c r="I62" s="15" t="n">
+      <c r="I62" s="7" t="n">
         <f aca="false">IF($C62="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J62" s="17" t="n">
+      <c r="J62" s="5" t="n">
         <f aca="false">IF($C62="Lease-koop",D62+p_SlotJr,IF($C62="Koop",D62,0))</f>
         <v>0</v>
       </c>
-      <c r="K62" s="15" t="n">
+      <c r="K62" s="7" t="n">
         <f aca="false">E62+F62+G62+H62+I62</f>
         <v>0</v>
       </c>
-      <c r="L62" s="17" t="n">
+      <c r="L62" s="5" t="n">
         <f aca="false">IF($C62="Lease-koop",p_Afschr,IF($C62="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A62,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M62" s="17" t="n">
+      <c r="M62" s="5" t="n">
         <f aca="false">IF($C62="Lease-koop",D62+p_Lev,IF(AND($C62="Koop",D62&gt;0),D62+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A62,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N62" s="15" t="n">
+      <c r="N62" s="7" t="n">
         <f aca="false">IF($C62="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D63" s="5"/>
-      <c r="E63" s="15" t="n">
+      <c r="E63" s="7" t="n">
         <f aca="false">IF($C63="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F63" s="15" t="n">
+      <c r="F63" s="7" t="n">
         <f aca="false">IF($C63="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G63" s="15" t="n">
+      <c r="G63" s="7" t="n">
         <f aca="false">IF($C63="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H63" s="7"/>
-      <c r="I63" s="15" t="n">
+      <c r="I63" s="7" t="n">
         <f aca="false">IF($C63="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J63" s="17" t="n">
+      <c r="J63" s="5" t="n">
         <f aca="false">IF($C63="Lease-koop",D63+p_SlotJr,IF($C63="Koop",D63,0))</f>
         <v>0</v>
       </c>
-      <c r="K63" s="15" t="n">
+      <c r="K63" s="7" t="n">
         <f aca="false">E63+F63+G63+H63+I63</f>
         <v>0</v>
       </c>
-      <c r="L63" s="17" t="n">
+      <c r="L63" s="5" t="n">
         <f aca="false">IF($C63="Lease-koop",p_Afschr,IF($C63="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A63,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M63" s="17" t="n">
+      <c r="M63" s="5" t="n">
         <f aca="false">IF($C63="Lease-koop",D63+p_Lev,IF(AND($C63="Koop",D63&gt;0),D63+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A63,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N63" s="15" t="n">
+      <c r="N63" s="7" t="n">
         <f aca="false">IF($C63="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D64" s="5"/>
-      <c r="E64" s="15" t="n">
+      <c r="E64" s="7" t="n">
         <f aca="false">IF($C64="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F64" s="15" t="n">
+      <c r="F64" s="7" t="n">
         <f aca="false">IF($C64="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G64" s="15" t="n">
+      <c r="G64" s="7" t="n">
         <f aca="false">IF($C64="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H64" s="7"/>
-      <c r="I64" s="15" t="n">
+      <c r="I64" s="7" t="n">
         <f aca="false">IF($C64="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J64" s="17" t="n">
+      <c r="J64" s="5" t="n">
         <f aca="false">IF($C64="Lease-koop",D64+p_SlotJr,IF($C64="Koop",D64,0))</f>
         <v>0</v>
       </c>
-      <c r="K64" s="15" t="n">
+      <c r="K64" s="7" t="n">
         <f aca="false">E64+F64+G64+H64+I64</f>
         <v>0</v>
       </c>
-      <c r="L64" s="17" t="n">
+      <c r="L64" s="5" t="n">
         <f aca="false">IF($C64="Lease-koop",p_Afschr,IF($C64="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A64,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M64" s="17" t="n">
+      <c r="M64" s="5" t="n">
         <f aca="false">IF($C64="Lease-koop",D64+p_Lev,IF(AND($C64="Koop",D64&gt;0),D64+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A64,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N64" s="15" t="n">
+      <c r="N64" s="7" t="n">
         <f aca="false">IF($C64="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D65" s="5"/>
-      <c r="E65" s="15" t="n">
+      <c r="E65" s="7" t="n">
         <f aca="false">IF($C65="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F65" s="15" t="n">
+      <c r="F65" s="7" t="n">
         <f aca="false">IF($C65="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G65" s="15" t="n">
+      <c r="G65" s="7" t="n">
         <f aca="false">IF($C65="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H65" s="7"/>
-      <c r="I65" s="15" t="n">
+      <c r="I65" s="7" t="n">
         <f aca="false">IF($C65="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J65" s="17" t="n">
+      <c r="J65" s="5" t="n">
         <f aca="false">IF($C65="Lease-koop",D65+p_SlotJr,IF($C65="Koop",D65,0))</f>
         <v>0</v>
       </c>
-      <c r="K65" s="15" t="n">
+      <c r="K65" s="7" t="n">
         <f aca="false">E65+F65+G65+H65+I65</f>
         <v>0</v>
       </c>
-      <c r="L65" s="17" t="n">
+      <c r="L65" s="5" t="n">
         <f aca="false">IF($C65="Lease-koop",p_Afschr,IF($C65="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A65,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M65" s="17" t="n">
+      <c r="M65" s="5" t="n">
         <f aca="false">IF($C65="Lease-koop",D65+p_Lev,IF(AND($C65="Koop",D65&gt;0),D65+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A65,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N65" s="15" t="n">
+      <c r="N65" s="7" t="n">
         <f aca="false">IF($C65="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D66" s="5"/>
-      <c r="E66" s="15" t="n">
+      <c r="E66" s="7" t="n">
         <f aca="false">IF($C66="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F66" s="15" t="n">
+      <c r="F66" s="7" t="n">
         <f aca="false">IF($C66="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G66" s="15" t="n">
+      <c r="G66" s="7" t="n">
         <f aca="false">IF($C66="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H66" s="7"/>
-      <c r="I66" s="15" t="n">
+      <c r="I66" s="7" t="n">
         <f aca="false">IF($C66="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J66" s="17" t="n">
+      <c r="J66" s="5" t="n">
         <f aca="false">IF($C66="Lease-koop",D66+p_SlotJr,IF($C66="Koop",D66,0))</f>
         <v>0</v>
       </c>
-      <c r="K66" s="15" t="n">
+      <c r="K66" s="7" t="n">
         <f aca="false">E66+F66+G66+H66+I66</f>
         <v>0</v>
       </c>
-      <c r="L66" s="17" t="n">
+      <c r="L66" s="5" t="n">
         <f aca="false">IF($C66="Lease-koop",p_Afschr,IF($C66="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A66,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M66" s="17" t="n">
+      <c r="M66" s="5" t="n">
         <f aca="false">IF($C66="Lease-koop",D66+p_Lev,IF(AND($C66="Koop",D66&gt;0),D66+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A66,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N66" s="15" t="n">
+      <c r="N66" s="7" t="n">
         <f aca="false">IF($C66="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D67" s="5"/>
-      <c r="E67" s="15" t="n">
+      <c r="E67" s="7" t="n">
         <f aca="false">IF($C67="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F67" s="15" t="n">
+      <c r="F67" s="7" t="n">
         <f aca="false">IF($C67="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G67" s="15" t="n">
+      <c r="G67" s="7" t="n">
         <f aca="false">IF($C67="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H67" s="7"/>
-      <c r="I67" s="15" t="n">
+      <c r="I67" s="7" t="n">
         <f aca="false">IF($C67="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J67" s="17" t="n">
+      <c r="J67" s="5" t="n">
         <f aca="false">IF($C67="Lease-koop",D67+p_SlotJr,IF($C67="Koop",D67,0))</f>
         <v>0</v>
       </c>
-      <c r="K67" s="15" t="n">
+      <c r="K67" s="7" t="n">
         <f aca="false">E67+F67+G67+H67+I67</f>
         <v>0</v>
       </c>
-      <c r="L67" s="17" t="n">
+      <c r="L67" s="5" t="n">
         <f aca="false">IF($C67="Lease-koop",p_Afschr,IF($C67="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A67,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M67" s="17" t="n">
+      <c r="M67" s="5" t="n">
         <f aca="false">IF($C67="Lease-koop",D67+p_Lev,IF(AND($C67="Koop",D67&gt;0),D67+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A67,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N67" s="15" t="n">
+      <c r="N67" s="7" t="n">
         <f aca="false">IF($C67="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D68" s="5"/>
-      <c r="E68" s="15" t="n">
+      <c r="E68" s="7" t="n">
         <f aca="false">IF($C68="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F68" s="15" t="n">
+      <c r="F68" s="7" t="n">
         <f aca="false">IF($C68="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G68" s="15" t="n">
+      <c r="G68" s="7" t="n">
         <f aca="false">IF($C68="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H68" s="7"/>
-      <c r="I68" s="15" t="n">
+      <c r="I68" s="7" t="n">
         <f aca="false">IF($C68="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J68" s="17" t="n">
+      <c r="J68" s="5" t="n">
         <f aca="false">IF($C68="Lease-koop",D68+p_SlotJr,IF($C68="Koop",D68,0))</f>
         <v>0</v>
       </c>
-      <c r="K68" s="15" t="n">
+      <c r="K68" s="7" t="n">
         <f aca="false">E68+F68+G68+H68+I68</f>
         <v>0</v>
       </c>
-      <c r="L68" s="17" t="n">
+      <c r="L68" s="5" t="n">
         <f aca="false">IF($C68="Lease-koop",p_Afschr,IF($C68="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A68,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M68" s="17" t="n">
+      <c r="M68" s="5" t="n">
         <f aca="false">IF($C68="Lease-koop",D68+p_Lev,IF(AND($C68="Koop",D68&gt;0),D68+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A68,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N68" s="15" t="n">
+      <c r="N68" s="7" t="n">
         <f aca="false">IF($C68="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D69" s="5"/>
-      <c r="E69" s="15" t="n">
+      <c r="E69" s="7" t="n">
         <f aca="false">IF($C69="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F69" s="15" t="n">
+      <c r="F69" s="7" t="n">
         <f aca="false">IF($C69="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G69" s="15" t="n">
+      <c r="G69" s="7" t="n">
         <f aca="false">IF($C69="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H69" s="7"/>
-      <c r="I69" s="15" t="n">
+      <c r="I69" s="7" t="n">
         <f aca="false">IF($C69="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J69" s="17" t="n">
+      <c r="J69" s="5" t="n">
         <f aca="false">IF($C69="Lease-koop",D69+p_SlotJr,IF($C69="Koop",D69,0))</f>
         <v>0</v>
       </c>
-      <c r="K69" s="15" t="n">
+      <c r="K69" s="7" t="n">
         <f aca="false">E69+F69+G69+H69+I69</f>
         <v>0</v>
       </c>
-      <c r="L69" s="17" t="n">
+      <c r="L69" s="5" t="n">
         <f aca="false">IF($C69="Lease-koop",p_Afschr,IF($C69="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A69,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M69" s="17" t="n">
+      <c r="M69" s="5" t="n">
         <f aca="false">IF($C69="Lease-koop",D69+p_Lev,IF(AND($C69="Koop",D69&gt;0),D69+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A69,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N69" s="15" t="n">
+      <c r="N69" s="7" t="n">
         <f aca="false">IF($C69="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D70" s="5"/>
-      <c r="E70" s="15" t="n">
+      <c r="E70" s="7" t="n">
         <f aca="false">IF($C70="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F70" s="15" t="n">
+      <c r="F70" s="7" t="n">
         <f aca="false">IF($C70="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G70" s="15" t="n">
+      <c r="G70" s="7" t="n">
         <f aca="false">IF($C70="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H70" s="7"/>
-      <c r="I70" s="15" t="n">
+      <c r="I70" s="7" t="n">
         <f aca="false">IF($C70="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J70" s="17" t="n">
+      <c r="J70" s="5" t="n">
         <f aca="false">IF($C70="Lease-koop",D70+p_SlotJr,IF($C70="Koop",D70,0))</f>
         <v>0</v>
       </c>
-      <c r="K70" s="15" t="n">
+      <c r="K70" s="7" t="n">
         <f aca="false">E70+F70+G70+H70+I70</f>
         <v>0</v>
       </c>
-      <c r="L70" s="17" t="n">
+      <c r="L70" s="5" t="n">
         <f aca="false">IF($C70="Lease-koop",p_Afschr,IF($C70="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A70,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M70" s="17" t="n">
+      <c r="M70" s="5" t="n">
         <f aca="false">IF($C70="Lease-koop",D70+p_Lev,IF(AND($C70="Koop",D70&gt;0),D70+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A70,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N70" s="15" t="n">
+      <c r="N70" s="7" t="n">
         <f aca="false">IF($C70="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D71" s="5"/>
-      <c r="E71" s="15" t="n">
+      <c r="E71" s="7" t="n">
         <f aca="false">IF($C71="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F71" s="15" t="n">
+      <c r="F71" s="7" t="n">
         <f aca="false">IF($C71="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G71" s="15" t="n">
+      <c r="G71" s="7" t="n">
         <f aca="false">IF($C71="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H71" s="7"/>
-      <c r="I71" s="15" t="n">
+      <c r="I71" s="7" t="n">
         <f aca="false">IF($C71="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J71" s="17" t="n">
+      <c r="J71" s="5" t="n">
         <f aca="false">IF($C71="Lease-koop",D71+p_SlotJr,IF($C71="Koop",D71,0))</f>
         <v>0</v>
       </c>
-      <c r="K71" s="15" t="n">
+      <c r="K71" s="7" t="n">
         <f aca="false">E71+F71+G71+H71+I71</f>
         <v>0</v>
       </c>
-      <c r="L71" s="17" t="n">
+      <c r="L71" s="5" t="n">
         <f aca="false">IF($C71="Lease-koop",p_Afschr,IF($C71="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A71,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M71" s="17" t="n">
+      <c r="M71" s="5" t="n">
         <f aca="false">IF($C71="Lease-koop",D71+p_Lev,IF(AND($C71="Koop",D71&gt;0),D71+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A71,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N71" s="15" t="n">
+      <c r="N71" s="7" t="n">
         <f aca="false">IF($C71="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D72" s="5"/>
-      <c r="E72" s="15" t="n">
+      <c r="E72" s="7" t="n">
         <f aca="false">IF($C72="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F72" s="15" t="n">
+      <c r="F72" s="7" t="n">
         <f aca="false">IF($C72="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G72" s="15" t="n">
+      <c r="G72" s="7" t="n">
         <f aca="false">IF($C72="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H72" s="7"/>
-      <c r="I72" s="15" t="n">
+      <c r="I72" s="7" t="n">
         <f aca="false">IF($C72="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J72" s="17" t="n">
+      <c r="J72" s="5" t="n">
         <f aca="false">IF($C72="Lease-koop",D72+p_SlotJr,IF($C72="Koop",D72,0))</f>
         <v>0</v>
       </c>
-      <c r="K72" s="15" t="n">
+      <c r="K72" s="7" t="n">
         <f aca="false">E72+F72+G72+H72+I72</f>
         <v>0</v>
       </c>
-      <c r="L72" s="17" t="n">
+      <c r="L72" s="5" t="n">
         <f aca="false">IF($C72="Lease-koop",p_Afschr,IF($C72="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A72,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M72" s="17" t="n">
+      <c r="M72" s="5" t="n">
         <f aca="false">IF($C72="Lease-koop",D72+p_Lev,IF(AND($C72="Koop",D72&gt;0),D72+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A72,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N72" s="15" t="n">
+      <c r="N72" s="7" t="n">
         <f aca="false">IF($C72="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D73" s="5"/>
-      <c r="E73" s="15" t="n">
+      <c r="E73" s="7" t="n">
         <f aca="false">IF($C73="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F73" s="15" t="n">
+      <c r="F73" s="7" t="n">
         <f aca="false">IF($C73="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G73" s="15" t="n">
+      <c r="G73" s="7" t="n">
         <f aca="false">IF($C73="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H73" s="7"/>
-      <c r="I73" s="15" t="n">
+      <c r="I73" s="7" t="n">
         <f aca="false">IF($C73="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J73" s="17" t="n">
+      <c r="J73" s="5" t="n">
         <f aca="false">IF($C73="Lease-koop",D73+p_SlotJr,IF($C73="Koop",D73,0))</f>
         <v>0</v>
       </c>
-      <c r="K73" s="15" t="n">
+      <c r="K73" s="7" t="n">
         <f aca="false">E73+F73+G73+H73+I73</f>
         <v>0</v>
       </c>
-      <c r="L73" s="17" t="n">
+      <c r="L73" s="5" t="n">
         <f aca="false">IF($C73="Lease-koop",p_Afschr,IF($C73="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A73,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M73" s="17" t="n">
+      <c r="M73" s="5" t="n">
         <f aca="false">IF($C73="Lease-koop",D73+p_Lev,IF(AND($C73="Koop",D73&gt;0),D73+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A73,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N73" s="15" t="n">
+      <c r="N73" s="7" t="n">
         <f aca="false">IF($C73="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D74" s="5"/>
-      <c r="E74" s="15" t="n">
+      <c r="E74" s="7" t="n">
         <f aca="false">IF($C74="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F74" s="15" t="n">
+      <c r="F74" s="7" t="n">
         <f aca="false">IF($C74="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G74" s="15" t="n">
+      <c r="G74" s="7" t="n">
         <f aca="false">IF($C74="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H74" s="7"/>
-      <c r="I74" s="15" t="n">
+      <c r="I74" s="7" t="n">
         <f aca="false">IF($C74="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J74" s="17" t="n">
+      <c r="J74" s="5" t="n">
         <f aca="false">IF($C74="Lease-koop",D74+p_SlotJr,IF($C74="Koop",D74,0))</f>
         <v>0</v>
       </c>
-      <c r="K74" s="15" t="n">
+      <c r="K74" s="7" t="n">
         <f aca="false">E74+F74+G74+H74+I74</f>
         <v>0</v>
       </c>
-      <c r="L74" s="17" t="n">
+      <c r="L74" s="5" t="n">
         <f aca="false">IF($C74="Lease-koop",p_Afschr,IF($C74="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A74,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M74" s="17" t="n">
+      <c r="M74" s="5" t="n">
         <f aca="false">IF($C74="Lease-koop",D74+p_Lev,IF(AND($C74="Koop",D74&gt;0),D74+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A74,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N74" s="15" t="n">
+      <c r="N74" s="7" t="n">
         <f aca="false">IF($C74="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D75" s="5"/>
-      <c r="E75" s="15" t="n">
+      <c r="E75" s="7" t="n">
         <f aca="false">IF($C75="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F75" s="15" t="n">
+      <c r="F75" s="7" t="n">
         <f aca="false">IF($C75="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G75" s="15" t="n">
+      <c r="G75" s="7" t="n">
         <f aca="false">IF($C75="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H75" s="7"/>
-      <c r="I75" s="15" t="n">
+      <c r="I75" s="7" t="n">
         <f aca="false">IF($C75="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J75" s="17" t="n">
+      <c r="J75" s="5" t="n">
         <f aca="false">IF($C75="Lease-koop",D75+p_SlotJr,IF($C75="Koop",D75,0))</f>
         <v>0</v>
       </c>
-      <c r="K75" s="15" t="n">
+      <c r="K75" s="7" t="n">
         <f aca="false">E75+F75+G75+H75+I75</f>
         <v>0</v>
       </c>
-      <c r="L75" s="17" t="n">
+      <c r="L75" s="5" t="n">
         <f aca="false">IF($C75="Lease-koop",p_Afschr,IF($C75="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A75,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M75" s="17" t="n">
+      <c r="M75" s="5" t="n">
         <f aca="false">IF($C75="Lease-koop",D75+p_Lev,IF(AND($C75="Koop",D75&gt;0),D75+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A75,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N75" s="15" t="n">
+      <c r="N75" s="7" t="n">
         <f aca="false">IF($C75="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D76" s="5"/>
-      <c r="E76" s="15" t="n">
+      <c r="E76" s="7" t="n">
         <f aca="false">IF($C76="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F76" s="15" t="n">
+      <c r="F76" s="7" t="n">
         <f aca="false">IF($C76="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G76" s="15" t="n">
+      <c r="G76" s="7" t="n">
         <f aca="false">IF($C76="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H76" s="7"/>
-      <c r="I76" s="15" t="n">
+      <c r="I76" s="7" t="n">
         <f aca="false">IF($C76="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J76" s="17" t="n">
+      <c r="J76" s="5" t="n">
         <f aca="false">IF($C76="Lease-koop",D76+p_SlotJr,IF($C76="Koop",D76,0))</f>
         <v>0</v>
       </c>
-      <c r="K76" s="15" t="n">
+      <c r="K76" s="7" t="n">
         <f aca="false">E76+F76+G76+H76+I76</f>
         <v>0</v>
       </c>
-      <c r="L76" s="17" t="n">
+      <c r="L76" s="5" t="n">
         <f aca="false">IF($C76="Lease-koop",p_Afschr,IF($C76="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A76,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M76" s="17" t="n">
+      <c r="M76" s="5" t="n">
         <f aca="false">IF($C76="Lease-koop",D76+p_Lev,IF(AND($C76="Koop",D76&gt;0),D76+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A76,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N76" s="15" t="n">
+      <c r="N76" s="7" t="n">
         <f aca="false">IF($C76="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D77" s="5"/>
-      <c r="E77" s="15" t="n">
+      <c r="E77" s="7" t="n">
         <f aca="false">IF($C77="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F77" s="15" t="n">
+      <c r="F77" s="7" t="n">
         <f aca="false">IF($C77="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G77" s="15" t="n">
+      <c r="G77" s="7" t="n">
         <f aca="false">IF($C77="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H77" s="7"/>
-      <c r="I77" s="15" t="n">
+      <c r="I77" s="7" t="n">
         <f aca="false">IF($C77="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J77" s="17" t="n">
+      <c r="J77" s="5" t="n">
         <f aca="false">IF($C77="Lease-koop",D77+p_SlotJr,IF($C77="Koop",D77,0))</f>
         <v>0</v>
       </c>
-      <c r="K77" s="15" t="n">
+      <c r="K77" s="7" t="n">
         <f aca="false">E77+F77+G77+H77+I77</f>
         <v>0</v>
       </c>
-      <c r="L77" s="17" t="n">
+      <c r="L77" s="5" t="n">
         <f aca="false">IF($C77="Lease-koop",p_Afschr,IF($C77="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A77,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M77" s="17" t="n">
+      <c r="M77" s="5" t="n">
         <f aca="false">IF($C77="Lease-koop",D77+p_Lev,IF(AND($C77="Koop",D77&gt;0),D77+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A77,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N77" s="15" t="n">
+      <c r="N77" s="7" t="n">
         <f aca="false">IF($C77="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D78" s="5"/>
-      <c r="E78" s="15" t="n">
+      <c r="E78" s="7" t="n">
         <f aca="false">IF($C78="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F78" s="15" t="n">
+      <c r="F78" s="7" t="n">
         <f aca="false">IF($C78="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G78" s="15" t="n">
+      <c r="G78" s="7" t="n">
         <f aca="false">IF($C78="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H78" s="7"/>
-      <c r="I78" s="15" t="n">
+      <c r="I78" s="7" t="n">
         <f aca="false">IF($C78="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J78" s="17" t="n">
+      <c r="J78" s="5" t="n">
         <f aca="false">IF($C78="Lease-koop",D78+p_SlotJr,IF($C78="Koop",D78,0))</f>
         <v>0</v>
       </c>
-      <c r="K78" s="15" t="n">
+      <c r="K78" s="7" t="n">
         <f aca="false">E78+F78+G78+H78+I78</f>
         <v>0</v>
       </c>
-      <c r="L78" s="17" t="n">
+      <c r="L78" s="5" t="n">
         <f aca="false">IF($C78="Lease-koop",p_Afschr,IF($C78="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A78,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M78" s="17" t="n">
+      <c r="M78" s="5" t="n">
         <f aca="false">IF($C78="Lease-koop",D78+p_Lev,IF(AND($C78="Koop",D78&gt;0),D78+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A78,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N78" s="15" t="n">
+      <c r="N78" s="7" t="n">
         <f aca="false">IF($C78="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D79" s="5"/>
-      <c r="E79" s="15" t="n">
+      <c r="E79" s="7" t="n">
         <f aca="false">IF($C79="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F79" s="15" t="n">
+      <c r="F79" s="7" t="n">
         <f aca="false">IF($C79="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G79" s="15" t="n">
+      <c r="G79" s="7" t="n">
         <f aca="false">IF($C79="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H79" s="7"/>
-      <c r="I79" s="15" t="n">
+      <c r="I79" s="7" t="n">
         <f aca="false">IF($C79="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J79" s="17" t="n">
+      <c r="J79" s="5" t="n">
         <f aca="false">IF($C79="Lease-koop",D79+p_SlotJr,IF($C79="Koop",D79,0))</f>
         <v>0</v>
       </c>
-      <c r="K79" s="15" t="n">
+      <c r="K79" s="7" t="n">
         <f aca="false">E79+F79+G79+H79+I79</f>
         <v>0</v>
       </c>
-      <c r="L79" s="17" t="n">
+      <c r="L79" s="5" t="n">
         <f aca="false">IF($C79="Lease-koop",p_Afschr,IF($C79="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A79,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M79" s="17" t="n">
+      <c r="M79" s="5" t="n">
         <f aca="false">IF($C79="Lease-koop",D79+p_Lev,IF(AND($C79="Koop",D79&gt;0),D79+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A79,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N79" s="15" t="n">
+      <c r="N79" s="7" t="n">
         <f aca="false">IF($C79="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D80" s="5"/>
-      <c r="E80" s="15" t="n">
+      <c r="E80" s="7" t="n">
         <f aca="false">IF($C80="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F80" s="15" t="n">
+      <c r="F80" s="7" t="n">
         <f aca="false">IF($C80="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G80" s="15" t="n">
+      <c r="G80" s="7" t="n">
         <f aca="false">IF($C80="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H80" s="7"/>
-      <c r="I80" s="15" t="n">
+      <c r="I80" s="7" t="n">
         <f aca="false">IF($C80="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J80" s="17" t="n">
+      <c r="J80" s="5" t="n">
         <f aca="false">IF($C80="Lease-koop",D80+p_SlotJr,IF($C80="Koop",D80,0))</f>
         <v>0</v>
       </c>
-      <c r="K80" s="15" t="n">
+      <c r="K80" s="7" t="n">
         <f aca="false">E80+F80+G80+H80+I80</f>
         <v>0</v>
       </c>
-      <c r="L80" s="17" t="n">
+      <c r="L80" s="5" t="n">
         <f aca="false">IF($C80="Lease-koop",p_Afschr,IF($C80="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A80,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M80" s="17" t="n">
+      <c r="M80" s="5" t="n">
         <f aca="false">IF($C80="Lease-koop",D80+p_Lev,IF(AND($C80="Koop",D80&gt;0),D80+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A80,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N80" s="15" t="n">
+      <c r="N80" s="7" t="n">
         <f aca="false">IF($C80="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D81" s="5"/>
-      <c r="E81" s="15" t="n">
+      <c r="E81" s="7" t="n">
         <f aca="false">IF($C81="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F81" s="15" t="n">
+      <c r="F81" s="7" t="n">
         <f aca="false">IF($C81="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G81" s="15" t="n">
+      <c r="G81" s="7" t="n">
         <f aca="false">IF($C81="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H81" s="7"/>
-      <c r="I81" s="15" t="n">
+      <c r="I81" s="7" t="n">
         <f aca="false">IF($C81="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J81" s="17" t="n">
+      <c r="J81" s="5" t="n">
         <f aca="false">IF($C81="Lease-koop",D81+p_SlotJr,IF($C81="Koop",D81,0))</f>
         <v>0</v>
       </c>
-      <c r="K81" s="15" t="n">
+      <c r="K81" s="7" t="n">
         <f aca="false">E81+F81+G81+H81+I81</f>
         <v>0</v>
       </c>
-      <c r="L81" s="17" t="n">
+      <c r="L81" s="5" t="n">
         <f aca="false">IF($C81="Lease-koop",p_Afschr,IF($C81="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A81,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M81" s="17" t="n">
+      <c r="M81" s="5" t="n">
         <f aca="false">IF($C81="Lease-koop",D81+p_Lev,IF(AND($C81="Koop",D81&gt;0),D81+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A81,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N81" s="15" t="n">
+      <c r="N81" s="7" t="n">
         <f aca="false">IF($C81="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D82" s="5"/>
-      <c r="E82" s="15" t="n">
+      <c r="E82" s="7" t="n">
         <f aca="false">IF($C82="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F82" s="15" t="n">
+      <c r="F82" s="7" t="n">
         <f aca="false">IF($C82="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G82" s="15" t="n">
+      <c r="G82" s="7" t="n">
         <f aca="false">IF($C82="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H82" s="7"/>
-      <c r="I82" s="15" t="n">
+      <c r="I82" s="7" t="n">
         <f aca="false">IF($C82="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J82" s="17" t="n">
+      <c r="J82" s="5" t="n">
         <f aca="false">IF($C82="Lease-koop",D82+p_SlotJr,IF($C82="Koop",D82,0))</f>
         <v>0</v>
       </c>
-      <c r="K82" s="15" t="n">
+      <c r="K82" s="7" t="n">
         <f aca="false">E82+F82+G82+H82+I82</f>
         <v>0</v>
       </c>
-      <c r="L82" s="17" t="n">
+      <c r="L82" s="5" t="n">
         <f aca="false">IF($C82="Lease-koop",p_Afschr,IF($C82="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A82,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M82" s="17" t="n">
+      <c r="M82" s="5" t="n">
         <f aca="false">IF($C82="Lease-koop",D82+p_Lev,IF(AND($C82="Koop",D82&gt;0),D82+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A82,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N82" s="15" t="n">
+      <c r="N82" s="7" t="n">
         <f aca="false">IF($C82="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D83" s="5"/>
-      <c r="E83" s="15" t="n">
+      <c r="E83" s="7" t="n">
         <f aca="false">IF($C83="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F83" s="15" t="n">
+      <c r="F83" s="7" t="n">
         <f aca="false">IF($C83="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G83" s="15" t="n">
+      <c r="G83" s="7" t="n">
         <f aca="false">IF($C83="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H83" s="7"/>
-      <c r="I83" s="15" t="n">
+      <c r="I83" s="7" t="n">
         <f aca="false">IF($C83="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J83" s="17" t="n">
+      <c r="J83" s="5" t="n">
         <f aca="false">IF($C83="Lease-koop",D83+p_SlotJr,IF($C83="Koop",D83,0))</f>
         <v>0</v>
       </c>
-      <c r="K83" s="15" t="n">
+      <c r="K83" s="7" t="n">
         <f aca="false">E83+F83+G83+H83+I83</f>
         <v>0</v>
       </c>
-      <c r="L83" s="17" t="n">
+      <c r="L83" s="5" t="n">
         <f aca="false">IF($C83="Lease-koop",p_Afschr,IF($C83="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A83,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M83" s="17" t="n">
+      <c r="M83" s="5" t="n">
         <f aca="false">IF($C83="Lease-koop",D83+p_Lev,IF(AND($C83="Koop",D83&gt;0),D83+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A83,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N83" s="15" t="n">
+      <c r="N83" s="7" t="n">
         <f aca="false">IF($C83="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D84" s="5"/>
-      <c r="E84" s="15" t="n">
+      <c r="E84" s="7" t="n">
         <f aca="false">IF($C84="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F84" s="15" t="n">
+      <c r="F84" s="7" t="n">
         <f aca="false">IF($C84="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G84" s="15" t="n">
+      <c r="G84" s="7" t="n">
         <f aca="false">IF($C84="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H84" s="7"/>
-      <c r="I84" s="15" t="n">
+      <c r="I84" s="7" t="n">
         <f aca="false">IF($C84="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J84" s="17" t="n">
+      <c r="J84" s="5" t="n">
         <f aca="false">IF($C84="Lease-koop",D84+p_SlotJr,IF($C84="Koop",D84,0))</f>
         <v>0</v>
       </c>
-      <c r="K84" s="15" t="n">
+      <c r="K84" s="7" t="n">
         <f aca="false">E84+F84+G84+H84+I84</f>
         <v>0</v>
       </c>
-      <c r="L84" s="17" t="n">
+      <c r="L84" s="5" t="n">
         <f aca="false">IF($C84="Lease-koop",p_Afschr,IF($C84="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A84,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M84" s="17" t="n">
+      <c r="M84" s="5" t="n">
         <f aca="false">IF($C84="Lease-koop",D84+p_Lev,IF(AND($C84="Koop",D84&gt;0),D84+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A84,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N84" s="15" t="n">
+      <c r="N84" s="7" t="n">
         <f aca="false">IF($C84="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D85" s="5"/>
-      <c r="E85" s="15" t="n">
+      <c r="E85" s="7" t="n">
         <f aca="false">IF($C85="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F85" s="15" t="n">
+      <c r="F85" s="7" t="n">
         <f aca="false">IF($C85="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G85" s="15" t="n">
+      <c r="G85" s="7" t="n">
         <f aca="false">IF($C85="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H85" s="7"/>
-      <c r="I85" s="15" t="n">
+      <c r="I85" s="7" t="n">
         <f aca="false">IF($C85="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J85" s="17" t="n">
+      <c r="J85" s="5" t="n">
         <f aca="false">IF($C85="Lease-koop",D85+p_SlotJr,IF($C85="Koop",D85,0))</f>
         <v>0</v>
       </c>
-      <c r="K85" s="15" t="n">
+      <c r="K85" s="7" t="n">
         <f aca="false">E85+F85+G85+H85+I85</f>
         <v>0</v>
       </c>
-      <c r="L85" s="17" t="n">
+      <c r="L85" s="5" t="n">
         <f aca="false">IF($C85="Lease-koop",p_Afschr,IF($C85="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A85,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M85" s="17" t="n">
+      <c r="M85" s="5" t="n">
         <f aca="false">IF($C85="Lease-koop",D85+p_Lev,IF(AND($C85="Koop",D85&gt;0),D85+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A85,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N85" s="15" t="n">
+      <c r="N85" s="7" t="n">
         <f aca="false">IF($C85="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D86" s="5"/>
-      <c r="E86" s="15" t="n">
+      <c r="E86" s="7" t="n">
         <f aca="false">IF($C86="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F86" s="15" t="n">
+      <c r="F86" s="7" t="n">
         <f aca="false">IF($C86="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G86" s="15" t="n">
+      <c r="G86" s="7" t="n">
         <f aca="false">IF($C86="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H86" s="7"/>
-      <c r="I86" s="15" t="n">
+      <c r="I86" s="7" t="n">
         <f aca="false">IF($C86="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J86" s="17" t="n">
+      <c r="J86" s="5" t="n">
         <f aca="false">IF($C86="Lease-koop",D86+p_SlotJr,IF($C86="Koop",D86,0))</f>
         <v>0</v>
       </c>
-      <c r="K86" s="15" t="n">
+      <c r="K86" s="7" t="n">
         <f aca="false">E86+F86+G86+H86+I86</f>
         <v>0</v>
       </c>
-      <c r="L86" s="17" t="n">
+      <c r="L86" s="5" t="n">
         <f aca="false">IF($C86="Lease-koop",p_Afschr,IF($C86="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A86,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M86" s="17" t="n">
+      <c r="M86" s="5" t="n">
         <f aca="false">IF($C86="Lease-koop",D86+p_Lev,IF(AND($C86="Koop",D86&gt;0),D86+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A86,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N86" s="15" t="n">
+      <c r="N86" s="7" t="n">
         <f aca="false">IF($C86="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D87" s="5"/>
-      <c r="E87" s="15" t="n">
+      <c r="E87" s="7" t="n">
         <f aca="false">IF($C87="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F87" s="15" t="n">
+      <c r="F87" s="7" t="n">
         <f aca="false">IF($C87="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G87" s="15" t="n">
+      <c r="G87" s="7" t="n">
         <f aca="false">IF($C87="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H87" s="7"/>
-      <c r="I87" s="15" t="n">
+      <c r="I87" s="7" t="n">
         <f aca="false">IF($C87="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J87" s="17" t="n">
+      <c r="J87" s="5" t="n">
         <f aca="false">IF($C87="Lease-koop",D87+p_SlotJr,IF($C87="Koop",D87,0))</f>
         <v>0</v>
       </c>
-      <c r="K87" s="15" t="n">
+      <c r="K87" s="7" t="n">
         <f aca="false">E87+F87+G87+H87+I87</f>
         <v>0</v>
       </c>
-      <c r="L87" s="17" t="n">
+      <c r="L87" s="5" t="n">
         <f aca="false">IF($C87="Lease-koop",p_Afschr,IF($C87="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A87,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M87" s="17" t="n">
+      <c r="M87" s="5" t="n">
         <f aca="false">IF($C87="Lease-koop",D87+p_Lev,IF(AND($C87="Koop",D87&gt;0),D87+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A87,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N87" s="15" t="n">
+      <c r="N87" s="7" t="n">
         <f aca="false">IF($C87="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D88" s="5"/>
-      <c r="E88" s="15" t="n">
+      <c r="E88" s="7" t="n">
         <f aca="false">IF($C88="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F88" s="15" t="n">
+      <c r="F88" s="7" t="n">
         <f aca="false">IF($C88="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G88" s="15" t="n">
+      <c r="G88" s="7" t="n">
         <f aca="false">IF($C88="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H88" s="7"/>
-      <c r="I88" s="15" t="n">
+      <c r="I88" s="7" t="n">
         <f aca="false">IF($C88="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J88" s="17" t="n">
+      <c r="J88" s="5" t="n">
         <f aca="false">IF($C88="Lease-koop",D88+p_SlotJr,IF($C88="Koop",D88,0))</f>
         <v>0</v>
       </c>
-      <c r="K88" s="15" t="n">
+      <c r="K88" s="7" t="n">
         <f aca="false">E88+F88+G88+H88+I88</f>
         <v>0</v>
       </c>
-      <c r="L88" s="17" t="n">
+      <c r="L88" s="5" t="n">
         <f aca="false">IF($C88="Lease-koop",p_Afschr,IF($C88="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A88,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M88" s="17" t="n">
+      <c r="M88" s="5" t="n">
         <f aca="false">IF($C88="Lease-koop",D88+p_Lev,IF(AND($C88="Koop",D88&gt;0),D88+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A88,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N88" s="15" t="n">
+      <c r="N88" s="7" t="n">
         <f aca="false">IF($C88="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D89" s="5"/>
-      <c r="E89" s="15" t="n">
+      <c r="E89" s="7" t="n">
         <f aca="false">IF($C89="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F89" s="15" t="n">
+      <c r="F89" s="7" t="n">
         <f aca="false">IF($C89="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G89" s="15" t="n">
+      <c r="G89" s="7" t="n">
         <f aca="false">IF($C89="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H89" s="7"/>
-      <c r="I89" s="15" t="n">
+      <c r="I89" s="7" t="n">
         <f aca="false">IF($C89="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J89" s="17" t="n">
+      <c r="J89" s="5" t="n">
         <f aca="false">IF($C89="Lease-koop",D89+p_SlotJr,IF($C89="Koop",D89,0))</f>
         <v>0</v>
       </c>
-      <c r="K89" s="15" t="n">
+      <c r="K89" s="7" t="n">
         <f aca="false">E89+F89+G89+H89+I89</f>
         <v>0</v>
       </c>
-      <c r="L89" s="17" t="n">
+      <c r="L89" s="5" t="n">
         <f aca="false">IF($C89="Lease-koop",p_Afschr,IF($C89="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A89,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M89" s="17" t="n">
+      <c r="M89" s="5" t="n">
         <f aca="false">IF($C89="Lease-koop",D89+p_Lev,IF(AND($C89="Koop",D89&gt;0),D89+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A89,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N89" s="15" t="n">
+      <c r="N89" s="7" t="n">
         <f aca="false">IF($C89="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D90" s="5"/>
-      <c r="E90" s="15" t="n">
+      <c r="E90" s="7" t="n">
         <f aca="false">IF($C90="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F90" s="15" t="n">
+      <c r="F90" s="7" t="n">
         <f aca="false">IF($C90="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G90" s="15" t="n">
+      <c r="G90" s="7" t="n">
         <f aca="false">IF($C90="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H90" s="7"/>
-      <c r="I90" s="15" t="n">
+      <c r="I90" s="7" t="n">
         <f aca="false">IF($C90="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J90" s="17" t="n">
+      <c r="J90" s="5" t="n">
         <f aca="false">IF($C90="Lease-koop",D90+p_SlotJr,IF($C90="Koop",D90,0))</f>
         <v>0</v>
       </c>
-      <c r="K90" s="15" t="n">
+      <c r="K90" s="7" t="n">
         <f aca="false">E90+F90+G90+H90+I90</f>
         <v>0</v>
       </c>
-      <c r="L90" s="17" t="n">
+      <c r="L90" s="5" t="n">
         <f aca="false">IF($C90="Lease-koop",p_Afschr,IF($C90="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A90,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M90" s="17" t="n">
+      <c r="M90" s="5" t="n">
         <f aca="false">IF($C90="Lease-koop",D90+p_Lev,IF(AND($C90="Koop",D90&gt;0),D90+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A90,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N90" s="15" t="n">
+      <c r="N90" s="7" t="n">
         <f aca="false">IF($C90="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D91" s="5"/>
-      <c r="E91" s="15" t="n">
+      <c r="E91" s="7" t="n">
         <f aca="false">IF($C91="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F91" s="15" t="n">
+      <c r="F91" s="7" t="n">
         <f aca="false">IF($C91="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G91" s="15" t="n">
+      <c r="G91" s="7" t="n">
         <f aca="false">IF($C91="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H91" s="7"/>
-      <c r="I91" s="15" t="n">
+      <c r="I91" s="7" t="n">
         <f aca="false">IF($C91="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J91" s="17" t="n">
+      <c r="J91" s="5" t="n">
         <f aca="false">IF($C91="Lease-koop",D91+p_SlotJr,IF($C91="Koop",D91,0))</f>
         <v>0</v>
       </c>
-      <c r="K91" s="15" t="n">
+      <c r="K91" s="7" t="n">
         <f aca="false">E91+F91+G91+H91+I91</f>
         <v>0</v>
       </c>
-      <c r="L91" s="17" t="n">
+      <c r="L91" s="5" t="n">
         <f aca="false">IF($C91="Lease-koop",p_Afschr,IF($C91="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A91,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M91" s="17" t="n">
+      <c r="M91" s="5" t="n">
         <f aca="false">IF($C91="Lease-koop",D91+p_Lev,IF(AND($C91="Koop",D91&gt;0),D91+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A91,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N91" s="15" t="n">
+      <c r="N91" s="7" t="n">
         <f aca="false">IF($C91="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D92" s="5"/>
-      <c r="E92" s="15" t="n">
+      <c r="E92" s="7" t="n">
         <f aca="false">IF($C92="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F92" s="15" t="n">
+      <c r="F92" s="7" t="n">
         <f aca="false">IF($C92="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G92" s="15" t="n">
+      <c r="G92" s="7" t="n">
         <f aca="false">IF($C92="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H92" s="7"/>
-      <c r="I92" s="15" t="n">
+      <c r="I92" s="7" t="n">
         <f aca="false">IF($C92="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J92" s="17" t="n">
+      <c r="J92" s="5" t="n">
         <f aca="false">IF($C92="Lease-koop",D92+p_SlotJr,IF($C92="Koop",D92,0))</f>
         <v>0</v>
       </c>
-      <c r="K92" s="15" t="n">
+      <c r="K92" s="7" t="n">
         <f aca="false">E92+F92+G92+H92+I92</f>
         <v>0</v>
       </c>
-      <c r="L92" s="17" t="n">
+      <c r="L92" s="5" t="n">
         <f aca="false">IF($C92="Lease-koop",p_Afschr,IF($C92="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A92,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M92" s="17" t="n">
+      <c r="M92" s="5" t="n">
         <f aca="false">IF($C92="Lease-koop",D92+p_Lev,IF(AND($C92="Koop",D92&gt;0),D92+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A92,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N92" s="15" t="n">
+      <c r="N92" s="7" t="n">
         <f aca="false">IF($C92="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D93" s="5"/>
-      <c r="E93" s="15" t="n">
+      <c r="E93" s="7" t="n">
         <f aca="false">IF($C93="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F93" s="15" t="n">
+      <c r="F93" s="7" t="n">
         <f aca="false">IF($C93="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G93" s="15" t="n">
+      <c r="G93" s="7" t="n">
         <f aca="false">IF($C93="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H93" s="7"/>
-      <c r="I93" s="15" t="n">
+      <c r="I93" s="7" t="n">
         <f aca="false">IF($C93="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J93" s="17" t="n">
+      <c r="J93" s="5" t="n">
         <f aca="false">IF($C93="Lease-koop",D93+p_SlotJr,IF($C93="Koop",D93,0))</f>
         <v>0</v>
       </c>
-      <c r="K93" s="15" t="n">
+      <c r="K93" s="7" t="n">
         <f aca="false">E93+F93+G93+H93+I93</f>
         <v>0</v>
       </c>
-      <c r="L93" s="17" t="n">
+      <c r="L93" s="5" t="n">
         <f aca="false">IF($C93="Lease-koop",p_Afschr,IF($C93="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A93,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M93" s="17" t="n">
+      <c r="M93" s="5" t="n">
         <f aca="false">IF($C93="Lease-koop",D93+p_Lev,IF(AND($C93="Koop",D93&gt;0),D93+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A93,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N93" s="15" t="n">
+      <c r="N93" s="7" t="n">
         <f aca="false">IF($C93="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D94" s="5"/>
-      <c r="E94" s="15" t="n">
+      <c r="E94" s="7" t="n">
         <f aca="false">IF($C94="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F94" s="15" t="n">
+      <c r="F94" s="7" t="n">
         <f aca="false">IF($C94="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G94" s="15" t="n">
+      <c r="G94" s="7" t="n">
         <f aca="false">IF($C94="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H94" s="7"/>
-      <c r="I94" s="15" t="n">
+      <c r="I94" s="7" t="n">
         <f aca="false">IF($C94="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J94" s="17" t="n">
+      <c r="J94" s="5" t="n">
         <f aca="false">IF($C94="Lease-koop",D94+p_SlotJr,IF($C94="Koop",D94,0))</f>
         <v>0</v>
       </c>
-      <c r="K94" s="15" t="n">
+      <c r="K94" s="7" t="n">
         <f aca="false">E94+F94+G94+H94+I94</f>
         <v>0</v>
       </c>
-      <c r="L94" s="17" t="n">
+      <c r="L94" s="5" t="n">
         <f aca="false">IF($C94="Lease-koop",p_Afschr,IF($C94="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A94,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M94" s="17" t="n">
+      <c r="M94" s="5" t="n">
         <f aca="false">IF($C94="Lease-koop",D94+p_Lev,IF(AND($C94="Koop",D94&gt;0),D94+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A94,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N94" s="15" t="n">
+      <c r="N94" s="7" t="n">
         <f aca="false">IF($C94="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D95" s="5"/>
-      <c r="E95" s="15" t="n">
+      <c r="E95" s="7" t="n">
         <f aca="false">IF($C95="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F95" s="15" t="n">
+      <c r="F95" s="7" t="n">
         <f aca="false">IF($C95="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G95" s="15" t="n">
+      <c r="G95" s="7" t="n">
         <f aca="false">IF($C95="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H95" s="7"/>
-      <c r="I95" s="15" t="n">
+      <c r="I95" s="7" t="n">
         <f aca="false">IF($C95="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J95" s="17" t="n">
+      <c r="J95" s="5" t="n">
         <f aca="false">IF($C95="Lease-koop",D95+p_SlotJr,IF($C95="Koop",D95,0))</f>
         <v>0</v>
       </c>
-      <c r="K95" s="15" t="n">
+      <c r="K95" s="7" t="n">
         <f aca="false">E95+F95+G95+H95+I95</f>
         <v>0</v>
       </c>
-      <c r="L95" s="17" t="n">
+      <c r="L95" s="5" t="n">
         <f aca="false">IF($C95="Lease-koop",p_Afschr,IF($C95="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A95,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M95" s="17" t="n">
+      <c r="M95" s="5" t="n">
         <f aca="false">IF($C95="Lease-koop",D95+p_Lev,IF(AND($C95="Koop",D95&gt;0),D95+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A95,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N95" s="15" t="n">
+      <c r="N95" s="7" t="n">
         <f aca="false">IF($C95="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D96" s="5"/>
-      <c r="E96" s="15" t="n">
+      <c r="E96" s="7" t="n">
         <f aca="false">IF($C96="Lease-koop",p_Aanbet,0)</f>
         <v>0</v>
       </c>
-      <c r="F96" s="15" t="n">
+      <c r="F96" s="7" t="n">
         <f aca="false">IF($C96="Lease-koop",p_Belet,0)</f>
         <v>0</v>
       </c>
-      <c r="G96" s="15" t="n">
+      <c r="G96" s="7" t="n">
         <f aca="false">IF($C96="Lease-koop",p_Opbouw,0)</f>
         <v>0</v>
       </c>
       <c r="H96" s="7"/>
-      <c r="I96" s="15" t="n">
+      <c r="I96" s="7" t="n">
         <f aca="false">IF($C96="Lease-koop",p_Slot,0)</f>
         <v>0</v>
       </c>
-      <c r="J96" s="17" t="n">
+      <c r="J96" s="5" t="n">
         <f aca="false">IF($C96="Lease-koop",D96+p_SlotJr,IF($C96="Koop",D96,0))</f>
         <v>0</v>
       </c>
-      <c r="K96" s="15" t="n">
+      <c r="K96" s="7" t="n">
         <f aca="false">E96+F96+G96+H96+I96</f>
         <v>0</v>
       </c>
-      <c r="L96" s="17" t="n">
+      <c r="L96" s="5" t="n">
         <f aca="false">IF($C96="Lease-koop",p_Afschr,IF($C96="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A96,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="M96" s="17" t="n">
+      <c r="M96" s="5" t="n">
         <f aca="false">IF($C96="Lease-koop",D96+p_Lev,IF(AND($C96="Koop",D96&gt;0),D96+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A96,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="N96" s="15" t="n">
+      <c r="N96" s="7" t="n">
         <f aca="false">IF($C96="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
@@ -6224,7 +6178,7 @@
       </c>
       <c r="N10" s="4"/>
       <c r="O10" s="7"/>
-      <c r="P10" s="18"/>
+      <c r="P10" s="14"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
@@ -6256,7 +6210,7 @@
       </c>
       <c r="N11" s="4"/>
       <c r="O11" s="7"/>
-      <c r="P11" s="18"/>
+      <c r="P11" s="14"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
@@ -6382,7 +6336,7 @@
       </c>
       <c r="N15" s="4"/>
       <c r="O15" s="7"/>
-      <c r="P15" s="18"/>
+      <c r="P15" s="14"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Wagenpark_beheer.xlsx: V28 aanbetaling en bijkomende kosten op gemiddelde
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013EaFTgzjMaNvZvWgFM9YZf
</commit_message>
<xml_diff>
--- a/Wagenpark_beheer.xlsx
+++ b/Wagenpark_beheer.xlsx
@@ -571,14 +571,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFDDEBF7"/>
+        <bgColor rgb="FFCCFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDDEBF7"/>
-        <bgColor rgb="FFCCFFFF"/>
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -653,19 +653,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -677,11 +677,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -693,7 +693,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -733,7 +733,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
+          <fgColor rgb="FF000000"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -741,7 +741,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
+          <fgColor rgb="FFFFFF00"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -2042,8 +2042,14 @@
         <v>8</v>
       </c>
       <c r="H30" s="8"/>
-      <c r="I30" s="9"/>
-      <c r="J30" s="9"/>
+      <c r="I30" s="8" t="n">
+        <f aca="false">p_Aanbet</f>
+        <v>10000</v>
+      </c>
+      <c r="J30" s="8" t="n">
+        <f aca="false">p_Belet+p_Opbouw</f>
+        <v>12000</v>
+      </c>
       <c r="K30" s="8" t="n">
         <f aca="false">p_Slot</f>
         <v>35000</v>
@@ -2091,43 +2097,43 @@
       <c r="O31" s="8"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G33" s="10" t="s">
+      <c r="G33" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="H33" s="11" t="n">
+      <c r="H33" s="10" t="n">
         <f aca="false">SUBTOTAL(109,H5:H31)</f>
         <v>1608161</v>
       </c>
-      <c r="I33" s="11" t="n">
+      <c r="I33" s="10" t="n">
         <f aca="false">SUBTOTAL(109,I5:I31)</f>
-        <v>68310</v>
-      </c>
-      <c r="J33" s="11" t="n">
+        <v>78310</v>
+      </c>
+      <c r="J33" s="10" t="n">
         <f aca="false">SUBTOTAL(109,J5:J31)</f>
-        <v>10260</v>
-      </c>
-      <c r="K33" s="11" t="n">
+        <v>22260</v>
+      </c>
+      <c r="K33" s="10" t="n">
         <f aca="false">SUBTOTAL(109,K5:K31)</f>
         <v>245000</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="10" t="s">
+      <c r="A35" s="9" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="12" t="s">
+      <c r="A36" s="11" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="12" t="s">
+      <c r="A37" s="11" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="12" t="s">
+      <c r="A38" s="11" t="s">
         <v>92</v>
       </c>
     </row>
@@ -2178,10 +2184,10 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="9" t="s">
         <v>95</v>
       </c>
     </row>
@@ -2189,7 +2195,7 @@
       <c r="A4" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="C4" s="9" t="n">
+      <c r="C4" s="12" t="n">
         <v>10000</v>
       </c>
       <c r="F4" s="13" t="n">
@@ -2228,10 +2234,10 @@
       <c r="A5" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="12" t="n">
         <v>5000</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="9" t="s">
         <v>98</v>
       </c>
       <c r="F5" s="14" t="n">
@@ -2271,7 +2277,7 @@
       <c r="A6" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C6" s="9" t="n">
+      <c r="C6" s="12" t="n">
         <v>7000</v>
       </c>
       <c r="E6" s="4" t="s">
@@ -2314,7 +2320,7 @@
       <c r="A7" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="12" t="n">
         <v>35000</v>
       </c>
     </row>
@@ -2346,15 +2352,15 @@
       <c r="A11" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="C11" s="9" t="n">
+      <c r="C11" s="12" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J13" s="10" t="s">
+      <c r="J13" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="K13" s="11" t="n">
+      <c r="K13" s="10" t="n">
         <f aca="false">SUM($K$15:$K$51)</f>
         <v>2047208</v>
       </c>
@@ -4223,22 +4229,22 @@
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="10" t="s">
+      <c r="A53" s="9" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="12" t="s">
+      <c r="A54" s="11" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="12" t="s">
+      <c r="A55" s="11" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="12" t="s">
+      <c r="A56" s="11" t="s">
         <v>121</v>
       </c>
     </row>
@@ -4701,7 +4707,7 @@
       <c r="P15" s="19"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="11" t="s">
         <v>149</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Wagenpark_beheer.xlsx: buiten gebruik teruggebracht tot zes kolommen
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013EaFTgzjMaNvZvWgFM9YZf
</commit_message>
<xml_diff>
--- a/Wagenpark_beheer.xlsx
+++ b/Wagenpark_beheer.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="146">
   <si>
     <t xml:space="preserve">Voertuigen in gebruik</t>
   </si>
@@ -431,9 +431,6 @@
     <t xml:space="preserve">05-SZ-NF</t>
   </si>
   <si>
-    <t xml:space="preserve">John Beerens</t>
-  </si>
-  <si>
     <t xml:space="preserve">6971005/434335/M05SZNF</t>
   </si>
   <si>
@@ -443,9 +440,6 @@
     <t xml:space="preserve">TFN-07-R</t>
   </si>
   <si>
-    <t xml:space="preserve">William vd Boomen</t>
-  </si>
-  <si>
     <t xml:space="preserve">6210601/434335</t>
   </si>
   <si>
@@ -455,9 +449,6 @@
     <t xml:space="preserve">VG-683-L</t>
   </si>
   <si>
-    <t xml:space="preserve">Ruud Liebregts</t>
-  </si>
-  <si>
     <t xml:space="preserve">V97</t>
   </si>
   <si>
@@ -474,9 +465,6 @@
   </si>
   <si>
     <t xml:space="preserve">VG-094-L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Willie v Dal</t>
   </si>
   <si>
     <t xml:space="preserve">6210102/434335</t>
@@ -815,25 +803,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblBuitenGebruik" displayName="tblBuitenGebruik" ref="A4:P15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A4:P15"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblBuitenGebruik" displayName="tblBuitenGebruik" ref="A4:F15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A4:F15"/>
+  <tableColumns count="6">
     <tableColumn id="1" name="V-nummer"/>
     <tableColumn id="2" name="Kredietnr."/>
     <tableColumn id="3" name="Kenteken"/>
-    <tableColumn id="4" name="Aanschafwijze"/>
-    <tableColumn id="5" name="Berijder"/>
-    <tableColumn id="6" name="Aanschafjaar"/>
-    <tableColumn id="7" name="Levensduur"/>
-    <tableColumn id="8" name="Aanschafkosten (werkelijk)"/>
-    <tableColumn id="9" name="Aanbetaling (raming)"/>
-    <tableColumn id="10" name="Bijkomende kosten (raming)"/>
-    <tableColumn id="11" name="Slotbetaling (raming)"/>
-    <tableColumn id="12" name="Te activeren in jaar"/>
-    <tableColumn id="13" name="Activakaart"/>
-    <tableColumn id="14" name="Exploitatienr."/>
-    <tableColumn id="15" name="Leasesom 1 jaar"/>
-    <tableColumn id="16" name="Jaar buiten gebruik"/>
+    <tableColumn id="4" name="Aanschafjaar"/>
+    <tableColumn id="5" name="Jaar buiten gebruik"/>
+    <tableColumn id="6" name="Activakaart"/>
   </tableColumns>
 </table>
 </file>
@@ -4272,21 +4250,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="9" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4294,14 +4265,6 @@
         <v>122</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-    </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
@@ -4313,143 +4276,65 @@
         <v>4</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>6</v>
+        <v>123</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="M4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="N4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="P4" s="3" t="s">
-        <v>123</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>48</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="F5" s="6" t="n">
+      <c r="D5" s="6" t="n">
         <v>2014</v>
       </c>
-      <c r="G5" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="8"/>
-      <c r="P5" s="6" t="n">
+      <c r="E5" s="6" t="n">
         <v>2026</v>
       </c>
+      <c r="F5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>59</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="F6" s="6" t="n">
+      <c r="D6" s="6" t="n">
         <v>2018</v>
       </c>
-      <c r="G6" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
-      <c r="O6" s="8"/>
-      <c r="P6" s="6" t="n">
+      <c r="E6" s="6" t="n">
         <v>2026</v>
       </c>
+      <c r="F6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>61</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="F7" s="6" t="n">
+      <c r="D7" s="6" t="n">
         <v>2013</v>
       </c>
-      <c r="G7" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-      <c r="O7" s="8"/>
-      <c r="P7" s="6" t="n">
+      <c r="E7" s="6" t="n">
         <v>2026</v>
       </c>
+      <c r="F7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="5" t="s">
         <v>83</v>
       </c>
       <c r="B8" s="5" t="n">
@@ -4458,263 +4343,132 @@
       <c r="C8" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="F8" s="6" t="n">
+      <c r="D8" s="6" t="n">
         <v>2017</v>
       </c>
-      <c r="G8" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="H8" s="8" t="n">
-        <v>80000</v>
-      </c>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="5"/>
-      <c r="O8" s="8"/>
-      <c r="P8" s="6" t="n">
+      <c r="E8" s="6" t="n">
         <v>2026</v>
       </c>
+      <c r="F8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="5" t="s">
         <v>128</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="F9" s="6" t="n">
+      <c r="D9" s="6" t="n">
         <v>2007</v>
       </c>
-      <c r="G9" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="H9" s="8" t="n">
-        <v>65000</v>
-      </c>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="8"/>
-      <c r="L9" s="6"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-      <c r="O9" s="8"/>
-      <c r="P9" s="6" t="n">
+      <c r="E9" s="6" t="n">
         <v>2026</v>
       </c>
+      <c r="F9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="5" t="s">
         <v>130</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="D10" s="5"/>
-      <c r="E10" s="4" t="s">
+      <c r="D10" s="6" t="n">
+        <v>2006</v>
+      </c>
+      <c r="E10" s="19"/>
+      <c r="F10" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="F10" s="6" t="n">
-        <v>2006</v>
-      </c>
-      <c r="G10" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="H10" s="8" t="n">
-        <v>43000</v>
-      </c>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="5" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
         <v>133</v>
-      </c>
-      <c r="N10" s="5"/>
-      <c r="O10" s="8"/>
-      <c r="P10" s="19"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>134</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E11" s="19"/>
+      <c r="F11" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="D11" s="5"/>
-      <c r="E11" s="4" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
         <v>136</v>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>2015</v>
-      </c>
-      <c r="G11" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="H11" s="8" t="n">
-        <v>240000</v>
-      </c>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
-      <c r="K11" s="8"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="N11" s="5"/>
-      <c r="O11" s="8"/>
-      <c r="P11" s="19"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>138</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="D12" s="5"/>
-      <c r="E12" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="F12" s="6" t="n">
+        <v>137</v>
+      </c>
+      <c r="D12" s="6" t="n">
         <v>2013</v>
       </c>
-      <c r="G12" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="H12" s="8" t="n">
-        <v>65000</v>
-      </c>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
-      <c r="K12" s="8"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-      <c r="O12" s="8"/>
-      <c r="P12" s="6" t="n">
+      <c r="E12" s="6" t="n">
         <v>2027</v>
       </c>
+      <c r="F12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>141</v>
+      <c r="A13" s="5" t="s">
+        <v>138</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D13" s="5"/>
-      <c r="E13" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="F13" s="6" t="n">
+        <v>139</v>
+      </c>
+      <c r="D13" s="6" t="n">
         <v>2013</v>
       </c>
-      <c r="G13" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="H13" s="8" t="n">
-        <v>65000</v>
-      </c>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
-      <c r="K13" s="8"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
-      <c r="O13" s="8"/>
-      <c r="P13" s="6" t="n">
+      <c r="E13" s="6" t="n">
         <v>2025</v>
       </c>
+      <c r="F13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
-        <v>143</v>
+      <c r="A14" s="5" t="s">
+        <v>140</v>
       </c>
       <c r="B14" s="5"/>
       <c r="C14" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="D14" s="5"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="6" t="n">
+        <v>141</v>
+      </c>
+      <c r="D14" s="6" t="n">
         <v>2013</v>
       </c>
-      <c r="G14" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="H14" s="8" t="n">
-        <v>65000</v>
-      </c>
-      <c r="I14" s="8"/>
-      <c r="J14" s="8"/>
-      <c r="K14" s="8"/>
-      <c r="L14" s="6"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-      <c r="O14" s="8"/>
-      <c r="P14" s="6" t="n">
+      <c r="E14" s="6" t="n">
         <v>2027</v>
       </c>
+      <c r="F14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>145</v>
+      <c r="A15" s="5" t="s">
+        <v>142</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="D15" s="5"/>
-      <c r="E15" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="F15" s="6" t="n">
+        <v>143</v>
+      </c>
+      <c r="D15" s="6" t="n">
         <v>2013</v>
       </c>
-      <c r="G15" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="H15" s="8" t="n">
-        <v>72000</v>
-      </c>
-      <c r="I15" s="8"/>
-      <c r="J15" s="8"/>
-      <c r="K15" s="8"/>
-      <c r="L15" s="6"/>
-      <c r="M15" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="N15" s="5"/>
-      <c r="O15" s="8"/>
-      <c r="P15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="5" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="I3:L3"/>
-  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Wagenpark_beheer.xlsx: alle personen- en bedrijfsauto's als lease-koop
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013EaFTgzjMaNvZvWgFM9YZf
</commit_message>
<xml_diff>
--- a/Wagenpark_beheer.xlsx
+++ b/Wagenpark_beheer.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="144">
   <si>
     <t xml:space="preserve">Voertuigen in gebruik</t>
   </si>
@@ -375,12 +375,6 @@
   </si>
   <si>
     <t xml:space="preserve">Opmerking</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Begroting 2027: koop.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Begroting 2027: koop. Daarna lease-koop.</t>
   </si>
   <si>
     <t xml:space="preserve">Uitgesteld naar 2028.</t>
@@ -2220,7 +2214,7 @@
       </c>
       <c r="F5" s="14" t="n">
         <f aca="false">SUMIF($D$15:$D$51,F$4,$E$15:$E$51)+SUMIF($D$15:$D$51,F$4,$F$15:$F$51)+SUMIF($D$15:$D$51,F$4,$G$15:$G$51)+SUMIF($D$15:$D$51,F$4,$H$15:$H$51)+SUMIF($J$15:$J$51,F$4,$I$15:$I$51)</f>
-        <v>322000</v>
+        <v>190000</v>
       </c>
       <c r="G5" s="14" t="n">
         <f aca="false">SUMIF($D$15:$D$51,G$4,$E$15:$E$51)+SUMIF($D$15:$D$51,G$4,$F$15:$F$51)+SUMIF($D$15:$D$51,G$4,$G$15:$G$51)+SUMIF($D$15:$D$51,G$4,$H$15:$H$51)+SUMIF($J$15:$J$51,G$4,$I$15:$I$51)</f>
@@ -2228,7 +2222,7 @@
       </c>
       <c r="H5" s="14" t="n">
         <f aca="false">SUMIF($D$15:$D$51,H$4,$E$15:$E$51)+SUMIF($D$15:$D$51,H$4,$F$15:$F$51)+SUMIF($D$15:$D$51,H$4,$G$15:$G$51)+SUMIF($D$15:$D$51,H$4,$H$15:$H$51)+SUMIF($J$15:$J$51,H$4,$I$15:$I$51)</f>
-        <v>157000</v>
+        <v>297000</v>
       </c>
       <c r="I5" s="14" t="n">
         <f aca="false">SUMIF($D$15:$D$51,I$4,$E$15:$E$51)+SUMIF($D$15:$D$51,I$4,$F$15:$F$51)+SUMIF($D$15:$D$51,I$4,$G$15:$G$51)+SUMIF($D$15:$D$51,I$4,$H$15:$H$51)+SUMIF($J$15:$J$51,I$4,$I$15:$I$51)</f>
@@ -2263,11 +2257,11 @@
       </c>
       <c r="F6" s="8" t="n">
         <f aca="false">SUMPRODUCT(($C$15:$C$51="Lease-koop")*($D$15:$D$51&lt;=F$4)*($J$15:$J$51&gt;F$4)*$N$15:$N$51)</f>
-        <v>12000</v>
+        <v>60000</v>
       </c>
       <c r="G6" s="8" t="n">
         <f aca="false">SUMPRODUCT(($C$15:$C$51="Lease-koop")*($D$15:$D$51&lt;=G$4)*($J$15:$J$51&gt;G$4)*$N$15:$N$51)</f>
-        <v>12000</v>
+        <v>60000</v>
       </c>
       <c r="H6" s="8" t="n">
         <f aca="false">SUMPRODUCT(($C$15:$C$51="Lease-koop")*($D$15:$D$51&lt;=H$4)*($J$15:$J$51&gt;H$4)*$N$15:$N$51)</f>
@@ -2340,7 +2334,7 @@
       </c>
       <c r="K13" s="10" t="n">
         <f aca="false">SUM($K$15:$K$51)</f>
-        <v>2047208</v>
+        <v>2055208</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2396,41 +2390,39 @@
       </c>
       <c r="B15" s="16"/>
       <c r="C15" s="5" t="s">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="D15" s="6" t="n">
         <v>2027</v>
       </c>
       <c r="E15" s="17" t="n">
         <f aca="false">IF($C15="Lease-koop",p_Aanbet,0)</f>
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="F15" s="17" t="n">
         <f aca="false">IF($C15="Lease-koop",p_Belet,0)</f>
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="G15" s="17" t="n">
         <f aca="false">IF($C15="Lease-koop",p_Opbouw,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="17" t="n">
-        <v>65000</v>
-      </c>
+        <v>7000</v>
+      </c>
+      <c r="H15" s="17"/>
       <c r="I15" s="17" t="n">
         <f aca="false">IF($C15="Lease-koop",p_Slot,0)</f>
-        <v>0</v>
+        <v>35000</v>
       </c>
       <c r="J15" s="6" t="n">
         <f aca="false">IF($C15="Lease-koop",D15+p_SlotJr,IF($C15="Koop",D15,0))</f>
-        <v>2027</v>
+        <v>2029</v>
       </c>
       <c r="K15" s="17" t="n">
         <f aca="false">E15+F15+G15+H15+I15</f>
-        <v>65000</v>
+        <v>57000</v>
       </c>
       <c r="L15" s="6" t="n">
         <f aca="false">IF($C15="Lease-koop",p_Afschr,IF($C15="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A15,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M15" s="6" t="n">
         <f aca="false">IF($C15="Lease-koop",D15+p_Lev,IF(AND($C15="Koop",D15&gt;0),D15+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A15,'In gebruik'!$A:$A,0)),0),0))</f>
@@ -2438,11 +2430,9 @@
       </c>
       <c r="N15" s="17" t="n">
         <f aca="false">IF($C15="Lease-koop",p_Lease,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O15" s="4" t="s">
-        <v>114</v>
-      </c>
+        <v>12000</v>
+      </c>
+      <c r="O15" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
@@ -2450,41 +2440,39 @@
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="5" t="s">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="D16" s="6" t="n">
         <v>2027</v>
       </c>
       <c r="E16" s="17" t="n">
         <f aca="false">IF($C16="Lease-koop",p_Aanbet,0)</f>
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="F16" s="17" t="n">
         <f aca="false">IF($C16="Lease-koop",p_Belet,0)</f>
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="G16" s="17" t="n">
         <f aca="false">IF($C16="Lease-koop",p_Opbouw,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H16" s="17" t="n">
-        <v>65000</v>
-      </c>
+        <v>7000</v>
+      </c>
+      <c r="H16" s="17"/>
       <c r="I16" s="17" t="n">
         <f aca="false">IF($C16="Lease-koop",p_Slot,0)</f>
-        <v>0</v>
+        <v>35000</v>
       </c>
       <c r="J16" s="6" t="n">
         <f aca="false">IF($C16="Lease-koop",D16+p_SlotJr,IF($C16="Koop",D16,0))</f>
-        <v>2027</v>
+        <v>2029</v>
       </c>
       <c r="K16" s="17" t="n">
         <f aca="false">E16+F16+G16+H16+I16</f>
-        <v>65000</v>
+        <v>57000</v>
       </c>
       <c r="L16" s="6" t="n">
         <f aca="false">IF($C16="Lease-koop",p_Afschr,IF($C16="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A16,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M16" s="6" t="n">
         <f aca="false">IF($C16="Lease-koop",D16+p_Lev,IF(AND($C16="Koop",D16&gt;0),D16+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A16,'In gebruik'!$A:$A,0)),0),0))</f>
@@ -2492,11 +2480,9 @@
       </c>
       <c r="N16" s="17" t="n">
         <f aca="false">IF($C16="Lease-koop",p_Lease,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O16" s="4" t="s">
-        <v>114</v>
-      </c>
+        <v>12000</v>
+      </c>
+      <c r="O16" s="4"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
@@ -2606,41 +2592,39 @@
       </c>
       <c r="B19" s="16"/>
       <c r="C19" s="5" t="s">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="D19" s="6" t="n">
         <v>2027</v>
       </c>
       <c r="E19" s="17" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Aanbet,0)</f>
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="F19" s="17" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Belet,0)</f>
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="G19" s="17" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Opbouw,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H19" s="17" t="n">
-        <v>45000</v>
-      </c>
+        <v>7000</v>
+      </c>
+      <c r="H19" s="17"/>
       <c r="I19" s="17" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Slot,0)</f>
-        <v>0</v>
+        <v>35000</v>
       </c>
       <c r="J19" s="6" t="n">
         <f aca="false">IF($C19="Lease-koop",D19+p_SlotJr,IF($C19="Koop",D19,0))</f>
-        <v>2027</v>
+        <v>2029</v>
       </c>
       <c r="K19" s="17" t="n">
         <f aca="false">E19+F19+G19+H19+I19</f>
-        <v>45000</v>
+        <v>57000</v>
       </c>
       <c r="L19" s="6" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Afschr,IF($C19="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A19,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M19" s="6" t="n">
         <f aca="false">IF($C19="Lease-koop",D19+p_Lev,IF(AND($C19="Koop",D19&gt;0),D19+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A19,'In gebruik'!$A:$A,0)),0),0))</f>
@@ -2648,11 +2632,9 @@
       </c>
       <c r="N19" s="17" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Lease,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O19" s="4" t="s">
-        <v>115</v>
-      </c>
+        <v>12000</v>
+      </c>
+      <c r="O19" s="4"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
@@ -2660,41 +2642,39 @@
       </c>
       <c r="B20" s="16"/>
       <c r="C20" s="5" t="s">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="D20" s="6" t="n">
         <v>2027</v>
       </c>
       <c r="E20" s="17" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Aanbet,0)</f>
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="F20" s="17" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Belet,0)</f>
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="G20" s="17" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Opbouw,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H20" s="17" t="n">
-        <v>45000</v>
-      </c>
+        <v>7000</v>
+      </c>
+      <c r="H20" s="17"/>
       <c r="I20" s="17" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Slot,0)</f>
-        <v>0</v>
+        <v>35000</v>
       </c>
       <c r="J20" s="6" t="n">
         <f aca="false">IF($C20="Lease-koop",D20+p_SlotJr,IF($C20="Koop",D20,0))</f>
-        <v>2027</v>
+        <v>2029</v>
       </c>
       <c r="K20" s="17" t="n">
         <f aca="false">E20+F20+G20+H20+I20</f>
-        <v>45000</v>
+        <v>57000</v>
       </c>
       <c r="L20" s="6" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Afschr,IF($C20="Koop",IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A20,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M20" s="6" t="n">
         <f aca="false">IF($C20="Lease-koop",D20+p_Lev,IF(AND($C20="Koop",D20&gt;0),D20+IFERROR(INDEX('In gebruik'!$G:$G,MATCH($A20,'In gebruik'!$A:$A,0)),0),0))</f>
@@ -2702,11 +2682,9 @@
       </c>
       <c r="N20" s="17" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Lease,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O20" s="4" t="s">
-        <v>115</v>
-      </c>
+        <v>12000</v>
+      </c>
+      <c r="O20" s="4"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
@@ -2759,7 +2737,7 @@
         <v>0</v>
       </c>
       <c r="O21" s="4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2972,7 +2950,7 @@
       </c>
       <c r="B26" s="5"/>
       <c r="C26" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D26" s="6" t="n">
         <v>2032</v>
@@ -3015,7 +2993,7 @@
         <v>0</v>
       </c>
       <c r="O26" s="4" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4213,17 +4191,17 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="11" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="11" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -4262,7 +4240,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4279,7 +4257,7 @@
         <v>7</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>14</v>
@@ -4291,7 +4269,7 @@
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D5" s="6" t="n">
         <v>2014</v>
@@ -4307,7 +4285,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>2018</v>
@@ -4323,7 +4301,7 @@
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="5" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>2013</v>
@@ -4341,7 +4319,7 @@
         <v>7205049</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>2017</v>
@@ -4353,11 +4331,11 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="5" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>2007</v>
@@ -4369,43 +4347,43 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="5" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D10" s="6" t="n">
         <v>2006</v>
       </c>
       <c r="E10" s="19"/>
       <c r="F10" s="5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D11" s="6" t="n">
         <v>2015</v>
       </c>
       <c r="E11" s="19"/>
       <c r="F11" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>2013</v>
@@ -4417,11 +4395,11 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D13" s="6" t="n">
         <v>2013</v>
@@ -4433,11 +4411,11 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B14" s="5"/>
       <c r="C14" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D14" s="6" t="n">
         <v>2013</v>
@@ -4449,23 +4427,23 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="5" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D15" s="6" t="n">
         <v>2013</v>
       </c>
       <c r="E15" s="19"/>
       <c r="F15" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Wagenpark_beheer.xlsx: kolomvolgorde vervangingsinvesteringen aangepast
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013EaFTgzjMaNvZvWgFM9YZf
</commit_message>
<xml_diff>
--- a/Wagenpark_beheer.xlsx
+++ b/Wagenpark_beheer.xlsx
@@ -401,16 +401,16 @@
     <t xml:space="preserve">Einde levensduur</t>
   </si>
   <si>
+    <t xml:space="preserve">Afschrijftermijn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Activanummer</t>
+  </si>
+  <si>
     <t xml:space="preserve">Te activeren</t>
   </si>
   <si>
     <t xml:space="preserve">Jaar activering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Afschrijftermijn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Activanummer</t>
   </si>
   <si>
     <t xml:space="preserve">Opmerking</t>
@@ -2271,13 +2271,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="12" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="5" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="50"/>
   </cols>
   <sheetData>
@@ -2356,12 +2355,12 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="L13" s="2" t="s">
+      <c r="F13" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
@@ -2379,38 +2378,38 @@
       <c r="E14" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="F14" s="14" t="n">
+        <v>2027</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <f aca="false">F14+1</f>
+        <v>2028</v>
+      </c>
+      <c r="H14" s="14" t="n">
+        <f aca="false">G14+1</f>
+        <v>2029</v>
+      </c>
+      <c r="I14" s="14" t="n">
+        <f aca="false">H14+1</f>
+        <v>2030</v>
+      </c>
+      <c r="J14" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="K14" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="H14" s="3" t="s">
+      <c r="L14" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="I14" s="3" t="s">
+      <c r="M14" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="N14" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="J14" s="3" t="s">
+      <c r="O14" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="K14" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="L14" s="14" t="n">
-        <v>2027</v>
-      </c>
-      <c r="M14" s="14" t="n">
-        <f aca="false">L14+1</f>
-        <v>2028</v>
-      </c>
-      <c r="N14" s="14" t="n">
-        <f aca="false">M14+1</f>
-        <v>2029</v>
-      </c>
-      <c r="O14" s="14" t="n">
-        <f aca="false">N14+1</f>
-        <v>2030</v>
       </c>
       <c r="P14" s="3" t="s">
         <v>126</v>
@@ -2435,41 +2434,41 @@
         <v>2035</v>
       </c>
       <c r="F15" s="15" t="n">
+        <f aca="false">IF($C15="Lease-koop",IF(F$14=$D15,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M15,p_Slot,0),IF(F$14=$D15,N($L15),0))</f>
+        <v>22000</v>
+      </c>
+      <c r="G15" s="15" t="n">
+        <f aca="false">IF($C15="Lease-koop",IF(G$14=$D15,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M15,p_Slot,0),IF(G$14=$D15,N($L15),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="15" t="n">
+        <f aca="false">IF($C15="Lease-koop",IF(H$14=$D15,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M15,p_Slot,0),IF(H$14=$D15,N($L15),0))</f>
+        <v>35000</v>
+      </c>
+      <c r="I15" s="15" t="n">
+        <f aca="false">IF($C15="Lease-koop",IF(I$14=$D15,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M15,p_Slot,0),IF(I$14=$D15,N($L15),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <f aca="false">IF($C15="Lease-koop",p_Afschr,IF($C15="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A15,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>6</v>
+      </c>
+      <c r="K15" s="16"/>
+      <c r="L15" s="15" t="n">
         <f aca="false">p_Aanbet+p_Belet+p_Opbouw+p_Slot</f>
         <v>57000</v>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="M15" s="6" t="n">
         <f aca="false">IF($C15="Lease-koop",D15+p_SlotJr,IF($C15="Koop",D15,0))</f>
         <v>2029</v>
       </c>
-      <c r="H15" s="6" t="n">
-        <f aca="false">IF($C15="Lease-koop",p_Afschr,IF($C15="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A15,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>6</v>
-      </c>
-      <c r="I15" s="15" t="n">
+      <c r="N15" s="15" t="n">
         <f aca="false">IF($C15="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
-      <c r="J15" s="5" t="str">
+      <c r="O15" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A15,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K15" s="16"/>
-      <c r="L15" s="15" t="n">
-        <f aca="false">IF($C15="Lease-koop",IF(L$14=$D15,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G15,p_Slot,0),IF(L$14=$D15,N($F15),0))</f>
-        <v>22000</v>
-      </c>
-      <c r="M15" s="15" t="n">
-        <f aca="false">IF($C15="Lease-koop",IF(M$14=$D15,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G15,p_Slot,0),IF(M$14=$D15,N($F15),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N15" s="15" t="n">
-        <f aca="false">IF($C15="Lease-koop",IF(N$14=$D15,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G15,p_Slot,0),IF(N$14=$D15,N($F15),0))</f>
-        <v>35000</v>
-      </c>
-      <c r="O15" s="15" t="n">
-        <f aca="false">IF($C15="Lease-koop",IF(O$14=$D15,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G15,p_Slot,0),IF(O$14=$D15,N($F15),0))</f>
-        <v>0</v>
       </c>
       <c r="P15" s="4"/>
     </row>
@@ -2492,41 +2491,41 @@
         <v>2035</v>
       </c>
       <c r="F16" s="15" t="n">
+        <f aca="false">IF($C16="Lease-koop",IF(F$14=$D16,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M16,p_Slot,0),IF(F$14=$D16,N($L16),0))</f>
+        <v>22000</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <f aca="false">IF($C16="Lease-koop",IF(G$14=$D16,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M16,p_Slot,0),IF(G$14=$D16,N($L16),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="15" t="n">
+        <f aca="false">IF($C16="Lease-koop",IF(H$14=$D16,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M16,p_Slot,0),IF(H$14=$D16,N($L16),0))</f>
+        <v>35000</v>
+      </c>
+      <c r="I16" s="15" t="n">
+        <f aca="false">IF($C16="Lease-koop",IF(I$14=$D16,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M16,p_Slot,0),IF(I$14=$D16,N($L16),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J16" s="6" t="n">
+        <f aca="false">IF($C16="Lease-koop",p_Afschr,IF($C16="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A16,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>6</v>
+      </c>
+      <c r="K16" s="16"/>
+      <c r="L16" s="15" t="n">
         <f aca="false">p_Aanbet+p_Belet+p_Opbouw+p_Slot</f>
         <v>57000</v>
       </c>
-      <c r="G16" s="6" t="n">
+      <c r="M16" s="6" t="n">
         <f aca="false">IF($C16="Lease-koop",D16+p_SlotJr,IF($C16="Koop",D16,0))</f>
         <v>2029</v>
       </c>
-      <c r="H16" s="6" t="n">
-        <f aca="false">IF($C16="Lease-koop",p_Afschr,IF($C16="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A16,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>6</v>
-      </c>
-      <c r="I16" s="15" t="n">
+      <c r="N16" s="15" t="n">
         <f aca="false">IF($C16="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
-      <c r="J16" s="5" t="str">
+      <c r="O16" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A16,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K16" s="16"/>
-      <c r="L16" s="15" t="n">
-        <f aca="false">IF($C16="Lease-koop",IF(L$14=$D16,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G16,p_Slot,0),IF(L$14=$D16,N($F16),0))</f>
-        <v>22000</v>
-      </c>
-      <c r="M16" s="15" t="n">
-        <f aca="false">IF($C16="Lease-koop",IF(M$14=$D16,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G16,p_Slot,0),IF(M$14=$D16,N($F16),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N16" s="15" t="n">
-        <f aca="false">IF($C16="Lease-koop",IF(N$14=$D16,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G16,p_Slot,0),IF(N$14=$D16,N($F16),0))</f>
-        <v>35000</v>
-      </c>
-      <c r="O16" s="15" t="n">
-        <f aca="false">IF($C16="Lease-koop",IF(O$14=$D16,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G16,p_Slot,0),IF(O$14=$D16,N($F16),0))</f>
-        <v>0</v>
       </c>
       <c r="P16" s="4"/>
     </row>
@@ -2549,41 +2548,41 @@
         <v>2035</v>
       </c>
       <c r="F17" s="15" t="n">
+        <f aca="false">IF($C17="Lease-koop",IF(F$14=$D17,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M17,p_Slot,0),IF(F$14=$D17,N($L17),0))</f>
+        <v>22000</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <f aca="false">IF($C17="Lease-koop",IF(G$14=$D17,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M17,p_Slot,0),IF(G$14=$D17,N($L17),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H17" s="15" t="n">
+        <f aca="false">IF($C17="Lease-koop",IF(H$14=$D17,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M17,p_Slot,0),IF(H$14=$D17,N($L17),0))</f>
+        <v>35000</v>
+      </c>
+      <c r="I17" s="15" t="n">
+        <f aca="false">IF($C17="Lease-koop",IF(I$14=$D17,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M17,p_Slot,0),IF(I$14=$D17,N($L17),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J17" s="6" t="n">
+        <f aca="false">IF($C17="Lease-koop",p_Afschr,IF($C17="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A17,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>6</v>
+      </c>
+      <c r="K17" s="16"/>
+      <c r="L17" s="15" t="n">
         <f aca="false">p_Aanbet+p_Belet+p_Opbouw+p_Slot</f>
         <v>57000</v>
       </c>
-      <c r="G17" s="6" t="n">
+      <c r="M17" s="6" t="n">
         <f aca="false">IF($C17="Lease-koop",D17+p_SlotJr,IF($C17="Koop",D17,0))</f>
         <v>2029</v>
       </c>
-      <c r="H17" s="6" t="n">
-        <f aca="false">IF($C17="Lease-koop",p_Afschr,IF($C17="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A17,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>6</v>
-      </c>
-      <c r="I17" s="15" t="n">
+      <c r="N17" s="15" t="n">
         <f aca="false">IF($C17="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
-      <c r="J17" s="5" t="str">
+      <c r="O17" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A17,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K17" s="16"/>
-      <c r="L17" s="15" t="n">
-        <f aca="false">IF($C17="Lease-koop",IF(L$14=$D17,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G17,p_Slot,0),IF(L$14=$D17,N($F17),0))</f>
-        <v>22000</v>
-      </c>
-      <c r="M17" s="15" t="n">
-        <f aca="false">IF($C17="Lease-koop",IF(M$14=$D17,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G17,p_Slot,0),IF(M$14=$D17,N($F17),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N17" s="15" t="n">
-        <f aca="false">IF($C17="Lease-koop",IF(N$14=$D17,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G17,p_Slot,0),IF(N$14=$D17,N($F17),0))</f>
-        <v>35000</v>
-      </c>
-      <c r="O17" s="15" t="n">
-        <f aca="false">IF($C17="Lease-koop",IF(O$14=$D17,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G17,p_Slot,0),IF(O$14=$D17,N($F17),0))</f>
-        <v>0</v>
       </c>
       <c r="P17" s="4"/>
     </row>
@@ -2606,40 +2605,40 @@
         <v>2042</v>
       </c>
       <c r="F18" s="15" t="n">
+        <f aca="false">IF($C18="Lease-koop",IF(F$14=$D18,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M18,p_Slot,0),IF(F$14=$D18,N($L18),0))</f>
         <v>80000</v>
       </c>
-      <c r="G18" s="6" t="n">
+      <c r="G18" s="15" t="n">
+        <f aca="false">IF($C18="Lease-koop",IF(G$14=$D18,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M18,p_Slot,0),IF(G$14=$D18,N($L18),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H18" s="15" t="n">
+        <f aca="false">IF($C18="Lease-koop",IF(H$14=$D18,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M18,p_Slot,0),IF(H$14=$D18,N($L18),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="15" t="n">
+        <f aca="false">IF($C18="Lease-koop",IF(I$14=$D18,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M18,p_Slot,0),IF(I$14=$D18,N($L18),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J18" s="6" t="n">
+        <f aca="false">IF($C18="Lease-koop",p_Afschr,IF($C18="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A18,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>15</v>
+      </c>
+      <c r="K18" s="16"/>
+      <c r="L18" s="15" t="n">
+        <v>80000</v>
+      </c>
+      <c r="M18" s="6" t="n">
         <f aca="false">IF($C18="Lease-koop",D18+p_SlotJr,IF($C18="Koop",D18,0))</f>
         <v>2027</v>
       </c>
-      <c r="H18" s="6" t="n">
-        <f aca="false">IF($C18="Lease-koop",p_Afschr,IF($C18="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A18,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>15</v>
-      </c>
-      <c r="I18" s="15" t="n">
+      <c r="N18" s="15" t="n">
         <f aca="false">IF($C18="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
-      <c r="J18" s="5" t="str">
+      <c r="O18" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A18,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="15" t="n">
-        <f aca="false">IF($C18="Lease-koop",IF(L$14=$D18,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G18,p_Slot,0),IF(L$14=$D18,N($F18),0))</f>
-        <v>80000</v>
-      </c>
-      <c r="M18" s="15" t="n">
-        <f aca="false">IF($C18="Lease-koop",IF(M$14=$D18,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G18,p_Slot,0),IF(M$14=$D18,N($F18),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N18" s="15" t="n">
-        <f aca="false">IF($C18="Lease-koop",IF(N$14=$D18,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G18,p_Slot,0),IF(N$14=$D18,N($F18),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O18" s="15" t="n">
-        <f aca="false">IF($C18="Lease-koop",IF(O$14=$D18,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G18,p_Slot,0),IF(O$14=$D18,N($F18),0))</f>
-        <v>0</v>
       </c>
       <c r="P18" s="4"/>
     </row>
@@ -2662,41 +2661,41 @@
         <v>2035</v>
       </c>
       <c r="F19" s="15" t="n">
+        <f aca="false">IF($C19="Lease-koop",IF(F$14=$D19,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M19,p_Slot,0),IF(F$14=$D19,N($L19),0))</f>
+        <v>22000</v>
+      </c>
+      <c r="G19" s="15" t="n">
+        <f aca="false">IF($C19="Lease-koop",IF(G$14=$D19,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M19,p_Slot,0),IF(G$14=$D19,N($L19),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H19" s="15" t="n">
+        <f aca="false">IF($C19="Lease-koop",IF(H$14=$D19,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M19,p_Slot,0),IF(H$14=$D19,N($L19),0))</f>
+        <v>35000</v>
+      </c>
+      <c r="I19" s="15" t="n">
+        <f aca="false">IF($C19="Lease-koop",IF(I$14=$D19,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M19,p_Slot,0),IF(I$14=$D19,N($L19),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J19" s="6" t="n">
+        <f aca="false">IF($C19="Lease-koop",p_Afschr,IF($C19="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A19,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>6</v>
+      </c>
+      <c r="K19" s="16"/>
+      <c r="L19" s="15" t="n">
         <f aca="false">p_Aanbet+p_Belet+p_Opbouw+p_Slot</f>
         <v>57000</v>
       </c>
-      <c r="G19" s="6" t="n">
+      <c r="M19" s="6" t="n">
         <f aca="false">IF($C19="Lease-koop",D19+p_SlotJr,IF($C19="Koop",D19,0))</f>
         <v>2029</v>
       </c>
-      <c r="H19" s="6" t="n">
-        <f aca="false">IF($C19="Lease-koop",p_Afschr,IF($C19="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A19,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>6</v>
-      </c>
-      <c r="I19" s="15" t="n">
+      <c r="N19" s="15" t="n">
         <f aca="false">IF($C19="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
-      <c r="J19" s="5" t="str">
+      <c r="O19" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A19,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K19" s="16"/>
-      <c r="L19" s="15" t="n">
-        <f aca="false">IF($C19="Lease-koop",IF(L$14=$D19,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G19,p_Slot,0),IF(L$14=$D19,N($F19),0))</f>
-        <v>22000</v>
-      </c>
-      <c r="M19" s="15" t="n">
-        <f aca="false">IF($C19="Lease-koop",IF(M$14=$D19,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G19,p_Slot,0),IF(M$14=$D19,N($F19),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N19" s="15" t="n">
-        <f aca="false">IF($C19="Lease-koop",IF(N$14=$D19,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G19,p_Slot,0),IF(N$14=$D19,N($F19),0))</f>
-        <v>35000</v>
-      </c>
-      <c r="O19" s="15" t="n">
-        <f aca="false">IF($C19="Lease-koop",IF(O$14=$D19,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G19,p_Slot,0),IF(O$14=$D19,N($F19),0))</f>
-        <v>0</v>
       </c>
       <c r="P19" s="4"/>
     </row>
@@ -2719,41 +2718,41 @@
         <v>2035</v>
       </c>
       <c r="F20" s="15" t="n">
+        <f aca="false">IF($C20="Lease-koop",IF(F$14=$D20,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M20,p_Slot,0),IF(F$14=$D20,N($L20),0))</f>
+        <v>22000</v>
+      </c>
+      <c r="G20" s="15" t="n">
+        <f aca="false">IF($C20="Lease-koop",IF(G$14=$D20,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M20,p_Slot,0),IF(G$14=$D20,N($L20),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H20" s="15" t="n">
+        <f aca="false">IF($C20="Lease-koop",IF(H$14=$D20,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M20,p_Slot,0),IF(H$14=$D20,N($L20),0))</f>
+        <v>35000</v>
+      </c>
+      <c r="I20" s="15" t="n">
+        <f aca="false">IF($C20="Lease-koop",IF(I$14=$D20,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M20,p_Slot,0),IF(I$14=$D20,N($L20),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J20" s="6" t="n">
+        <f aca="false">IF($C20="Lease-koop",p_Afschr,IF($C20="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A20,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>6</v>
+      </c>
+      <c r="K20" s="16"/>
+      <c r="L20" s="15" t="n">
         <f aca="false">p_Aanbet+p_Belet+p_Opbouw+p_Slot</f>
         <v>57000</v>
       </c>
-      <c r="G20" s="6" t="n">
+      <c r="M20" s="6" t="n">
         <f aca="false">IF($C20="Lease-koop",D20+p_SlotJr,IF($C20="Koop",D20,0))</f>
         <v>2029</v>
       </c>
-      <c r="H20" s="6" t="n">
-        <f aca="false">IF($C20="Lease-koop",p_Afschr,IF($C20="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A20,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>6</v>
-      </c>
-      <c r="I20" s="15" t="n">
+      <c r="N20" s="15" t="n">
         <f aca="false">IF($C20="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
-      <c r="J20" s="5" t="str">
+      <c r="O20" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A20,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K20" s="16"/>
-      <c r="L20" s="15" t="n">
-        <f aca="false">IF($C20="Lease-koop",IF(L$14=$D20,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G20,p_Slot,0),IF(L$14=$D20,N($F20),0))</f>
-        <v>22000</v>
-      </c>
-      <c r="M20" s="15" t="n">
-        <f aca="false">IF($C20="Lease-koop",IF(M$14=$D20,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G20,p_Slot,0),IF(M$14=$D20,N($F20),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N20" s="15" t="n">
-        <f aca="false">IF($C20="Lease-koop",IF(N$14=$D20,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G20,p_Slot,0),IF(N$14=$D20,N($F20),0))</f>
-        <v>35000</v>
-      </c>
-      <c r="O20" s="15" t="n">
-        <f aca="false">IF($C20="Lease-koop",IF(O$14=$D20,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G20,p_Slot,0),IF(O$14=$D20,N($F20),0))</f>
-        <v>0</v>
       </c>
       <c r="P20" s="4"/>
     </row>
@@ -2776,40 +2775,40 @@
         <v>2036</v>
       </c>
       <c r="F21" s="15" t="n">
+        <f aca="false">IF($C21="Lease-koop",IF(F$14=$D21,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M21,p_Slot,0),IF(F$14=$D21,N($L21),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="15" t="n">
+        <f aca="false">IF($C21="Lease-koop",IF(G$14=$D21,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M21,p_Slot,0),IF(G$14=$D21,N($L21),0))</f>
         <v>50000</v>
       </c>
-      <c r="G21" s="6" t="n">
+      <c r="H21" s="15" t="n">
+        <f aca="false">IF($C21="Lease-koop",IF(H$14=$D21,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M21,p_Slot,0),IF(H$14=$D21,N($L21),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I21" s="15" t="n">
+        <f aca="false">IF($C21="Lease-koop",IF(I$14=$D21,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M21,p_Slot,0),IF(I$14=$D21,N($L21),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J21" s="6" t="n">
+        <f aca="false">IF($C21="Lease-koop",p_Afschr,IF($C21="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A21,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>8</v>
+      </c>
+      <c r="K21" s="16"/>
+      <c r="L21" s="15" t="n">
+        <v>50000</v>
+      </c>
+      <c r="M21" s="6" t="n">
         <f aca="false">IF($C21="Lease-koop",D21+p_SlotJr,IF($C21="Koop",D21,0))</f>
         <v>2028</v>
       </c>
-      <c r="H21" s="6" t="n">
-        <f aca="false">IF($C21="Lease-koop",p_Afschr,IF($C21="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A21,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>8</v>
-      </c>
-      <c r="I21" s="15" t="n">
+      <c r="N21" s="15" t="n">
         <f aca="false">IF($C21="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
-      <c r="J21" s="5" t="str">
+      <c r="O21" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A21,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K21" s="16"/>
-      <c r="L21" s="15" t="n">
-        <f aca="false">IF($C21="Lease-koop",IF(L$14=$D21,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G21,p_Slot,0),IF(L$14=$D21,N($F21),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M21" s="15" t="n">
-        <f aca="false">IF($C21="Lease-koop",IF(M$14=$D21,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G21,p_Slot,0),IF(M$14=$D21,N($F21),0))</f>
-        <v>50000</v>
-      </c>
-      <c r="N21" s="15" t="n">
-        <f aca="false">IF($C21="Lease-koop",IF(N$14=$D21,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G21,p_Slot,0),IF(N$14=$D21,N($F21),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O21" s="15" t="n">
-        <f aca="false">IF($C21="Lease-koop",IF(O$14=$D21,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G21,p_Slot,0),IF(O$14=$D21,N($F21),0))</f>
-        <v>0</v>
       </c>
       <c r="P21" s="4" t="s">
         <v>127</v>
@@ -2834,41 +2833,41 @@
         <v>2037</v>
       </c>
       <c r="F22" s="15" t="n">
+        <f aca="false">IF($C22="Lease-koop",IF(F$14=$D22,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M22,p_Slot,0),IF(F$14=$D22,N($L22),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G22" s="15" t="n">
+        <f aca="false">IF($C22="Lease-koop",IF(G$14=$D22,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M22,p_Slot,0),IF(G$14=$D22,N($L22),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H22" s="15" t="n">
+        <f aca="false">IF($C22="Lease-koop",IF(H$14=$D22,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M22,p_Slot,0),IF(H$14=$D22,N($L22),0))</f>
+        <v>22000</v>
+      </c>
+      <c r="I22" s="15" t="n">
+        <f aca="false">IF($C22="Lease-koop",IF(I$14=$D22,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M22,p_Slot,0),IF(I$14=$D22,N($L22),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J22" s="6" t="n">
+        <f aca="false">IF($C22="Lease-koop",p_Afschr,IF($C22="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A22,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>6</v>
+      </c>
+      <c r="K22" s="16"/>
+      <c r="L22" s="15" t="n">
         <f aca="false">p_Aanbet+p_Belet+p_Opbouw+p_Slot</f>
         <v>57000</v>
       </c>
-      <c r="G22" s="6" t="n">
+      <c r="M22" s="6" t="n">
         <f aca="false">IF($C22="Lease-koop",D22+p_SlotJr,IF($C22="Koop",D22,0))</f>
         <v>2031</v>
       </c>
-      <c r="H22" s="6" t="n">
-        <f aca="false">IF($C22="Lease-koop",p_Afschr,IF($C22="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A22,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>6</v>
-      </c>
-      <c r="I22" s="15" t="n">
+      <c r="N22" s="15" t="n">
         <f aca="false">IF($C22="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
-      <c r="J22" s="5" t="str">
+      <c r="O22" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A22,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="15" t="n">
-        <f aca="false">IF($C22="Lease-koop",IF(L$14=$D22,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G22,p_Slot,0),IF(L$14=$D22,N($F22),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M22" s="15" t="n">
-        <f aca="false">IF($C22="Lease-koop",IF(M$14=$D22,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G22,p_Slot,0),IF(M$14=$D22,N($F22),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N22" s="15" t="n">
-        <f aca="false">IF($C22="Lease-koop",IF(N$14=$D22,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G22,p_Slot,0),IF(N$14=$D22,N($F22),0))</f>
-        <v>22000</v>
-      </c>
-      <c r="O22" s="15" t="n">
-        <f aca="false">IF($C22="Lease-koop",IF(O$14=$D22,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G22,p_Slot,0),IF(O$14=$D22,N($F22),0))</f>
-        <v>0</v>
       </c>
       <c r="P22" s="4"/>
     </row>
@@ -2891,40 +2890,40 @@
         <v>2049</v>
       </c>
       <c r="F23" s="15" t="n">
+        <f aca="false">IF($C23="Lease-koop",IF(F$14=$D23,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M23,p_Slot,0),IF(F$14=$D23,N($L23),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G23" s="15" t="n">
+        <f aca="false">IF($C23="Lease-koop",IF(G$14=$D23,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M23,p_Slot,0),IF(G$14=$D23,N($L23),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H23" s="15" t="n">
+        <f aca="false">IF($C23="Lease-koop",IF(H$14=$D23,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M23,p_Slot,0),IF(H$14=$D23,N($L23),0))</f>
         <v>100000</v>
       </c>
-      <c r="G23" s="6" t="n">
+      <c r="I23" s="15" t="n">
+        <f aca="false">IF($C23="Lease-koop",IF(I$14=$D23,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M23,p_Slot,0),IF(I$14=$D23,N($L23),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J23" s="6" t="n">
+        <f aca="false">IF($C23="Lease-koop",p_Afschr,IF($C23="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A23,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>20</v>
+      </c>
+      <c r="K23" s="16"/>
+      <c r="L23" s="15" t="n">
+        <v>100000</v>
+      </c>
+      <c r="M23" s="6" t="n">
         <f aca="false">IF($C23="Lease-koop",D23+p_SlotJr,IF($C23="Koop",D23,0))</f>
         <v>2029</v>
       </c>
-      <c r="H23" s="6" t="n">
-        <f aca="false">IF($C23="Lease-koop",p_Afschr,IF($C23="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A23,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>20</v>
-      </c>
-      <c r="I23" s="15" t="n">
+      <c r="N23" s="15" t="n">
         <f aca="false">IF($C23="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
-      <c r="J23" s="5" t="str">
+      <c r="O23" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A23,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K23" s="16"/>
-      <c r="L23" s="15" t="n">
-        <f aca="false">IF($C23="Lease-koop",IF(L$14=$D23,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G23,p_Slot,0),IF(L$14=$D23,N($F23),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M23" s="15" t="n">
-        <f aca="false">IF($C23="Lease-koop",IF(M$14=$D23,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G23,p_Slot,0),IF(M$14=$D23,N($F23),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N23" s="15" t="n">
-        <f aca="false">IF($C23="Lease-koop",IF(N$14=$D23,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G23,p_Slot,0),IF(N$14=$D23,N($F23),0))</f>
-        <v>100000</v>
-      </c>
-      <c r="O23" s="15" t="n">
-        <f aca="false">IF($C23="Lease-koop",IF(O$14=$D23,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G23,p_Slot,0),IF(O$14=$D23,N($F23),0))</f>
-        <v>0</v>
       </c>
       <c r="P23" s="4"/>
     </row>
@@ -2947,41 +2946,41 @@
         <v>2039</v>
       </c>
       <c r="F24" s="15" t="n">
+        <f aca="false">IF($C24="Lease-koop",IF(F$14=$D24,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M24,p_Slot,0),IF(F$14=$D24,N($L24),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G24" s="15" t="n">
+        <f aca="false">IF($C24="Lease-koop",IF(G$14=$D24,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M24,p_Slot,0),IF(G$14=$D24,N($L24),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="15" t="n">
+        <f aca="false">IF($C24="Lease-koop",IF(H$14=$D24,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M24,p_Slot,0),IF(H$14=$D24,N($L24),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I24" s="15" t="n">
+        <f aca="false">IF($C24="Lease-koop",IF(I$14=$D24,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M24,p_Slot,0),IF(I$14=$D24,N($L24),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J24" s="6" t="n">
+        <f aca="false">IF($C24="Lease-koop",p_Afschr,IF($C24="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A24,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>6</v>
+      </c>
+      <c r="K24" s="16"/>
+      <c r="L24" s="15" t="n">
         <f aca="false">p_Aanbet+p_Belet+p_Opbouw+p_Slot</f>
         <v>57000</v>
       </c>
-      <c r="G24" s="6" t="n">
+      <c r="M24" s="6" t="n">
         <f aca="false">IF($C24="Lease-koop",D24+p_SlotJr,IF($C24="Koop",D24,0))</f>
         <v>2033</v>
       </c>
-      <c r="H24" s="6" t="n">
-        <f aca="false">IF($C24="Lease-koop",p_Afschr,IF($C24="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A24,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>6</v>
-      </c>
-      <c r="I24" s="15" t="n">
+      <c r="N24" s="15" t="n">
         <f aca="false">IF($C24="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
-      <c r="J24" s="5" t="str">
+      <c r="O24" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A24,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K24" s="16"/>
-      <c r="L24" s="15" t="n">
-        <f aca="false">IF($C24="Lease-koop",IF(L$14=$D24,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G24,p_Slot,0),IF(L$14=$D24,N($F24),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M24" s="15" t="n">
-        <f aca="false">IF($C24="Lease-koop",IF(M$14=$D24,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G24,p_Slot,0),IF(M$14=$D24,N($F24),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N24" s="15" t="n">
-        <f aca="false">IF($C24="Lease-koop",IF(N$14=$D24,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G24,p_Slot,0),IF(N$14=$D24,N($F24),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O24" s="15" t="n">
-        <f aca="false">IF($C24="Lease-koop",IF(O$14=$D24,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G24,p_Slot,0),IF(O$14=$D24,N($F24),0))</f>
-        <v>0</v>
       </c>
       <c r="P24" s="4"/>
     </row>
@@ -3004,40 +3003,40 @@
         <v>2040</v>
       </c>
       <c r="F25" s="15" t="n">
+        <f aca="false">IF($C25="Lease-koop",IF(F$14=$D25,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M25,p_Slot,0),IF(F$14=$D25,N($L25),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="15" t="n">
+        <f aca="false">IF($C25="Lease-koop",IF(G$14=$D25,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M25,p_Slot,0),IF(G$14=$D25,N($L25),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="15" t="n">
+        <f aca="false">IF($C25="Lease-koop",IF(H$14=$D25,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M25,p_Slot,0),IF(H$14=$D25,N($L25),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I25" s="15" t="n">
+        <f aca="false">IF($C25="Lease-koop",IF(I$14=$D25,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M25,p_Slot,0),IF(I$14=$D25,N($L25),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J25" s="6" t="n">
+        <f aca="false">IF($C25="Lease-koop",p_Afschr,IF($C25="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A25,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>8</v>
+      </c>
+      <c r="K25" s="16"/>
+      <c r="L25" s="15" t="n">
         <v>248960</v>
       </c>
-      <c r="G25" s="6" t="n">
+      <c r="M25" s="6" t="n">
         <f aca="false">IF($C25="Lease-koop",D25+p_SlotJr,IF($C25="Koop",D25,0))</f>
         <v>2032</v>
       </c>
-      <c r="H25" s="6" t="n">
-        <f aca="false">IF($C25="Lease-koop",p_Afschr,IF($C25="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A25,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>8</v>
-      </c>
-      <c r="I25" s="15" t="n">
+      <c r="N25" s="15" t="n">
         <f aca="false">IF($C25="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
-      <c r="J25" s="5" t="str">
+      <c r="O25" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A25,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K25" s="16"/>
-      <c r="L25" s="15" t="n">
-        <f aca="false">IF($C25="Lease-koop",IF(L$14=$D25,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G25,p_Slot,0),IF(L$14=$D25,N($F25),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M25" s="15" t="n">
-        <f aca="false">IF($C25="Lease-koop",IF(M$14=$D25,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G25,p_Slot,0),IF(M$14=$D25,N($F25),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N25" s="15" t="n">
-        <f aca="false">IF($C25="Lease-koop",IF(N$14=$D25,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G25,p_Slot,0),IF(N$14=$D25,N($F25),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O25" s="15" t="n">
-        <f aca="false">IF($C25="Lease-koop",IF(O$14=$D25,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G25,p_Slot,0),IF(O$14=$D25,N($F25),0))</f>
-        <v>0</v>
       </c>
       <c r="P25" s="4"/>
     </row>
@@ -3059,39 +3058,39 @@
         <f aca="false">IF($C26="Lease-koop",D26+p_Lev,IF($C26="Koop",D26+IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A26,'In gebruik'!$A:$A,0)),0),0))</f>
         <v>0</v>
       </c>
-      <c r="F26" s="15"/>
-      <c r="G26" s="6" t="n">
+      <c r="F26" s="15" t="n">
+        <f aca="false">IF($C26="Lease-koop",IF(F$14=$D26,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M26,p_Slot,0),IF(F$14=$D26,N($L26),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="15" t="n">
+        <f aca="false">IF($C26="Lease-koop",IF(G$14=$D26,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M26,p_Slot,0),IF(G$14=$D26,N($L26),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="15" t="n">
+        <f aca="false">IF($C26="Lease-koop",IF(H$14=$D26,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M26,p_Slot,0),IF(H$14=$D26,N($L26),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I26" s="15" t="n">
+        <f aca="false">IF($C26="Lease-koop",IF(I$14=$D26,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M26,p_Slot,0),IF(I$14=$D26,N($L26),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J26" s="6" t="n">
+        <f aca="false">IF($C26="Lease-koop",p_Afschr,IF($C26="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A26,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>0</v>
+      </c>
+      <c r="K26" s="5"/>
+      <c r="L26" s="15"/>
+      <c r="M26" s="6" t="n">
         <f aca="false">IF($C26="Lease-koop",D26+p_SlotJr,IF($C26="Koop",D26,0))</f>
         <v>0</v>
       </c>
-      <c r="H26" s="6" t="n">
-        <f aca="false">IF($C26="Lease-koop",p_Afschr,IF($C26="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A26,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>0</v>
-      </c>
-      <c r="I26" s="15" t="n">
+      <c r="N26" s="15" t="n">
         <f aca="false">IF($C26="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
-      <c r="J26" s="5" t="str">
+      <c r="O26" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A26,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K26" s="5"/>
-      <c r="L26" s="15" t="n">
-        <f aca="false">IF($C26="Lease-koop",IF(L$14=$D26,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G26,p_Slot,0),IF(L$14=$D26,N($F26),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M26" s="15" t="n">
-        <f aca="false">IF($C26="Lease-koop",IF(M$14=$D26,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G26,p_Slot,0),IF(M$14=$D26,N($F26),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N26" s="15" t="n">
-        <f aca="false">IF($C26="Lease-koop",IF(N$14=$D26,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G26,p_Slot,0),IF(N$14=$D26,N($F26),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O26" s="15" t="n">
-        <f aca="false">IF($C26="Lease-koop",IF(O$14=$D26,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G26,p_Slot,0),IF(O$14=$D26,N($F26),0))</f>
-        <v>0</v>
       </c>
       <c r="P26" s="4" t="s">
         <v>129</v>
@@ -3116,41 +3115,41 @@
         <v>2040</v>
       </c>
       <c r="F27" s="15" t="n">
+        <f aca="false">IF($C27="Lease-koop",IF(F$14=$D27,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M27,p_Slot,0),IF(F$14=$D27,N($L27),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G27" s="15" t="n">
+        <f aca="false">IF($C27="Lease-koop",IF(G$14=$D27,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M27,p_Slot,0),IF(G$14=$D27,N($L27),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="15" t="n">
+        <f aca="false">IF($C27="Lease-koop",IF(H$14=$D27,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M27,p_Slot,0),IF(H$14=$D27,N($L27),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I27" s="15" t="n">
+        <f aca="false">IF($C27="Lease-koop",IF(I$14=$D27,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M27,p_Slot,0),IF(I$14=$D27,N($L27),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J27" s="6" t="n">
+        <f aca="false">IF($C27="Lease-koop",p_Afschr,IF($C27="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A27,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>6</v>
+      </c>
+      <c r="K27" s="16"/>
+      <c r="L27" s="15" t="n">
         <f aca="false">p_Aanbet+p_Belet+p_Opbouw+p_Slot</f>
         <v>57000</v>
       </c>
-      <c r="G27" s="6" t="n">
+      <c r="M27" s="6" t="n">
         <f aca="false">IF($C27="Lease-koop",D27+p_SlotJr,IF($C27="Koop",D27,0))</f>
         <v>2034</v>
       </c>
-      <c r="H27" s="6" t="n">
-        <f aca="false">IF($C27="Lease-koop",p_Afschr,IF($C27="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A27,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>6</v>
-      </c>
-      <c r="I27" s="15" t="n">
+      <c r="N27" s="15" t="n">
         <f aca="false">IF($C27="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
-      <c r="J27" s="5" t="str">
+      <c r="O27" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A27,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K27" s="16"/>
-      <c r="L27" s="15" t="n">
-        <f aca="false">IF($C27="Lease-koop",IF(L$14=$D27,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G27,p_Slot,0),IF(L$14=$D27,N($F27),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M27" s="15" t="n">
-        <f aca="false">IF($C27="Lease-koop",IF(M$14=$D27,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G27,p_Slot,0),IF(M$14=$D27,N($F27),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N27" s="15" t="n">
-        <f aca="false">IF($C27="Lease-koop",IF(N$14=$D27,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G27,p_Slot,0),IF(N$14=$D27,N($F27),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O27" s="15" t="n">
-        <f aca="false">IF($C27="Lease-koop",IF(O$14=$D27,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G27,p_Slot,0),IF(O$14=$D27,N($F27),0))</f>
-        <v>0</v>
       </c>
       <c r="P27" s="4"/>
     </row>
@@ -3173,41 +3172,41 @@
         <v>2040</v>
       </c>
       <c r="F28" s="15" t="n">
+        <f aca="false">IF($C28="Lease-koop",IF(F$14=$D28,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M28,p_Slot,0),IF(F$14=$D28,N($L28),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G28" s="15" t="n">
+        <f aca="false">IF($C28="Lease-koop",IF(G$14=$D28,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M28,p_Slot,0),IF(G$14=$D28,N($L28),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H28" s="15" t="n">
+        <f aca="false">IF($C28="Lease-koop",IF(H$14=$D28,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M28,p_Slot,0),IF(H$14=$D28,N($L28),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I28" s="15" t="n">
+        <f aca="false">IF($C28="Lease-koop",IF(I$14=$D28,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M28,p_Slot,0),IF(I$14=$D28,N($L28),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J28" s="6" t="n">
+        <f aca="false">IF($C28="Lease-koop",p_Afschr,IF($C28="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A28,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>6</v>
+      </c>
+      <c r="K28" s="16"/>
+      <c r="L28" s="15" t="n">
         <f aca="false">p_Aanbet+p_Belet+p_Opbouw+p_Slot</f>
         <v>57000</v>
       </c>
-      <c r="G28" s="6" t="n">
+      <c r="M28" s="6" t="n">
         <f aca="false">IF($C28="Lease-koop",D28+p_SlotJr,IF($C28="Koop",D28,0))</f>
         <v>2034</v>
       </c>
-      <c r="H28" s="6" t="n">
-        <f aca="false">IF($C28="Lease-koop",p_Afschr,IF($C28="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A28,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>6</v>
-      </c>
-      <c r="I28" s="15" t="n">
+      <c r="N28" s="15" t="n">
         <f aca="false">IF($C28="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
-      <c r="J28" s="5" t="str">
+      <c r="O28" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A28,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="15" t="n">
-        <f aca="false">IF($C28="Lease-koop",IF(L$14=$D28,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G28,p_Slot,0),IF(L$14=$D28,N($F28),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M28" s="15" t="n">
-        <f aca="false">IF($C28="Lease-koop",IF(M$14=$D28,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G28,p_Slot,0),IF(M$14=$D28,N($F28),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N28" s="15" t="n">
-        <f aca="false">IF($C28="Lease-koop",IF(N$14=$D28,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G28,p_Slot,0),IF(N$14=$D28,N($F28),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O28" s="15" t="n">
-        <f aca="false">IF($C28="Lease-koop",IF(O$14=$D28,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G28,p_Slot,0),IF(O$14=$D28,N($F28),0))</f>
-        <v>0</v>
       </c>
       <c r="P28" s="4"/>
     </row>
@@ -3230,41 +3229,41 @@
         <v>2040</v>
       </c>
       <c r="F29" s="15" t="n">
+        <f aca="false">IF($C29="Lease-koop",IF(F$14=$D29,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M29,p_Slot,0),IF(F$14=$D29,N($L29),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G29" s="15" t="n">
+        <f aca="false">IF($C29="Lease-koop",IF(G$14=$D29,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M29,p_Slot,0),IF(G$14=$D29,N($L29),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="15" t="n">
+        <f aca="false">IF($C29="Lease-koop",IF(H$14=$D29,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M29,p_Slot,0),IF(H$14=$D29,N($L29),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I29" s="15" t="n">
+        <f aca="false">IF($C29="Lease-koop",IF(I$14=$D29,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M29,p_Slot,0),IF(I$14=$D29,N($L29),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J29" s="6" t="n">
+        <f aca="false">IF($C29="Lease-koop",p_Afschr,IF($C29="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A29,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>6</v>
+      </c>
+      <c r="K29" s="16"/>
+      <c r="L29" s="15" t="n">
         <f aca="false">p_Aanbet+p_Belet+p_Opbouw+p_Slot</f>
         <v>57000</v>
       </c>
-      <c r="G29" s="6" t="n">
+      <c r="M29" s="6" t="n">
         <f aca="false">IF($C29="Lease-koop",D29+p_SlotJr,IF($C29="Koop",D29,0))</f>
         <v>2034</v>
       </c>
-      <c r="H29" s="6" t="n">
-        <f aca="false">IF($C29="Lease-koop",p_Afschr,IF($C29="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A29,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>6</v>
-      </c>
-      <c r="I29" s="15" t="n">
+      <c r="N29" s="15" t="n">
         <f aca="false">IF($C29="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
-      <c r="J29" s="5" t="str">
+      <c r="O29" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A29,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K29" s="16"/>
-      <c r="L29" s="15" t="n">
-        <f aca="false">IF($C29="Lease-koop",IF(L$14=$D29,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G29,p_Slot,0),IF(L$14=$D29,N($F29),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M29" s="15" t="n">
-        <f aca="false">IF($C29="Lease-koop",IF(M$14=$D29,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G29,p_Slot,0),IF(M$14=$D29,N($F29),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N29" s="15" t="n">
-        <f aca="false">IF($C29="Lease-koop",IF(N$14=$D29,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G29,p_Slot,0),IF(N$14=$D29,N($F29),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O29" s="15" t="n">
-        <f aca="false">IF($C29="Lease-koop",IF(O$14=$D29,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G29,p_Slot,0),IF(O$14=$D29,N($F29),0))</f>
-        <v>0</v>
       </c>
       <c r="P29" s="4"/>
     </row>
@@ -3287,41 +3286,41 @@
         <v>2041</v>
       </c>
       <c r="F30" s="15" t="n">
+        <f aca="false">IF($C30="Lease-koop",IF(F$14=$D30,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M30,p_Slot,0),IF(F$14=$D30,N($L30),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G30" s="15" t="n">
+        <f aca="false">IF($C30="Lease-koop",IF(G$14=$D30,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M30,p_Slot,0),IF(G$14=$D30,N($L30),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H30" s="15" t="n">
+        <f aca="false">IF($C30="Lease-koop",IF(H$14=$D30,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M30,p_Slot,0),IF(H$14=$D30,N($L30),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I30" s="15" t="n">
+        <f aca="false">IF($C30="Lease-koop",IF(I$14=$D30,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M30,p_Slot,0),IF(I$14=$D30,N($L30),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J30" s="6" t="n">
+        <f aca="false">IF($C30="Lease-koop",p_Afschr,IF($C30="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A30,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>6</v>
+      </c>
+      <c r="K30" s="16"/>
+      <c r="L30" s="15" t="n">
         <f aca="false">p_Aanbet+p_Belet+p_Opbouw+p_Slot</f>
         <v>57000</v>
       </c>
-      <c r="G30" s="6" t="n">
+      <c r="M30" s="6" t="n">
         <f aca="false">IF($C30="Lease-koop",D30+p_SlotJr,IF($C30="Koop",D30,0))</f>
         <v>2035</v>
       </c>
-      <c r="H30" s="6" t="n">
-        <f aca="false">IF($C30="Lease-koop",p_Afschr,IF($C30="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A30,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>6</v>
-      </c>
-      <c r="I30" s="15" t="n">
+      <c r="N30" s="15" t="n">
         <f aca="false">IF($C30="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
-      <c r="J30" s="5" t="str">
+      <c r="O30" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A30,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K30" s="16"/>
-      <c r="L30" s="15" t="n">
-        <f aca="false">IF($C30="Lease-koop",IF(L$14=$D30,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G30,p_Slot,0),IF(L$14=$D30,N($F30),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M30" s="15" t="n">
-        <f aca="false">IF($C30="Lease-koop",IF(M$14=$D30,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G30,p_Slot,0),IF(M$14=$D30,N($F30),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N30" s="15" t="n">
-        <f aca="false">IF($C30="Lease-koop",IF(N$14=$D30,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G30,p_Slot,0),IF(N$14=$D30,N($F30),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O30" s="15" t="n">
-        <f aca="false">IF($C30="Lease-koop",IF(O$14=$D30,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G30,p_Slot,0),IF(O$14=$D30,N($F30),0))</f>
-        <v>0</v>
       </c>
       <c r="P30" s="4"/>
     </row>
@@ -3344,40 +3343,40 @@
         <v>2043</v>
       </c>
       <c r="F31" s="15" t="n">
+        <f aca="false">IF($C31="Lease-koop",IF(F$14=$D31,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M31,p_Slot,0),IF(F$14=$D31,N($L31),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G31" s="15" t="n">
+        <f aca="false">IF($C31="Lease-koop",IF(G$14=$D31,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M31,p_Slot,0),IF(G$14=$D31,N($L31),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H31" s="15" t="n">
+        <f aca="false">IF($C31="Lease-koop",IF(H$14=$D31,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M31,p_Slot,0),IF(H$14=$D31,N($L31),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I31" s="15" t="n">
+        <f aca="false">IF($C31="Lease-koop",IF(I$14=$D31,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M31,p_Slot,0),IF(I$14=$D31,N($L31),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J31" s="6" t="n">
+        <f aca="false">IF($C31="Lease-koop",p_Afschr,IF($C31="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A31,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>10</v>
+      </c>
+      <c r="K31" s="16"/>
+      <c r="L31" s="15" t="n">
         <v>19000</v>
       </c>
-      <c r="G31" s="6" t="n">
+      <c r="M31" s="6" t="n">
         <f aca="false">IF($C31="Lease-koop",D31+p_SlotJr,IF($C31="Koop",D31,0))</f>
         <v>2033</v>
       </c>
-      <c r="H31" s="6" t="n">
-        <f aca="false">IF($C31="Lease-koop",p_Afschr,IF($C31="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A31,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>10</v>
-      </c>
-      <c r="I31" s="15" t="n">
+      <c r="N31" s="15" t="n">
         <f aca="false">IF($C31="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
-      <c r="J31" s="5" t="str">
+      <c r="O31" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A31,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K31" s="16"/>
-      <c r="L31" s="15" t="n">
-        <f aca="false">IF($C31="Lease-koop",IF(L$14=$D31,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G31,p_Slot,0),IF(L$14=$D31,N($F31),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M31" s="15" t="n">
-        <f aca="false">IF($C31="Lease-koop",IF(M$14=$D31,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G31,p_Slot,0),IF(M$14=$D31,N($F31),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N31" s="15" t="n">
-        <f aca="false">IF($C31="Lease-koop",IF(N$14=$D31,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G31,p_Slot,0),IF(N$14=$D31,N($F31),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O31" s="15" t="n">
-        <f aca="false">IF($C31="Lease-koop",IF(O$14=$D31,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G31,p_Slot,0),IF(O$14=$D31,N($F31),0))</f>
-        <v>0</v>
       </c>
       <c r="P31" s="4"/>
     </row>
@@ -3400,41 +3399,41 @@
         <v>2042</v>
       </c>
       <c r="F32" s="15" t="n">
+        <f aca="false">IF($C32="Lease-koop",IF(F$14=$D32,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M32,p_Slot,0),IF(F$14=$D32,N($L32),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G32" s="15" t="n">
+        <f aca="false">IF($C32="Lease-koop",IF(G$14=$D32,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M32,p_Slot,0),IF(G$14=$D32,N($L32),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H32" s="15" t="n">
+        <f aca="false">IF($C32="Lease-koop",IF(H$14=$D32,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M32,p_Slot,0),IF(H$14=$D32,N($L32),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I32" s="15" t="n">
+        <f aca="false">IF($C32="Lease-koop",IF(I$14=$D32,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M32,p_Slot,0),IF(I$14=$D32,N($L32),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J32" s="6" t="n">
+        <f aca="false">IF($C32="Lease-koop",p_Afschr,IF($C32="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A32,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>6</v>
+      </c>
+      <c r="K32" s="16"/>
+      <c r="L32" s="15" t="n">
         <f aca="false">p_Aanbet+p_Belet+p_Opbouw+p_Slot</f>
         <v>57000</v>
       </c>
-      <c r="G32" s="6" t="n">
+      <c r="M32" s="6" t="n">
         <f aca="false">IF($C32="Lease-koop",D32+p_SlotJr,IF($C32="Koop",D32,0))</f>
         <v>2036</v>
       </c>
-      <c r="H32" s="6" t="n">
-        <f aca="false">IF($C32="Lease-koop",p_Afschr,IF($C32="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A32,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>6</v>
-      </c>
-      <c r="I32" s="15" t="n">
+      <c r="N32" s="15" t="n">
         <f aca="false">IF($C32="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
-      <c r="J32" s="5" t="str">
+      <c r="O32" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A32,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v>635901</v>
-      </c>
-      <c r="K32" s="16"/>
-      <c r="L32" s="15" t="n">
-        <f aca="false">IF($C32="Lease-koop",IF(L$14=$D32,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G32,p_Slot,0),IF(L$14=$D32,N($F32),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M32" s="15" t="n">
-        <f aca="false">IF($C32="Lease-koop",IF(M$14=$D32,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G32,p_Slot,0),IF(M$14=$D32,N($F32),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N32" s="15" t="n">
-        <f aca="false">IF($C32="Lease-koop",IF(N$14=$D32,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G32,p_Slot,0),IF(N$14=$D32,N($F32),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O32" s="15" t="n">
-        <f aca="false">IF($C32="Lease-koop",IF(O$14=$D32,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G32,p_Slot,0),IF(O$14=$D32,N($F32),0))</f>
-        <v>0</v>
       </c>
       <c r="P32" s="4"/>
     </row>
@@ -3457,41 +3456,41 @@
         <v>2042</v>
       </c>
       <c r="F33" s="15" t="n">
+        <f aca="false">IF($C33="Lease-koop",IF(F$14=$D33,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M33,p_Slot,0),IF(F$14=$D33,N($L33),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G33" s="15" t="n">
+        <f aca="false">IF($C33="Lease-koop",IF(G$14=$D33,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M33,p_Slot,0),IF(G$14=$D33,N($L33),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H33" s="15" t="n">
+        <f aca="false">IF($C33="Lease-koop",IF(H$14=$D33,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M33,p_Slot,0),IF(H$14=$D33,N($L33),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I33" s="15" t="n">
+        <f aca="false">IF($C33="Lease-koop",IF(I$14=$D33,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M33,p_Slot,0),IF(I$14=$D33,N($L33),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J33" s="6" t="n">
+        <f aca="false">IF($C33="Lease-koop",p_Afschr,IF($C33="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A33,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>6</v>
+      </c>
+      <c r="K33" s="16"/>
+      <c r="L33" s="15" t="n">
         <f aca="false">p_Aanbet+p_Belet+p_Opbouw+p_Slot</f>
         <v>57000</v>
       </c>
-      <c r="G33" s="6" t="n">
+      <c r="M33" s="6" t="n">
         <f aca="false">IF($C33="Lease-koop",D33+p_SlotJr,IF($C33="Koop",D33,0))</f>
         <v>2036</v>
       </c>
-      <c r="H33" s="6" t="n">
-        <f aca="false">IF($C33="Lease-koop",p_Afschr,IF($C33="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A33,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>6</v>
-      </c>
-      <c r="I33" s="15" t="n">
+      <c r="N33" s="15" t="n">
         <f aca="false">IF($C33="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
-      <c r="J33" s="5" t="str">
+      <c r="O33" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A33,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v>617901</v>
-      </c>
-      <c r="K33" s="16"/>
-      <c r="L33" s="15" t="n">
-        <f aca="false">IF($C33="Lease-koop",IF(L$14=$D33,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G33,p_Slot,0),IF(L$14=$D33,N($F33),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M33" s="15" t="n">
-        <f aca="false">IF($C33="Lease-koop",IF(M$14=$D33,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G33,p_Slot,0),IF(M$14=$D33,N($F33),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N33" s="15" t="n">
-        <f aca="false">IF($C33="Lease-koop",IF(N$14=$D33,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G33,p_Slot,0),IF(N$14=$D33,N($F33),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O33" s="15" t="n">
-        <f aca="false">IF($C33="Lease-koop",IF(O$14=$D33,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G33,p_Slot,0),IF(O$14=$D33,N($F33),0))</f>
-        <v>0</v>
       </c>
       <c r="P33" s="4"/>
     </row>
@@ -3514,41 +3513,41 @@
         <v>2042</v>
       </c>
       <c r="F34" s="15" t="n">
+        <f aca="false">IF($C34="Lease-koop",IF(F$14=$D34,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M34,p_Slot,0),IF(F$14=$D34,N($L34),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G34" s="15" t="n">
+        <f aca="false">IF($C34="Lease-koop",IF(G$14=$D34,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M34,p_Slot,0),IF(G$14=$D34,N($L34),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H34" s="15" t="n">
+        <f aca="false">IF($C34="Lease-koop",IF(H$14=$D34,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M34,p_Slot,0),IF(H$14=$D34,N($L34),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I34" s="15" t="n">
+        <f aca="false">IF($C34="Lease-koop",IF(I$14=$D34,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M34,p_Slot,0),IF(I$14=$D34,N($L34),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J34" s="6" t="n">
+        <f aca="false">IF($C34="Lease-koop",p_Afschr,IF($C34="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A34,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>6</v>
+      </c>
+      <c r="K34" s="16"/>
+      <c r="L34" s="15" t="n">
         <f aca="false">p_Aanbet+p_Belet+p_Opbouw+p_Slot</f>
         <v>57000</v>
       </c>
-      <c r="G34" s="6" t="n">
+      <c r="M34" s="6" t="n">
         <f aca="false">IF($C34="Lease-koop",D34+p_SlotJr,IF($C34="Koop",D34,0))</f>
         <v>2036</v>
       </c>
-      <c r="H34" s="6" t="n">
-        <f aca="false">IF($C34="Lease-koop",p_Afschr,IF($C34="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A34,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>6</v>
-      </c>
-      <c r="I34" s="15" t="n">
+      <c r="N34" s="15" t="n">
         <f aca="false">IF($C34="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
-      <c r="J34" s="5" t="str">
+      <c r="O34" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A34,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v>635901</v>
-      </c>
-      <c r="K34" s="16"/>
-      <c r="L34" s="15" t="n">
-        <f aca="false">IF($C34="Lease-koop",IF(L$14=$D34,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G34,p_Slot,0),IF(L$14=$D34,N($F34),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M34" s="15" t="n">
-        <f aca="false">IF($C34="Lease-koop",IF(M$14=$D34,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G34,p_Slot,0),IF(M$14=$D34,N($F34),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N34" s="15" t="n">
-        <f aca="false">IF($C34="Lease-koop",IF(N$14=$D34,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G34,p_Slot,0),IF(N$14=$D34,N($F34),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O34" s="15" t="n">
-        <f aca="false">IF($C34="Lease-koop",IF(O$14=$D34,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G34,p_Slot,0),IF(O$14=$D34,N($F34),0))</f>
-        <v>0</v>
       </c>
       <c r="P34" s="4"/>
     </row>
@@ -3571,41 +3570,41 @@
         <v>2042</v>
       </c>
       <c r="F35" s="15" t="n">
+        <f aca="false">IF($C35="Lease-koop",IF(F$14=$D35,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M35,p_Slot,0),IF(F$14=$D35,N($L35),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G35" s="15" t="n">
+        <f aca="false">IF($C35="Lease-koop",IF(G$14=$D35,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M35,p_Slot,0),IF(G$14=$D35,N($L35),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H35" s="15" t="n">
+        <f aca="false">IF($C35="Lease-koop",IF(H$14=$D35,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M35,p_Slot,0),IF(H$14=$D35,N($L35),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I35" s="15" t="n">
+        <f aca="false">IF($C35="Lease-koop",IF(I$14=$D35,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M35,p_Slot,0),IF(I$14=$D35,N($L35),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J35" s="6" t="n">
+        <f aca="false">IF($C35="Lease-koop",p_Afschr,IF($C35="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A35,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>6</v>
+      </c>
+      <c r="K35" s="16"/>
+      <c r="L35" s="15" t="n">
         <f aca="false">p_Aanbet+p_Belet+p_Opbouw+p_Slot</f>
         <v>57000</v>
       </c>
-      <c r="G35" s="6" t="n">
+      <c r="M35" s="6" t="n">
         <f aca="false">IF($C35="Lease-koop",D35+p_SlotJr,IF($C35="Koop",D35,0))</f>
         <v>2036</v>
       </c>
-      <c r="H35" s="6" t="n">
-        <f aca="false">IF($C35="Lease-koop",p_Afschr,IF($C35="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A35,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>6</v>
-      </c>
-      <c r="I35" s="15" t="n">
+      <c r="N35" s="15" t="n">
         <f aca="false">IF($C35="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
-      <c r="J35" s="5" t="str">
+      <c r="O35" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A35,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v>604901</v>
-      </c>
-      <c r="K35" s="16"/>
-      <c r="L35" s="15" t="n">
-        <f aca="false">IF($C35="Lease-koop",IF(L$14=$D35,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G35,p_Slot,0),IF(L$14=$D35,N($F35),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M35" s="15" t="n">
-        <f aca="false">IF($C35="Lease-koop",IF(M$14=$D35,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G35,p_Slot,0),IF(M$14=$D35,N($F35),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N35" s="15" t="n">
-        <f aca="false">IF($C35="Lease-koop",IF(N$14=$D35,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G35,p_Slot,0),IF(N$14=$D35,N($F35),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O35" s="15" t="n">
-        <f aca="false">IF($C35="Lease-koop",IF(O$14=$D35,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G35,p_Slot,0),IF(O$14=$D35,N($F35),0))</f>
-        <v>0</v>
       </c>
       <c r="P35" s="4"/>
     </row>
@@ -3628,41 +3627,41 @@
         <v>2042</v>
       </c>
       <c r="F36" s="15" t="n">
+        <f aca="false">IF($C36="Lease-koop",IF(F$14=$D36,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M36,p_Slot,0),IF(F$14=$D36,N($L36),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G36" s="15" t="n">
+        <f aca="false">IF($C36="Lease-koop",IF(G$14=$D36,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M36,p_Slot,0),IF(G$14=$D36,N($L36),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H36" s="15" t="n">
+        <f aca="false">IF($C36="Lease-koop",IF(H$14=$D36,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M36,p_Slot,0),IF(H$14=$D36,N($L36),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I36" s="15" t="n">
+        <f aca="false">IF($C36="Lease-koop",IF(I$14=$D36,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M36,p_Slot,0),IF(I$14=$D36,N($L36),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J36" s="6" t="n">
+        <f aca="false">IF($C36="Lease-koop",p_Afschr,IF($C36="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A36,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>6</v>
+      </c>
+      <c r="K36" s="16"/>
+      <c r="L36" s="15" t="n">
         <f aca="false">p_Aanbet+p_Belet+p_Opbouw+p_Slot</f>
         <v>57000</v>
       </c>
-      <c r="G36" s="6" t="n">
+      <c r="M36" s="6" t="n">
         <f aca="false">IF($C36="Lease-koop",D36+p_SlotJr,IF($C36="Koop",D36,0))</f>
         <v>2036</v>
       </c>
-      <c r="H36" s="6" t="n">
-        <f aca="false">IF($C36="Lease-koop",p_Afschr,IF($C36="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A36,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>6</v>
-      </c>
-      <c r="I36" s="15" t="n">
+      <c r="N36" s="15" t="n">
         <f aca="false">IF($C36="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
-      <c r="J36" s="5" t="str">
+      <c r="O36" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A36,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v>630901</v>
-      </c>
-      <c r="K36" s="16"/>
-      <c r="L36" s="15" t="n">
-        <f aca="false">IF($C36="Lease-koop",IF(L$14=$D36,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G36,p_Slot,0),IF(L$14=$D36,N($F36),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M36" s="15" t="n">
-        <f aca="false">IF($C36="Lease-koop",IF(M$14=$D36,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G36,p_Slot,0),IF(M$14=$D36,N($F36),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N36" s="15" t="n">
-        <f aca="false">IF($C36="Lease-koop",IF(N$14=$D36,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G36,p_Slot,0),IF(N$14=$D36,N($F36),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O36" s="15" t="n">
-        <f aca="false">IF($C36="Lease-koop",IF(O$14=$D36,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G36,p_Slot,0),IF(O$14=$D36,N($F36),0))</f>
-        <v>0</v>
       </c>
       <c r="P36" s="4"/>
     </row>
@@ -3685,41 +3684,41 @@
         <v>2042</v>
       </c>
       <c r="F37" s="15" t="n">
+        <f aca="false">IF($C37="Lease-koop",IF(F$14=$D37,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M37,p_Slot,0),IF(F$14=$D37,N($L37),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G37" s="15" t="n">
+        <f aca="false">IF($C37="Lease-koop",IF(G$14=$D37,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M37,p_Slot,0),IF(G$14=$D37,N($L37),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H37" s="15" t="n">
+        <f aca="false">IF($C37="Lease-koop",IF(H$14=$D37,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M37,p_Slot,0),IF(H$14=$D37,N($L37),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I37" s="15" t="n">
+        <f aca="false">IF($C37="Lease-koop",IF(I$14=$D37,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M37,p_Slot,0),IF(I$14=$D37,N($L37),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J37" s="6" t="n">
+        <f aca="false">IF($C37="Lease-koop",p_Afschr,IF($C37="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A37,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>6</v>
+      </c>
+      <c r="K37" s="16"/>
+      <c r="L37" s="15" t="n">
         <f aca="false">p_Aanbet+p_Belet+p_Opbouw+p_Slot</f>
         <v>57000</v>
       </c>
-      <c r="G37" s="6" t="n">
+      <c r="M37" s="6" t="n">
         <f aca="false">IF($C37="Lease-koop",D37+p_SlotJr,IF($C37="Koop",D37,0))</f>
         <v>2036</v>
       </c>
-      <c r="H37" s="6" t="n">
-        <f aca="false">IF($C37="Lease-koop",p_Afschr,IF($C37="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A37,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>6</v>
-      </c>
-      <c r="I37" s="15" t="n">
+      <c r="N37" s="15" t="n">
         <f aca="false">IF($C37="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
-      <c r="J37" s="5" t="str">
+      <c r="O37" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A37,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v>604901</v>
-      </c>
-      <c r="K37" s="16"/>
-      <c r="L37" s="15" t="n">
-        <f aca="false">IF($C37="Lease-koop",IF(L$14=$D37,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G37,p_Slot,0),IF(L$14=$D37,N($F37),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M37" s="15" t="n">
-        <f aca="false">IF($C37="Lease-koop",IF(M$14=$D37,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G37,p_Slot,0),IF(M$14=$D37,N($F37),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N37" s="15" t="n">
-        <f aca="false">IF($C37="Lease-koop",IF(N$14=$D37,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G37,p_Slot,0),IF(N$14=$D37,N($F37),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O37" s="15" t="n">
-        <f aca="false">IF($C37="Lease-koop",IF(O$14=$D37,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G37,p_Slot,0),IF(O$14=$D37,N($F37),0))</f>
-        <v>0</v>
       </c>
       <c r="P37" s="4"/>
     </row>
@@ -3742,40 +3741,40 @@
         <v>2044</v>
       </c>
       <c r="F38" s="15" t="n">
+        <f aca="false">IF($C38="Lease-koop",IF(F$14=$D38,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M38,p_Slot,0),IF(F$14=$D38,N($L38),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G38" s="15" t="n">
+        <f aca="false">IF($C38="Lease-koop",IF(G$14=$D38,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M38,p_Slot,0),IF(G$14=$D38,N($L38),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H38" s="15" t="n">
+        <f aca="false">IF($C38="Lease-koop",IF(H$14=$D38,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M38,p_Slot,0),IF(H$14=$D38,N($L38),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I38" s="15" t="n">
+        <f aca="false">IF($C38="Lease-koop",IF(I$14=$D38,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M38,p_Slot,0),IF(I$14=$D38,N($L38),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J38" s="6" t="n">
+        <f aca="false">IF($C38="Lease-koop",p_Afschr,IF($C38="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A38,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>10</v>
+      </c>
+      <c r="K38" s="16"/>
+      <c r="L38" s="15" t="n">
         <v>51100</v>
       </c>
-      <c r="G38" s="6" t="n">
+      <c r="M38" s="6" t="n">
         <f aca="false">IF($C38="Lease-koop",D38+p_SlotJr,IF($C38="Koop",D38,0))</f>
         <v>2034</v>
       </c>
-      <c r="H38" s="6" t="n">
-        <f aca="false">IF($C38="Lease-koop",p_Afschr,IF($C38="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A38,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>10</v>
-      </c>
-      <c r="I38" s="15" t="n">
+      <c r="N38" s="15" t="n">
         <f aca="false">IF($C38="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
-      <c r="J38" s="5" t="str">
+      <c r="O38" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A38,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K38" s="16"/>
-      <c r="L38" s="15" t="n">
-        <f aca="false">IF($C38="Lease-koop",IF(L$14=$D38,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G38,p_Slot,0),IF(L$14=$D38,N($F38),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M38" s="15" t="n">
-        <f aca="false">IF($C38="Lease-koop",IF(M$14=$D38,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G38,p_Slot,0),IF(M$14=$D38,N($F38),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N38" s="15" t="n">
-        <f aca="false">IF($C38="Lease-koop",IF(N$14=$D38,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G38,p_Slot,0),IF(N$14=$D38,N($F38),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O38" s="15" t="n">
-        <f aca="false">IF($C38="Lease-koop",IF(O$14=$D38,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G38,p_Slot,0),IF(O$14=$D38,N($F38),0))</f>
-        <v>0</v>
       </c>
       <c r="P38" s="4"/>
     </row>
@@ -3798,41 +3797,41 @@
         <v>2042</v>
       </c>
       <c r="F39" s="15" t="n">
+        <f aca="false">IF($C39="Lease-koop",IF(F$14=$D39,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M39,p_Slot,0),IF(F$14=$D39,N($L39),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G39" s="15" t="n">
+        <f aca="false">IF($C39="Lease-koop",IF(G$14=$D39,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M39,p_Slot,0),IF(G$14=$D39,N($L39),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H39" s="15" t="n">
+        <f aca="false">IF($C39="Lease-koop",IF(H$14=$D39,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M39,p_Slot,0),IF(H$14=$D39,N($L39),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I39" s="15" t="n">
+        <f aca="false">IF($C39="Lease-koop",IF(I$14=$D39,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M39,p_Slot,0),IF(I$14=$D39,N($L39),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J39" s="6" t="n">
+        <f aca="false">IF($C39="Lease-koop",p_Afschr,IF($C39="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A39,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>6</v>
+      </c>
+      <c r="K39" s="16"/>
+      <c r="L39" s="15" t="n">
         <f aca="false">p_Aanbet+p_Belet+p_Opbouw+p_Slot</f>
         <v>57000</v>
       </c>
-      <c r="G39" s="6" t="n">
+      <c r="M39" s="6" t="n">
         <f aca="false">IF($C39="Lease-koop",D39+p_SlotJr,IF($C39="Koop",D39,0))</f>
         <v>2036</v>
       </c>
-      <c r="H39" s="6" t="n">
-        <f aca="false">IF($C39="Lease-koop",p_Afschr,IF($C39="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A39,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>6</v>
-      </c>
-      <c r="I39" s="15" t="n">
+      <c r="N39" s="15" t="n">
         <f aca="false">IF($C39="Lease-koop",p_Lease,0)</f>
         <v>12000</v>
       </c>
-      <c r="J39" s="5" t="str">
+      <c r="O39" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A39,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K39" s="16"/>
-      <c r="L39" s="15" t="n">
-        <f aca="false">IF($C39="Lease-koop",IF(L$14=$D39,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G39,p_Slot,0),IF(L$14=$D39,N($F39),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M39" s="15" t="n">
-        <f aca="false">IF($C39="Lease-koop",IF(M$14=$D39,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G39,p_Slot,0),IF(M$14=$D39,N($F39),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N39" s="15" t="n">
-        <f aca="false">IF($C39="Lease-koop",IF(N$14=$D39,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G39,p_Slot,0),IF(N$14=$D39,N($F39),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O39" s="15" t="n">
-        <f aca="false">IF($C39="Lease-koop",IF(O$14=$D39,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G39,p_Slot,0),IF(O$14=$D39,N($F39),0))</f>
-        <v>0</v>
       </c>
       <c r="P39" s="4"/>
     </row>
@@ -3855,40 +3854,40 @@
         <v>2047</v>
       </c>
       <c r="F40" s="15" t="n">
+        <f aca="false">IF($C40="Lease-koop",IF(F$14=$D40,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M40,p_Slot,0),IF(F$14=$D40,N($L40),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G40" s="15" t="n">
+        <f aca="false">IF($C40="Lease-koop",IF(G$14=$D40,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M40,p_Slot,0),IF(G$14=$D40,N($L40),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H40" s="15" t="n">
+        <f aca="false">IF($C40="Lease-koop",IF(H$14=$D40,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M40,p_Slot,0),IF(H$14=$D40,N($L40),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I40" s="15" t="n">
+        <f aca="false">IF($C40="Lease-koop",IF(I$14=$D40,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M40,p_Slot,0),IF(I$14=$D40,N($L40),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J40" s="6" t="n">
+        <f aca="false">IF($C40="Lease-koop",p_Afschr,IF($C40="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A40,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>12</v>
+      </c>
+      <c r="K40" s="16"/>
+      <c r="L40" s="15" t="n">
         <v>358180</v>
       </c>
-      <c r="G40" s="6" t="n">
+      <c r="M40" s="6" t="n">
         <f aca="false">IF($C40="Lease-koop",D40+p_SlotJr,IF($C40="Koop",D40,0))</f>
         <v>2035</v>
       </c>
-      <c r="H40" s="6" t="n">
-        <f aca="false">IF($C40="Lease-koop",p_Afschr,IF($C40="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A40,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>12</v>
-      </c>
-      <c r="I40" s="15" t="n">
+      <c r="N40" s="15" t="n">
         <f aca="false">IF($C40="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
-      <c r="J40" s="5" t="str">
+      <c r="O40" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A40,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K40" s="16"/>
-      <c r="L40" s="15" t="n">
-        <f aca="false">IF($C40="Lease-koop",IF(L$14=$D40,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G40,p_Slot,0),IF(L$14=$D40,N($F40),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M40" s="15" t="n">
-        <f aca="false">IF($C40="Lease-koop",IF(M$14=$D40,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G40,p_Slot,0),IF(M$14=$D40,N($F40),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N40" s="15" t="n">
-        <f aca="false">IF($C40="Lease-koop",IF(N$14=$D40,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G40,p_Slot,0),IF(N$14=$D40,N($F40),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O40" s="15" t="n">
-        <f aca="false">IF($C40="Lease-koop",IF(O$14=$D40,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G40,p_Slot,0),IF(O$14=$D40,N($F40),0))</f>
-        <v>0</v>
       </c>
       <c r="P40" s="4"/>
     </row>
@@ -3911,40 +3910,40 @@
         <v>2053</v>
       </c>
       <c r="F41" s="15" t="n">
+        <f aca="false">IF($C41="Lease-koop",IF(F$14=$D41,p_Aanbet+p_Belet+p_Opbouw,0)+IF(F$14=$M41,p_Slot,0),IF(F$14=$D41,N($L41),0))</f>
+        <v>0</v>
+      </c>
+      <c r="G41" s="15" t="n">
+        <f aca="false">IF($C41="Lease-koop",IF(G$14=$D41,p_Aanbet+p_Belet+p_Opbouw,0)+IF(G$14=$M41,p_Slot,0),IF(G$14=$D41,N($L41),0))</f>
+        <v>0</v>
+      </c>
+      <c r="H41" s="15" t="n">
+        <f aca="false">IF($C41="Lease-koop",IF(H$14=$D41,p_Aanbet+p_Belet+p_Opbouw,0)+IF(H$14=$M41,p_Slot,0),IF(H$14=$D41,N($L41),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I41" s="15" t="n">
+        <f aca="false">IF($C41="Lease-koop",IF(I$14=$D41,p_Aanbet+p_Belet+p_Opbouw,0)+IF(I$14=$M41,p_Slot,0),IF(I$14=$D41,N($L41),0))</f>
+        <v>0</v>
+      </c>
+      <c r="J41" s="6" t="n">
+        <f aca="false">IF($C41="Lease-koop",p_Afschr,IF($C41="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A41,'In gebruik'!$A:$A,0)),0),0))</f>
+        <v>15</v>
+      </c>
+      <c r="K41" s="16"/>
+      <c r="L41" s="15" t="n">
         <v>121968</v>
       </c>
-      <c r="G41" s="6" t="n">
+      <c r="M41" s="6" t="n">
         <f aca="false">IF($C41="Lease-koop",D41+p_SlotJr,IF($C41="Koop",D41,0))</f>
         <v>2038</v>
       </c>
-      <c r="H41" s="6" t="n">
-        <f aca="false">IF($C41="Lease-koop",p_Afschr,IF($C41="Koop",IFERROR(INDEX('In gebruik'!$H:$H,MATCH($A41,'In gebruik'!$A:$A,0)),0),0))</f>
-        <v>15</v>
-      </c>
-      <c r="I41" s="15" t="n">
+      <c r="N41" s="15" t="n">
         <f aca="false">IF($C41="Lease-koop",p_Lease,0)</f>
         <v>0</v>
       </c>
-      <c r="J41" s="5" t="str">
+      <c r="O41" s="5" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$O:$O,MATCH($A41,'In gebruik'!$A:$A,0))&amp;"","")</f>
         <v/>
-      </c>
-      <c r="K41" s="16"/>
-      <c r="L41" s="15" t="n">
-        <f aca="false">IF($C41="Lease-koop",IF(L$14=$D41,p_Aanbet+p_Belet+p_Opbouw,0)+IF(L$14=$G41,p_Slot,0),IF(L$14=$D41,N($F41),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M41" s="15" t="n">
-        <f aca="false">IF($C41="Lease-koop",IF(M$14=$D41,p_Aanbet+p_Belet+p_Opbouw,0)+IF(M$14=$G41,p_Slot,0),IF(M$14=$D41,N($F41),0))</f>
-        <v>0</v>
-      </c>
-      <c r="N41" s="15" t="n">
-        <f aca="false">IF($C41="Lease-koop",IF(N$14=$D41,p_Aanbet+p_Belet+p_Opbouw,0)+IF(N$14=$G41,p_Slot,0),IF(N$14=$D41,N($F41),0))</f>
-        <v>0</v>
-      </c>
-      <c r="O41" s="15" t="n">
-        <f aca="false">IF($C41="Lease-koop",IF(O$14=$D41,p_Aanbet+p_Belet+p_Opbouw,0)+IF(O$14=$G41,p_Slot,0),IF(O$14=$D41,N($F41),0))</f>
-        <v>0</v>
       </c>
       <c r="P41" s="4"/>
     </row>
@@ -3958,29 +3957,29 @@
       <c r="E42" s="18"/>
       <c r="F42" s="10" t="n">
         <f aca="false">SUM(F15:F41)</f>
-        <v>2055208</v>
-      </c>
-      <c r="G42" s="18"/>
-      <c r="H42" s="18"/>
-      <c r="I42" s="18"/>
+        <v>190000</v>
+      </c>
+      <c r="G42" s="10" t="n">
+        <f aca="false">SUM(G15:G41)</f>
+        <v>50000</v>
+      </c>
+      <c r="H42" s="10" t="n">
+        <f aca="false">SUM(H15:H41)</f>
+        <v>297000</v>
+      </c>
+      <c r="I42" s="10" t="n">
+        <f aca="false">SUM(I15:I41)</f>
+        <v>0</v>
+      </c>
       <c r="J42" s="18"/>
       <c r="K42" s="18"/>
       <c r="L42" s="10" t="n">
         <f aca="false">SUM(L15:L41)</f>
-        <v>190000</v>
-      </c>
-      <c r="M42" s="10" t="n">
-        <f aca="false">SUM(M15:M41)</f>
-        <v>50000</v>
-      </c>
-      <c r="N42" s="10" t="n">
-        <f aca="false">SUM(N15:N41)</f>
-        <v>297000</v>
-      </c>
-      <c r="O42" s="10" t="n">
-        <f aca="false">SUM(O15:O41)</f>
-        <v>0</v>
-      </c>
+        <v>2055208</v>
+      </c>
+      <c r="M42" s="18"/>
+      <c r="N42" s="18"/>
+      <c r="O42" s="18"/>
       <c r="P42" s="18"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4011,7 +4010,7 @@
   </sheetData>
   <autoFilter ref="A14:P41"/>
   <mergeCells count="1">
-    <mergeCell ref="L13:O13"/>
+    <mergeCell ref="F13:I13"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C15:C62" type="list">

</xml_diff>

<commit_message>
Wagenpark_beheer.xlsx: kolomvolgorde in gebruik en gebruiksdoel ingevuld
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013EaFTgzjMaNvZvWgFM9YZf
</commit_message>
<xml_diff>
--- a/Wagenpark_beheer.xlsx
+++ b/Wagenpark_beheer.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="160">
   <si>
     <t xml:space="preserve">Voertuigen in gebruik</t>
   </si>
@@ -68,6 +68,12 @@
     <t xml:space="preserve">Aanschafkosten (werkelijk)</t>
   </si>
   <si>
+    <t xml:space="preserve">Te activeren in jaar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Activakaart</t>
+  </si>
+  <si>
     <t xml:space="preserve">Aanbetaling (raming)</t>
   </si>
   <si>
@@ -77,12 +83,6 @@
     <t xml:space="preserve">Slotbetaling (raming)</t>
   </si>
   <si>
-    <t xml:space="preserve">Te activeren in jaar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Activakaart</t>
-  </si>
-  <si>
     <t xml:space="preserve">Exploitatienr.</t>
   </si>
   <si>
@@ -95,7 +95,7 @@
     <t xml:space="preserve">26-BXG-9</t>
   </si>
   <si>
-    <t xml:space="preserve">Vrachtwagen</t>
+    <t xml:space="preserve">Openbare ruimte</t>
   </si>
   <si>
     <t xml:space="preserve">Koop</t>
@@ -110,7 +110,7 @@
     <t xml:space="preserve">06-BVN-2</t>
   </si>
   <si>
-    <t xml:space="preserve">Rioolvoertuig</t>
+    <t xml:space="preserve">Riolering</t>
   </si>
   <si>
     <t xml:space="preserve">Lau/William</t>
@@ -122,6 +122,9 @@
     <t xml:space="preserve">BZ-TZ-45</t>
   </si>
   <si>
+    <t xml:space="preserve">Gladheidsbestrijding</t>
+  </si>
+  <si>
     <t xml:space="preserve">STROOIEN</t>
   </si>
   <si>
@@ -131,7 +134,7 @@
     <t xml:space="preserve">V-88-FPL</t>
   </si>
   <si>
-    <t xml:space="preserve">Stratenmakers</t>
+    <t xml:space="preserve">Openbare ruimte (straatwerk)</t>
   </si>
   <si>
     <t xml:space="preserve">Marnick/Henry</t>
@@ -233,7 +236,7 @@
     <t xml:space="preserve">V-603-LV</t>
   </si>
   <si>
-    <t xml:space="preserve">Speelt/groen</t>
+    <t xml:space="preserve">Speeltoestellen / groen</t>
   </si>
   <si>
     <t xml:space="preserve">Ruud Liebrechts</t>
@@ -263,7 +266,7 @@
     <t xml:space="preserve">V-73-NRS</t>
   </si>
   <si>
-    <t xml:space="preserve">Timmerman</t>
+    <t xml:space="preserve">Gebouwen (timmerman)</t>
   </si>
   <si>
     <t xml:space="preserve">Arie v Dijk</t>
@@ -302,7 +305,7 @@
     <t xml:space="preserve">geen</t>
   </si>
   <si>
-    <t xml:space="preserve">Werf</t>
+    <t xml:space="preserve">Gemeentewerf</t>
   </si>
   <si>
     <t xml:space="preserve">V25</t>
@@ -314,7 +317,7 @@
     <t xml:space="preserve">RG-730-S</t>
   </si>
   <si>
-    <t xml:space="preserve">Algemeen</t>
+    <t xml:space="preserve">Algemeen (dienstauto)</t>
   </si>
   <si>
     <t xml:space="preserve">Dienstauto</t>
@@ -353,7 +356,7 @@
     <t xml:space="preserve">Toelichting</t>
   </si>
   <si>
-    <t xml:space="preserve">Koop: kolom I = werkelijk betaald. Lease-koop: kolom J t/m M, kolom I blijft leeg.</t>
+    <t xml:space="preserve">Koop: kolom I = werkelijk betaald. Lease-koop: kolom J en L t/m N, kolom I blijft leeg.</t>
   </si>
   <si>
     <t xml:space="preserve">Uitgaven vanaf 2027 staan op het gemiddelde; overschrijven met de werkelijke uitgave zodra bekend.</t>
@@ -467,9 +470,6 @@
     <t xml:space="preserve">05-SZ-NF</t>
   </si>
   <si>
-    <t xml:space="preserve">Tijdelijk kantoor</t>
-  </si>
-  <si>
     <t xml:space="preserve">6971005/434335/M05SZNF</t>
   </si>
   <si>
@@ -479,7 +479,7 @@
     <t xml:space="preserve">TFN-07-R</t>
   </si>
   <si>
-    <t xml:space="preserve">Veegwagen</t>
+    <t xml:space="preserve">Straatreiniging</t>
   </si>
   <si>
     <t xml:space="preserve">6210601/434335</t>
@@ -491,9 +491,6 @@
     <t xml:space="preserve">VG-683-L</t>
   </si>
   <si>
-    <t xml:space="preserve">Speelwerktuigen</t>
-  </si>
-  <si>
     <t xml:space="preserve">V97</t>
   </si>
   <si>
@@ -510,9 +507,6 @@
   </si>
   <si>
     <t xml:space="preserve">VG-094-L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIJDELIJK alg dienst</t>
   </si>
   <si>
     <t xml:space="preserve">6210102/434335</t>
@@ -870,11 +864,11 @@
     <tableColumn id="7" name="Aanschafjaar"/>
     <tableColumn id="8" name="Levensduur"/>
     <tableColumn id="9" name="Aanschafkosten (werkelijk)"/>
-    <tableColumn id="10" name="Aanbetaling (raming)"/>
-    <tableColumn id="11" name="Bijkomende kosten (raming)"/>
-    <tableColumn id="12" name="Slotbetaling (raming)"/>
-    <tableColumn id="13" name="Te activeren in jaar"/>
-    <tableColumn id="14" name="Activakaart"/>
+    <tableColumn id="10" name="Te activeren in jaar"/>
+    <tableColumn id="11" name="Activakaart"/>
+    <tableColumn id="12" name="Aanbetaling (raming)"/>
+    <tableColumn id="13" name="Bijkomende kosten (raming)"/>
+    <tableColumn id="14" name="Slotbetaling (raming)"/>
     <tableColumn id="15" name="Exploitatienr."/>
     <tableColumn id="16" name="Leasesom 1 jaar"/>
   </tableColumns>
@@ -1072,9 +1066,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="10" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="12" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="12"/>
   </cols>
@@ -1085,12 +1079,11 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J3" s="2" t="s">
+      <c r="L3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
       <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
@@ -1170,13 +1163,13 @@
       <c r="I5" s="8" t="n">
         <v>248960</v>
       </c>
-      <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="5" t="n">
+        <v>119</v>
+      </c>
       <c r="L5" s="8"/>
-      <c r="M5" s="6"/>
-      <c r="N5" s="5" t="n">
-        <v>119</v>
-      </c>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
       <c r="O5" s="5"/>
       <c r="P5" s="8"/>
     </row>
@@ -1208,13 +1201,13 @@
       <c r="I6" s="8" t="n">
         <v>358180</v>
       </c>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="5" t="n">
+        <v>625</v>
+      </c>
       <c r="L6" s="8"/>
-      <c r="M6" s="6"/>
-      <c r="N6" s="5" t="n">
-        <v>625</v>
-      </c>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
       <c r="O6" s="5"/>
       <c r="P6" s="8"/>
     </row>
@@ -1227,45 +1220,45 @@
         <v>28</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G7" s="6" t="n">
         <v>2012</v>
       </c>
       <c r="H7" s="7"/>
       <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="5"/>
       <c r="L7" s="8"/>
-      <c r="M7" s="6"/>
-      <c r="N7" s="5"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
       <c r="O7" s="5"/>
       <c r="P7" s="8"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B8" s="5" t="n">
         <v>7205035</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G8" s="6" t="n">
         <v>2024</v>
@@ -1276,34 +1269,34 @@
       <c r="I8" s="8" t="n">
         <v>72896</v>
       </c>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="5" t="n">
+        <v>632</v>
+      </c>
       <c r="L8" s="8"/>
-      <c r="M8" s="6"/>
-      <c r="N8" s="5" t="n">
-        <v>632</v>
-      </c>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
       <c r="O8" s="5"/>
       <c r="P8" s="8"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B9" s="5" t="n">
         <v>7205053</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G9" s="6" t="n">
         <v>2021</v>
@@ -1314,32 +1307,32 @@
       <c r="I9" s="8" t="n">
         <v>65000</v>
       </c>
-      <c r="J9" s="8"/>
-      <c r="K9" s="8"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="5"/>
       <c r="L9" s="8"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="5"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
       <c r="O9" s="5"/>
       <c r="P9" s="8"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B10" s="5" t="n">
         <v>7205045</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G10" s="6" t="n">
         <v>2026</v>
@@ -1348,20 +1341,20 @@
         <v>8</v>
       </c>
       <c r="I10" s="8"/>
-      <c r="J10" s="8" t="n">
+      <c r="J10" s="6" t="n">
+        <v>2028</v>
+      </c>
+      <c r="K10" s="5"/>
+      <c r="L10" s="8" t="n">
         <v>11000</v>
       </c>
-      <c r="K10" s="8" t="n">
+      <c r="M10" s="8" t="n">
         <v>3420</v>
       </c>
-      <c r="L10" s="8" t="n">
+      <c r="N10" s="8" t="n">
         <f aca="false">p_Slot</f>
         <v>35000</v>
       </c>
-      <c r="M10" s="6" t="n">
-        <v>2028</v>
-      </c>
-      <c r="N10" s="5"/>
       <c r="O10" s="5" t="n">
         <v>635901</v>
       </c>
@@ -1371,22 +1364,22 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B11" s="5" t="n">
         <v>7205051</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G11" s="6" t="n">
         <v>2013</v>
@@ -1397,34 +1390,34 @@
       <c r="I11" s="8" t="n">
         <v>65000</v>
       </c>
-      <c r="J11" s="8"/>
-      <c r="K11" s="8"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="5" t="n">
+        <v>803</v>
+      </c>
       <c r="L11" s="8"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="5" t="n">
-        <v>803</v>
-      </c>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
       <c r="O11" s="5"/>
       <c r="P11" s="8"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>7205048</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G12" s="6" t="n">
         <v>2026</v>
@@ -1433,22 +1426,22 @@
         <v>8</v>
       </c>
       <c r="I12" s="8"/>
-      <c r="J12" s="8" t="n">
+      <c r="J12" s="6" t="n">
+        <v>2028</v>
+      </c>
+      <c r="K12" s="5" t="n">
+        <v>648</v>
+      </c>
+      <c r="L12" s="8" t="n">
         <v>11000</v>
       </c>
-      <c r="K12" s="8" t="n">
+      <c r="M12" s="8" t="n">
         <v>3420</v>
       </c>
-      <c r="L12" s="8" t="n">
+      <c r="N12" s="8" t="n">
         <f aca="false">p_Slot</f>
         <v>35000</v>
       </c>
-      <c r="M12" s="6" t="n">
-        <v>2028</v>
-      </c>
-      <c r="N12" s="5" t="n">
-        <v>648</v>
-      </c>
       <c r="O12" s="5" t="n">
         <v>617901</v>
       </c>
@@ -1458,22 +1451,22 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B13" s="5" t="n">
         <v>7205039</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G13" s="6" t="n">
         <v>2024</v>
@@ -1484,34 +1477,34 @@
       <c r="I13" s="8" t="n">
         <v>38664</v>
       </c>
-      <c r="J13" s="8"/>
-      <c r="K13" s="8"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="5" t="n">
+        <v>472</v>
+      </c>
       <c r="L13" s="8"/>
-      <c r="M13" s="6"/>
-      <c r="N13" s="5" t="n">
-        <v>472</v>
-      </c>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
       <c r="O13" s="5"/>
       <c r="P13" s="8"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B14" s="5" t="n">
         <v>7205043</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G14" s="6" t="n">
         <v>2025</v>
@@ -1522,32 +1515,32 @@
       <c r="I14" s="8" t="n">
         <v>30093</v>
       </c>
-      <c r="J14" s="8"/>
-      <c r="K14" s="8"/>
+      <c r="J14" s="6"/>
+      <c r="K14" s="5" t="n">
+        <v>461</v>
+      </c>
       <c r="L14" s="8"/>
-      <c r="M14" s="6"/>
-      <c r="N14" s="5" t="n">
-        <v>461</v>
-      </c>
+      <c r="M14" s="8"/>
+      <c r="N14" s="8"/>
       <c r="O14" s="5"/>
       <c r="P14" s="8"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B15" s="5" t="n">
         <v>7205046</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G15" s="6" t="n">
         <v>2026</v>
@@ -1556,20 +1549,20 @@
         <v>8</v>
       </c>
       <c r="I15" s="8"/>
-      <c r="J15" s="8" t="n">
+      <c r="J15" s="6" t="n">
+        <v>2028</v>
+      </c>
+      <c r="K15" s="5"/>
+      <c r="L15" s="8" t="n">
         <v>11000</v>
       </c>
-      <c r="K15" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="8" t="n">
+      <c r="M15" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="8" t="n">
         <f aca="false">p_Slot</f>
         <v>35000</v>
       </c>
-      <c r="M15" s="6" t="n">
-        <v>2028</v>
-      </c>
-      <c r="N15" s="5"/>
       <c r="O15" s="5" t="n">
         <v>635901</v>
       </c>
@@ -1579,22 +1572,22 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B16" s="5" t="n">
         <v>7205044</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G16" s="6" t="n">
         <v>2024</v>
@@ -1605,34 +1598,34 @@
       <c r="I16" s="8" t="n">
         <v>65770</v>
       </c>
-      <c r="J16" s="8"/>
-      <c r="K16" s="8"/>
+      <c r="J16" s="6"/>
+      <c r="K16" s="5" t="n">
+        <v>465</v>
+      </c>
       <c r="L16" s="8"/>
-      <c r="M16" s="6"/>
-      <c r="N16" s="5" t="n">
-        <v>465</v>
-      </c>
+      <c r="M16" s="8"/>
+      <c r="N16" s="8"/>
       <c r="O16" s="5"/>
       <c r="P16" s="8"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B17" s="5" t="n">
         <v>7205052</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G17" s="6" t="n">
         <v>2017</v>
@@ -1643,34 +1636,34 @@
       <c r="I17" s="8" t="n">
         <v>65000</v>
       </c>
-      <c r="J17" s="8"/>
-      <c r="K17" s="8"/>
+      <c r="J17" s="6"/>
+      <c r="K17" s="5" t="n">
+        <v>520</v>
+      </c>
       <c r="L17" s="8"/>
-      <c r="M17" s="6"/>
-      <c r="N17" s="5" t="n">
-        <v>520</v>
-      </c>
+      <c r="M17" s="8"/>
+      <c r="N17" s="8"/>
       <c r="O17" s="5"/>
       <c r="P17" s="8"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B18" s="5" t="n">
         <v>7205058</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G18" s="6" t="n">
         <v>2018</v>
@@ -1681,30 +1674,30 @@
       <c r="I18" s="8" t="n">
         <v>45000</v>
       </c>
-      <c r="J18" s="8"/>
-      <c r="K18" s="8"/>
+      <c r="J18" s="6"/>
+      <c r="K18" s="5"/>
       <c r="L18" s="8"/>
-      <c r="M18" s="6"/>
-      <c r="N18" s="5"/>
+      <c r="M18" s="8"/>
+      <c r="N18" s="8"/>
       <c r="O18" s="5"/>
       <c r="P18" s="8"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B19" s="5" t="n">
         <v>7205033</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G19" s="6" t="n">
         <v>2026</v>
@@ -1713,22 +1706,22 @@
         <v>8</v>
       </c>
       <c r="I19" s="8"/>
-      <c r="J19" s="8" t="n">
+      <c r="J19" s="6" t="n">
+        <v>2028</v>
+      </c>
+      <c r="K19" s="5" t="n">
+        <v>463</v>
+      </c>
+      <c r="L19" s="8" t="n">
         <v>11000</v>
       </c>
-      <c r="K19" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" s="8" t="n">
+      <c r="M19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="8" t="n">
         <f aca="false">p_Slot</f>
         <v>35000</v>
       </c>
-      <c r="M19" s="6" t="n">
-        <v>2028</v>
-      </c>
-      <c r="N19" s="5" t="n">
-        <v>463</v>
-      </c>
       <c r="O19" s="5" t="n">
         <v>604901</v>
       </c>
@@ -1738,20 +1731,20 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B20" s="5" t="n">
         <v>7205032</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G20" s="6" t="n">
         <v>2026</v>
@@ -1760,22 +1753,22 @@
         <v>8</v>
       </c>
       <c r="I20" s="8"/>
-      <c r="J20" s="8" t="n">
+      <c r="J20" s="6" t="n">
+        <v>2028</v>
+      </c>
+      <c r="K20" s="5" t="n">
+        <v>776</v>
+      </c>
+      <c r="L20" s="8" t="n">
         <v>13310</v>
       </c>
-      <c r="K20" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" s="8" t="n">
+      <c r="M20" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="8" t="n">
         <f aca="false">p_Slot</f>
         <v>35000</v>
       </c>
-      <c r="M20" s="6" t="n">
-        <v>2028</v>
-      </c>
-      <c r="N20" s="5" t="n">
-        <v>776</v>
-      </c>
       <c r="O20" s="5" t="n">
         <v>630901</v>
       </c>
@@ -1785,22 +1778,22 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B21" s="5" t="n">
         <v>7205047</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G21" s="6" t="n">
         <v>2026</v>
@@ -1809,22 +1802,22 @@
         <v>8</v>
       </c>
       <c r="I21" s="8"/>
-      <c r="J21" s="8" t="n">
+      <c r="J21" s="6" t="n">
+        <v>2028</v>
+      </c>
+      <c r="K21" s="5" t="n">
+        <v>647</v>
+      </c>
+      <c r="L21" s="8" t="n">
         <v>11000</v>
       </c>
-      <c r="K21" s="8" t="n">
+      <c r="M21" s="8" t="n">
         <v>3420</v>
       </c>
-      <c r="L21" s="8" t="n">
+      <c r="N21" s="8" t="n">
         <f aca="false">p_Slot</f>
         <v>35000</v>
       </c>
-      <c r="M21" s="6" t="n">
-        <v>2028</v>
-      </c>
-      <c r="N21" s="5" t="n">
-        <v>647</v>
-      </c>
       <c r="O21" s="5" t="n">
         <v>604901</v>
       </c>
@@ -1834,16 +1827,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B22" s="5" t="n">
         <v>7205027</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>21</v>
@@ -1858,34 +1851,34 @@
       <c r="I22" s="8" t="n">
         <v>121968</v>
       </c>
-      <c r="J22" s="8"/>
-      <c r="K22" s="8"/>
+      <c r="J22" s="6"/>
+      <c r="K22" s="5" t="n">
+        <v>458</v>
+      </c>
       <c r="L22" s="8"/>
-      <c r="M22" s="6"/>
-      <c r="N22" s="5" t="n">
-        <v>458</v>
-      </c>
+      <c r="M22" s="8"/>
+      <c r="N22" s="8"/>
       <c r="O22" s="5"/>
       <c r="P22" s="8"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B23" s="5" t="n">
         <v>7205057</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G23" s="6" t="n">
         <v>2012</v>
@@ -1896,32 +1889,32 @@
       <c r="I23" s="8" t="n">
         <v>80000</v>
       </c>
-      <c r="J23" s="8"/>
-      <c r="K23" s="8"/>
+      <c r="J23" s="6"/>
+      <c r="K23" s="5" t="n">
+        <v>823</v>
+      </c>
       <c r="L23" s="8"/>
-      <c r="M23" s="6"/>
-      <c r="N23" s="5" t="n">
-        <v>823</v>
-      </c>
+      <c r="M23" s="8"/>
+      <c r="N23" s="8"/>
       <c r="O23" s="5"/>
       <c r="P23" s="8"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B24" s="5"/>
       <c r="C24" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G24" s="6" t="n">
         <v>2009</v>
@@ -1932,32 +1925,32 @@
       <c r="I24" s="8" t="n">
         <v>100000</v>
       </c>
-      <c r="J24" s="8"/>
-      <c r="K24" s="8"/>
+      <c r="J24" s="6"/>
+      <c r="K24" s="5"/>
       <c r="L24" s="8"/>
-      <c r="M24" s="6"/>
-      <c r="N24" s="5"/>
+      <c r="M24" s="8"/>
+      <c r="N24" s="8"/>
       <c r="O24" s="5"/>
       <c r="P24" s="8"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B25" s="5" t="n">
         <v>7205041</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G25" s="6" t="n">
         <v>2024</v>
@@ -1968,32 +1961,32 @@
       <c r="I25" s="8" t="n">
         <v>51100</v>
       </c>
-      <c r="J25" s="8"/>
-      <c r="K25" s="8"/>
+      <c r="J25" s="6"/>
+      <c r="K25" s="5" t="n">
+        <v>518</v>
+      </c>
       <c r="L25" s="8"/>
-      <c r="M25" s="6"/>
-      <c r="N25" s="5" t="n">
-        <v>518</v>
-      </c>
+      <c r="M25" s="8"/>
+      <c r="N25" s="8"/>
       <c r="O25" s="5"/>
       <c r="P25" s="8"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B26" s="5"/>
       <c r="C26" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E26" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G26" s="6" t="n">
         <v>2023</v>
@@ -2004,32 +1997,32 @@
       <c r="I26" s="8" t="n">
         <v>19000</v>
       </c>
-      <c r="J26" s="8"/>
-      <c r="K26" s="8"/>
+      <c r="J26" s="6"/>
+      <c r="K26" s="5"/>
       <c r="L26" s="8"/>
-      <c r="M26" s="6"/>
-      <c r="N26" s="5"/>
+      <c r="M26" s="8"/>
+      <c r="N26" s="8"/>
       <c r="O26" s="5"/>
       <c r="P26" s="8"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B27" s="5" t="n">
         <v>7205056</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G27" s="6" t="n">
         <v>2007</v>
@@ -2040,32 +2033,32 @@
       <c r="I27" s="8" t="n">
         <v>50000</v>
       </c>
-      <c r="J27" s="8"/>
-      <c r="K27" s="8"/>
+      <c r="J27" s="6"/>
+      <c r="K27" s="5"/>
       <c r="L27" s="8"/>
-      <c r="M27" s="6"/>
-      <c r="N27" s="5"/>
+      <c r="M27" s="8"/>
+      <c r="N27" s="8"/>
       <c r="O27" s="5"/>
       <c r="P27" s="8"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B28" s="5" t="n">
         <v>7205054</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G28" s="6" t="n">
         <v>2017</v>
@@ -2076,32 +2069,32 @@
       <c r="I28" s="8" t="n">
         <v>45000</v>
       </c>
-      <c r="J28" s="8"/>
-      <c r="K28" s="8"/>
+      <c r="J28" s="6"/>
+      <c r="K28" s="5"/>
       <c r="L28" s="8"/>
-      <c r="M28" s="6"/>
-      <c r="N28" s="5"/>
+      <c r="M28" s="8"/>
+      <c r="N28" s="8"/>
       <c r="O28" s="5"/>
       <c r="P28" s="8"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B29" s="5" t="n">
         <v>7205055</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G29" s="6" t="n">
         <v>2017</v>
@@ -2112,30 +2105,30 @@
       <c r="I29" s="8" t="n">
         <v>45000</v>
       </c>
-      <c r="J29" s="8"/>
-      <c r="K29" s="8"/>
+      <c r="J29" s="6"/>
+      <c r="K29" s="5"/>
       <c r="L29" s="8"/>
-      <c r="M29" s="6"/>
-      <c r="N29" s="5"/>
+      <c r="M29" s="8"/>
+      <c r="N29" s="8"/>
       <c r="O29" s="5"/>
       <c r="P29" s="8"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B30" s="5"/>
       <c r="C30" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G30" s="6" t="n">
         <v>2026</v>
@@ -2144,43 +2137,43 @@
         <v>8</v>
       </c>
       <c r="I30" s="8"/>
-      <c r="J30" s="8" t="n">
+      <c r="J30" s="6" t="n">
+        <v>2028</v>
+      </c>
+      <c r="K30" s="5"/>
+      <c r="L30" s="8" t="n">
         <f aca="false">p_Aanbet</f>
         <v>10000</v>
       </c>
-      <c r="K30" s="8" t="n">
+      <c r="M30" s="8" t="n">
         <f aca="false">p_Belet+p_Opbouw</f>
         <v>12000</v>
       </c>
-      <c r="L30" s="8" t="n">
+      <c r="N30" s="8" t="n">
         <f aca="false">p_Slot</f>
         <v>35000</v>
       </c>
-      <c r="M30" s="6" t="n">
-        <v>2028</v>
-      </c>
-      <c r="N30" s="5"/>
       <c r="O30" s="5"/>
       <c r="P30" s="8"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B31" s="5" t="n">
         <v>7205036</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E31" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G31" s="6" t="n">
         <v>2023</v>
@@ -2191,60 +2184,60 @@
       <c r="I31" s="8" t="n">
         <v>41530</v>
       </c>
-      <c r="J31" s="8"/>
-      <c r="K31" s="8"/>
+      <c r="J31" s="6"/>
+      <c r="K31" s="5" t="n">
+        <v>631</v>
+      </c>
       <c r="L31" s="8"/>
-      <c r="M31" s="6"/>
-      <c r="N31" s="5" t="n">
-        <v>631</v>
-      </c>
+      <c r="M31" s="8"/>
+      <c r="N31" s="8"/>
       <c r="O31" s="5"/>
       <c r="P31" s="8"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H33" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I33" s="10" t="n">
         <f aca="false">SUBTOTAL(109,I5:I31)</f>
         <v>1608161</v>
       </c>
-      <c r="J33" s="10" t="n">
-        <f aca="false">SUBTOTAL(109,J5:J31)</f>
-        <v>78310</v>
-      </c>
-      <c r="K33" s="10" t="n">
-        <f aca="false">SUBTOTAL(109,K5:K31)</f>
-        <v>22260</v>
-      </c>
       <c r="L33" s="10" t="n">
         <f aca="false">SUBTOTAL(109,L5:L31)</f>
+        <v>78310</v>
+      </c>
+      <c r="M33" s="10" t="n">
+        <f aca="false">SUBTOTAL(109,M5:M31)</f>
+        <v>22260</v>
+      </c>
+      <c r="N33" s="10" t="n">
+        <f aca="false">SUBTOTAL(109,N5:N31)</f>
         <v>245000</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="J3:M3"/>
+    <mergeCell ref="L3:N3"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2282,17 +2275,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C4" s="12" t="n">
         <v>10000</v>
@@ -2300,7 +2293,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C5" s="12" t="n">
         <v>5000</v>
@@ -2308,7 +2301,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C6" s="12" t="n">
         <v>7000</v>
@@ -2316,7 +2309,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C7" s="12" t="n">
         <v>35000</v>
@@ -2324,7 +2317,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>2</v>
@@ -2332,7 +2325,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>8</v>
@@ -2340,7 +2333,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>6</v>
@@ -2348,7 +2341,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C11" s="12" t="n">
         <v>12000</v>
@@ -2356,7 +2349,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F13" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -2370,13 +2363,13 @@
         <v>5</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F14" s="14" t="n">
         <v>2027</v>
@@ -2394,30 +2387,30 @@
         <v>2030</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="N14" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="O14" s="3" t="s">
         <v>16</v>
       </c>
       <c r="P14" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B15" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A15,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -2474,7 +2467,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B16" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A16,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -2531,11 +2524,11 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B17" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A17,'In gebruik'!$A:$A,0))&amp;"","")</f>
-        <v>Speelt/groen</v>
+        <v>Speeltoestellen / groen</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>1</v>
@@ -2588,7 +2581,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B18" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A18,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -2644,11 +2637,11 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B19" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A19,'In gebruik'!$A:$A,0))&amp;"","")</f>
-        <v>Algemeen</v>
+        <v>Algemeen (dienstauto)</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>1</v>
@@ -2701,7 +2694,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B20" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A20,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -2758,11 +2751,11 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B21" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A21,'In gebruik'!$A:$A,0))&amp;"","")</f>
-        <v>Werf</v>
+        <v>Gemeentewerf</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>21</v>
@@ -2811,12 +2804,12 @@
         <v/>
       </c>
       <c r="P21" s="4" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B22" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A22,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -2873,7 +2866,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B23" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A23,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -2929,7 +2922,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B24" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A24,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -2990,7 +2983,7 @@
       </c>
       <c r="B25" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A25,'In gebruik'!$A:$A,0))&amp;"","")</f>
-        <v>Vrachtwagen</v>
+        <v>Openbare ruimte</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>21</v>
@@ -3046,10 +3039,10 @@
       </c>
       <c r="B26" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A26,'In gebruik'!$A:$A,0))&amp;"","")</f>
-        <v>Vrachtwagen</v>
+        <v>Gladheidsbestrijding</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D26" s="6" t="n">
         <v>2032</v>
@@ -3093,16 +3086,16 @@
         <v/>
       </c>
       <c r="P26" s="4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B27" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A27,'In gebruik'!$A:$A,0))&amp;"","")</f>
-        <v>Stratenmakers</v>
+        <v>Openbare ruimte (straatwerk)</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>1</v>
@@ -3155,7 +3148,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B28" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A28,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3212,7 +3205,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B29" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A29,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3269,7 +3262,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B30" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A30,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3326,11 +3319,11 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B31" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A31,'In gebruik'!$A:$A,0))&amp;"","")</f>
-        <v>Werf</v>
+        <v>Gemeentewerf</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>21</v>
@@ -3382,7 +3375,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B32" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A32,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3439,11 +3432,11 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B33" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A33,'In gebruik'!$A:$A,0))&amp;"","")</f>
-        <v>Stratenmakers</v>
+        <v>Openbare ruimte (straatwerk)</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>1</v>
@@ -3496,7 +3489,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B34" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A34,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3553,7 +3546,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B35" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A35,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3610,7 +3603,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B36" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A36,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3667,11 +3660,11 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B37" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A37,'In gebruik'!$A:$A,0))&amp;"","")</f>
-        <v>Timmerman</v>
+        <v>Gebouwen (timmerman)</v>
       </c>
       <c r="C37" s="5" t="s">
         <v>1</v>
@@ -3724,7 +3717,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B38" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A38,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3780,7 +3773,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B39" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A39,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3841,7 +3834,7 @@
       </c>
       <c r="B40" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A40,'In gebruik'!$A:$A,0))&amp;"","")</f>
-        <v>Rioolvoertuig</v>
+        <v>Riolering</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>21</v>
@@ -3893,7 +3886,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B41" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A41,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3949,7 +3942,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="17" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B42" s="18"/>
       <c r="C42" s="18"/>
@@ -3984,27 +3977,27 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="11" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="11" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -4047,7 +4040,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4067,22 +4060,22 @@
         <v>8</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>2014</v>
@@ -4094,14 +4087,14 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E6" s="6" t="n">
         <v>2018</v>
@@ -4113,14 +4106,14 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>2013</v>
@@ -4132,16 +4125,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B8" s="5" t="n">
         <v>7205049</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>2017</v>
@@ -4153,14 +4146,14 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>2007</v>
@@ -4172,14 +4165,14 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>144</v>
+        <v>37</v>
       </c>
       <c r="E10" s="6" t="n">
         <v>2006</v>
@@ -4217,7 +4210,7 @@
         <v>151</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>152</v>
+        <v>67</v>
       </c>
       <c r="E12" s="6" t="n">
         <v>2013</v>
@@ -4229,14 +4222,14 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E13" s="6" t="n">
         <v>2013</v>
@@ -4248,14 +4241,14 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B14" s="5"/>
       <c r="C14" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>2013</v>
@@ -4267,26 +4260,26 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>159</v>
+        <v>45</v>
       </c>
       <c r="E15" s="6" t="n">
         <v>2013</v>
       </c>
       <c r="F15" s="19"/>
       <c r="G15" s="5" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Wagenpark_beheer.xlsx: V01 gebruiksdoel gladheidsbestrijding
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013EaFTgzjMaNvZvWgFM9YZf
</commit_message>
<xml_diff>
--- a/Wagenpark_beheer.xlsx
+++ b/Wagenpark_beheer.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="159">
   <si>
     <t xml:space="preserve">Voertuigen in gebruik</t>
   </si>
@@ -95,7 +95,7 @@
     <t xml:space="preserve">26-BXG-9</t>
   </si>
   <si>
-    <t xml:space="preserve">Openbare ruimte</t>
+    <t xml:space="preserve">Gladheidsbestrijding</t>
   </si>
   <si>
     <t xml:space="preserve">Koop</t>
@@ -120,9 +120,6 @@
   </si>
   <si>
     <t xml:space="preserve">BZ-TZ-45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gladheidsbestrijding</t>
   </si>
   <si>
     <t xml:space="preserve">STROOIEN</t>
@@ -1220,13 +1217,13 @@
         <v>28</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G7" s="6" t="n">
         <v>2012</v>
@@ -1243,22 +1240,22 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B8" s="5" t="n">
         <v>7205035</v>
       </c>
       <c r="C8" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>32</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>33</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G8" s="6" t="n">
         <v>2024</v>
@@ -1281,22 +1278,22 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B9" s="5" t="n">
         <v>7205053</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>37</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G9" s="6" t="n">
         <v>2021</v>
@@ -1317,22 +1314,22 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B10" s="5" t="n">
         <v>7205045</v>
       </c>
       <c r="C10" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>41</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G10" s="6" t="n">
         <v>2026</v>
@@ -1364,22 +1361,22 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B11" s="5" t="n">
         <v>7205051</v>
       </c>
       <c r="C11" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>44</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>45</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G11" s="6" t="n">
         <v>2013</v>
@@ -1402,22 +1399,22 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>7205048</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G12" s="6" t="n">
         <v>2026</v>
@@ -1451,22 +1448,22 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B13" s="5" t="n">
         <v>7205039</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G13" s="6" t="n">
         <v>2024</v>
@@ -1489,22 +1486,22 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B14" s="5" t="n">
         <v>7205043</v>
       </c>
       <c r="C14" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>54</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>55</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G14" s="6" t="n">
         <v>2025</v>
@@ -1527,20 +1524,20 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B15" s="5" t="n">
         <v>7205046</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G15" s="6" t="n">
         <v>2026</v>
@@ -1572,22 +1569,22 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B16" s="5" t="n">
         <v>7205044</v>
       </c>
       <c r="C16" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>59</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>60</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G16" s="6" t="n">
         <v>2024</v>
@@ -1610,22 +1607,22 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B17" s="5" t="n">
         <v>7205052</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G17" s="6" t="n">
         <v>2017</v>
@@ -1648,22 +1645,22 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B18" s="5" t="n">
         <v>7205058</v>
       </c>
       <c r="C18" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>66</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>67</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G18" s="6" t="n">
         <v>2018</v>
@@ -1684,20 +1681,20 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B19" s="5" t="n">
         <v>7205033</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G19" s="6" t="n">
         <v>2026</v>
@@ -1731,20 +1728,20 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B20" s="5" t="n">
         <v>7205032</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G20" s="6" t="n">
         <v>2026</v>
@@ -1778,22 +1775,22 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B21" s="5" t="n">
         <v>7205047</v>
       </c>
       <c r="C21" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D21" s="4" t="s">
         <v>76</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>77</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G21" s="6" t="n">
         <v>2026</v>
@@ -1827,16 +1824,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B22" s="5" t="n">
         <v>7205027</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>21</v>
@@ -1863,22 +1860,22 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B23" s="5" t="n">
         <v>7205057</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G23" s="6" t="n">
         <v>2012</v>
@@ -1901,20 +1898,20 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B24" s="5"/>
       <c r="C24" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G24" s="6" t="n">
         <v>2009</v>
@@ -1935,22 +1932,22 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B25" s="5" t="n">
         <v>7205041</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G25" s="6" t="n">
         <v>2024</v>
@@ -1973,20 +1970,20 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B26" s="5"/>
       <c r="C26" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>89</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>90</v>
       </c>
       <c r="E26" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G26" s="6" t="n">
         <v>2023</v>
@@ -2007,22 +2004,22 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B27" s="5" t="n">
         <v>7205056</v>
       </c>
       <c r="C27" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="D27" s="4" t="s">
         <v>89</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>90</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G27" s="6" t="n">
         <v>2007</v>
@@ -2043,22 +2040,22 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B28" s="5" t="n">
         <v>7205054</v>
       </c>
       <c r="C28" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D28" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>94</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G28" s="6" t="n">
         <v>2017</v>
@@ -2079,22 +2076,22 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B29" s="5" t="n">
         <v>7205055</v>
       </c>
       <c r="C29" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D29" s="4" t="s">
         <v>97</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>98</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G29" s="6" t="n">
         <v>2017</v>
@@ -2115,20 +2112,20 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B30" s="5"/>
       <c r="C30" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D30" s="4" t="s">
         <v>100</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>101</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G30" s="6" t="n">
         <v>2026</v>
@@ -2158,22 +2155,22 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B31" s="5" t="n">
         <v>7205036</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E31" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G31" s="6" t="n">
         <v>2023</v>
@@ -2196,7 +2193,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H33" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I33" s="10" t="n">
         <f aca="false">SUBTOTAL(109,I5:I31)</f>
@@ -2217,22 +2214,22 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -2275,17 +2272,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C4" s="12" t="n">
         <v>10000</v>
@@ -2293,7 +2290,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C5" s="12" t="n">
         <v>5000</v>
@@ -2301,7 +2298,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C6" s="12" t="n">
         <v>7000</v>
@@ -2309,7 +2306,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C7" s="12" t="n">
         <v>35000</v>
@@ -2317,7 +2314,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>2</v>
@@ -2325,7 +2322,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>8</v>
@@ -2333,7 +2330,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>6</v>
@@ -2341,7 +2338,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C11" s="12" t="n">
         <v>12000</v>
@@ -2349,7 +2346,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F13" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -2363,13 +2360,13 @@
         <v>5</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F14" s="14" t="n">
         <v>2027</v>
@@ -2387,30 +2384,30 @@
         <v>2030</v>
       </c>
       <c r="J14" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="K14" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="K14" s="3" t="s">
+      <c r="L14" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="L14" s="3" t="s">
+      <c r="M14" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="M14" s="3" t="s">
-        <v>126</v>
-      </c>
       <c r="N14" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="O14" s="3" t="s">
         <v>16</v>
       </c>
       <c r="P14" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B15" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A15,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -2467,7 +2464,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B16" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A16,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -2524,7 +2521,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B17" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A17,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -2581,7 +2578,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B18" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A18,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -2637,7 +2634,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B19" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A19,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -2694,7 +2691,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B20" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A20,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -2751,7 +2748,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B21" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A21,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -2804,12 +2801,12 @@
         <v/>
       </c>
       <c r="P21" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B22" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A22,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -2866,7 +2863,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B23" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A23,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -2922,7 +2919,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B24" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A24,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -2983,7 +2980,7 @@
       </c>
       <c r="B25" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A25,'In gebruik'!$A:$A,0))&amp;"","")</f>
-        <v>Openbare ruimte</v>
+        <v>Gladheidsbestrijding</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>21</v>
@@ -3042,7 +3039,7 @@
         <v>Gladheidsbestrijding</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D26" s="6" t="n">
         <v>2032</v>
@@ -3086,12 +3083,12 @@
         <v/>
       </c>
       <c r="P26" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B27" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A27,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3148,7 +3145,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B28" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A28,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3205,7 +3202,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B29" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A29,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3262,7 +3259,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B30" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A30,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3319,7 +3316,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B31" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A31,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3375,7 +3372,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B32" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A32,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3432,7 +3429,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B33" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A33,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3489,7 +3486,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B34" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A34,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3546,7 +3543,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B35" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A35,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3603,7 +3600,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B36" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A36,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3660,7 +3657,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B37" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A37,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3717,7 +3714,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B38" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A38,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3773,7 +3770,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B39" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A39,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3886,7 +3883,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B41" s="4" t="str">
         <f aca="false">IFERROR(INDEX('In gebruik'!$D:$D,MATCH($A41,'In gebruik'!$A:$A,0))&amp;"","")</f>
@@ -3942,7 +3939,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="17" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B42" s="18"/>
       <c r="C42" s="18"/>
@@ -3977,27 +3974,27 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="11" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -4040,7 +4037,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4060,7 +4057,7 @@
         <v>8</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>12</v>
@@ -4068,14 +4065,14 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>2014</v>
@@ -4087,14 +4084,14 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E6" s="6" t="n">
         <v>2018</v>
@@ -4106,14 +4103,14 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>2013</v>
@@ -4125,16 +4122,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B8" s="5" t="n">
         <v>7205049</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>2017</v>
@@ -4146,14 +4143,14 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>2007</v>
@@ -4165,52 +4162,52 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E10" s="6" t="n">
         <v>2006</v>
       </c>
       <c r="F10" s="19"/>
       <c r="G10" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>147</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>148</v>
       </c>
       <c r="E11" s="6" t="n">
         <v>2015</v>
       </c>
       <c r="F11" s="19"/>
       <c r="G11" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E12" s="6" t="n">
         <v>2013</v>
@@ -4222,14 +4219,14 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E13" s="6" t="n">
         <v>2013</v>
@@ -4241,14 +4238,14 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B14" s="5"/>
       <c r="C14" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>2013</v>
@@ -4260,26 +4257,26 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E15" s="6" t="n">
         <v>2013</v>
       </c>
       <c r="F15" s="19"/>
       <c r="G15" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Wagenpark_beheer.xlsx: zachte invulkleur en controleblok op dashboard
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013EaFTgzjMaNvZvWgFM9YZf
</commit_message>
<xml_diff>
--- a/Wagenpark_beheer.xlsx
+++ b/Wagenpark_beheer.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="235">
   <si>
     <t xml:space="preserve">Dashboard wagenpark</t>
   </si>
@@ -111,6 +111,51 @@
     <t xml:space="preserve">Investeringen volgend jaar</t>
   </si>
   <si>
+    <t xml:space="preserve">Controle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aantal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jaarovergang bijgewerkt (lopend jaar = huidig jaar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In gebruik: kenteken ontbreekt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In gebruik: kredietnummer ontbreekt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In gebruik: activakaart ontbreekt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In gebruik: aanschafkosten ontbreken (koop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In gebruik: lease-koop bedragen ontbreken</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In gebruik: levensduur verstreken</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In gebruik: V-nummer dubbel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Te vervangen dit jaar: nog niet bevestigd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vervangingsinvesteringen: activanummer ontbreekt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vervangingsinvesteringen: koopprijs ontbreekt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buiten gebruik: datum/jaar ontbreekt</t>
+  </si>
+  <si>
     <t xml:space="preserve">Werkwijze</t>
   </si>
   <si>
@@ -181,9 +226,6 @@
   </si>
   <si>
     <t xml:space="preserve">Leasesom 1 jaar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status</t>
   </si>
   <si>
     <t xml:space="preserve">V01-01</t>
@@ -794,13 +836,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDDEBF7"/>
-        <bgColor rgb="FFCCFFFF"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
     <fill>
@@ -942,7 +984,21 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="6">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -968,15 +1024,8 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
+          <fgColor rgb="FFE2EFDA"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1018,7 +1067,7 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFE2EFDA"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
@@ -1237,7 +1286,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:H30"/>
+  <dimension ref="B1:H44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -1376,38 +1425,213 @@
       <c r="B24" s="3" t="s">
         <v>21</v>
       </c>
+      <c r="C24" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="5" t="s">
-        <v>22</v>
+      <c r="B25" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C25" s="9" t="n">
+        <f aca="true">IF(LopendJaar=YEAR(TODAY()),0,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D25" s="8" t="str">
+        <f aca="false">IF(C25=0,"OK","Actie")</f>
+        <v>OK</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="5" t="s">
-        <v>23</v>
+      <c r="B26" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C26" s="9" t="n">
+        <f aca="false">COUNTIFS('Voertuigen 2026'!$Q$5:$Q$300,"In gebruik",'Voertuigen 2026'!$C$5:$C$300,"")+COUNTIFS('Voertuigen 2026'!$Q$5:$Q$300,"In gebruik",'Voertuigen 2026'!$C$5:$C$300,"n.n.b.")</f>
+        <v>3</v>
+      </c>
+      <c r="D26" s="8" t="str">
+        <f aca="false">IF(C26=0,"OK","Actie")</f>
+        <v>Actie</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="5" t="s">
-        <v>24</v>
+      <c r="B27" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C27" s="9" t="n">
+        <f aca="false">COUNTIFS('Voertuigen 2026'!$Q$5:$Q$300,"In gebruik",'Voertuigen 2026'!$B$5:$B$300,"")+COUNTIFS('Voertuigen 2026'!$Q$5:$Q$300,"In gebruik",'Voertuigen 2026'!$B$5:$B$300,"n.n.b.")</f>
+        <v>4</v>
+      </c>
+      <c r="D27" s="8" t="str">
+        <f aca="false">IF(C27=0,"OK","Actie")</f>
+        <v>Actie</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="5" t="s">
-        <v>25</v>
+      <c r="B28" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28" s="9" t="n">
+        <f aca="false">COUNTIFS('Voertuigen 2026'!$Q$5:$Q$300,"In gebruik",'Voertuigen 2026'!$K$5:$K$300,"")+COUNTIFS('Voertuigen 2026'!$Q$5:$Q$300,"In gebruik",'Voertuigen 2026'!$K$5:$K$300,"n.n.b.")</f>
+        <v>11</v>
+      </c>
+      <c r="D28" s="8" t="str">
+        <f aca="false">IF(C28=0,"OK","Actie")</f>
+        <v>Actie</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C29" s="9" t="n">
+        <f aca="false">COUNTIFS('Voertuigen 2026'!$Q$5:$Q$300,"In gebruik",'Voertuigen 2026'!$E$5:$E$300,"Koop",'Voertuigen 2026'!$I$5:$I$300,"")</f>
+        <v>1</v>
+      </c>
+      <c r="D29" s="8" t="str">
+        <f aca="false">IF(C29=0,"OK","Actie")</f>
+        <v>Actie</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C30" s="9" t="n">
+        <f aca="false">COUNTIFS('Voertuigen 2026'!$Q$5:$Q$300,"In gebruik",'Voertuigen 2026'!$E$5:$E$300,"Lease-koop",'Voertuigen 2026'!$L$5:$L$300,"")+COUNTIFS('Voertuigen 2026'!$Q$5:$Q$300,"In gebruik",'Voertuigen 2026'!$E$5:$E$300,"Lease-koop",'Voertuigen 2026'!$N$5:$N$300,"")</f>
+        <v>0</v>
+      </c>
+      <c r="D30" s="8" t="str">
+        <f aca="false">IF(C30=0,"OK","Actie")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C31" s="9" t="n">
+        <f aca="false">SUMPRODUCT(('Voertuigen 2026'!$Q$5:$Q$300="In gebruik")*('Voertuigen 2026'!$H$5:$H$300&gt;0)*('Voertuigen 2026'!$G$5:$G$300+'Voertuigen 2026'!$H$5:$H$300&lt;=LopendJaar))</f>
+        <v>6</v>
+      </c>
+      <c r="D31" s="8" t="str">
+        <f aca="false">IF(C31=0,"OK","Actie")</f>
+        <v>Actie</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C32" s="9" t="n">
+        <f aca="false">SUMPRODUCT(('Voertuigen 2026'!$Q$5:$Q$300="In gebruik")*(COUNTIFS('Voertuigen 2026'!$A$5:$A$300,'Voertuigen 2026'!$A$5:$A$300,'Voertuigen 2026'!$Q$5:$Q$300,"In gebruik")&gt;1))</f>
+        <v>0</v>
+      </c>
+      <c r="D32" s="8" t="str">
+        <f aca="false">IF(C32=0,"OK","Actie")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C33" s="9" t="n">
+        <f aca="false">COUNTIF('Voertuigen 2026'!$Q$5:$Q$300,"Te vervangen*")</f>
+        <v>0</v>
+      </c>
+      <c r="D33" s="8" t="str">
+        <f aca="false">IF(C33=0,"OK","Actie")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C34" s="9" t="n">
+        <f aca="false">COUNTIFS(Vervangingsinvesteringen!$A$5:$A$300,"V*",Vervangingsinvesteringen!$C$5:$C$300,"&lt;&gt;Doorschuiven",Vervangingsinvesteringen!$K$5:$K$300,"")</f>
         <v>26</v>
       </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="5" t="s">
-        <v>27</v>
+      <c r="D34" s="8" t="str">
+        <f aca="false">IF(C34=0,"OK","Actie")</f>
+        <v>Actie</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C35" s="9" t="n">
+        <f aca="false">COUNTIFS(Vervangingsinvesteringen!$C$5:$C$300,"Koop",Vervangingsinvesteringen!$L$5:$L$300,"")</f>
+        <v>0</v>
+      </c>
+      <c r="D35" s="8" t="str">
+        <f aca="false">IF(C35=0,"OK","Actie")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C36" s="9" t="n">
+        <f aca="false">COUNTIFS('Buiten gebruik'!$A$5:$A$300,"V*",'Buiten gebruik'!$F$5:$F$300,"")</f>
+        <v>3</v>
+      </c>
+      <c r="D36" s="8" t="str">
+        <f aca="false">IF(C36=0,"OK","Actie")</f>
+        <v>Actie</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B39" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B42" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B43" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B44" s="5" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="D25:D36">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>D25="OK"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>D25="Actie"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C7" type="list">
       <formula1>$H$2:$H$60</formula1>
@@ -1450,80 +1674,80 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="K4" s="11" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="L4" s="11" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="N4" s="11" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="O4" s="11" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="P4" s="11" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="Q4" s="11" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>7205037</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="G5" s="12" t="n">
         <v>2024</v>
@@ -1544,27 +1768,27 @@
       <c r="O5" s="8"/>
       <c r="P5" s="13"/>
       <c r="Q5" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>7205034</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="G6" s="12" t="n">
         <v>2023</v>
@@ -1585,25 +1809,25 @@
       <c r="O6" s="8"/>
       <c r="P6" s="13"/>
       <c r="Q6" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G7" s="12" t="n">
         <v>2012</v>
@@ -1618,27 +1842,27 @@
       <c r="O7" s="8"/>
       <c r="P7" s="13"/>
       <c r="Q7" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>7205035</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="G8" s="12" t="n">
         <v>2024</v>
@@ -1659,27 +1883,27 @@
       <c r="O8" s="8"/>
       <c r="P8" s="13"/>
       <c r="Q8" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>63</v>
+        <v>77</v>
       </c>
       <c r="B9" s="8" t="n">
         <v>7205053</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="G9" s="12" t="n">
         <v>2021</v>
@@ -1698,27 +1922,27 @@
       <c r="O9" s="8"/>
       <c r="P9" s="13"/>
       <c r="Q9" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>7205045</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="G10" s="12" t="n">
         <v>2026</v>
@@ -1748,27 +1972,27 @@
         <v>11786.52</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="B11" s="8" t="n">
         <v>7205051</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="G11" s="12" t="n">
         <v>2013</v>
@@ -1789,27 +2013,27 @@
       <c r="O11" s="8"/>
       <c r="P11" s="13"/>
       <c r="Q11" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="B12" s="8" t="n">
         <v>7205048</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="G12" s="12" t="n">
         <v>2026</v>
@@ -1841,27 +2065,27 @@
         <v>11786.52</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="B13" s="8" t="n">
         <v>7205039</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="G13" s="12" t="n">
         <v>2024</v>
@@ -1882,27 +2106,27 @@
       <c r="O13" s="8"/>
       <c r="P13" s="13"/>
       <c r="Q13" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>7205043</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="G14" s="12" t="n">
         <v>2025</v>
@@ -1923,25 +2147,25 @@
       <c r="O14" s="8"/>
       <c r="P14" s="13"/>
       <c r="Q14" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="B15" s="8" t="n">
         <v>7205046</v>
       </c>
       <c r="C15" s="8"/>
       <c r="D15" s="2" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="G15" s="12" t="n">
         <v>2026</v>
@@ -1971,27 +2195,27 @@
         <v>13448.5289256198</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="B16" s="8" t="n">
         <v>7205044</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="G16" s="12" t="n">
         <v>2024</v>
@@ -2012,27 +2236,27 @@
       <c r="O16" s="8"/>
       <c r="P16" s="13"/>
       <c r="Q16" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="B17" s="8" t="n">
         <v>7205052</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="G17" s="12" t="n">
         <v>2017</v>
@@ -2053,27 +2277,27 @@
       <c r="O17" s="8"/>
       <c r="P17" s="13"/>
       <c r="Q17" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>7205058</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="G18" s="12" t="n">
         <v>2018</v>
@@ -2092,25 +2316,25 @@
       <c r="O18" s="8"/>
       <c r="P18" s="13"/>
       <c r="Q18" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="B19" s="8" t="n">
         <v>7205033</v>
       </c>
       <c r="C19" s="8"/>
       <c r="D19" s="2" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="G19" s="12" t="n">
         <v>2026</v>
@@ -2142,25 +2366,25 @@
         <v>11641.6859504132</v>
       </c>
       <c r="Q19" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="B20" s="8" t="n">
         <v>7205032</v>
       </c>
       <c r="C20" s="8"/>
       <c r="D20" s="2" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="G20" s="12" t="n">
         <v>2026</v>
@@ -2192,27 +2416,27 @@
         <v>14085.84</v>
       </c>
       <c r="Q20" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="B21" s="8" t="n">
         <v>7205047</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="G21" s="12" t="n">
         <v>2026</v>
@@ -2244,24 +2468,24 @@
         <v>11786.52</v>
       </c>
       <c r="Q21" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="B22" s="8" t="n">
         <v>7205027</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="12" t="n">
@@ -2283,27 +2507,27 @@
       <c r="O22" s="8"/>
       <c r="P22" s="13"/>
       <c r="Q22" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="B23" s="8" t="n">
         <v>7205057</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="G23" s="12" t="n">
         <v>2012</v>
@@ -2324,25 +2548,25 @@
       <c r="O23" s="8"/>
       <c r="P23" s="13"/>
       <c r="Q23" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="8" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="G24" s="12" t="n">
         <v>2009</v>
@@ -2361,27 +2585,27 @@
       <c r="O24" s="8"/>
       <c r="P24" s="13"/>
       <c r="Q24" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="B25" s="8" t="n">
         <v>7205041</v>
       </c>
       <c r="C25" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="D25" s="2" t="s">
-        <v>102</v>
-      </c>
       <c r="E25" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="G25" s="12" t="n">
         <v>2024</v>
@@ -2402,25 +2626,25 @@
       <c r="O25" s="8"/>
       <c r="P25" s="13"/>
       <c r="Q25" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="8" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="G26" s="12" t="n">
         <v>2023</v>
@@ -2439,27 +2663,27 @@
       <c r="O26" s="8"/>
       <c r="P26" s="13"/>
       <c r="Q26" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="B27" s="8" t="n">
         <v>7205056</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="G27" s="12" t="n">
         <v>2007</v>
@@ -2478,27 +2702,27 @@
       <c r="O27" s="8"/>
       <c r="P27" s="13"/>
       <c r="Q27" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="B28" s="8" t="n">
         <v>7205054</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="G28" s="12" t="n">
         <v>2017</v>
@@ -2517,27 +2741,27 @@
       <c r="O28" s="8"/>
       <c r="P28" s="13"/>
       <c r="Q28" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="B29" s="8" t="n">
         <v>7205055</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="G29" s="12" t="n">
         <v>2017</v>
@@ -2556,25 +2780,25 @@
       <c r="O29" s="8"/>
       <c r="P29" s="13"/>
       <c r="Q29" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="8" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="G30" s="12" t="n">
         <v>2026</v>
@@ -2602,27 +2826,27 @@
       <c r="O30" s="8"/>
       <c r="P30" s="13"/>
       <c r="Q30" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="B31" s="8" t="n">
         <v>7205036</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="G31" s="12" t="n">
         <v>2023</v>
@@ -2643,12 +2867,12 @@
       <c r="O31" s="8"/>
       <c r="P31" s="13"/>
       <c r="Q31" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
       <c r="I33" s="14" t="n">
         <f aca="false">SUMIF($Q$5:$Q$31,"In gebruik",I5:I31)</f>
@@ -2669,7 +2893,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="I34" s="14" t="n">
         <f aca="false">SUMIF($Q$5:$Q$31,"Te vervangen*",I5:I31)</f>
@@ -2690,28 +2914,28 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q31"/>
   <conditionalFormatting sqref="A5:Q500">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>LEFT($Q5,12)="Te vervangen"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2750,24 +2974,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="F4" s="15" t="n">
         <f aca="false">LopendJaar+1</f>
@@ -2786,36 +3010,36 @@
         <v>2030</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>143</v>
+        <v>157</v>
       </c>
       <c r="K4" s="11" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="L4" s="11" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="N4" s="11" t="s">
-        <v>147</v>
+        <v>161</v>
       </c>
       <c r="O4" s="11" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="P4" s="11" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D5" s="12" t="n">
         <v>2027</v>
@@ -2862,13 +3086,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D6" s="12" t="n">
         <v>2027</v>
@@ -2915,13 +3139,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D7" s="12" t="n">
         <v>2027</v>
@@ -2968,13 +3192,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="D8" s="12" t="n">
         <v>2027</v>
@@ -3019,13 +3243,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D9" s="12" t="n">
         <v>2027</v>
@@ -3072,13 +3296,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D10" s="12" t="n">
         <v>2027</v>
@@ -3125,13 +3349,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="D11" s="12" t="n">
         <v>2028</v>
@@ -3173,18 +3397,18 @@
       </c>
       <c r="O11" s="8"/>
       <c r="P11" s="2" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D12" s="12" t="n">
         <v>2029</v>
@@ -3231,13 +3455,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>158</v>
+        <v>172</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="D13" s="12" t="n">
         <v>2029</v>
@@ -3282,13 +3506,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>159</v>
+        <v>173</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D14" s="12" t="n">
         <v>2031</v>
@@ -3335,13 +3559,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="D15" s="12" t="n">
         <v>2032</v>
@@ -3386,13 +3610,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
       <c r="D16" s="12" t="n">
         <v>2032</v>
@@ -3430,18 +3654,18 @@
       </c>
       <c r="O16" s="8"/>
       <c r="P16" s="2" t="s">
-        <v>163</v>
+        <v>177</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>164</v>
+        <v>178</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D17" s="12" t="n">
         <v>2032</v>
@@ -3488,13 +3712,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D18" s="12" t="n">
         <v>2032</v>
@@ -3541,13 +3765,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D19" s="12" t="n">
         <v>2032</v>
@@ -3594,13 +3818,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C20" s="8" t="s">
         <v>84</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>70</v>
       </c>
       <c r="D20" s="12" t="n">
         <v>2033</v>
@@ -3647,13 +3871,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="D21" s="12" t="n">
         <v>2033</v>
@@ -3698,13 +3922,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D22" s="12" t="n">
         <v>2034</v>
@@ -3753,13 +3977,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D23" s="12" t="n">
         <v>2034</v>
@@ -3808,13 +4032,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>171</v>
+        <v>185</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D24" s="12" t="n">
         <v>2034</v>
@@ -3863,13 +4087,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D25" s="12" t="n">
         <v>2034</v>
@@ -3918,13 +4142,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D26" s="12" t="n">
         <v>2034</v>
@@ -3973,13 +4197,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>174</v>
+        <v>188</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D27" s="12" t="n">
         <v>2034</v>
@@ -4028,13 +4252,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>175</v>
+        <v>189</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="D28" s="12" t="n">
         <v>2034</v>
@@ -4079,13 +4303,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>176</v>
+        <v>190</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D29" s="12" t="n">
         <v>2034</v>
@@ -4132,13 +4356,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>177</v>
+        <v>191</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="D30" s="12" t="n">
         <v>2035</v>
@@ -4183,13 +4407,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>178</v>
+        <v>192</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="D31" s="12" t="n">
         <v>2038</v>
@@ -4234,7 +4458,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="17" t="s">
-        <v>179</v>
+        <v>193</v>
       </c>
       <c r="B33" s="18"/>
       <c r="C33" s="18"/>
@@ -4269,37 +4493,37 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>180</v>
+        <v>194</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>181</v>
+        <v>195</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>182</v>
+        <v>196</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>183</v>
+        <v>197</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>184</v>
+        <v>198</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
       <c r="C42" s="19" t="n">
         <v>10000</v>
@@ -4307,7 +4531,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>186</v>
+        <v>200</v>
       </c>
       <c r="C43" s="19" t="n">
         <v>5000</v>
@@ -4315,7 +4539,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>187</v>
+        <v>201</v>
       </c>
       <c r="C44" s="19" t="n">
         <v>7000</v>
@@ -4323,7 +4547,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="C45" s="19" t="n">
         <v>35000</v>
@@ -4331,7 +4555,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="C46" s="20" t="n">
         <v>2</v>
@@ -4339,7 +4563,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="C47" s="20" t="n">
         <v>8</v>
@@ -4347,7 +4571,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>191</v>
+        <v>205</v>
       </c>
       <c r="C48" s="20" t="n">
         <v>6</v>
@@ -4355,7 +4579,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>147</v>
+        <v>161</v>
       </c>
       <c r="C49" s="19" t="n">
         <v>12000</v>
@@ -4397,42 +4621,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>192</v>
+        <v>206</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>194</v>
+        <v>208</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="E5" s="12" t="n">
         <v>2014</v>
@@ -4444,14 +4668,14 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>196</v>
+        <v>210</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
-        <v>197</v>
+        <v>211</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="E6" s="12" t="n">
         <v>2018</v>
@@ -4463,14 +4687,14 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
-        <v>199</v>
+        <v>213</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="E7" s="12" t="n">
         <v>2013</v>
@@ -4482,16 +4706,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>200</v>
+        <v>214</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>7205049</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>201</v>
+        <v>215</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="E8" s="12" t="n">
         <v>2017</v>
@@ -4503,14 +4727,14 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
       <c r="B9" s="8"/>
       <c r="C9" s="8" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="E9" s="12" t="n">
         <v>2007</v>
@@ -4522,52 +4746,52 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="8" t="s">
-        <v>205</v>
+        <v>219</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="E10" s="12" t="n">
         <v>2006</v>
       </c>
       <c r="F10" s="21"/>
       <c r="G10" s="8" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>207</v>
+        <v>221</v>
       </c>
       <c r="B11" s="8"/>
       <c r="C11" s="8" t="s">
-        <v>208</v>
+        <v>222</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="E11" s="12" t="n">
         <v>2015</v>
       </c>
       <c r="F11" s="21"/>
       <c r="G11" s="8" t="s">
-        <v>210</v>
+        <v>224</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>211</v>
+        <v>225</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="8" t="s">
-        <v>212</v>
+        <v>226</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="E12" s="12" t="n">
         <v>2013</v>
@@ -4579,14 +4803,14 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>213</v>
+        <v>227</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8" t="s">
-        <v>214</v>
+        <v>228</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="E13" s="12" t="n">
         <v>2013</v>
@@ -4598,14 +4822,14 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>215</v>
+        <v>229</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="8" t="s">
-        <v>216</v>
+        <v>230</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="E14" s="12" t="n">
         <v>2013</v>
@@ -4617,26 +4841,26 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>217</v>
+        <v>231</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8" t="s">
-        <v>218</v>
+        <v>232</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="E15" s="12" t="n">
         <v>2013</v>
       </c>
       <c r="F15" s="21"/>
       <c r="G15" s="8" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>